<commit_message>
chore: tracker - admin comp-invite button as future addon
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E189"/>
+  <dimension ref="A1:E190"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="1" min="1" max="1"/>
@@ -4636,27 +4636,27 @@
     <row r="172">
       <c r="A172" s="27" t="inlineStr">
         <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   16 items</t>
+          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   17 items</t>
         </is>
       </c>
       <c r="B172" s="27" t="inlineStr">
         <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   16 items</t>
+          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   17 items</t>
         </is>
       </c>
       <c r="C172" s="27" t="inlineStr">
         <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   16 items</t>
+          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   17 items</t>
         </is>
       </c>
       <c r="D172" s="27" t="inlineStr">
         <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   16 items</t>
+          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   17 items</t>
         </is>
       </c>
       <c r="E172" s="27" t="inlineStr">
         <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   16 items</t>
+          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   17 items</t>
         </is>
       </c>
     </row>
@@ -4744,314 +4744,314 @@
     <row r="176">
       <c r="A176" s="28" t="inlineStr">
         <is>
-          <t>Mike Perez: account cleanup + re-join link at $150 founding</t>
+          <t>Admin 'Invite comp member' button - form (name, company, email, phone, comp note), creates comp'd account + sends welcome email, note auto-attached to billing view (member + admin); v1 invite flow built without UI, button is the addon</t>
         </is>
       </c>
       <c r="B176" s="28" t="inlineStr">
         <is>
-          <t>After Adam's conversation: clean up Mike's canceled/failed-billing account and send a founding-rate $150 re-join link.</t>
+          <t>Admin UI button/form to invite a complimentary business member: name, company, email, phone, and comp note. Creates the comp'd account, sends the welcome email, and attaches the note to the billing view for both member and admin.</t>
         </is>
       </c>
       <c r="C176" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM conversation first. Then cleanup + founding $150 checkout/re-join link.</t>
+          <t>Addon after v1 invite flow (API/ops path without UI). Build the Invite comp member button + form once the headless invite path exists.</t>
         </is>
       </c>
       <c r="D176" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: conversation first</t>
+          <t>QUEUED</t>
         </is>
       </c>
       <c r="E176" s="28" t="inlineStr">
         <is>
-          <t>Founding $150; conversation first.</t>
+          <t>v1 invite flow built without UI; this button is the future addon.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="28" t="inlineStr">
         <is>
-          <t>Zane Mackey comp_reason entry</t>
+          <t>Mike Perez: account cleanup + re-join link at $150 founding</t>
         </is>
       </c>
       <c r="B177" s="28" t="inlineStr">
         <is>
-          <t>Record a one-phrase comp_reason on Zane Mackey's profile now that the column exists.</t>
+          <t>After Adam's conversation: clean up Mike's canceled/failed-billing account and send a founding-rate $150 re-join link.</t>
         </is>
       </c>
       <c r="C177" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: one phrase for comp_reason.</t>
+          <t>WAITING ON ADAM conversation first. Then cleanup + founding $150 checkout/re-join link.</t>
         </is>
       </c>
       <c r="D177" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: one phrase</t>
+          <t>WAITING ON ADAM: conversation first</t>
         </is>
       </c>
       <c r="E177" s="28" t="inlineStr">
         <is>
-          <t>One phrase for comp_reason.</t>
+          <t>Founding $150; conversation first.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="28" t="inlineStr">
         <is>
-          <t>Zach Trusky renewal ~Nov/Dec 2026 — honored $1,034 annual</t>
+          <t>Zane Mackey comp_reason entry</t>
         </is>
       </c>
       <c r="B178" s="28" t="inlineStr">
         <is>
-          <t>Zach's annual amount lives outside Stripe ($1,034 honored). Need reminder + collection path decision around Nov/Dec 2026.</t>
+          <t>Record a one-phrase comp_reason on Zane Mackey's profile now that the column exists.</t>
         </is>
       </c>
       <c r="C178" s="28" t="inlineStr">
         <is>
-          <t>Schedule reminder; decide collection path (manual invoice vs Stripe annual vs override).</t>
+          <t>WAITING ON ADAM: one phrase for comp_reason.</t>
         </is>
       </c>
       <c r="D178" s="28" t="inlineStr">
         <is>
-          <t>SCHEDULED NOV 2026</t>
+          <t>WAITING ON ADAM: one phrase</t>
         </is>
       </c>
       <c r="E178" s="28" t="inlineStr">
         <is>
-          <t>Honored $1,034 annual; no Stripe customer today.</t>
+          <t>One phrase for comp_reason.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="28" t="inlineStr">
         <is>
-          <t>Security: unknown third-party script (batatatech.com) on Glue Up admin pages</t>
+          <t>Zach Trusky renewal ~Nov/Dec 2026 — honored $1,034 annual</t>
         </is>
       </c>
       <c r="B179" s="28" t="inlineStr">
         <is>
-          <t>Unknown batatatech.com script firing on Glue Up admin pages — treat as extension/malware until proven otherwise; audit browsers + rotate passwords.</t>
+          <t>Zach's annual amount lives outside Stripe ($1,034 honored). Need reminder + collection path decision around Nov/Dec 2026.</t>
         </is>
       </c>
       <c r="C179" s="28" t="inlineStr">
         <is>
-          <t>Browser extension audit on machines that use Glue Up admin; password rotation for affected accounts.</t>
+          <t>Schedule reminder; decide collection path (manual invoice vs Stripe annual vs override).</t>
         </is>
       </c>
       <c r="D179" s="28" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>SCHEDULED NOV 2026</t>
         </is>
       </c>
       <c r="E179" s="28" t="inlineStr">
         <is>
-          <t>Extension audit + password rotation.</t>
+          <t>Honored $1,034 annual; no Stripe customer today.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="28" t="inlineStr">
         <is>
-          <t>Stripe support ticket: typed promo codes rejected account-wide</t>
+          <t>Security: unknown third-party script (batatatech.com) on Glue Up admin pages</t>
         </is>
       </c>
       <c r="B180" s="28" t="inlineStr">
         <is>
-          <t>Typed promo codes are rejected account-wide on hosted Checkout (CLTBUCKETLIST / apartment codes path). Needs a Stripe support ticket.</t>
+          <t>Unknown batatatech.com script firing on Glue Up admin pages — treat as extension/malware until proven otherwise; audit browsers + rotate passwords.</t>
         </is>
       </c>
       <c r="C180" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM to file the Stripe support ticket.</t>
+          <t>Browser extension audit on machines that use Glue Up admin; password rotation for affected accounts.</t>
         </is>
       </c>
       <c r="D180" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="E180" s="28" t="inlineStr">
         <is>
-          <t>Account-wide hosted checkout rejection of typed promos.</t>
+          <t>Extension audit + password rotation.</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="28" t="inlineStr">
         <is>
-          <t>Calendar update-leg verification via throwaway event</t>
+          <t>Stripe support ticket: typed promo codes rejected account-wide</t>
         </is>
       </c>
       <c r="B181" s="28" t="inlineStr">
         <is>
-          <t>Verify that event-edit REQUEST invites actually move real calendars (ICS sequence / update leg) using a throwaway event.</t>
+          <t>Typed promo codes are rejected account-wide on hosted Checkout (CLTBUCKETLIST / apartment codes path). Needs a Stripe support ticket.</t>
         </is>
       </c>
       <c r="C181" s="28" t="inlineStr">
         <is>
-          <t>Create throwaway event, subscribe, edit, confirm calendars update; then delete throwaway.</t>
+          <t>WAITING ON ADAM to file the Stripe support ticket.</t>
         </is>
       </c>
       <c r="D181" s="28" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>WAITING ON ADAM</t>
         </is>
       </c>
       <c r="E181" s="28" t="inlineStr">
         <is>
-          <t>Throwaway event verification of REQUEST/update path.</t>
+          <t>Account-wide hosted checkout rejection of typed promos.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="28" t="inlineStr">
         <is>
-          <t>Ticket-checkout promo codes — same server-side attach as membership</t>
+          <t>Calendar update-leg verification via throwaway event</t>
         </is>
       </c>
       <c r="B182" s="28" t="inlineStr">
         <is>
-          <t>Ticket checkout should attach promo codes server-side the same way membership checkout does.</t>
+          <t>Verify that event-edit REQUEST invites actually move real calendars (ICS sequence / update leg) using a throwaway event.</t>
         </is>
       </c>
       <c r="C182" s="28" t="inlineStr">
         <is>
-          <t>FAST FOLLOW after membership promo attach path is solid; mirror server-side attach on create-ticket-checkout.</t>
+          <t>Create throwaway event, subscribe, edit, confirm calendars update; then delete throwaway.</t>
         </is>
       </c>
       <c r="D182" s="28" t="inlineStr">
         <is>
-          <t>FAST FOLLOW</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="E182" s="28" t="inlineStr">
         <is>
-          <t>Mirror membership server-side promo attach.</t>
+          <t>Throwaway event verification of REQUEST/update path.</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="28" t="inlineStr">
         <is>
-          <t>Resend click-tracking subdomain (DNS)</t>
+          <t>Ticket-checkout promo codes — same server-side attach as membership</t>
         </is>
       </c>
       <c r="B183" s="28" t="inlineStr">
         <is>
-          <t>Configure Resend click-tracking subdomain — Adam hands / DNS.</t>
+          <t>Ticket checkout should attach promo codes server-side the same way membership checkout does.</t>
         </is>
       </c>
       <c r="C183" s="28" t="inlineStr">
         <is>
-          <t>ADAM: DNS records for Resend click-tracking subdomain.</t>
+          <t>FAST FOLLOW after membership promo attach path is solid; mirror server-side attach on create-ticket-checkout.</t>
         </is>
       </c>
       <c r="D183" s="28" t="inlineStr">
         <is>
-          <t>ADAM - DNS</t>
+          <t>FAST FOLLOW</t>
         </is>
       </c>
       <c r="E183" s="28" t="inlineStr">
         <is>
-          <t>Adam hands / DNS.</t>
+          <t>Mirror membership server-side promo attach.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="28" t="inlineStr">
         <is>
-          <t>Catherine W password nudge via IG</t>
+          <t>Resend click-tracking subdomain (DNS)</t>
         </is>
       </c>
       <c r="B184" s="28" t="inlineStr">
         <is>
-          <t>Nudge Catherine W to reset/set password via Instagram.</t>
+          <t>Configure Resend click-tracking subdomain — Adam hands / DNS.</t>
         </is>
       </c>
       <c r="C184" s="28" t="inlineStr">
         <is>
-          <t>ADAM: send IG nudge.</t>
+          <t>ADAM: DNS records for Resend click-tracking subdomain.</t>
         </is>
       </c>
       <c r="D184" s="28" t="inlineStr">
         <is>
-          <t>ADAM - IG</t>
+          <t>ADAM - DNS</t>
         </is>
       </c>
       <c r="E184" s="28" t="inlineStr">
         <is>
-          <t>Via Instagram.</t>
+          <t>Adam hands / DNS.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="28" t="inlineStr">
         <is>
-          <t>Apartment campaign relaunch — codes work for the first time</t>
+          <t>Catherine W password nudge via IG</t>
         </is>
       </c>
       <c r="B185" s="28" t="inlineStr">
         <is>
-          <t>Apartment promo codes verified working for the first time; flyers can go out.</t>
+          <t>Nudge Catherine W to reset/set password via Instagram.</t>
         </is>
       </c>
       <c r="C185" s="28" t="inlineStr">
         <is>
-          <t>TIMI/GABBI: relaunch flyers / apartment campaign distribution.</t>
+          <t>ADAM: send IG nudge.</t>
         </is>
       </c>
       <c r="D185" s="28" t="inlineStr">
         <is>
-          <t>TIMI/GABBI</t>
+          <t>ADAM - IG</t>
         </is>
       </c>
       <c r="E185" s="28" t="inlineStr">
         <is>
-          <t>Codes verified; flyers can go out.</t>
+          <t>Via Instagram.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="28" t="inlineStr">
         <is>
-          <t>/welcome checkout-flow coverage on develop</t>
+          <t>Apartment campaign relaunch — codes work for the first time</t>
         </is>
       </c>
       <c r="B186" s="28" t="inlineStr">
         <is>
-          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
+          <t>Apartment promo codes verified working for the first time; flyers can go out.</t>
         </is>
       </c>
       <c r="C186" s="28" t="inlineStr">
         <is>
-          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
+          <t>TIMI/GABBI: relaunch flyers / apartment campaign distribution.</t>
         </is>
       </c>
       <c r="D186" s="28" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>TIMI/GABBI</t>
         </is>
       </c>
       <c r="E186" s="28" t="inlineStr">
         <is>
-          <t>Untested on develop; no Stripe checkout env.</t>
+          <t>Codes verified; flyers can go out.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="28" t="inlineStr">
         <is>
-          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
+          <t>/welcome checkout-flow coverage on develop</t>
         </is>
       </c>
       <c r="B187" s="28" t="inlineStr">
         <is>
-          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
+          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
         </is>
       </c>
       <c r="C187" s="28" t="inlineStr">
         <is>
-          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
+          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
         </is>
       </c>
       <c r="D187" s="28" t="inlineStr">
@@ -5061,59 +5061,86 @@
       </c>
       <c r="E187" s="28" t="inlineStr">
         <is>
-          <t>Revisit in identity-bridge work.</t>
+          <t>Untested on develop; no Stripe checkout env.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="28" t="inlineStr">
         <is>
-          <t>Retire the Google Sheets tracker path</t>
+          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
         </is>
       </c>
       <c r="B188" s="28" t="inlineStr">
         <is>
-          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
+          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
         </is>
       </c>
       <c r="C188" s="28" t="inlineStr">
         <is>
-          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
+          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
         </is>
       </c>
       <c r="D188" s="28" t="inlineStr">
         <is>
-          <t>QUEUED - cleanup</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="E188" s="28" t="inlineStr">
         <is>
-          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
+          <t>Revisit in identity-bridge work.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="28" t="inlineStr">
         <is>
+          <t>Retire the Google Sheets tracker path</t>
+        </is>
+      </c>
+      <c r="B189" s="28" t="inlineStr">
+        <is>
+          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
+        </is>
+      </c>
+      <c r="C189" s="28" t="inlineStr">
+        <is>
+          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
+        </is>
+      </c>
+      <c r="D189" s="28" t="inlineStr">
+        <is>
+          <t>QUEUED - cleanup</t>
+        </is>
+      </c>
+      <c r="E189" s="28" t="inlineStr">
+        <is>
+          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="28" t="inlineStr">
+        <is>
           <t>Admin card PATCH date normalization - external dates should save as noon UTC to avoid timezone off-by-one (Zach precedent)</t>
         </is>
       </c>
-      <c r="B189" s="28" t="inlineStr">
+      <c r="B190" s="28" t="inlineStr">
         <is>
           <t>external_paid_through saved as midnight UTC displays as prior calendar day in US Eastern (Zach showed Nov 30 instead of Dec 1). Admin billing PATCH should normalize date-only inputs to noon UTC.</t>
         </is>
       </c>
-      <c r="C189" s="28" t="inlineStr">
+      <c r="C190" s="28" t="inlineStr">
         <is>
           <t>In PATCH /api/admin/members/[id]/billing (and any similar writers), coerce external_paid_through date-only values to YYYY-MM-DDT12:00:00.000Z before save. SMALL.</t>
         </is>
       </c>
-      <c r="D189" s="28" t="inlineStr">
+      <c r="D190" s="28" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="E189" s="28" t="inlineStr">
+      <c r="E190" s="28" t="inlineStr">
         <is>
           <t>SMALL/OPEN. Precedent: Zach Trusky external_paid_through 2026-12-01T00:00:00Z → Nov 30 in America/New_York.</t>
         </is>

</xml_diff>

<commit_message>
chore: tracker - close 2 items, annotate 3 verified items
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E190"/>
+  <dimension ref="A1:E188"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="1" min="1" max="1"/>
@@ -4636,27 +4636,27 @@
     <row r="172">
       <c r="A172" s="27" t="inlineStr">
         <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   17 items</t>
+          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
       <c r="B172" s="27" t="inlineStr">
         <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   17 items</t>
+          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
       <c r="C172" s="27" t="inlineStr">
         <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   17 items</t>
+          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
       <c r="D172" s="27" t="inlineStr">
         <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   17 items</t>
+          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
       <c r="E172" s="27" t="inlineStr">
         <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   17 items</t>
+          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
     </row>
@@ -4867,12 +4867,12 @@
       </c>
       <c r="D180" s="28" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - Adam chrome://extensions only</t>
         </is>
       </c>
       <c r="E180" s="28" t="inlineStr">
         <is>
-          <t>Extension audit + password rotation.</t>
+          <t>repo confirmed clean 8/4 - scope is Adam's chrome://extensions only</t>
         </is>
       </c>
     </row>
@@ -4889,17 +4889,17 @@
       </c>
       <c r="C181" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM to file the Stripe support ticket.</t>
+          <t>OPTIONAL: file Stripe ticket only if we want Stripe's diagnosis for future ticket-checkout native-box trust. Membership path uses server-side attach.</t>
         </is>
       </c>
       <c r="D181" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM</t>
+          <t>OPTIONAL</t>
         </is>
       </c>
       <c r="E181" s="28" t="inlineStr">
         <is>
-          <t>Account-wide hosted checkout rejection of typed promos.</t>
+          <t>OPTIONAL - native box re-verified still broken 8/4; our server-side attach is the permanent fix; ticket only decides future ticket-checkout trust</t>
         </is>
       </c>
     </row>
@@ -4970,7 +4970,7 @@
       </c>
       <c r="C184" s="28" t="inlineStr">
         <is>
-          <t>ADAM: DNS records for Resend click-tracking subdomain.</t>
+          <t>ADAM DNS: add Resend click-tracking subdomain CNAME + add Resend to SPF include (current SPF is Google-only). Confirmed missing 8/4.</t>
         </is>
       </c>
       <c r="D184" s="28" t="inlineStr">
@@ -4980,167 +4980,113 @@
       </c>
       <c r="E184" s="28" t="inlineStr">
         <is>
-          <t>Adam hands / DNS.</t>
+          <t>confirmed NOT configured 8/4; also add Resend to SPF include during same DNS visit</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="28" t="inlineStr">
         <is>
-          <t>Catherine W password nudge via IG</t>
+          <t>/welcome checkout-flow coverage on develop</t>
         </is>
       </c>
       <c r="B185" s="28" t="inlineStr">
         <is>
-          <t>Nudge Catherine W to reset/set password via Instagram.</t>
+          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
         </is>
       </c>
       <c r="C185" s="28" t="inlineStr">
         <is>
-          <t>ADAM: send IG nudge.</t>
+          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
         </is>
       </c>
       <c r="D185" s="28" t="inlineStr">
         <is>
-          <t>ADAM - IG</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="E185" s="28" t="inlineStr">
         <is>
-          <t>Via Instagram.</t>
+          <t>Untested on develop; no Stripe checkout env.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="28" t="inlineStr">
         <is>
-          <t>Apartment campaign relaunch — codes work for the first time</t>
+          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
         </is>
       </c>
       <c r="B186" s="28" t="inlineStr">
         <is>
-          <t>Apartment promo codes verified working for the first time; flyers can go out.</t>
+          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
         </is>
       </c>
       <c r="C186" s="28" t="inlineStr">
         <is>
-          <t>TIMI/GABBI: relaunch flyers / apartment campaign distribution.</t>
+          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
         </is>
       </c>
       <c r="D186" s="28" t="inlineStr">
         <is>
-          <t>TIMI/GABBI</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="E186" s="28" t="inlineStr">
         <is>
-          <t>Codes verified; flyers can go out.</t>
+          <t>Revisit in identity-bridge work.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="28" t="inlineStr">
         <is>
-          <t>/welcome checkout-flow coverage on develop</t>
+          <t>Retire the Google Sheets tracker path</t>
         </is>
       </c>
       <c r="B187" s="28" t="inlineStr">
         <is>
-          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
+          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
         </is>
       </c>
       <c r="C187" s="28" t="inlineStr">
         <is>
-          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
+          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
         </is>
       </c>
       <c r="D187" s="28" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>QUEUED - cleanup</t>
         </is>
       </c>
       <c r="E187" s="28" t="inlineStr">
         <is>
-          <t>Untested on develop; no Stripe checkout env.</t>
+          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="28" t="inlineStr">
         <is>
-          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
+          <t>Admin card PATCH date normalization - external dates should save as noon UTC to avoid timezone off-by-one (Zach precedent)</t>
         </is>
       </c>
       <c r="B188" s="28" t="inlineStr">
         <is>
-          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
+          <t>external_paid_through saved as midnight UTC displays as prior calendar day in US Eastern (Zach showed Nov 30 instead of Dec 1). Admin billing PATCH should normalize date-only inputs to noon UTC.</t>
         </is>
       </c>
       <c r="C188" s="28" t="inlineStr">
         <is>
-          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
+          <t>In PATCH /api/admin/members/[id]/billing (and any similar writers), coerce external_paid_through date-only values to YYYY-MM-DDT12:00:00.000Z before save. SMALL.</t>
         </is>
       </c>
       <c r="D188" s="28" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="E188" s="28" t="inlineStr">
-        <is>
-          <t>Revisit in identity-bridge work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" s="28" t="inlineStr">
-        <is>
-          <t>Retire the Google Sheets tracker path</t>
-        </is>
-      </c>
-      <c r="B189" s="28" t="inlineStr">
-        <is>
-          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
-        </is>
-      </c>
-      <c r="C189" s="28" t="inlineStr">
-        <is>
-          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
-        </is>
-      </c>
-      <c r="D189" s="28" t="inlineStr">
-        <is>
-          <t>QUEUED - cleanup</t>
-        </is>
-      </c>
-      <c r="E189" s="28" t="inlineStr">
-        <is>
-          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="28" t="inlineStr">
-        <is>
-          <t>Admin card PATCH date normalization - external dates should save as noon UTC to avoid timezone off-by-one (Zach precedent)</t>
-        </is>
-      </c>
-      <c r="B190" s="28" t="inlineStr">
-        <is>
-          <t>external_paid_through saved as midnight UTC displays as prior calendar day in US Eastern (Zach showed Nov 30 instead of Dec 1). Admin billing PATCH should normalize date-only inputs to noon UTC.</t>
-        </is>
-      </c>
-      <c r="C190" s="28" t="inlineStr">
-        <is>
-          <t>In PATCH /api/admin/members/[id]/billing (and any similar writers), coerce external_paid_through date-only values to YYYY-MM-DDT12:00:00.000Z before save. SMALL.</t>
-        </is>
-      </c>
-      <c r="D190" s="28" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E190" s="28" t="inlineStr">
         <is>
           <t>SMALL/OPEN. Precedent: Zach Trusky external_paid_through 2026-12-01T00:00:00Z → Nov 30 in America/New_York.</t>
         </is>

</xml_diff>

<commit_message>
chore: tracker - promo system endstate, close 2 items
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E188"/>
+  <dimension ref="A1:E187"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="1" min="1" max="1"/>
@@ -4877,29 +4877,29 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="28" t="inlineStr">
-        <is>
-          <t>Stripe support ticket: typed promo codes rejected account-wide</t>
-        </is>
-      </c>
-      <c r="B181" s="28" t="inlineStr">
-        <is>
-          <t>Typed promo codes are rejected account-wide on hosted Checkout (CLTBUCKETLIST / apartment codes path). Needs a Stripe support ticket.</t>
-        </is>
-      </c>
-      <c r="C181" s="28" t="inlineStr">
-        <is>
-          <t>OPTIONAL: file Stripe ticket only if we want Stripe's diagnosis for future ticket-checkout native-box trust. Membership path uses server-side attach.</t>
-        </is>
-      </c>
-      <c r="D181" s="28" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="E181" s="28" t="inlineStr">
-        <is>
-          <t>OPTIONAL - native box re-verified still broken 8/4; our server-side attach is the permanent fix; ticket only decides future ticket-checkout trust</t>
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>[DONE] Promo system endstate 8/5</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Supersedes Stripe support ticket + ticket-checkout promo fast-follow (removed).</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
         </is>
       </c>
     </row>
@@ -4933,71 +4933,71 @@
     <row r="183">
       <c r="A183" s="28" t="inlineStr">
         <is>
-          <t>Ticket-checkout promo codes — same server-side attach as membership</t>
+          <t>Resend click-tracking subdomain (DNS)</t>
         </is>
       </c>
       <c r="B183" s="28" t="inlineStr">
         <is>
-          <t>Ticket checkout should attach promo codes server-side the same way membership checkout does.</t>
+          <t>Configure Resend click-tracking subdomain — Adam hands / DNS.</t>
         </is>
       </c>
       <c r="C183" s="28" t="inlineStr">
         <is>
-          <t>FAST FOLLOW after membership promo attach path is solid; mirror server-side attach on create-ticket-checkout.</t>
+          <t>ADAM DNS: add Resend click-tracking subdomain CNAME + add Resend to SPF include (current SPF is Google-only). Confirmed missing 8/4.</t>
         </is>
       </c>
       <c r="D183" s="28" t="inlineStr">
         <is>
-          <t>FAST FOLLOW</t>
+          <t>ADAM - DNS</t>
         </is>
       </c>
       <c r="E183" s="28" t="inlineStr">
         <is>
-          <t>Mirror membership server-side promo attach.</t>
+          <t>confirmed NOT configured 8/4; also add Resend to SPF include during same DNS visit</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="28" t="inlineStr">
         <is>
-          <t>Resend click-tracking subdomain (DNS)</t>
+          <t>/welcome checkout-flow coverage on develop</t>
         </is>
       </c>
       <c r="B184" s="28" t="inlineStr">
         <is>
-          <t>Configure Resend click-tracking subdomain — Adam hands / DNS.</t>
+          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
         </is>
       </c>
       <c r="C184" s="28" t="inlineStr">
         <is>
-          <t>ADAM DNS: add Resend click-tracking subdomain CNAME + add Resend to SPF include (current SPF is Google-only). Confirmed missing 8/4.</t>
+          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
         </is>
       </c>
       <c r="D184" s="28" t="inlineStr">
         <is>
-          <t>ADAM - DNS</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="E184" s="28" t="inlineStr">
         <is>
-          <t>confirmed NOT configured 8/4; also add Resend to SPF include during same DNS visit</t>
+          <t>Untested on develop; no Stripe checkout env.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="28" t="inlineStr">
         <is>
-          <t>/welcome checkout-flow coverage on develop</t>
+          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
         </is>
       </c>
       <c r="B185" s="28" t="inlineStr">
         <is>
-          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
+          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
         </is>
       </c>
       <c r="C185" s="28" t="inlineStr">
         <is>
-          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
+          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
         </is>
       </c>
       <c r="D185" s="28" t="inlineStr">
@@ -5007,86 +5007,59 @@
       </c>
       <c r="E185" s="28" t="inlineStr">
         <is>
-          <t>Untested on develop; no Stripe checkout env.</t>
+          <t>Revisit in identity-bridge work.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="28" t="inlineStr">
         <is>
-          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
+          <t>Retire the Google Sheets tracker path</t>
         </is>
       </c>
       <c r="B186" s="28" t="inlineStr">
         <is>
-          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
+          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
         </is>
       </c>
       <c r="C186" s="28" t="inlineStr">
         <is>
-          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
+          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
         </is>
       </c>
       <c r="D186" s="28" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>QUEUED - cleanup</t>
         </is>
       </c>
       <c r="E186" s="28" t="inlineStr">
         <is>
-          <t>Revisit in identity-bridge work.</t>
+          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="28" t="inlineStr">
         <is>
-          <t>Retire the Google Sheets tracker path</t>
+          <t>Admin card PATCH date normalization - external dates should save as noon UTC to avoid timezone off-by-one (Zach precedent)</t>
         </is>
       </c>
       <c r="B187" s="28" t="inlineStr">
         <is>
-          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
+          <t>external_paid_through saved as midnight UTC displays as prior calendar day in US Eastern (Zach showed Nov 30 instead of Dec 1). Admin billing PATCH should normalize date-only inputs to noon UTC.</t>
         </is>
       </c>
       <c r="C187" s="28" t="inlineStr">
         <is>
-          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
+          <t>In PATCH /api/admin/members/[id]/billing (and any similar writers), coerce external_paid_through date-only values to YYYY-MM-DDT12:00:00.000Z before save. SMALL.</t>
         </is>
       </c>
       <c r="D187" s="28" t="inlineStr">
         <is>
-          <t>QUEUED - cleanup</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="E187" s="28" t="inlineStr">
-        <is>
-          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="28" t="inlineStr">
-        <is>
-          <t>Admin card PATCH date normalization - external dates should save as noon UTC to avoid timezone off-by-one (Zach precedent)</t>
-        </is>
-      </c>
-      <c r="B188" s="28" t="inlineStr">
-        <is>
-          <t>external_paid_through saved as midnight UTC displays as prior calendar day in US Eastern (Zach showed Nov 30 instead of Dec 1). Admin billing PATCH should normalize date-only inputs to noon UTC.</t>
-        </is>
-      </c>
-      <c r="C188" s="28" t="inlineStr">
-        <is>
-          <t>In PATCH /api/admin/members/[id]/billing (and any similar writers), coerce external_paid_through date-only values to YYYY-MM-DDT12:00:00.000Z before save. SMALL.</t>
-        </is>
-      </c>
-      <c r="D188" s="28" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E188" s="28" t="inlineStr">
         <is>
           <t>SMALL/OPEN. Precedent: Zach Trusky external_paid_through 2026-12-01T00:00:00Z → Nov 30 in America/New_York.</t>
         </is>

</xml_diff>

<commit_message>
chore: tracker - add branded auth links + password hardening under AUTH
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E187"/>
+  <dimension ref="A1:E189"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="1" min="1" max="1"/>
@@ -2743,7 +2743,7 @@
     <row r="90" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>AUTH   ·   5 items</t>
+          <t>AUTH   ·   7 items</t>
         </is>
       </c>
       <c r="B90" s="29" t="n"/>
@@ -2871,31 +2871,63 @@
       <c r="E95" s="6" t="n"/>
     </row>
     <row r="96" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A96" s="4" t="inlineStr">
-        <is>
-          <t>BUSINESS   ·   1 item</t>
-        </is>
-      </c>
-      <c r="B96" s="29" t="n"/>
-      <c r="C96" s="29" t="n"/>
-      <c r="D96" s="29" t="n"/>
-      <c r="E96" s="30" t="n"/>
-    </row>
-    <row r="97" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>Branded auth links (stop showing supabase.co URLs)</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Every auth link we send (invite, password reset, magic link) points at bnmtynevbuplqpuqvmna.supabase.co. Looks untrustworthy in texts and emails, and the domain mismatch hurts link reputation with Gmail and Outlook.</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>Ship Option A first: a server-side /invite route on 704collective.com that accepts only a token and redirects to the hardcoded Supabase verify URL. No open-redirect parameter. Rehearse on develop, desktop 1440x900 and mobile 390x844. ENDGAME is Option B, the Supabase custom auth domain add-on (auth.704collective.com), which fixes every auth email with no redirect hop. Option B changes the project auth URL and touches env vars, redirect allow-lists and the JWT issuer, so it needs a planned window and a rollback plan.</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E96" s="6" t="inlineStr">
+        <is>
+          <t>Raised 2026-08-06 while hand-minting comp-invite links for Brandon Aruta and Davis Baxter to send by text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A97" s="7" t="inlineStr">
         <is>
-          <t>Verify the business application approval works</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="n"/>
-      <c r="C97" s="5" t="n"/>
-      <c r="D97" s="5" t="n"/>
-      <c r="E97" s="6" t="n"/>
+          <t>Password rules hardening (min length 6 to 8, leaked-password check)</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Supabase minimum password length is 6 and the leaked-password check is off. Both are weaker than they should be for a paid membership platform.</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>Do the UI copy FIRST, then the dashboard toggles. Update /setup-password and every password field to state the real rule before raising the server minimum to 8, otherwise members get rejected by a rule the screen never showed them. Then enable Prevent use of leaked passwords and confirm the rejection message renders cleanly. Leave Require current password when updating OFF, it breaks the no-password comp-invite setup flow. Rehearse on develop both viewports.</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="inlineStr">
+        <is>
+          <t>Raised 2026-08-06 during the Email OTP expiration change (3600 to 86400).</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>FINANCIALS   ·   6 items</t>
+          <t>BUSINESS   ·   1 item</t>
         </is>
       </c>
       <c r="B98" s="29" t="n"/>
@@ -2906,125 +2938,93 @@
     <row r="99" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A99" s="7" t="inlineStr">
         <is>
-          <t>Verify the financial dashboard</t>
-        </is>
-      </c>
-      <c r="B99" s="8" t="inlineStr">
-        <is>
-          <t>Confirm it reports MRR, churn, and revenue by tier correctly (churn once showed 2055%).</t>
-        </is>
-      </c>
-      <c r="C99" s="8" t="inlineStr">
-        <is>
-          <t>Verify financial dashboard accuracy.</t>
-        </is>
-      </c>
-      <c r="D99" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E99" s="8" t="inlineStr">
-        <is>
-          <t>Built in Lovable originally — accuracy unconfirmed.</t>
-        </is>
-      </c>
+          <t>Verify the business application approval works</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="n"/>
+      <c r="C99" s="5" t="n"/>
+      <c r="D99" s="5" t="n"/>
+      <c r="E99" s="6" t="n"/>
     </row>
     <row r="100" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A100" s="7" t="inlineStr">
-        <is>
-          <t>Verify the admin financial data function</t>
-        </is>
-      </c>
-      <c r="B100" s="8" t="inlineStr">
-        <is>
-          <t>Confirm the edge function feeding admin financials returns correct numbers.</t>
-        </is>
-      </c>
-      <c r="C100" s="8" t="inlineStr">
-        <is>
-          <t>Verify admin-financial-data.</t>
-        </is>
-      </c>
-      <c r="D100" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E100" s="8" t="inlineStr">
-        <is>
-          <t>Confirm the numbers it returns are correct.</t>
-        </is>
-      </c>
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>FINANCIALS   ·   6 items</t>
+        </is>
+      </c>
+      <c r="B100" s="29" t="n"/>
+      <c r="C100" s="29" t="n"/>
+      <c r="D100" s="29" t="n"/>
+      <c r="E100" s="30" t="n"/>
     </row>
     <row r="101" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A101" s="7" t="inlineStr">
         <is>
-          <t>Three-bucket revenue view</t>
+          <t>Verify the financial dashboard</t>
         </is>
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>Show revenue split three ways.</t>
+          <t>Confirm it reports MRR, churn, and revenue by tier correctly (churn once showed 2055%).</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t>Collected / projected / churned split.</t>
-        </is>
-      </c>
-      <c r="D101" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
+          <t>Verify financial dashboard accuracy.</t>
+        </is>
+      </c>
+      <c r="D101" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
         <is>
-          <t>Collected / projected / churned.</t>
+          <t>Built in Lovable originally — accuracy unconfirmed.</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A102" s="7" t="inlineStr">
         <is>
-          <t>Member-facing financial widget</t>
+          <t>Verify the admin financial data function</t>
         </is>
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>A small financial widget members can see.</t>
+          <t>Confirm the edge function feeding admin financials returns correct numbers.</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Member-facing billing-status widget.</t>
-        </is>
-      </c>
-      <c r="D102" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
+          <t>Verify admin-financial-data.</t>
+        </is>
+      </c>
+      <c r="D102" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t>Small billing-status widget for members.</t>
+          <t>Confirm the numbers it returns are correct.</t>
         </is>
       </c>
     </row>
     <row r="103" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A103" s="7" t="inlineStr">
         <is>
-          <t>Reduce redundant Stripe scans</t>
+          <t>Three-bucket revenue view</t>
         </is>
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>Cut how often the system scans Stripe, for performance/cost.</t>
+          <t>Show revenue split three ways.</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Reduce Stripe API scan frequency.</t>
+          <t>Collected / projected / churned split.</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
@@ -3034,100 +3034,100 @@
       </c>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t>Cut scan frequency for cost / performance.</t>
+          <t>Collected / projected / churned.</t>
         </is>
       </c>
     </row>
     <row r="104" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A104" s="7" t="inlineStr">
         <is>
-          <t>Past-due dismissal flow</t>
-        </is>
-      </c>
-      <c r="B104" s="5" t="n"/>
-      <c r="C104" s="5" t="n"/>
-      <c r="D104" s="5" t="n"/>
-      <c r="E104" s="6" t="n"/>
+          <t>Member-facing financial widget</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t>A small financial widget members can see.</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>Member-facing billing-status widget.</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E104" s="8" t="inlineStr">
+        <is>
+          <t>Small billing-status widget for members.</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A105" s="4" t="inlineStr">
-        <is>
-          <t>EMAIL &amp; DRIP   ·   13 items</t>
-        </is>
-      </c>
-      <c r="B105" s="29" t="n"/>
-      <c r="C105" s="29" t="n"/>
-      <c r="D105" s="29" t="n"/>
-      <c r="E105" s="30" t="n"/>
+      <c r="A105" s="7" t="inlineStr">
+        <is>
+          <t>Reduce redundant Stripe scans</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>Cut how often the system scans Stripe, for performance/cost.</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>Reduce Stripe API scan frequency.</t>
+        </is>
+      </c>
+      <c r="D105" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>Cut scan frequency for cost / performance.</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t>Drip email health banner</t>
-        </is>
-      </c>
-      <c r="B106" s="8" t="inlineStr">
-        <is>
-          <t>A banner flagging when drips are silently failing or stalled.</t>
-        </is>
-      </c>
-      <c r="C106" s="8" t="inlineStr">
-        <is>
-          <t>Drip health-check banner.</t>
-        </is>
-      </c>
-      <c r="D106" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E106" s="8" t="inlineStr">
-        <is>
-          <t>Flags silently failing / stalled drips.</t>
-        </is>
-      </c>
+          <t>Past-due dismissal flow</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="n"/>
+      <c r="C106" s="5" t="n"/>
+      <c r="D106" s="5" t="n"/>
+      <c r="E106" s="6" t="n"/>
     </row>
     <row r="107" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A107" s="7" t="inlineStr">
-        <is>
-          <t>Guest follow-up drip (7 + 20 day)</t>
-        </is>
-      </c>
-      <c r="B107" s="8" t="inlineStr">
-        <is>
-          <t>Automatic emails to guests at day 7 and 20 to convert them.</t>
-        </is>
-      </c>
-      <c r="C107" s="8" t="inlineStr">
-        <is>
-          <t>Guest 7-day + 20-day drip.</t>
-        </is>
-      </c>
-      <c r="D107" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E107" s="8" t="inlineStr">
-        <is>
-          <t>Converts guests at day 7 and 20.</t>
-        </is>
-      </c>
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>EMAIL &amp; DRIP   ·   13 items</t>
+        </is>
+      </c>
+      <c r="B107" s="29" t="n"/>
+      <c r="C107" s="29" t="n"/>
+      <c r="D107" s="29" t="n"/>
+      <c r="E107" s="30" t="n"/>
     </row>
     <row r="108" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t>14-day RSVP prompt for new members</t>
+          <t>Drip email health banner</t>
         </is>
       </c>
       <c r="B108" s="8" t="inlineStr">
         <is>
-          <t>Nudge new members who haven't RSVP'd within 14 days.</t>
+          <t>A banner flagging when drips are silently failing or stalled.</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t>14-day RSVP prompt drip.</t>
+          <t>Drip health-check banner.</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
@@ -3137,24 +3137,24 @@
       </c>
       <c r="E108" s="8" t="inlineStr">
         <is>
-          <t>Nudges new members who haven't RSVP'd.</t>
+          <t>Flags silently failing / stalled drips.</t>
         </is>
       </c>
     </row>
     <row r="109" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A109" s="7" t="inlineStr">
         <is>
-          <t>Confirm the email log matches actual sends</t>
+          <t>Guest follow-up drip (7 + 20 day)</t>
         </is>
       </c>
       <c r="B109" s="8" t="inlineStr">
         <is>
-          <t>Today failures are swallowed; make 'did this send' provable.</t>
+          <t>Automatic emails to guests at day 7 and 20 to convert them.</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t>email_log row matching; stop swallowing failures.</t>
+          <t>Guest 7-day + 20-day drip.</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
@@ -3164,24 +3164,24 @@
       </c>
       <c r="E109" s="8" t="inlineStr">
         <is>
-          <t>Stop swallowing failures so 'did this send' is provable.</t>
+          <t>Converts guests at day 7 and 20.</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t>Per-email open/click analytics</t>
+          <t>14-day RSVP prompt for new members</t>
         </is>
       </c>
       <c r="B110" s="8" t="inlineStr">
         <is>
-          <t>Track opens/clicks per template so we know what works.</t>
+          <t>Nudge new members who haven't RSVP'd within 14 days.</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t>Per-template email analytics.</t>
+          <t>14-day RSVP prompt drip.</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
@@ -3191,24 +3191,24 @@
       </c>
       <c r="E110" s="8" t="inlineStr">
         <is>
-          <t>Per-template open / click tracking.</t>
+          <t>Nudges new members who haven't RSVP'd.</t>
         </is>
       </c>
     </row>
     <row r="111" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A111" s="7" t="inlineStr">
         <is>
-          <t>Per-member engagement scoring</t>
+          <t>Confirm the email log matches actual sends</t>
         </is>
       </c>
       <c r="B111" s="8" t="inlineStr">
         <is>
-          <t>Score each member's engagement from email/event activity.</t>
+          <t>Today failures are swallowed; make 'did this send' provable.</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t>Engagement scoring per member.</t>
+          <t>email_log row matching; stop swallowing failures.</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
@@ -3218,24 +3218,24 @@
       </c>
       <c r="E111" s="8" t="inlineStr">
         <is>
-          <t>Score members from email / event activity.</t>
+          <t>Stop swallowing failures so 'did this send' is provable.</t>
         </is>
       </c>
     </row>
     <row r="112" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t>Category-level unsubscribe preferences</t>
+          <t>Per-email open/click analytics</t>
         </is>
       </c>
       <c r="B112" s="8" t="inlineStr">
         <is>
-          <t>Let members opt out of specific categories, not all-or-nothing; builds on the one-flag fix.</t>
+          <t>Track opens/clicks per template so we know what works.</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t>Per-category opt-out prefs + a member settings page.</t>
+          <t>Per-template email analytics.</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
@@ -3245,24 +3245,24 @@
       </c>
       <c r="E112" s="8" t="inlineStr">
         <is>
-          <t>Builds on the one-flag opt-out fix.</t>
+          <t>Per-template open / click tracking.</t>
         </is>
       </c>
     </row>
     <row r="113" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A113" s="7" t="inlineStr">
         <is>
-          <t>Branching drips based on opens/clicks</t>
+          <t>Per-member engagement scoring</t>
         </is>
       </c>
       <c r="B113" s="8" t="inlineStr">
         <is>
-          <t>Drip sequences that branch on open/click.</t>
+          <t>Score each member's engagement from email/event activity.</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t>Open/click-branching drips.</t>
+          <t>Engagement scoring per member.</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
@@ -3272,24 +3272,24 @@
       </c>
       <c r="E113" s="8" t="inlineStr">
         <is>
-          <t>Branch sequences on open / click.</t>
+          <t>Score members from email / event activity.</t>
         </is>
       </c>
     </row>
     <row r="114" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A114" s="7" t="inlineStr">
         <is>
-          <t>Send email from a contact record</t>
+          <t>Category-level unsubscribe preferences</t>
         </is>
       </c>
       <c r="B114" s="8" t="inlineStr">
         <is>
-          <t>Let an admin email directly from a member/contact record.</t>
+          <t>Let members opt out of specific categories, not all-or-nothing; builds on the one-flag fix.</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t>Send-email action on the contact record.</t>
+          <t>Per-category opt-out prefs + a member settings page.</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
@@ -3299,24 +3299,24 @@
       </c>
       <c r="E114" s="8" t="inlineStr">
         <is>
-          <t>Admin emails directly from a member record.</t>
+          <t>Builds on the one-flag opt-out fix.</t>
         </is>
       </c>
     </row>
     <row r="115" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A115" s="7" t="inlineStr">
         <is>
-          <t>Attachments and images on event email campaigns</t>
+          <t>Branching drips based on opens/clicks</t>
         </is>
       </c>
       <c r="B115" s="8" t="inlineStr">
         <is>
-          <t>Let campaign emails include attachments and images.</t>
+          <t>Drip sequences that branch on open/click.</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t>Extend the campaign editor for attachments + images.</t>
+          <t>Open/click-branching drips.</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
@@ -3326,51 +3326,51 @@
       </c>
       <c r="E115" s="8" t="inlineStr">
         <is>
-          <t>Extend the campaign editor.</t>
+          <t>Branch sequences on open / click.</t>
         </is>
       </c>
     </row>
     <row r="116" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>Live test the guest-pass drip</t>
+          <t>Send email from a contact record</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
         <is>
-          <t>Confirm the drip fires correctly on a guest pass.</t>
+          <t>Let an admin email directly from a member/contact record.</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t>Live test the drip on guest_pass.</t>
-        </is>
-      </c>
-      <c r="D116" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
+          <t>Send-email action on the contact record.</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
         <is>
-          <t>Confirm it fires on a guest pass.</t>
+          <t>Admin emails directly from a member record.</t>
         </is>
       </c>
     </row>
     <row r="117" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t>Merge guest follow-up into the drip processor</t>
+          <t>Attachments and images on event email campaigns</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
         <is>
-          <t>Retire the separate guest-followup function and fold it into the main processor.</t>
+          <t>Let campaign emails include attachments and images.</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t>Consolidate guest-followup into process-drips.</t>
+          <t>Extend the campaign editor for attachments + images.</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
@@ -3380,241 +3380,241 @@
       </c>
       <c r="E117" s="8" t="inlineStr">
         <is>
-          <t>Fold guest-followup into process-drips.</t>
+          <t>Extend the campaign editor.</t>
         </is>
       </c>
     </row>
     <row r="118" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A118" s="7" t="inlineStr">
         <is>
+          <t>Live test the guest-pass drip</t>
+        </is>
+      </c>
+      <c r="B118" s="8" t="inlineStr">
+        <is>
+          <t>Confirm the drip fires correctly on a guest pass.</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>Live test the drip on guest_pass.</t>
+        </is>
+      </c>
+      <c r="D118" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E118" s="8" t="inlineStr">
+        <is>
+          <t>Confirm it fires on a guest pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="15" customFormat="1" customHeight="1" s="2">
+      <c r="A119" s="7" t="inlineStr">
+        <is>
+          <t>Merge guest follow-up into the drip processor</t>
+        </is>
+      </c>
+      <c r="B119" s="8" t="inlineStr">
+        <is>
+          <t>Retire the separate guest-followup function and fold it into the main processor.</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>Consolidate guest-followup into process-drips.</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E119" s="8" t="inlineStr">
+        <is>
+          <t>Fold guest-followup into process-drips.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
           <t>Push current members to subscribe to the calendar + add their pass</t>
         </is>
       </c>
-      <c r="B118" s="5" t="n"/>
-      <c r="C118" s="5" t="n"/>
-      <c r="D118" s="5" t="n"/>
-      <c r="E118" s="6" t="n"/>
-    </row>
-    <row r="119" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A119" s="4" t="inlineStr">
+      <c r="B120" s="5" t="n"/>
+      <c r="C120" s="5" t="n"/>
+      <c r="D120" s="5" t="n"/>
+      <c r="E120" s="6" t="n"/>
+    </row>
+    <row r="121" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A121" s="4" t="inlineStr">
         <is>
           <t>DATA &amp; CLEANUP   ·   6 items</t>
         </is>
       </c>
-      <c r="B119" s="29" t="n"/>
-      <c r="C119" s="29" t="n"/>
-      <c r="D119" s="29" t="n"/>
-      <c r="E119" s="30" t="n"/>
-    </row>
-    <row r="120" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A120" s="17" t="inlineStr">
+      <c r="B121" s="29" t="n"/>
+      <c r="C121" s="29" t="n"/>
+      <c r="D121" s="29" t="n"/>
+      <c r="E121" s="30" t="n"/>
+    </row>
+    <row r="122" ht="21.75" customFormat="1" customHeight="1" s="2">
+      <c r="A122" s="17" t="inlineStr">
         <is>
           <t>Add CHECK constraints incrementally (enums REJECTED — too risky)</t>
         </is>
       </c>
-      <c r="B120" s="15" t="inlineStr">
+      <c r="B122" s="15" t="inlineStr">
         <is>
           <t>Was 'convert status text -&gt; enums'. DIAGNOSED Jul 9 as too risky: ~35 tables / 60+ write paths, and profiles.subscription_status is fed by the Stripe webhook with Stripe's full status vocabulary (trialing/paused/incomplete/etc). An enum built from observed values would make the webhook UPDATE throw on the first unseen status — silent breakage in the PAYMENT path. Enums rejected.</t>
         </is>
       </c>
-      <c r="C120" s="15" t="inlineStr">
+      <c r="C122" s="15" t="inlineStr">
         <is>
           <t>If typo-prevention is wanted later: add per-table CHECK constraints (NOT enums), table-by-table, starting with attendance_credentials (values: active/used/voided). Trivially reversible. Its own scoped task — never wholesale.</t>
         </is>
       </c>
-      <c r="D120" s="18" t="inlineStr">
+      <c r="D122" s="18" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
       </c>
-      <c r="E120" s="15" t="inlineStr">
+      <c r="E122" s="15" t="inlineStr">
         <is>
           <t>Reclassified Jul 9. Do NOT rush — payment-path risk. CHECK constraints are the safe 80/20 if revisited.</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A121" s="17" t="inlineStr">
+    <row r="123" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A123" s="17" t="inlineStr">
         <is>
           <t>RSVP attribution by event ID</t>
         </is>
       </c>
-      <c r="B121" s="15" t="inlineStr">
+      <c r="B123" s="15" t="inlineStr">
         <is>
           <t>DIAGNOSED Jul 9: bigger than 'add a column'. Per-event RSVP tagging is DEAD — the code that slug-tagged events was removed; since Apr 21 a public RSVP only gets a generic 'free-event-rsvp' tag, so you can't segment 'RSVP'd to event X' for any recent event. 6 frozen slug-tags remain (105 rows) and rot on rename. contact_tags has NO event_id column.</t>
         </is>
       </c>
-      <c r="C121" s="15" t="inlineStr">
+      <c r="C123" s="15" t="inlineStr">
         <is>
           <t>HALF-DAY scoped task (not a quick close): (1) migration add nullable event_id uuid REFERENCES events(id) to contact_tags; (2) re-add per-event tagging in capture-public-rsvp (event_id already in scope) + optionally create-guest-pass; (3) backfill — 5 of 6 slug-tags map to real event_ids by title-slug match (1 unmatched: coffee-and-connect-tabbris-co-working). Deploys + tests.</t>
         </is>
       </c>
-      <c r="D121" s="19" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E121" s="15" t="inlineStr">
+      <c r="D123" s="19" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E123" s="15" t="inlineStr">
         <is>
           <t>Jul 9: revives dead per-event attribution. Own task, budget a half-day. Backfill mostly possible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A122" s="7" t="inlineStr">
-        <is>
-          <t>Drop ~35 empty leftover tables</t>
-        </is>
-      </c>
-      <c r="B122" s="8" t="inlineStr">
-        <is>
-          <t>~35 empty scaffolding tables (old CRM, social manager, feed, DMs).</t>
-        </is>
-      </c>
-      <c r="C122" s="8" t="inlineStr">
-        <is>
-          <t>Export copies as a receipt, then drop.</t>
-        </is>
-      </c>
-      <c r="D122" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E122" s="8" t="inlineStr">
-        <is>
-          <t>Don't drop without exporting copies first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A123" s="7" t="inlineStr">
-        <is>
-          <t>Drop old backup tables after soak</t>
-        </is>
-      </c>
-      <c r="B123" s="8" t="inlineStr">
-        <is>
-          <t>Backup tables from recent migrations await a 2-4 week no-regression soak.</t>
-        </is>
-      </c>
-      <c r="C123" s="8" t="inlineStr">
-        <is>
-          <t>Drop dated backup_* tables after soak; confirm stability first.</t>
-        </is>
-      </c>
-      <c r="D123" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E123" s="8" t="inlineStr">
-        <is>
-          <t>Only after a 2-4 week no-regression soak.</t>
         </is>
       </c>
     </row>
     <row r="124" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A124" s="7" t="inlineStr">
         <is>
-          <t>Delete dead admin member components</t>
-        </is>
-      </c>
-      <c r="B124" s="5" t="n"/>
-      <c r="C124" s="5" t="n"/>
-      <c r="D124" s="5" t="n"/>
-      <c r="E124" s="6" t="n"/>
+          <t>Drop ~35 empty leftover tables</t>
+        </is>
+      </c>
+      <c r="B124" s="8" t="inlineStr">
+        <is>
+          <t>~35 empty scaffolding tables (old CRM, social manager, feed, DMs).</t>
+        </is>
+      </c>
+      <c r="C124" s="8" t="inlineStr">
+        <is>
+          <t>Export copies as a receipt, then drop.</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E124" s="8" t="inlineStr">
+        <is>
+          <t>Don't drop without exporting copies first.</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A125" s="4" t="inlineStr">
-        <is>
-          <t>MARKETING &amp; FRONT-END   ·   10 items</t>
-        </is>
-      </c>
-      <c r="B125" s="5" t="n"/>
-      <c r="C125" s="5" t="n"/>
-      <c r="D125" s="5" t="n"/>
-      <c r="E125" s="6" t="n"/>
+      <c r="A125" s="7" t="inlineStr">
+        <is>
+          <t>Drop old backup tables after soak</t>
+        </is>
+      </c>
+      <c r="B125" s="8" t="inlineStr">
+        <is>
+          <t>Backup tables from recent migrations await a 2-4 week no-regression soak.</t>
+        </is>
+      </c>
+      <c r="C125" s="8" t="inlineStr">
+        <is>
+          <t>Drop dated backup_* tables after soak; confirm stability first.</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E125" s="8" t="inlineStr">
+        <is>
+          <t>Only after a 2-4 week no-regression soak.</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A126" s="7" t="inlineStr">
         <is>
-          <t>SEO + schema markup + pre-rendering (all front pages + 4 hub landers)</t>
-        </is>
-      </c>
-      <c r="B126" s="29" t="n"/>
-      <c r="C126" s="29" t="n"/>
-      <c r="D126" s="29" t="n"/>
-      <c r="E126" s="30" t="n"/>
+          <t>Delete dead admin member components</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="n"/>
+      <c r="C126" s="5" t="n"/>
+      <c r="D126" s="5" t="n"/>
+      <c r="E126" s="6" t="n"/>
     </row>
     <row r="127" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
-      <c r="A127" s="7" t="inlineStr">
-        <is>
-          <t>Homepage hero rebuild + image optimization</t>
-        </is>
-      </c>
-      <c r="B127" s="8" t="inlineStr">
-        <is>
-          <t>Rebuild the hero and compress oversized hero images (currently 24-30MB, should be 200-800KB).</t>
-        </is>
-      </c>
-      <c r="C127" s="8" t="inlineStr">
-        <is>
-          <t>Hero rebuild + compress images.</t>
-        </is>
-      </c>
-      <c r="D127" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E127" s="8" t="inlineStr">
-        <is>
-          <t>Includes compressing 24-30MB hero images to 200-800KB.</t>
-        </is>
-      </c>
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>MARKETING &amp; FRONT-END   ·   10 items</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="n"/>
+      <c r="C127" s="5" t="n"/>
+      <c r="D127" s="5" t="n"/>
+      <c r="E127" s="6" t="n"/>
     </row>
     <row r="128" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A128" s="7" t="inlineStr">
         <is>
-          <t>Homepage copy rewrite + slogan</t>
-        </is>
-      </c>
-      <c r="B128" s="8" t="inlineStr">
-        <is>
-          <t>Rewrite homepage body/section copy and update the slogan.</t>
-        </is>
-      </c>
-      <c r="C128" s="8" t="inlineStr">
-        <is>
-          <t>Body + section copy + slogan.</t>
-        </is>
-      </c>
-      <c r="D128" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E128" s="8" t="inlineStr">
-        <is>
-          <t>Needs the copy spec.</t>
-        </is>
-      </c>
+          <t>SEO + schema markup + pre-rendering (all front pages + 4 hub landers)</t>
+        </is>
+      </c>
+      <c r="B128" s="29" t="n"/>
+      <c r="C128" s="29" t="n"/>
+      <c r="D128" s="29" t="n"/>
+      <c r="E128" s="30" t="n"/>
     </row>
     <row r="129" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A129" s="7" t="inlineStr">
         <is>
-          <t>Fix the mobile hero sliding bug</t>
+          <t>Homepage hero rebuild + image optimization</t>
         </is>
       </c>
       <c r="B129" s="8" t="inlineStr">
         <is>
-          <t>A visual bug where the hero image slides on mobile.</t>
+          <t>Rebuild the hero and compress oversized hero images (currently 24-30MB, should be 200-800KB).</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
         <is>
-          <t>Mobile hero sliding fix.</t>
+          <t>Hero rebuild + compress images.</t>
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr">
@@ -3624,24 +3624,24 @@
       </c>
       <c r="E129" s="8" t="inlineStr">
         <is>
-          <t>Fix the hero sliding on mobile.</t>
+          <t>Includes compressing 24-30MB hero images to 200-800KB.</t>
         </is>
       </c>
     </row>
     <row r="130" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A130" s="7" t="inlineStr">
         <is>
-          <t>The Exchange page</t>
+          <t>Homepage copy rewrite + slogan</t>
         </is>
       </c>
       <c r="B130" s="8" t="inlineStr">
         <is>
-          <t>Build The Exchange page (speaker-driven business event product page).</t>
+          <t>Rewrite homepage body/section copy and update the slogan.</t>
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr">
         <is>
-          <t>The Exchange page.</t>
+          <t>Body + section copy + slogan.</t>
         </is>
       </c>
       <c r="D130" s="10" t="inlineStr">
@@ -3651,24 +3651,24 @@
       </c>
       <c r="E130" s="8" t="inlineStr">
         <is>
-          <t>Speaker-driven business-event product page.</t>
+          <t>Needs the copy spec.</t>
         </is>
       </c>
     </row>
     <row r="131" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A131" s="7" t="inlineStr">
         <is>
-          <t>Sponsor page (likely folds into /business)</t>
+          <t>Fix the mobile hero sliding bug</t>
         </is>
       </c>
       <c r="B131" s="8" t="inlineStr">
         <is>
-          <t>Sponsor functionality — likely folds into the /business application routing.</t>
+          <t>A visual bug where the hero image slides on mobile.</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
         <is>
-          <t>Probably absorbed by the /business rebuild.</t>
+          <t>Mobile hero sliding fix.</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr">
@@ -3678,24 +3678,24 @@
       </c>
       <c r="E131" s="8" t="inlineStr">
         <is>
-          <t>Likely folds into the /business rebuild — confirm first.</t>
+          <t>Fix the hero sliding on mobile.</t>
         </is>
       </c>
     </row>
     <row r="132" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A132" s="7" t="inlineStr">
         <is>
-          <t>/business page rebuild with dynamic application</t>
+          <t>The Exchange page</t>
         </is>
       </c>
       <c r="B132" s="8" t="inlineStr">
         <is>
-          <t>Rebuild /business as one page with a dynamic application routing prospects to membership, Preferred Business, or sponsorship by their answers.</t>
+          <t>Build The Exchange page (speaker-driven business event product page).</t>
         </is>
       </c>
       <c r="C132" s="8" t="inlineStr">
         <is>
-          <t>Dynamic diagnose-before-offer application.</t>
+          <t>The Exchange page.</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr">
@@ -3705,24 +3705,24 @@
       </c>
       <c r="E132" s="8" t="inlineStr">
         <is>
-          <t>Routes prospects to membership, Preferred Business, or sponsorship.</t>
+          <t>Speaker-driven business-event product page.</t>
         </is>
       </c>
     </row>
     <row r="133" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A133" s="7" t="inlineStr">
         <is>
-          <t>Charlotte hub landing sites (4 public landers)</t>
+          <t>Sponsor page (likely folds into /business)</t>
         </is>
       </c>
       <c r="B133" s="8" t="inlineStr">
         <is>
-          <t>Four audience-specific public landers (cltarrival / cltfounded / clteatsandevents / cltreset) that funnel Charlotte audiences into the club.</t>
+          <t>Sponsor functionality — likely folds into the /business application routing.</t>
         </is>
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t>4 public landers, shared skeleton, own design pass, fully pre-rendered + schema (see SEO item). They feed The Network.</t>
+          <t>Probably absorbed by the /business rebuild.</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr">
@@ -3732,24 +3732,24 @@
       </c>
       <c r="E133" s="8" t="inlineStr">
         <is>
-          <t>Public landers can ship earlier; they pair with The Network below.</t>
+          <t>Likely folds into the /business rebuild — confirm first.</t>
         </is>
       </c>
     </row>
     <row r="134" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A134" s="7" t="inlineStr">
         <is>
-          <t>The Network — four hubs + members rolled up</t>
+          <t>/business page rebuild with dynamic application</t>
         </is>
       </c>
       <c r="B134" s="8" t="inlineStr">
         <is>
-          <t>The four hubs rolled up into one view, plus all members. Two faces reading the same data: a PUBLIC face (the hub landers + business/partner listings — the sales asset) and an INTERNAL in-portal view that rolls up everyone. Social members appear ONLY on the internal in-portal view — never on the public hubs.</t>
+          <t>Rebuild /business as one page with a dynamic application routing prospects to membership, Preferred Business, or sponsorship by their answers.</t>
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr">
         <is>
-          <t>Roll the four hubs into one Network view + members. Public face = hubs / business + partner listings (social members excluded). Internal face = full rolled-up view including social members. Reads the same hub data as the landers.</t>
+          <t>Dynamic diagnose-before-offer application.</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
@@ -3759,294 +3759,294 @@
       </c>
       <c r="E134" s="8" t="inlineStr">
         <is>
-          <t>Depends on the portal + identity foundation. Social members are internal-only on The Network. Separate from the member directory (people-only).</t>
+          <t>Routes prospects to membership, Preferred Business, or sponsorship.</t>
         </is>
       </c>
     </row>
     <row r="135" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
       <c r="A135" s="7" t="inlineStr">
         <is>
-          <t>Instagram comment auto-DM (ManyChat)</t>
-        </is>
-      </c>
-      <c r="B135" s="5" t="n"/>
-      <c r="C135" s="5" t="n"/>
-      <c r="D135" s="5" t="n"/>
-      <c r="E135" s="6" t="n"/>
+          <t>Charlotte hub landing sites (4 public landers)</t>
+        </is>
+      </c>
+      <c r="B135" s="8" t="inlineStr">
+        <is>
+          <t>Four audience-specific public landers (cltarrival / cltfounded / clteatsandevents / cltreset) that funnel Charlotte audiences into the club.</t>
+        </is>
+      </c>
+      <c r="C135" s="8" t="inlineStr">
+        <is>
+          <t>4 public landers, shared skeleton, own design pass, fully pre-rendered + schema (see SEO item). They feed The Network.</t>
+        </is>
+      </c>
+      <c r="D135" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E135" s="8" t="inlineStr">
+        <is>
+          <t>Public landers can ship earlier; they pair with The Network below.</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A136" s="4" t="inlineStr">
-        <is>
-          <t>AI / AGENTS (LATER EFFORT)   ·   2 items</t>
-        </is>
-      </c>
-      <c r="B136" s="5" t="n"/>
-      <c r="C136" s="5" t="n"/>
-      <c r="D136" s="5" t="n"/>
-      <c r="E136" s="6" t="n"/>
+      <c r="A136" s="7" t="inlineStr">
+        <is>
+          <t>The Network — four hubs + members rolled up</t>
+        </is>
+      </c>
+      <c r="B136" s="8" t="inlineStr">
+        <is>
+          <t>The four hubs rolled up into one view, plus all members. Two faces reading the same data: a PUBLIC face (the hub landers + business/partner listings — the sales asset) and an INTERNAL in-portal view that rolls up everyone. Social members appear ONLY on the internal in-portal view — never on the public hubs.</t>
+        </is>
+      </c>
+      <c r="C136" s="8" t="inlineStr">
+        <is>
+          <t>Roll the four hubs into one Network view + members. Public face = hubs / business + partner listings (social members excluded). Internal face = full rolled-up view including social members. Reads the same hub data as the landers.</t>
+        </is>
+      </c>
+      <c r="D136" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E136" s="8" t="inlineStr">
+        <is>
+          <t>Depends on the portal + identity foundation. Social members are internal-only on The Network. Separate from the member directory (people-only).</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A137" s="7" t="inlineStr">
         <is>
+          <t>Instagram comment auto-DM (ManyChat)</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="n"/>
+      <c r="C137" s="5" t="n"/>
+      <c r="D137" s="5" t="n"/>
+      <c r="E137" s="6" t="n"/>
+    </row>
+    <row r="138" ht="35.05" customFormat="1" customHeight="1" s="2">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>AI / AGENTS (LATER EFFORT)   ·   2 items</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="n"/>
+      <c r="C138" s="5" t="n"/>
+      <c r="D138" s="5" t="n"/>
+      <c r="E138" s="6" t="n"/>
+    </row>
+    <row r="139" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A139" s="7" t="inlineStr">
+        <is>
           <t>AI concierge + agent platform</t>
         </is>
       </c>
-      <c r="B137" s="29" t="n"/>
-      <c r="C137" s="29" t="n"/>
-      <c r="D137" s="29" t="n"/>
-      <c r="E137" s="30" t="n"/>
-    </row>
-    <row r="138" ht="35.05" customFormat="1" customHeight="1" s="2">
-      <c r="A138" s="7" t="inlineStr">
-        <is>
-          <t>AI foundations (memory, embeddings, coordination)</t>
-        </is>
-      </c>
-      <c r="B138" s="8" t="inlineStr">
-        <is>
-          <t>Supporting infra for the agents: shared memory, member embeddings, multi-agent coordination, model routing.</t>
-        </is>
-      </c>
-      <c r="C138" s="8" t="inlineStr">
-        <is>
-          <t>pgvector + embeddings, agent_memory, multi-agent coordination, model routing.</t>
-        </is>
-      </c>
-      <c r="D138" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E138" s="8" t="inlineStr">
-        <is>
-          <t>A later effort; supports the agents (embeddings, memory, routing).</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A139" s="4" t="inlineStr">
-        <is>
-          <t>EVENT DISCUSSION &amp; NOTIFICATIONS + JUL-5/6 FINDINGS — IN-HOUSE (NOT ON THE DEVELOPER SHEET)   ·   10 items</t>
-        </is>
-      </c>
-      <c r="B139" s="1" t="n"/>
-      <c r="D139" s="1" t="n"/>
-      <c r="E139" s="1" t="n"/>
+      <c r="B139" s="29" t="n"/>
+      <c r="C139" s="29" t="n"/>
+      <c r="D139" s="29" t="n"/>
+      <c r="E139" s="30" t="n"/>
     </row>
     <row r="140" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A140" s="7" t="inlineStr">
         <is>
-          <t>Rotate the R2 media token (exposed key)</t>
+          <t>AI foundations (memory, embeddings, coordination)</t>
         </is>
       </c>
       <c r="B140" s="8" t="inlineStr">
         <is>
-          <t>The R2 Access Key ID + Secret for bucket 704-discussion-media were exposed in a working chat (screenshot/paste). Scope = that one media bucket only — low blast radius, but rotate.</t>
+          <t>Supporting infra for the agents: shared memory, member embeddings, multi-agent coordination, model routing.</t>
         </is>
       </c>
       <c r="C140" s="8" t="inlineStr">
         <is>
-          <t>After 6c ships: Cloudflare -&gt; R2 -&gt; API tokens -&gt; re-create 704-discussion-upload (Object Read &amp; Write, bucket-scoped) -&gt; supabase secrets set the two new values -&gt; confirm an upload still works.</t>
-        </is>
-      </c>
-      <c r="D140" s="20" t="inlineStr">
-        <is>
-          <t>Declined</t>
+          <t>pgvector + embeddings, agent_memory, multi-agent coordination, model routing.</t>
+        </is>
+      </c>
+      <c r="D140" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
         </is>
       </c>
       <c r="E140" s="8" t="inlineStr">
         <is>
-          <t>Adam declined rotation Jul 5 - standing watch item. Key scope = one media bucket only (no member data / money / DB). Say 'rotate' anytime: ~2 min.</t>
+          <t>A later effort; supports the agents (embeddings, memory, routing).</t>
         </is>
       </c>
     </row>
     <row r="141" ht="113.4" customFormat="1" customHeight="1" s="2">
-      <c r="A141" s="7" t="inlineStr">
-        <is>
-          <t>Verify/finish the Alerts page (full history, discussion types)</t>
-        </is>
-      </c>
-      <c r="B141" s="8" t="inlineStr">
-        <is>
-          <t>Locked: bell badge clears on open, items dismiss via X, but the ALERTS PAGE keeps every notification forever - markable read (single + all). PARTIAL Jul 5: /dashboard/notifications now honors action_url (deep-links verified end to end). Remaining: full-history + mark-read behavior verification.</t>
-        </is>
-      </c>
-      <c r="C141" s="8" t="inlineStr">
-        <is>
-          <t>Read the Alerts page code; verify full-history + mark-read behavior and that all discussion notification types display with correct deep-links; fix gaps. Desktop + mobile test.</t>
-        </is>
-      </c>
-      <c r="D141" s="20" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E141" s="8" t="inlineStr">
-        <is>
-          <t>Deep-links fixed+verified Jul 5 (commit e9f6250). Remaining: verify full-history retention + mark-read (single + all).</t>
-        </is>
-      </c>
+      <c r="A141" s="4" t="inlineStr">
+        <is>
+          <t>EVENT DISCUSSION &amp; NOTIFICATIONS + JUL-5/6 FINDINGS — IN-HOUSE (NOT ON THE DEVELOPER SHEET)   ·   10 items</t>
+        </is>
+      </c>
+      <c r="B141" s="1" t="n"/>
+      <c r="D141" s="1" t="n"/>
+      <c r="E141" s="1" t="n"/>
     </row>
     <row r="142" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A142" s="7" t="inlineStr">
         <is>
-          <t>Messaging: bells for messages in existing conversations</t>
+          <t>Rotate the R2 media token (exposed key)</t>
         </is>
       </c>
       <c r="B142" s="8" t="inlineStr">
         <is>
-          <t>Messaging was resurrected Jul 5 (DMs/groups had NEVER worked since launch: RETURNING/RLS deadlock, participants-insert policy tautology, content-vs-body + title-vs-name schema mismatches, 4 missing messages columns - all fixed and verified end to end). Remaining gap: notifyNewConversation only fires on conversation CREATION, so messages into an existing thread produce no bell.</t>
+          <t>The R2 Access Key ID + Secret for bucket 704-discussion-media were exposed in a working chat (screenshot/paste). Scope = that one media bucket only — low blast radius, but rotate.</t>
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t>Add a new_message bell per message into an existing conversation, throttled (e.g. skip if an unread new_message bell for that conversation already exists).</t>
+          <t>After 6c ships: Cloudflare -&gt; R2 -&gt; API tokens -&gt; re-create 704-discussion-upload (Object Read &amp; Write, bucket-scoped) -&gt; supabase secrets set the two new values -&gt; confirm an upload still works.</t>
         </is>
       </c>
       <c r="D142" s="20" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Declined</t>
         </is>
       </c>
       <c r="E142" s="8" t="inlineStr">
         <is>
-          <t>Follow-on to the Jul 5 messaging resurrection. Recipients currently only get notified on the first-ever message.</t>
+          <t>Adam declined rotation Jul 5 - standing watch item. Key scope = one media bucket only (no member data / money / DB). Say 'rotate' anytime: ~2 min.</t>
         </is>
       </c>
     </row>
     <row r="143" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A143" s="7" t="inlineStr">
         <is>
-          <t>Messaging: attachment uploads (images/files)</t>
+          <t>Verify/finish the Alerts page (full history, discussion types)</t>
         </is>
       </c>
       <c r="B143" s="8" t="inlineStr">
         <is>
-          <t>MessagingView has image/file upload code paths and messages now has image_urls/file_urls/file_names columns (added Jul 5), but the storage wiring (bucket, upload flow) has never been tested and may not exist.</t>
+          <t>Locked: bell badge clears on open, items dismiss via X, but the ALERTS PAGE keeps every notification forever - markable read (single + all). PARTIAL Jul 5: /dashboard/notifications now honors action_url (deep-links verified end to end). Remaining: full-history + mark-read behavior verification.</t>
         </is>
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t>Audit the attachment path end to end: storage bucket, upload call, render. Fix or wire what's missing. Desktop + mobile test.</t>
+          <t>Read the Alerts page code; verify full-history + mark-read behavior and that all discussion notification types display with correct deep-links; fix gaps. Desktop + mobile test.</t>
         </is>
       </c>
       <c r="D143" s="20" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Verify</t>
         </is>
       </c>
       <c r="E143" s="8" t="inlineStr">
         <is>
-          <t>Text messaging + edits verified Jul 5; attachments explicitly skipped in that test.</t>
+          <t>Deep-links fixed+verified Jul 5 (commit e9f6250). Remaining: verify full-history retention + mark-read (single + all).</t>
         </is>
       </c>
     </row>
     <row r="144" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A144" s="7" t="inlineStr">
         <is>
+          <t>Messaging: bells for messages in existing conversations</t>
+        </is>
+      </c>
+      <c r="B144" s="8" t="inlineStr">
+        <is>
+          <t>Messaging was resurrected Jul 5 (DMs/groups had NEVER worked since launch: RETURNING/RLS deadlock, participants-insert policy tautology, content-vs-body + title-vs-name schema mismatches, 4 missing messages columns - all fixed and verified end to end). Remaining gap: notifyNewConversation only fires on conversation CREATION, so messages into an existing thread produce no bell.</t>
+        </is>
+      </c>
+      <c r="C144" s="8" t="inlineStr">
+        <is>
+          <t>Add a new_message bell per message into an existing conversation, throttled (e.g. skip if an unread new_message bell for that conversation already exists).</t>
+        </is>
+      </c>
+      <c r="D144" s="20" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E144" s="8" t="inlineStr">
+        <is>
+          <t>Follow-on to the Jul 5 messaging resurrection. Recipients currently only get notified on the first-ever message.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="46.25" customFormat="1" customHeight="1" s="2">
+      <c r="A145" s="7" t="inlineStr">
+        <is>
+          <t>Messaging: attachment uploads (images/files)</t>
+        </is>
+      </c>
+      <c r="B145" s="8" t="inlineStr">
+        <is>
+          <t>MessagingView has image/file upload code paths and messages now has image_urls/file_urls/file_names columns (added Jul 5), but the storage wiring (bucket, upload flow) has never been tested and may not exist.</t>
+        </is>
+      </c>
+      <c r="C145" s="8" t="inlineStr">
+        <is>
+          <t>Audit the attachment path end to end: storage bucket, upload call, render. Fix or wire what's missing. Desktop + mobile test.</t>
+        </is>
+      </c>
+      <c r="D145" s="20" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E145" s="8" t="inlineStr">
+        <is>
+          <t>Text messaging + edits verified Jul 5; attachments explicitly skipped in that test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="57.45" customFormat="1" customHeight="1" s="2">
+      <c r="A146" s="7" t="inlineStr">
+        <is>
           <t>Verify the first real-money admin refund (Remove &amp; Refund)</t>
         </is>
       </c>
-      <c r="B144" s="8" t="inlineStr">
+      <c r="B146" s="8" t="inlineStr">
         <is>
           <t>Admin Remove &amp; Refund shipped Jul 5 (edge fn admin-refund-ticket: admin gate, Stripe refund, void credential, seat freed; + attendee-dialog button, mobile-safe). Every branch proven EXCEPT the successful real-money refund line: void-only path, 403 gate, already-voided idempotency, and the Stripe-failure 502 fail-safe (no seat freed without money returned) all tested live.</t>
         </is>
       </c>
-      <c r="C144" s="8" t="inlineStr">
+      <c r="C146" s="8" t="inlineStr">
         <is>
           <t>WAIT mode: on the next genuine member refund request, use Remove &amp; Refund in the event attendee dialog and verify: Stripe refunded, credential voided, seat freed, toast correct.</t>
         </is>
       </c>
-      <c r="D144" s="20" t="inlineStr">
+      <c r="D146" s="20" t="inlineStr">
         <is>
           <t>Verify</t>
         </is>
       </c>
-      <c r="E144" s="8" t="inlineStr">
+      <c r="E146" s="8" t="inlineStr">
         <is>
           <t>Zero-cost proof on the next real request. Sacred Walker (Jul 5) handled manually pre-feature; her case is the template.</t>
         </is>
       </c>
     </row>
-    <row r="145" ht="46.25" customFormat="1" customHeight="1" s="2">
-      <c r="A145" s="21" t="inlineStr">
+    <row r="147" ht="57.45" customFormat="1" customHeight="1" s="2">
+      <c r="A147" s="21" t="inlineStr">
         <is>
           <t>SESSION LOG — JUL 7–9 2026 (COMPLETED; kept as record, esp. the security fix)</t>
         </is>
       </c>
-      <c r="B145" s="22" t="n"/>
-      <c r="C145" s="22" t="n"/>
-      <c r="D145" s="22" t="n"/>
-      <c r="E145" s="22" t="n"/>
-    </row>
-    <row r="146" ht="57.45" customFormat="1" customHeight="1" s="2">
-      <c r="A146" s="16" t="inlineStr">
-        <is>
-          <t>[DONE] Security: dropped anon-readable active_members view + locked event_participants_view</t>
-        </is>
-      </c>
-      <c r="B146" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL FIX Jul 9: active_members and event_participants_view were SECURITY DEFINER views with ALL privileges granted to anon — an unauthenticated internet caller could read every member's email/phone/Stripe customer ID + all attendee contact info, AND active_members (auto-updatable single-table view) exposed an anon WRITE path into profiles. active_members had ZERO callers -&gt; DROPPED. event_participants_view -&gt; security_invoker=true + REVOKE anon/authenticated (sole caller send-campaign uses service-role, unaffected). member_counts left as-is (intentional).</t>
-        </is>
-      </c>
-      <c r="C146" s="23" t="inlineStr">
-        <is>
-          <t>DONE via SQL. Verified from OUTSIDE with anon key: active_members=404, event_participants_view=401 permission denied. No rows leaked. send-campaign confirmed still works.</t>
-        </is>
-      </c>
-      <c r="D146" s="24" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E146" s="23" t="inlineStr">
-        <is>
-          <t>Biggest find of the session. Was disguised as a 'review Security Definer flags' tracker row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="57.45" customFormat="1" customHeight="1" s="2">
-      <c r="A147" s="16" t="inlineStr">
-        <is>
-          <t>[DONE] Nine-job cron auth resurrection + 2 guards, all 10 jobs healthy</t>
-        </is>
-      </c>
-      <c r="B147" s="23" t="inlineStr">
-        <is>
-          <t>Full audit found NINE broken crons (sheet knew of 2). Fixed: Vault key was legacy JWT but runtime injects sb_secret_ (updated Vault); SQL typo value-&gt;decrypted_secret on jobs 3/4/13; event-reminder had no service-key path + a no-auth-header mass-email hole (both fixed, commit 09d637d). Then built 2 guards: business-profile-reminder 14-day cooldown via contact_activity + internal-account exclusion (503548c); guest-event-match at-capacity exclusion (d722800). Both jobs 2 &amp; 10 re-enabled. All 10 cron jobs now active + healthy.</t>
-        </is>
-      </c>
-      <c r="C147" s="23" t="inlineStr">
-        <is>
-          <t>All confirmed 200 on live ticks. Guards dry-run/logic verified. WATCH: first live ticks of job 2 (14:00 UTC every 2 days) + job 10 (13:00 UTC daily) — read-only confirm right people emailed.</t>
-        </is>
-      </c>
-      <c r="D147" s="24" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E147" s="23" t="inlineStr">
-        <is>
-          <t>Commits 09d637d, 503548c, d722800 + Vault + SQL. event-reminder security hole closed.</t>
-        </is>
-      </c>
+      <c r="B147" s="22" t="n"/>
+      <c r="C147" s="22" t="n"/>
+      <c r="D147" s="22" t="n"/>
+      <c r="E147" s="22" t="n"/>
     </row>
     <row r="148" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A148" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Sentry error monitoring — live + verified in prod</t>
+          <t>[DONE] Security: dropped anon-readable active_members view + locked event_participants_view</t>
         </is>
       </c>
       <c r="B148" s="23" t="inlineStr">
         <is>
-          <t>@sentry/nextjs wired (client+server+API+global-error), CSP allowance, instrumentation moved into src/ (Next ignores root-level with a src/ dir), DSN + source-map auth token in Vercel, /admin/sentry page activated. Prod capture VERIFIED (smoke-test error landed in feed).</t>
+          <t>CRITICAL FIX Jul 9: active_members and event_participants_view were SECURITY DEFINER views with ALL privileges granted to anon — an unauthenticated internet caller could read every member's email/phone/Stripe customer ID + all attendee contact info, AND active_members (auto-updatable single-table view) exposed an anon WRITE path into profiles. active_members had ZERO callers -&gt; DROPPED. event_participants_view -&gt; security_invoker=true + REVOKE anon/authenticated (sole caller send-campaign uses service-role, unaffected). member_counts left as-is (intentional).</t>
         </is>
       </c>
       <c r="C148" s="23" t="inlineStr">
         <is>
-          <t>Verified. WATCH: confirm Sentry project SLUG is exactly '704-collective' in a Vercel build log (source-map upload) — if wrong, traces stay minified (one-word fix).</t>
+          <t>DONE via SQL. Verified from OUTSIDE with anon key: active_members=404, event_participants_view=401 permission denied. No rows leaked. send-campaign confirmed still works.</t>
         </is>
       </c>
       <c r="D148" s="24" t="inlineStr">
@@ -4056,24 +4056,24 @@
       </c>
       <c r="E148" s="23" t="inlineStr">
         <is>
-          <t>Commits 417fb37/d779885/5d12aac/b437166. The safety net — Stage 1 complete.</t>
+          <t>Biggest find of the session. Was disguised as a 'review Security Definer flags' tracker row.</t>
         </is>
       </c>
     </row>
     <row r="149" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A149" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Josh Ahart full removal (exit workstream)</t>
+          <t>[DONE] Nine-job cron auth resurrection + 2 guards, all 10 jobs healthy</t>
         </is>
       </c>
       <c r="B149" s="23" t="inlineStr">
         <is>
-          <t>De-privileged (super_admin-&gt;lead), permanent ban, all 8 sessions + 64 tokens killed, profile deactivated, ambassador row disabled, removed from public /about page (0cc8c66), 2 dormant test dupe accounts hard-deleted. Stripe sub cancelled + Connect account rejected (Adam, dashboard). Platform passwords rotated (Adam).</t>
+          <t>Full audit found NINE broken crons (sheet knew of 2). Fixed: Vault key was legacy JWT but runtime injects sb_secret_ (updated Vault); SQL typo value-&gt;decrypted_secret on jobs 3/4/13; event-reminder had no service-key path + a no-auth-header mass-email hole (both fixed, commit 09d637d). Then built 2 guards: business-profile-reminder 14-day cooldown via contact_activity + internal-account exclusion (503548c); guest-event-match at-capacity exclusion (d722800). Both jobs 2 &amp; 10 re-enabled. All 10 cron jobs now active + healthy.</t>
         </is>
       </c>
       <c r="C149" s="23" t="inlineStr">
         <is>
-          <t>Verified: role=lead, 0 sessions/tokens, banned. Public site scrubbed. Dashboard-member removal confirmed by Adam.</t>
+          <t>All confirmed 200 on live ticks. Guards dry-run/logic verified. WATCH: first live ticks of job 2 (14:00 UTC every 2 days) + job 10 (13:00 UTC daily) — read-only confirm right people emailed.</t>
         </is>
       </c>
       <c r="D149" s="24" t="inlineStr">
@@ -4083,24 +4083,24 @@
       </c>
       <c r="E149" s="23" t="inlineStr">
         <is>
-          <t>NOT on the build sheet — exit workstream. Recorded here for completeness.</t>
+          <t>Commits 09d637d, 503548c, d722800 + Vault + SQL. event-reminder security hole closed.</t>
         </is>
       </c>
     </row>
     <row r="150" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A150" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Member status batch (Jul 9)</t>
+          <t>[DONE] Sentry error monitoring — live + verified in prod</t>
         </is>
       </c>
       <c r="B150" s="23" t="inlineStr">
         <is>
-          <t>Nicholas Stathopoulos + Robert Villante -&gt; non_member/inactive/override off/lead (Nick admin revoked + sessions killed). Whitney Cleland + Brenna Dunne + Kaelah Torres -&gt; ERASED (auth+profile+people+credentials deleted; all comped, no Stripe to cancel). More status changes flagged as coming.</t>
+          <t>@sentry/nextjs wired (client+server+API+global-error), CSP allowance, instrumentation moved into src/ (Next ignores root-level with a src/ dir), DSN + source-map auth token in Vercel, /admin/sentry page activated. Prod capture VERIFIED (smoke-test error landed in feed).</t>
         </is>
       </c>
       <c r="C150" s="23" t="inlineStr">
         <is>
-          <t>All verified via SQL (zeros on erase). Read-first footprint audit confirmed safe (no owned content cascaded).</t>
+          <t>Verified. WATCH: confirm Sentry project SLUG is exactly '704-collective' in a Vercel build log (source-map upload) — if wrong, traces stay minified (one-word fix).</t>
         </is>
       </c>
       <c r="D150" s="24" t="inlineStr">
@@ -4110,24 +4110,24 @@
       </c>
       <c r="E150" s="23" t="inlineStr">
         <is>
-          <t>Adam noted more member changes coming next session.</t>
+          <t>Commits 417fb37/d779885/5d12aac/b437166. The safety net — Stage 1 complete.</t>
         </is>
       </c>
     </row>
     <row r="151" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A151" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Business-event RSVP tier leak — closed + Annslee voided</t>
+          <t>[DONE] Josh Ahart full removal (exit workstream)</t>
         </is>
       </c>
       <c r="B151" s="23" t="inlineStr">
         <is>
-          <t>Social members could RSVP business-only events: create-member-rsvp never checked required_tier, and the mobile sticky RSVP bar bypassed the desktop gate. Fixed: server-side tier gate in the edge function (ff20ba9, admins exempt) + mobile CTA respects canRsvp (952fbb2). Annslee Bottoms' live breach credential on Jul-14 Business Member Meeting VOIDED. Past legacy breaches intentionally left (real attendance history).</t>
+          <t>De-privileged (super_admin-&gt;lead), permanent ban, all 8 sessions + 64 tokens killed, profile deactivated, ambassador row disabled, removed from public /about page (0cc8c66), 2 dormant test dupe accounts hard-deleted. Stripe sub cancelled + Connect account rejected (Adam, dashboard). Platform passwords rotated (Adam).</t>
         </is>
       </c>
       <c r="C151" s="23" t="inlineStr">
         <is>
-          <t>Verified: socialtest gets 403 'business members only' + red toast; direct-invoke blocked; Annslee active count on event = 0.</t>
+          <t>Verified: role=lead, 0 sessions/tokens, banned. Public site scrubbed. Dashboard-member removal confirmed by Adam.</t>
         </is>
       </c>
       <c r="D151" s="24" t="inlineStr">
@@ -4137,24 +4137,24 @@
       </c>
       <c r="E151" s="23" t="inlineStr">
         <is>
-          <t>Commits ff20ba9, 952fbb2. Guest-side email opt-out gap noted -&gt; folds into unsubscribe policy work.</t>
+          <t>NOT on the build sheet — exit workstream. Recorded here for completeness.</t>
         </is>
       </c>
     </row>
     <row r="152" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A152" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Discussion edit/delete (comments+posts+photos) + admin always-on access</t>
+          <t>[DONE] Member status batch (Jul 9)</t>
         </is>
       </c>
       <c r="B152" s="23" t="inlineStr">
         <is>
-          <t>Owners + admins can now edit/delete their own discussion comments (ecec3f8), posts (1e3adc1), and remove their own gallery photos (bcf746f); admins moderate anyone's. '(edited)' marker, soft-delete, silent removal. Also: admins now see the discussion link on any open event regardless of RSVP (583b343 — backend was already admin-exempt; was a missing-link discovery bug). Feed/comment/DM URL linkify (561403e).</t>
+          <t>Nicholas Stathopoulos + Robert Villante -&gt; non_member/inactive/override off/lead (Nick admin revoked + sessions killed). Whitney Cleland + Brenna Dunne + Kaelah Torres -&gt; ERASED (auth+profile+people+credentials deleted; all comped, no Stripe to cancel). More status changes flagged as coming.</t>
         </is>
       </c>
       <c r="C152" s="23" t="inlineStr">
         <is>
-          <t>All browser-tested desktop+mobile. Backend RLS already permitted; these were frontend gaps.</t>
+          <t>All verified via SQL (zeros on erase). Read-first footprint audit confirmed safe (no owned content cascaded).</t>
         </is>
       </c>
       <c r="D152" s="24" t="inlineStr">
@@ -4164,122 +4164,122 @@
       </c>
       <c r="E152" s="23" t="inlineStr">
         <is>
-          <t>5 commits. Discussion feature now fully moderatable.</t>
+          <t>Adam noted more member changes coming next session.</t>
         </is>
       </c>
     </row>
     <row r="153" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A153" s="16" t="inlineStr">
         <is>
+          <t>[DONE] Business-event RSVP tier leak — closed + Annslee voided</t>
+        </is>
+      </c>
+      <c r="B153" s="23" t="inlineStr">
+        <is>
+          <t>Social members could RSVP business-only events: create-member-rsvp never checked required_tier, and the mobile sticky RSVP bar bypassed the desktop gate. Fixed: server-side tier gate in the edge function (ff20ba9, admins exempt) + mobile CTA respects canRsvp (952fbb2). Annslee Bottoms' live breach credential on Jul-14 Business Member Meeting VOIDED. Past legacy breaches intentionally left (real attendance history).</t>
+        </is>
+      </c>
+      <c r="C153" s="23" t="inlineStr">
+        <is>
+          <t>Verified: socialtest gets 403 'business members only' + red toast; direct-invoke blocked; Annslee active count on event = 0.</t>
+        </is>
+      </c>
+      <c r="D153" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E153" s="23" t="inlineStr">
+        <is>
+          <t>Commits ff20ba9, 952fbb2. Guest-side email opt-out gap noted -&gt; folds into unsubscribe policy work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A154" s="16" t="inlineStr">
+        <is>
+          <t>[DONE] Discussion edit/delete (comments+posts+photos) + admin always-on access</t>
+        </is>
+      </c>
+      <c r="B154" s="23" t="inlineStr">
+        <is>
+          <t>Owners + admins can now edit/delete their own discussion comments (ecec3f8), posts (1e3adc1), and remove their own gallery photos (bcf746f); admins moderate anyone's. '(edited)' marker, soft-delete, silent removal. Also: admins now see the discussion link on any open event regardless of RSVP (583b343 — backend was already admin-exempt; was a missing-link discovery bug). Feed/comment/DM URL linkify (561403e).</t>
+        </is>
+      </c>
+      <c r="C154" s="23" t="inlineStr">
+        <is>
+          <t>All browser-tested desktop+mobile. Backend RLS already permitted; these were frontend gaps.</t>
+        </is>
+      </c>
+      <c r="D154" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E154" s="23" t="inlineStr">
+        <is>
+          <t>5 commits. Discussion feature now fully moderatable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A155" s="16" t="inlineStr">
+        <is>
           <t>[DONE] Small fixes: hubs 404, week_label, dead components, partners 400, org_settings, last_attended</t>
         </is>
       </c>
-      <c r="B153" s="23" t="inlineStr">
+      <c r="B155" s="23" t="inlineStr">
         <is>
           <t>hubs preview widget queried non-existent 'business_hubs' -&gt; fixed to 'hubs' (a00cc50, restored a silently-broken business-tier feature). ambassador-payout phantom week_label column removed (1f46e88). 3 dead admin components deleted, 1376 lines (306efa4). partners 400 fixed via column aliasing (d95a337, latent partner-disappearing bug). organization_settings tracker row was STALE (schema fine, closed). last_attended already built+firing -&gt; backfilled 17 pre-trigger rows, closed.</t>
         </is>
       </c>
-      <c r="C153" s="23" t="inlineStr">
+      <c r="C155" s="23" t="inlineStr">
         <is>
           <t>All tsc+browser verified. org_settings &amp; last_attended were already-done rows.</t>
         </is>
       </c>
-      <c r="D153" s="24" t="inlineStr">
+      <c r="D155" s="24" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="E153" s="23" t="inlineStr">
+      <c r="E155" s="23" t="inlineStr">
         <is>
           <t>Commits a00cc50, 1f46e88, 306efa4, d95a337 + 2 SQL closes.</t>
         </is>
       </c>
     </row>
-    <row r="154" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A154" s="25" t="inlineStr">
+    <row r="156" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A156" s="25" t="inlineStr">
         <is>
           <t>PHASE 2  ·  MAJOR BUILDS (each gets its own detailed scope before build)</t>
         </is>
       </c>
-      <c r="B154" s="5" t="n"/>
-      <c r="C154" s="5" t="n"/>
-      <c r="D154" s="5" t="n"/>
-      <c r="E154" s="6" t="n"/>
-    </row>
-    <row r="155" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A155" s="4" t="inlineStr">
+      <c r="B156" s="5" t="n"/>
+      <c r="C156" s="5" t="n"/>
+      <c r="D156" s="5" t="n"/>
+      <c r="E156" s="6" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
         <is>
           <t>MAJOR BUILDS — EACH GETS ITS OWN DETAILED SCOPE BEFORE BUILD   ·   7 items</t>
         </is>
       </c>
-      <c r="B155" s="5" t="n"/>
-      <c r="C155" s="5" t="n"/>
-      <c r="D155" s="5" t="n"/>
-      <c r="E155" s="6" t="n"/>
-    </row>
-    <row r="156" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A156" s="7" t="inlineStr">
-        <is>
-          <t>CRM system</t>
-        </is>
-      </c>
-      <c r="B156" s="8" t="inlineStr">
-        <is>
-          <t>Full customer-relationship system built ON the merged person record: 360-degree member view, segments/audiences, lifecycle tracking. The internal data model IS the CRM (not a re-introduced external tool).</t>
-        </is>
-      </c>
-      <c r="C156" s="8" t="inlineStr">
-        <is>
-          <t>Own detailed scope before build.</t>
-        </is>
-      </c>
-      <c r="D156" s="26" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="E156" s="8" t="inlineStr">
-        <is>
-          <t>Built on the canonical person record from Phase 1. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag (carve-out keeps /admin/crm/campaigns live for the newsletter).</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="7" t="inlineStr">
-        <is>
-          <t>Preferred Business Network</t>
-        </is>
-      </c>
-      <c r="B157" s="8" t="inlineStr">
-        <is>
-          <t>New paid product: vetted local-business listings, $300/mo to be listed. Lives in the portal first, public domains later. Includes the internal 'Seats' system. Social members browse this to find services.</t>
-        </is>
-      </c>
-      <c r="C157" s="8" t="inlineStr">
-        <is>
-          <t>Own detailed scope before build.</t>
-        </is>
-      </c>
-      <c r="D157" s="26" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="E157" s="8" t="inlineStr">
-        <is>
-          <t>Plugs into The Network surface built in Phase 1.</t>
-        </is>
-      </c>
+      <c r="B157" s="5" t="n"/>
+      <c r="C157" s="5" t="n"/>
+      <c r="D157" s="5" t="n"/>
+      <c r="E157" s="6" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
         <is>
-          <t>Partner Portal (audit, then repurpose or remove)</t>
+          <t>CRM system</t>
         </is>
       </c>
       <c r="B158" s="8" t="inlineStr">
         <is>
-          <t>An existing, mostly-built partner portal of unclear purpose. Audit it, then either repurpose it as the Preferred Business Network management surface or remove it. Frozen until then.</t>
+          <t>Full customer-relationship system built ON the merged person record: 360-degree member view, segments/audiences, lifecycle tracking. The internal data model IS the CRM (not a re-introduced external tool).</t>
         </is>
       </c>
       <c r="C158" s="8" t="inlineStr">
@@ -4294,19 +4294,19 @@
       </c>
       <c r="E158" s="8" t="inlineStr">
         <is>
-          <t>Audit first; likely becomes the Preferred Business Network management surface. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag.</t>
+          <t>Built on the canonical person record from Phase 1. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag (carve-out keeps /admin/crm/campaigns live for the newsletter).</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
         <is>
-          <t>Task center for admins (lite project tool)</t>
+          <t>Preferred Business Network</t>
         </is>
       </c>
       <c r="B159" s="8" t="inlineStr">
         <is>
-          <t>A super-light ClickUp-style task center for admins/super-admins: create, assign, track tasks.</t>
+          <t>New paid product: vetted local-business listings, $300/mo to be listed. Lives in the portal first, public domains later. Includes the internal 'Seats' system. Social members browse this to find services.</t>
         </is>
       </c>
       <c r="C159" s="8" t="inlineStr">
@@ -4321,19 +4321,19 @@
       </c>
       <c r="E159" s="8" t="inlineStr">
         <is>
-          <t>Lite task assignment + tracking for admin / super-admin.</t>
+          <t>Plugs into The Network surface built in Phase 1.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
         <is>
-          <t>Shared email inbox view for super-admins</t>
+          <t>Partner Portal (audit, then repurpose or remove)</t>
         </is>
       </c>
       <c r="B160" s="8" t="inlineStr">
         <is>
-          <t>A shared inbox view so super-admins can see the team email (hello@) in one place.</t>
+          <t>An existing, mostly-built partner portal of unclear purpose. Audit it, then either repurpose it as the Preferred Business Network management surface or remove it. Frozen until then.</t>
         </is>
       </c>
       <c r="C160" s="8" t="inlineStr">
@@ -4348,19 +4348,19 @@
       </c>
       <c r="E160" s="8" t="inlineStr">
         <is>
-          <t>Super-admin visibility into hello@.</t>
+          <t>Audit first; likely becomes the Preferred Business Network management surface. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
         <is>
-          <t>Corporate / bulk-sales floating-seats portal</t>
+          <t>Task center for admins (lite project tool)</t>
         </is>
       </c>
       <c r="B161" s="8" t="inlineStr">
         <is>
-          <t>A portal for selling memberships in bulk to companies, with reassignable 'floating' seats.</t>
+          <t>A super-light ClickUp-style task center for admins/super-admins: create, assign, track tasks.</t>
         </is>
       </c>
       <c r="C161" s="8" t="inlineStr">
@@ -4375,19 +4375,19 @@
       </c>
       <c r="E161" s="8" t="inlineStr">
         <is>
-          <t>Reassignable floating seats for companies.</t>
+          <t>Lite task assignment + tracking for admin / super-admin.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
         <is>
-          <t>Full mobile app</t>
+          <t>Shared email inbox view for super-admins</t>
         </is>
       </c>
       <c r="B162" s="8" t="inlineStr">
         <is>
-          <t>A full native mobile application. The largest Phase 2 build.</t>
+          <t>A shared inbox view so super-admins can see the team email (hello@) in one place.</t>
         </is>
       </c>
       <c r="C162" s="8" t="inlineStr">
@@ -4402,89 +4402,89 @@
       </c>
       <c r="E162" s="8" t="inlineStr">
         <is>
-          <t>The final, largest Phase 2 effort.</t>
+          <t>Super-admin visibility into hello@.</t>
         </is>
       </c>
     </row>
     <row r="163" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A163" s="4" t="inlineStr">
-        <is>
-          <t>OPEN WATCH ITEMS — ADDED 2026-07-19   ·   8 items</t>
-        </is>
-      </c>
-      <c r="B163" s="29" t="n"/>
-      <c r="C163" s="29" t="n"/>
-      <c r="D163" s="29" t="n"/>
-      <c r="E163" s="30" t="n"/>
+      <c r="A163" s="7" t="inlineStr">
+        <is>
+          <t>Corporate / bulk-sales floating-seats portal</t>
+        </is>
+      </c>
+      <c r="B163" s="8" t="inlineStr">
+        <is>
+          <t>A portal for selling memberships in bulk to companies, with reassignable 'floating' seats.</t>
+        </is>
+      </c>
+      <c r="C163" s="8" t="inlineStr">
+        <is>
+          <t>Own detailed scope before build.</t>
+        </is>
+      </c>
+      <c r="D163" s="26" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="E163" s="8" t="inlineStr">
+        <is>
+          <t>Reassignable floating seats for companies.</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
         <is>
-          <t>Stage 5 Wave 4 - classify the ~204 guest/lead reverse-orphan profiles</t>
+          <t>Full mobile app</t>
         </is>
       </c>
       <c r="B164" s="8" t="inlineStr">
         <is>
-          <t>Waves 1-3 linked/minted the clear identity cases; the residual ~204 profiles are guests or leads that never became members and must be classified, not minted as members.</t>
+          <t>A full native mobile application. The largest Phase 2 build.</t>
         </is>
       </c>
       <c r="C164" s="8" t="inlineStr">
         <is>
-          <t>Decide the guest-vs-lead-vs-skip rule; mint people rows with the correct non-active member_status; reuse the Wave 3 additive/reversible pattern (metadata.created_by). Rehearse on develop first.</t>
-        </is>
-      </c>
-      <c r="D164" s="9" t="inlineStr">
-        <is>
-          <t>Build</t>
+          <t>Own detailed scope before build.</t>
+        </is>
+      </c>
+      <c r="D164" s="26" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="E164" s="8" t="inlineStr">
         <is>
-          <t>Waves 1-3 applied to prod. Wave 4 is the guest/lead bucket - needs a classification rule before any minting.</t>
+          <t>The final, largest Phase 2 effort.</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="7" t="inlineStr">
-        <is>
-          <t>Refill the Vercel NEXT_PUBLIC_TURNSTILE_SITE_KEY value (hardcode fallback active)</t>
-        </is>
-      </c>
-      <c r="B165" s="8" t="inlineStr">
-        <is>
-          <t>The prod env var was set to an empty string, which made the Turnstile widget render nothing and locked members out during an incident. A hardcoded public site-key fallback in TurnstileWidget.tsx currently masks the missing value.</t>
-        </is>
-      </c>
-      <c r="C165" s="8" t="inlineStr">
-        <is>
-          <t>Set the real public site key for NEXT_PUBLIC_TURNSTILE_SITE_KEY in Vercel (production), redeploy, confirm the widget renders from the env var, then optionally remove the hardcoded fallback.</t>
-        </is>
-      </c>
-      <c r="D165" s="9" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E165" s="8" t="inlineStr">
-        <is>
-          <t>Public site key (safe): 0x4AAAAAAD3gqCivsYyImeUH. Fallback keeps login working today; refill so config isn't hidden in code.</t>
-        </is>
-      </c>
+      <c r="A165" s="4" t="inlineStr">
+        <is>
+          <t>OPEN WATCH ITEMS — ADDED 2026-07-19   ·   8 items</t>
+        </is>
+      </c>
+      <c r="B165" s="29" t="n"/>
+      <c r="C165" s="29" t="n"/>
+      <c r="D165" s="29" t="n"/>
+      <c r="E165" s="30" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
         <is>
-          <t>Resolve the capacity-trigger split-brain (tickets vs attendance_credentials counting)</t>
+          <t>Stage 5 Wave 4 - classify the ~204 guest/lead reverse-orphan profiles</t>
         </is>
       </c>
       <c r="B166" s="8" t="inlineStr">
         <is>
-          <t>Event capacity is enforced by triggers on two tables (attendance_credentials and legacy tickets) that count independently, so the seated count can disagree depending on the write path.</t>
+          <t>Waves 1-3 linked/minted the clear identity cases; the residual ~204 profiles are guests or leads that never became members and must be classified, not minted as members.</t>
         </is>
       </c>
       <c r="C166" s="8" t="inlineStr">
         <is>
-          <t>Pick one source of truth (attendance_credentials); make both trigger families count consistently, or retire the legacy tickets capacity path once tickets is fully retired. Coordinates with 'Finish retiring the old ticket tables'.</t>
+          <t>Decide the guest-vs-lead-vs-skip rule; mint people rows with the correct non-active member_status; reuse the Wave 3 additive/reversible pattern (metadata.created_by). Rehearse on develop first.</t>
         </is>
       </c>
       <c r="D166" s="9" t="inlineStr">
@@ -4494,24 +4494,24 @@
       </c>
       <c r="E166" s="8" t="inlineStr">
         <is>
-          <t>The admin_override bypass now spans both trigger families; the underlying counting split remains until tickets is retired.</t>
+          <t>Waves 1-3 applied to prod. Wave 4 is the guest/lead bucket - needs a classification rule before any minting.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
         <is>
-          <t>Q6 canceled-but-paying tripwire (canceled-drift detection)</t>
+          <t>Refill the Vercel NEXT_PUBLIC_TURNSTILE_SITE_KEY value (hardcode fallback active)</t>
         </is>
       </c>
       <c r="B167" s="8" t="inlineStr">
         <is>
-          <t>Members whose app status shows canceled while Stripe still bills them (or the inverse) - a billing/status drift that should trip an alert instead of going silent.</t>
+          <t>The prod env var was set to an empty string, which made the Turnstile widget render nothing and locked members out during an incident. A hardcoded public site-key fallback in TurnstileWidget.tsx currently masks the missing value.</t>
         </is>
       </c>
       <c r="C167" s="8" t="inlineStr">
         <is>
-          <t>Add a scheduled check comparing profiles.subscription_status vs the live Stripe subscription state; alert on canceled-in-app-but-active-in-Stripe and the inverse.</t>
+          <t>Set the real public site key for NEXT_PUBLIC_TURNSTILE_SITE_KEY in Vercel (production), redeploy, confirm the widget renders from the env var, then optionally remove the hardcoded fallback.</t>
         </is>
       </c>
       <c r="D167" s="9" t="inlineStr">
@@ -4521,24 +4521,24 @@
       </c>
       <c r="E167" s="8" t="inlineStr">
         <is>
-          <t>The develop seed carries a canceled-drift (Q6) dummy for rehearsal. Folds into the DB/Stripe drift watch + admin health dashboard.</t>
+          <t>Public site key (safe): 0x4AAAAAAD3gqCivsYyImeUH. Fallback keeps login working today; refill so config isn't hidden in code.</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
         <is>
-          <t>Delete the stray Stripe Connect account</t>
+          <t>Resolve the capacity-trigger split-brain (tickets vs attendance_credentials counting)</t>
         </is>
       </c>
       <c r="B168" s="8" t="inlineStr">
         <is>
-          <t>A leftover Stripe Connect (Express) account from the ambassador / exit workstream needs removing so it doesn't linger.</t>
+          <t>Event capacity is enforced by triggers on two tables (attendance_credentials and legacy tickets) that count independently, so the seated count can disagree depending on the write path.</t>
         </is>
       </c>
       <c r="C168" s="8" t="inlineStr">
         <is>
-          <t>Confirm the account has no pending balance or payouts, then delete/reject it in the Stripe dashboard. Owner task.</t>
+          <t>Pick one source of truth (attendance_credentials); make both trigger families count consistently, or retire the legacy tickets capacity path once tickets is fully retired. Coordinates with 'Finish retiring the old ticket tables'.</t>
         </is>
       </c>
       <c r="D168" s="9" t="inlineStr">
@@ -4548,24 +4548,24 @@
       </c>
       <c r="E168" s="8" t="inlineStr">
         <is>
-          <t>Cleanup item from the ambassador / Connect work; low blast radius.</t>
+          <t>The admin_override bypass now spans both trigger families; the underlying counting split remains until tickets is retired.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
         <is>
-          <t>ManyChat - disconnect the Instagram-side integration</t>
+          <t>Q6 canceled-but-paying tripwire (canceled-drift detection)</t>
         </is>
       </c>
       <c r="B169" s="8" t="inlineStr">
         <is>
-          <t>The IG-side ManyChat connection needs to be disconnected / cleaned up. This is teardown of the current Instagram link, separate from the auto-DM build.</t>
+          <t>Members whose app status shows canceled while Stripe still bills them (or the inverse) - a billing/status drift that should trip an alert instead of going silent.</t>
         </is>
       </c>
       <c r="C169" s="8" t="inlineStr">
         <is>
-          <t>Disconnect the Instagram account from ManyChat (owner task in ManyChat / Meta); confirm no active automations still reference it.</t>
+          <t>Add a scheduled check comparing profiles.subscription_status vs the live Stripe subscription state; alert on canceled-in-app-but-active-in-Stripe and the inverse.</t>
         </is>
       </c>
       <c r="D169" s="9" t="inlineStr">
@@ -4575,491 +4575,545 @@
       </c>
       <c r="E169" s="8" t="inlineStr">
         <is>
-          <t>Distinct from the 'Instagram comment auto-DM (ManyChat)' build row above - that row stays as-is.</t>
+          <t>The develop seed carries a canceled-drift (Q6) dummy for rehearsal. Folds into the DB/Stripe drift watch + admin health dashboard.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
         <is>
-          <t>DB / Stripe drift watch items</t>
+          <t>Delete the stray Stripe Connect account</t>
         </is>
       </c>
       <c r="B170" s="8" t="inlineStr">
         <is>
-          <t>Ongoing watch on the places where the database and Stripe can drift out of sync: subscription statuses, customer email on email-change, retired legacy prices, orphaned Stripe customers.</t>
+          <t>A leftover Stripe Connect (Express) account from the ambassador / exit workstream needs removing so it doesn't linger.</t>
         </is>
       </c>
       <c r="C170" s="8" t="inlineStr">
         <is>
-          <t>Track and periodically reconcile; surface on the admin health dashboard. Pairs with the Q6 tripwire and the 'email change keeps Stripe billing in sync' verify.</t>
+          <t>Confirm the account has no pending balance or payouts, then delete/reject it in the Stripe dashboard. Owner task.</t>
         </is>
       </c>
       <c r="D170" s="9" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="E170" s="8" t="inlineStr">
         <is>
-          <t>Umbrella watch item; individual drifts get their own rows as they surface.</t>
+          <t>Cleanup item from the ambassador / Connect work; low blast radius.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
         <is>
+          <t>ManyChat - disconnect the Instagram-side integration</t>
+        </is>
+      </c>
+      <c r="B171" s="8" t="inlineStr">
+        <is>
+          <t>The IG-side ManyChat connection needs to be disconnected / cleaned up. This is teardown of the current Instagram link, separate from the auto-DM build.</t>
+        </is>
+      </c>
+      <c r="C171" s="8" t="inlineStr">
+        <is>
+          <t>Disconnect the Instagram account from ManyChat (owner task in ManyChat / Meta); confirm no active automations still reference it.</t>
+        </is>
+      </c>
+      <c r="D171" s="9" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E171" s="8" t="inlineStr">
+        <is>
+          <t>Distinct from the 'Instagram comment auto-DM (ManyChat)' build row above - that row stays as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="7" t="inlineStr">
+        <is>
+          <t>DB / Stripe drift watch items</t>
+        </is>
+      </c>
+      <c r="B172" s="8" t="inlineStr">
+        <is>
+          <t>Ongoing watch on the places where the database and Stripe can drift out of sync: subscription statuses, customer email on email-change, retired legacy prices, orphaned Stripe customers.</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="inlineStr">
+        <is>
+          <t>Track and periodically reconcile; surface on the admin health dashboard. Pairs with the Q6 tripwire and the 'email change keeps Stripe billing in sync' verify.</t>
+        </is>
+      </c>
+      <c r="D172" s="9" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="E172" s="8" t="inlineStr">
+        <is>
+          <t>Umbrella watch item; individual drifts get their own rows as they surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="7" t="inlineStr">
+        <is>
           <t>Waitlist claim links - monitor first real-world use</t>
         </is>
       </c>
-      <c r="B171" s="8" t="inlineStr">
+      <c r="B173" s="8" t="inlineStr">
         <is>
           <t>Cancel frees a seat -&gt; the first waitlister is emailed a 24h claim link -&gt; they claim it. Rehearsed as a full matrix on develop and shipped to prod; needs a read-only confirm on its first genuine use.</t>
         </is>
       </c>
-      <c r="C171" s="8" t="inlineStr">
+      <c r="C173" s="8" t="inlineStr">
         <is>
           <t>On the next real cancellation that frees a seat on a full, waitlisted event, confirm: notified_at/expires_at stamped, the email sent, the claimant claimed (member_rsvp with metadata source=waitlist_claim), and the waitlist row deleted.</t>
         </is>
       </c>
-      <c r="D171" s="9" t="inlineStr">
+      <c r="D173" s="9" t="inlineStr">
         <is>
           <t>Verify</t>
         </is>
       </c>
-      <c r="E171" s="8" t="inlineStr">
+      <c r="E173" s="8" t="inlineStr">
         <is>
           <t>Shipped 2026-07-19. Zero-cost proof on first real use, like the Remove &amp; Refund WAIT-mode row.</t>
         </is>
       </c>
     </row>
-    <row r="172">
-      <c r="A172" s="27" t="inlineStr">
+    <row r="174">
+      <c r="A174" s="27" t="inlineStr">
         <is>
           <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
-      <c r="B172" s="27" t="inlineStr">
+      <c r="B174" s="27" t="inlineStr">
         <is>
           <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
-      <c r="C172" s="27" t="inlineStr">
+      <c r="C174" s="27" t="inlineStr">
         <is>
           <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
-      <c r="D172" s="27" t="inlineStr">
+      <c r="D174" s="27" t="inlineStr">
         <is>
           <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
-      <c r="E172" s="27" t="inlineStr">
+      <c r="E174" s="27" t="inlineStr">
         <is>
           <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="28" t="inlineStr">
-        <is>
-          <t>Billing views: admin billing panel + member price/renewal display</t>
-        </is>
-      </c>
-      <c r="B173" s="28" t="inlineStr">
-        <is>
-          <t>Admin contact billing panel + member-facing price/renewal display. Three new profile columns (comp_reason, external_paid_through, external_payment_note) are live on both DBs; the UI/code build is in flight.</t>
-        </is>
-      </c>
-      <c r="C173" s="28" t="inlineStr">
-        <is>
-          <t>Extend admin contact detail with live Stripe billing; surface price/renewal/discount on member settings; wire the three new profile columns into admin editors.</t>
-        </is>
-      </c>
-      <c r="D173" s="28" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
-        </is>
-      </c>
-      <c r="E173" s="28" t="inlineStr">
-        <is>
-          <t>Columns live both DBs; code build in flight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="28" t="inlineStr">
-        <is>
-          <t>Report builder: admin/super_admin any-filter member/payment reports</t>
-        </is>
-      </c>
-      <c r="B174" s="28" t="inlineStr">
-        <is>
-          <t>Admin/super_admin reporting with arbitrary filters over members and payments. Data-cleanup prerequisite is DONE; build after billing views.</t>
-        </is>
-      </c>
-      <c r="C174" s="28" t="inlineStr">
-        <is>
-          <t>Build after billing views lands. Admin/super_admin only; any-filter member + payment reports.</t>
-        </is>
-      </c>
-      <c r="D174" s="28" t="inlineStr">
-        <is>
-          <t>QUEUED-BACKLOGGED</t>
-        </is>
-      </c>
-      <c r="E174" s="28" t="inlineStr">
-        <is>
-          <t>v1 proposal complete and approved-in-principle (DB-only cut, 3 entities, column picker, CSV export, 4 presets, server-paginated, ~7 files); resume at build sign-off. Cheap adds discussed: ambassador-referred, price tier, cancel reasons.</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="28" t="inlineStr">
         <is>
-          <t>Business comp invite flow: welcome template + admin invite tool</t>
+          <t>Billing views: admin billing panel + member price/renewal display</t>
         </is>
       </c>
       <c r="B175" s="28" t="inlineStr">
         <is>
-          <t>Welcome email template plus an admin tool to invite a business member (comp path).</t>
+          <t>Admin contact billing panel + member-facing price/renewal display. Three new profile columns (comp_reason, external_paid_through, external_payment_note) are live on both DBs; the UI/code build is in flight.</t>
         </is>
       </c>
       <c r="C175" s="28" t="inlineStr">
         <is>
-          <t>Blocked on Adam: invitee list + design answers. Then template + admin invite UI.</t>
+          <t>Extend admin contact detail with live Stripe billing; surface price/renewal/discount on member settings; wire the three new profile columns into admin editors.</t>
         </is>
       </c>
       <c r="D175" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: list + design answers</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="E175" s="28" t="inlineStr">
         <is>
-          <t>Needs invitee list + design answers from Adam.</t>
+          <t>Columns live both DBs; code build in flight.</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="28" t="inlineStr">
         <is>
-          <t>Admin 'Invite comp member' button - form (name, company, email, phone, comp note), creates comp'd account + sends welcome email, note auto-attached to billing view (member + admin); v1 invite flow built without UI, button is the addon</t>
+          <t>Report builder: admin/super_admin any-filter member/payment reports</t>
         </is>
       </c>
       <c r="B176" s="28" t="inlineStr">
         <is>
-          <t>Admin UI button/form to invite a complimentary business member: name, company, email, phone, and comp note. Creates the comp'd account, sends the welcome email, and attaches the note to the billing view for both member and admin.</t>
+          <t>Admin/super_admin reporting with arbitrary filters over members and payments. Data-cleanup prerequisite is DONE; build after billing views.</t>
         </is>
       </c>
       <c r="C176" s="28" t="inlineStr">
         <is>
-          <t>Addon after v1 invite flow (API/ops path without UI). Build the Invite comp member button + form once the headless invite path exists.</t>
+          <t>Build after billing views lands. Admin/super_admin only; any-filter member + payment reports.</t>
         </is>
       </c>
       <c r="D176" s="28" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>QUEUED-BACKLOGGED</t>
         </is>
       </c>
       <c r="E176" s="28" t="inlineStr">
         <is>
-          <t>v1 invite flow built without UI; this button is the future addon.</t>
+          <t>v1 proposal complete and approved-in-principle (DB-only cut, 3 entities, column picker, CSV export, 4 presets, server-paginated, ~7 files); resume at build sign-off. Cheap adds discussed: ambassador-referred, price tier, cancel reasons.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="28" t="inlineStr">
         <is>
-          <t>Mike Perez: account cleanup + re-join link at $150 founding</t>
+          <t>Business comp invite flow: welcome template + admin invite tool</t>
         </is>
       </c>
       <c r="B177" s="28" t="inlineStr">
         <is>
-          <t>After Adam's conversation: clean up Mike's canceled/failed-billing account and send a founding-rate $150 re-join link.</t>
+          <t>Welcome email template plus an admin tool to invite a business member (comp path).</t>
         </is>
       </c>
       <c r="C177" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM conversation first. Then cleanup + founding $150 checkout/re-join link.</t>
+          <t>Blocked on Adam: invitee list + design answers. Then template + admin invite UI.</t>
         </is>
       </c>
       <c r="D177" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: conversation first</t>
+          <t>WAITING ON ADAM: list + design answers</t>
         </is>
       </c>
       <c r="E177" s="28" t="inlineStr">
         <is>
-          <t>Founding $150; conversation first.</t>
+          <t>Needs invitee list + design answers from Adam.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="28" t="inlineStr">
         <is>
-          <t>Zane Mackey comp_reason entry</t>
+          <t>Admin 'Invite comp member' button - form (name, company, email, phone, comp note), creates comp'd account + sends welcome email, note auto-attached to billing view (member + admin); v1 invite flow built without UI, button is the addon</t>
         </is>
       </c>
       <c r="B178" s="28" t="inlineStr">
         <is>
-          <t>Record a one-phrase comp_reason on Zane Mackey's profile now that the column exists.</t>
+          <t>Admin UI button/form to invite a complimentary business member: name, company, email, phone, and comp note. Creates the comp'd account, sends the welcome email, and attaches the note to the billing view for both member and admin.</t>
         </is>
       </c>
       <c r="C178" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: one phrase for comp_reason.</t>
+          <t>Addon after v1 invite flow (API/ops path without UI). Build the Invite comp member button + form once the headless invite path exists.</t>
         </is>
       </c>
       <c r="D178" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: one phrase</t>
+          <t>QUEUED</t>
         </is>
       </c>
       <c r="E178" s="28" t="inlineStr">
         <is>
-          <t>One phrase for comp_reason.</t>
+          <t>v1 invite flow built without UI; this button is the future addon.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="28" t="inlineStr">
         <is>
-          <t>Zach Trusky renewal ~Nov/Dec 2026 — honored $1,034 annual</t>
+          <t>Mike Perez: account cleanup + re-join link at $150 founding</t>
         </is>
       </c>
       <c r="B179" s="28" t="inlineStr">
         <is>
-          <t>Zach's annual amount lives outside Stripe ($1,034 honored). Need reminder + collection path decision around Nov/Dec 2026.</t>
+          <t>After Adam's conversation: clean up Mike's canceled/failed-billing account and send a founding-rate $150 re-join link.</t>
         </is>
       </c>
       <c r="C179" s="28" t="inlineStr">
         <is>
-          <t>Schedule reminder; decide collection path (manual invoice vs Stripe annual vs override).</t>
+          <t>WAITING ON ADAM conversation first. Then cleanup + founding $150 checkout/re-join link.</t>
         </is>
       </c>
       <c r="D179" s="28" t="inlineStr">
         <is>
-          <t>SCHEDULED NOV 2026</t>
+          <t>WAITING ON ADAM: conversation first</t>
         </is>
       </c>
       <c r="E179" s="28" t="inlineStr">
         <is>
-          <t>Honored $1,034 annual; no Stripe customer today.</t>
+          <t>Founding $150; conversation first.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="28" t="inlineStr">
         <is>
-          <t>Security: unknown third-party script (batatatech.com) on Glue Up admin pages</t>
+          <t>Zane Mackey comp_reason entry</t>
         </is>
       </c>
       <c r="B180" s="28" t="inlineStr">
         <is>
-          <t>Unknown batatatech.com script firing on Glue Up admin pages — treat as extension/malware until proven otherwise; audit browsers + rotate passwords.</t>
+          <t>Record a one-phrase comp_reason on Zane Mackey's profile now that the column exists.</t>
         </is>
       </c>
       <c r="C180" s="28" t="inlineStr">
         <is>
-          <t>Browser extension audit on machines that use Glue Up admin; password rotation for affected accounts.</t>
+          <t>WAITING ON ADAM: one phrase for comp_reason.</t>
         </is>
       </c>
       <c r="D180" s="28" t="inlineStr">
         <is>
-          <t>OPEN - Adam chrome://extensions only</t>
+          <t>WAITING ON ADAM: one phrase</t>
         </is>
       </c>
       <c r="E180" s="28" t="inlineStr">
         <is>
-          <t>repo confirmed clean 8/4 - scope is Adam's chrome://extensions only</t>
+          <t>One phrase for comp_reason.</t>
         </is>
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>[DONE] Promo system endstate 8/5</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>Supersedes Stripe support ticket + ticket-checkout promo fast-follow (removed).</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
+      <c r="A181" s="28" t="inlineStr">
+        <is>
+          <t>Zach Trusky renewal ~Nov/Dec 2026 — honored $1,034 annual</t>
+        </is>
+      </c>
+      <c r="B181" s="28" t="inlineStr">
+        <is>
+          <t>Zach's annual amount lives outside Stripe ($1,034 honored). Need reminder + collection path decision around Nov/Dec 2026.</t>
+        </is>
+      </c>
+      <c r="C181" s="28" t="inlineStr">
+        <is>
+          <t>Schedule reminder; decide collection path (manual invoice vs Stripe annual vs override).</t>
+        </is>
+      </c>
+      <c r="D181" s="28" t="inlineStr">
+        <is>
+          <t>SCHEDULED NOV 2026</t>
+        </is>
+      </c>
+      <c r="E181" s="28" t="inlineStr">
+        <is>
+          <t>Honored $1,034 annual; no Stripe customer today.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="28" t="inlineStr">
         <is>
-          <t>Calendar update-leg verification via throwaway event</t>
+          <t>Security: unknown third-party script (batatatech.com) on Glue Up admin pages</t>
         </is>
       </c>
       <c r="B182" s="28" t="inlineStr">
         <is>
-          <t>Verify that event-edit REQUEST invites actually move real calendars (ICS sequence / update leg) using a throwaway event.</t>
+          <t>Unknown batatatech.com script firing on Glue Up admin pages — treat as extension/malware until proven otherwise; audit browsers + rotate passwords.</t>
         </is>
       </c>
       <c r="C182" s="28" t="inlineStr">
         <is>
-          <t>Create throwaway event, subscribe, edit, confirm calendars update; then delete throwaway.</t>
+          <t>Browser extension audit on machines that use Glue Up admin; password rotation for affected accounts.</t>
         </is>
       </c>
       <c r="D182" s="28" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - Adam chrome://extensions only</t>
         </is>
       </c>
       <c r="E182" s="28" t="inlineStr">
         <is>
-          <t>Throwaway event verification of REQUEST/update path.</t>
+          <t>repo confirmed clean 8/4 - scope is Adam's chrome://extensions only</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="28" t="inlineStr">
-        <is>
-          <t>Resend click-tracking subdomain (DNS)</t>
-        </is>
-      </c>
-      <c r="B183" s="28" t="inlineStr">
-        <is>
-          <t>Configure Resend click-tracking subdomain — Adam hands / DNS.</t>
-        </is>
-      </c>
-      <c r="C183" s="28" t="inlineStr">
-        <is>
-          <t>ADAM DNS: add Resend click-tracking subdomain CNAME + add Resend to SPF include (current SPF is Google-only). Confirmed missing 8/4.</t>
-        </is>
-      </c>
-      <c r="D183" s="28" t="inlineStr">
-        <is>
-          <t>ADAM - DNS</t>
-        </is>
-      </c>
-      <c r="E183" s="28" t="inlineStr">
-        <is>
-          <t>confirmed NOT configured 8/4; also add Resend to SPF include during same DNS visit</t>
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>[DONE] Promo system endstate 8/5</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Supersedes Stripe support ticket + ticket-checkout promo fast-follow (removed).</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="28" t="inlineStr">
         <is>
-          <t>/welcome checkout-flow coverage on develop</t>
+          <t>Calendar update-leg verification via throwaway event</t>
         </is>
       </c>
       <c r="B184" s="28" t="inlineStr">
         <is>
-          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
+          <t>Verify that event-edit REQUEST invites actually move real calendars (ICS sequence / update leg) using a throwaway event.</t>
         </is>
       </c>
       <c r="C184" s="28" t="inlineStr">
         <is>
-          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
+          <t>Create throwaway event, subscribe, edit, confirm calendars update; then delete throwaway.</t>
         </is>
       </c>
       <c r="D184" s="28" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="E184" s="28" t="inlineStr">
         <is>
-          <t>Untested on develop; no Stripe checkout env.</t>
+          <t>Throwaway event verification of REQUEST/update path.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="28" t="inlineStr">
         <is>
-          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
+          <t>Resend click-tracking subdomain (DNS)</t>
         </is>
       </c>
       <c r="B185" s="28" t="inlineStr">
         <is>
-          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
+          <t>Configure Resend click-tracking subdomain — Adam hands / DNS.</t>
         </is>
       </c>
       <c r="C185" s="28" t="inlineStr">
         <is>
-          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
+          <t>ADAM DNS: add Resend click-tracking subdomain CNAME + add Resend to SPF include (current SPF is Google-only). Confirmed missing 8/4.</t>
         </is>
       </c>
       <c r="D185" s="28" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>ADAM - DNS</t>
         </is>
       </c>
       <c r="E185" s="28" t="inlineStr">
         <is>
-          <t>Revisit in identity-bridge work.</t>
+          <t>confirmed NOT configured 8/4; also add Resend to SPF include during same DNS visit</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="28" t="inlineStr">
         <is>
-          <t>Retire the Google Sheets tracker path</t>
+          <t>/welcome checkout-flow coverage on develop</t>
         </is>
       </c>
       <c r="B186" s="28" t="inlineStr">
         <is>
-          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
+          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
         </is>
       </c>
       <c r="C186" s="28" t="inlineStr">
         <is>
-          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
+          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
         </is>
       </c>
       <c r="D186" s="28" t="inlineStr">
         <is>
-          <t>QUEUED - cleanup</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="E186" s="28" t="inlineStr">
         <is>
-          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
+          <t>Untested on develop; no Stripe checkout env.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="28" t="inlineStr">
         <is>
+          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
+        </is>
+      </c>
+      <c r="B187" s="28" t="inlineStr">
+        <is>
+          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
+        </is>
+      </c>
+      <c r="C187" s="28" t="inlineStr">
+        <is>
+          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
+        </is>
+      </c>
+      <c r="D187" s="28" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="E187" s="28" t="inlineStr">
+        <is>
+          <t>Revisit in identity-bridge work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="28" t="inlineStr">
+        <is>
+          <t>Retire the Google Sheets tracker path</t>
+        </is>
+      </c>
+      <c r="B188" s="28" t="inlineStr">
+        <is>
+          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
+        </is>
+      </c>
+      <c r="C188" s="28" t="inlineStr">
+        <is>
+          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
+        </is>
+      </c>
+      <c r="D188" s="28" t="inlineStr">
+        <is>
+          <t>QUEUED - cleanup</t>
+        </is>
+      </c>
+      <c r="E188" s="28" t="inlineStr">
+        <is>
+          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="28" t="inlineStr">
+        <is>
           <t>Admin card PATCH date normalization - external dates should save as noon UTC to avoid timezone off-by-one (Zach precedent)</t>
         </is>
       </c>
-      <c r="B187" s="28" t="inlineStr">
+      <c r="B189" s="28" t="inlineStr">
         <is>
           <t>external_paid_through saved as midnight UTC displays as prior calendar day in US Eastern (Zach showed Nov 30 instead of Dec 1). Admin billing PATCH should normalize date-only inputs to noon UTC.</t>
         </is>
       </c>
-      <c r="C187" s="28" t="inlineStr">
+      <c r="C189" s="28" t="inlineStr">
         <is>
           <t>In PATCH /api/admin/members/[id]/billing (and any similar writers), coerce external_paid_through date-only values to YYYY-MM-DDT12:00:00.000Z before save. SMALL.</t>
         </is>
       </c>
-      <c r="D187" s="28" t="inlineStr">
+      <c r="D189" s="28" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="E187" s="28" t="inlineStr">
+      <c r="E189" s="28" t="inlineStr">
         <is>
           <t>SMALL/OPEN. Precedent: Zach Trusky external_paid_through 2026-12-01T00:00:00Z → Nov 30 in America/New_York.</t>
         </is>

</xml_diff>

<commit_message>
chore: tracker - repair merged cell ranges, set row 96 status
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -2124,10 +2124,10 @@
           <t>ADMIN &amp; OPERATIONS   ·   10 items</t>
         </is>
       </c>
-      <c r="B64" s="5" t="n"/>
-      <c r="C64" s="5" t="n"/>
-      <c r="D64" s="5" t="n"/>
-      <c r="E64" s="6" t="n"/>
+      <c r="B64" s="29" t="n"/>
+      <c r="C64" s="29" t="n"/>
+      <c r="D64" s="29" t="n"/>
+      <c r="E64" s="30" t="n"/>
     </row>
     <row r="65" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A65" s="7" t="inlineStr">
@@ -2876,24 +2876,9 @@
           <t>Branded auth links (stop showing supabase.co URLs)</t>
         </is>
       </c>
-      <c r="B96" s="5" t="inlineStr">
-        <is>
-          <t>Every auth link we send (invite, password reset, magic link) points at bnmtynevbuplqpuqvmna.supabase.co. Looks untrustworthy in texts and emails, and the domain mismatch hurts link reputation with Gmail and Outlook.</t>
-        </is>
-      </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>Ship Option A first: a server-side /invite route on 704collective.com that accepts only a token and redirects to the hardcoded Supabase verify URL. No open-redirect parameter. Rehearse on develop, desktop 1440x900 and mobile 390x844. ENDGAME is Option B, the Supabase custom auth domain add-on (auth.704collective.com), which fixes every auth email with no redirect hop. Option B changes the project auth URL and touches env vars, redirect allow-lists and the JWT issuer, so it needs a planned window and a rollback plan.</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E96" s="6" t="inlineStr">
-        <is>
-          <t>Raised 2026-08-06 while hand-minting comp-invite links for Brandon Aruta and Davis Baxter to send by text.</t>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Build</t>
         </is>
       </c>
     </row>
@@ -3071,26 +3056,6 @@
           <t>Reduce redundant Stripe scans</t>
         </is>
       </c>
-      <c r="B105" s="8" t="inlineStr">
-        <is>
-          <t>Cut how often the system scans Stripe, for performance/cost.</t>
-        </is>
-      </c>
-      <c r="C105" s="8" t="inlineStr">
-        <is>
-          <t>Reduce Stripe API scan frequency.</t>
-        </is>
-      </c>
-      <c r="D105" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E105" s="8" t="inlineStr">
-        <is>
-          <t>Cut scan frequency for cost / performance.</t>
-        </is>
-      </c>
     </row>
     <row r="106" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A106" s="7" t="inlineStr">
@@ -3417,26 +3382,6 @@
           <t>Merge guest follow-up into the drip processor</t>
         </is>
       </c>
-      <c r="B119" s="8" t="inlineStr">
-        <is>
-          <t>Retire the separate guest-followup function and fold it into the main processor.</t>
-        </is>
-      </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t>Consolidate guest-followup into process-drips.</t>
-        </is>
-      </c>
-      <c r="D119" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E119" s="8" t="inlineStr">
-        <is>
-          <t>Fold guest-followup into process-drips.</t>
-        </is>
-      </c>
     </row>
     <row r="120" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A120" s="7" t="inlineStr">
@@ -3574,10 +3519,6 @@
           <t>Delete dead admin member components</t>
         </is>
       </c>
-      <c r="B126" s="5" t="n"/>
-      <c r="C126" s="5" t="n"/>
-      <c r="D126" s="5" t="n"/>
-      <c r="E126" s="6" t="n"/>
     </row>
     <row r="127" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
       <c r="A127" s="4" t="inlineStr">
@@ -3585,10 +3526,10 @@
           <t>MARKETING &amp; FRONT-END   ·   10 items</t>
         </is>
       </c>
-      <c r="B127" s="5" t="n"/>
-      <c r="C127" s="5" t="n"/>
-      <c r="D127" s="5" t="n"/>
-      <c r="E127" s="6" t="n"/>
+      <c r="B127" s="29" t="n"/>
+      <c r="C127" s="29" t="n"/>
+      <c r="D127" s="29" t="n"/>
+      <c r="E127" s="30" t="n"/>
     </row>
     <row r="128" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A128" s="7" t="inlineStr">
@@ -3823,10 +3764,6 @@
           <t>Instagram comment auto-DM (ManyChat)</t>
         </is>
       </c>
-      <c r="B137" s="5" t="n"/>
-      <c r="C137" s="5" t="n"/>
-      <c r="D137" s="5" t="n"/>
-      <c r="E137" s="6" t="n"/>
     </row>
     <row r="138" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A138" s="4" t="inlineStr">
@@ -3834,10 +3771,10 @@
           <t>AI / AGENTS (LATER EFFORT)   ·   2 items</t>
         </is>
       </c>
-      <c r="B138" s="5" t="n"/>
-      <c r="C138" s="5" t="n"/>
-      <c r="D138" s="5" t="n"/>
-      <c r="E138" s="6" t="n"/>
+      <c r="B138" s="29" t="n"/>
+      <c r="C138" s="29" t="n"/>
+      <c r="D138" s="29" t="n"/>
+      <c r="E138" s="30" t="n"/>
     </row>
     <row r="139" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A139" s="7" t="inlineStr">
@@ -3883,9 +3820,10 @@
           <t>EVENT DISCUSSION &amp; NOTIFICATIONS + JUL-5/6 FINDINGS — IN-HOUSE (NOT ON THE DEVELOPER SHEET)   ·   10 items</t>
         </is>
       </c>
-      <c r="B141" s="1" t="n"/>
-      <c r="D141" s="1" t="n"/>
-      <c r="E141" s="1" t="n"/>
+      <c r="B141" s="29" t="n"/>
+      <c r="C141" s="29" t="n"/>
+      <c r="D141" s="29" t="n"/>
+      <c r="E141" s="30" t="n"/>
     </row>
     <row r="142" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A142" s="7" t="inlineStr">
@@ -4028,10 +3966,6 @@
           <t>SESSION LOG — JUL 7–9 2026 (COMPLETED; kept as record, esp. the security fix)</t>
         </is>
       </c>
-      <c r="B147" s="22" t="n"/>
-      <c r="C147" s="22" t="n"/>
-      <c r="D147" s="22" t="n"/>
-      <c r="E147" s="22" t="n"/>
     </row>
     <row r="148" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A148" s="16" t="inlineStr">
@@ -4255,10 +4189,10 @@
           <t>PHASE 2  ·  MAJOR BUILDS (each gets its own detailed scope before build)</t>
         </is>
       </c>
-      <c r="B156" s="5" t="n"/>
-      <c r="C156" s="5" t="n"/>
-      <c r="D156" s="5" t="n"/>
-      <c r="E156" s="6" t="n"/>
+      <c r="B156" s="29" t="n"/>
+      <c r="C156" s="29" t="n"/>
+      <c r="D156" s="29" t="n"/>
+      <c r="E156" s="30" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -4266,10 +4200,10 @@
           <t>MAJOR BUILDS — EACH GETS ITS OWN DETAILED SCOPE BEFORE BUILD   ·   7 items</t>
         </is>
       </c>
-      <c r="B157" s="5" t="n"/>
-      <c r="C157" s="5" t="n"/>
-      <c r="D157" s="5" t="n"/>
-      <c r="E157" s="6" t="n"/>
+      <c r="B157" s="29" t="n"/>
+      <c r="C157" s="29" t="n"/>
+      <c r="D157" s="29" t="n"/>
+      <c r="E157" s="30" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -4410,26 +4344,6 @@
       <c r="A163" s="7" t="inlineStr">
         <is>
           <t>Corporate / bulk-sales floating-seats portal</t>
-        </is>
-      </c>
-      <c r="B163" s="8" t="inlineStr">
-        <is>
-          <t>A portal for selling memberships in bulk to companies, with reassignable 'floating' seats.</t>
-        </is>
-      </c>
-      <c r="C163" s="8" t="inlineStr">
-        <is>
-          <t>Own detailed scope before build.</t>
-        </is>
-      </c>
-      <c r="D163" s="26" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="E163" s="8" t="inlineStr">
-        <is>
-          <t>Reassignable floating seats for companies.</t>
         </is>
       </c>
     </row>
@@ -4693,26 +4607,6 @@
           <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
-      <c r="B174" s="27" t="inlineStr">
-        <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
-        </is>
-      </c>
-      <c r="C174" s="27" t="inlineStr">
-        <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
-        </is>
-      </c>
-      <c r="D174" s="27" t="inlineStr">
-        <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
-        </is>
-      </c>
-      <c r="E174" s="27" t="inlineStr">
-        <is>
-          <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" s="28" t="inlineStr">
@@ -5120,28 +5014,33 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="26">
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A157:E157"/>
+    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="A98:E98"/>
     <mergeCell ref="A60:E60"/>
-    <mergeCell ref="A98:E98"/>
     <mergeCell ref="A51:E51"/>
-    <mergeCell ref="A119:E119"/>
+    <mergeCell ref="A107:E107"/>
+    <mergeCell ref="A138:E138"/>
     <mergeCell ref="A90:E90"/>
-    <mergeCell ref="A137:E137"/>
+    <mergeCell ref="A174:E174"/>
     <mergeCell ref="A84:E84"/>
     <mergeCell ref="A74:E74"/>
-    <mergeCell ref="A105:E105"/>
     <mergeCell ref="A55:E55"/>
-    <mergeCell ref="A163:E163"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A126:E126"/>
-    <mergeCell ref="A96:E96"/>
-    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A141:E141"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A100:E100"/>
+    <mergeCell ref="A156:E156"/>
+    <mergeCell ref="A147:E147"/>
+    <mergeCell ref="A165:E165"/>
+    <mergeCell ref="A121:E121"/>
     <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A127:E127"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
chore: tracker - add Exchange intake viewer and send-campaign member exclusion as top priorities
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E189"/>
+  <dimension ref="A1:E191"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="1" min="1" max="1"/>
@@ -2121,7 +2121,7 @@
     <row r="64" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>ADMIN &amp; OPERATIONS   ·   10 items</t>
+          <t>ADMIN &amp; OPERATIONS   ·   12 items</t>
         </is>
       </c>
       <c r="B64" s="29" t="n"/>
@@ -2132,17 +2132,17 @@
     <row r="65" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>Add a private notes section on each member</t>
+          <t>PRIORITY 1: Exchange intake viewer (admin)</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>Internal request: a notes area per member for context (e.g. 'comped through August').</t>
+          <t>The Exchange intake forms are live and collecting registrations into the exchange_intake table, but there is NO way to see any of it in the admin UI. Right now the only way to read who registered, what they answered, or how full each pool is, is to run raw SQL. This is needed before Aug 27 and is the foundation the speed-networking matching engine will read from.</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>Read: admin + super-admin. Write/edit: super-admin only. Not member-visible.</t>
+          <t>Build an admin page (suggested /admin/exchange or a tab on the event detail admin view) that lists exchange_intake rows for a given event. Must show: name, email, phone, form_variant (public / commonwealth / invited), pool (house / commonwealth), participation (business_and_social / social_only), member_status_at_submit, status (invited / submitted), submitted_at, and all four free-text answers (q_role_title, q_company, q_years_charlotte, q_seeking). Needs: live pool counters (house X of 60, commonwealth Y of 60), filter by pool and participation, CSV export, and a view of which invited members have not yet submitted. RLS already allows admin/super_admin SELECT on exchange_intake. Read before write - the table already exists on both prod and develop.</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
@@ -2152,24 +2152,24 @@
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>Internal-only; super-admin writes, admins read, members never see it.</t>
+          <t>TOP PRIORITY. Raised 2026-08-12 immediately after the intake forms shipped. Event is Aug 27 2026. Table: exchange_intake, event id 02afde72-33c4-4c99-8dba-0ea5a8c0a723.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>Build the admin health dashboard</t>
+          <t>PRIORITY 2: send-campaign all_contacts audience includes paying members</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>One screen showing system health at a glance; catches silent failures before members do.</t>
+          <t>The 'All Contacts' audience in the campaign tool pulls every row from the contacts table and filters ONLY on unsubscribed. It does not exclude members. On prod, 89 of 207 contacts are also active members (over 40 percent overlap), so any All Contacts campaign sends prospect-facing copy to people who already pay. A 'join 704 Collective' style blast would pitch membership to existing members.</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>5 widgets — cron, webhooks, drip health, email tracking, payment sync. Sits on /api/health.</t>
+          <t>In supabase/functions/send-campaign/index.ts, the all_contacts branch (approx lines 478-489) selects contacts where unsubscribed is null or false, with no membership filter. Add an exclusion so contacts whose email matches a non-deleted profile with subscription_status active or trialing or membership_override true are removed from that audience. Consider whether the segment audience (tag-based, approx lines 490-506) needs the same treatment. Related dead code found the same night: converted_to_member_id is never written by any code, so the conversion-rate report on /admin/crm/reports measures nothing, and the campaigns audience preview counts contact_type = 'guest' which zero rows have, so it always shows 0. Rehearse on develop both viewports before shipping.</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
@@ -2179,24 +2179,24 @@
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>Reads /api/health + checks; surfaces silent failures.</t>
+          <t>Raised 2026-08-12 during a contacts table audit. Not known whether any past campaign used this audience. Timi should be told to avoid All Contacts until fixed.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>Let admins change a member's tier and have billing follow</t>
+          <t>Add a private notes section on each member</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>App-side tier change/comp exists; the Stripe billing side doesn't follow.</t>
+          <t>Internal request: a notes area per member for context (e.g. 'comped through August').</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Wire admin tier-change to Stripe subscription cancel/modify/start.</t>
+          <t>Read: admin + super-admin. Write/edit: super-admin only. Not member-visible.</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
@@ -2206,24 +2206,24 @@
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>App-side override already exists; this is the Stripe billing reconciliation.</t>
+          <t>Internal-only; super-admin writes, admins read, members never see it.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>Harden the admin cancel-subscription flow</t>
+          <t>Build the admin health dashboard</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>Make admin cancel safe (running twice shouldn't double-act).</t>
+          <t>One screen showing system health at a glance; catches silent failures before members do.</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>Add idempotency + structured logging + alert to admin-cancel-subscription.</t>
+          <t>5 widgets — cron, webhooks, drip health, email tracking, payment sync. Sits on /api/health.</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
@@ -2233,24 +2233,24 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>Idempotent + logged + alerted so a double-run can't double-act.</t>
+          <t>Reads /api/health + checks; surfaces silent failures.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>Build the admin area into clean sections</t>
+          <t>Let admins change a member's tier and have billing follow</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>Reorganize admin into Today / People / Events / Network / Money / Messages / Settings with one source of truth per question.</t>
+          <t>App-side tier change/comp exists; the Stripe billing side doesn't follow.</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>7-section IA; folds in nav cleanup, per-event check-in start, financial accuracy, tier tools, and guest upload.</t>
+          <t>Wire admin tier-change to Stripe subscription cancel/modify/start.</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
@@ -2260,24 +2260,24 @@
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>The Messages section is where the texting inbox lives.</t>
+          <t>App-side override already exists; this is the Stripe billing reconciliation.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>Shared admin navigation config</t>
+          <t>Harden the admin cancel-subscription flow</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>One shared config for admin nav so it's consistent and not duplicated.</t>
+          <t>Make admin cancel safe (running twice shouldn't double-act).</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Single adminNav config; remove duplicated nav definitions.</t>
+          <t>Add idempotency + structured logging + alert to admin-cancel-subscription.</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
@@ -2287,24 +2287,24 @@
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>One config; removes duplicated nav definitions.</t>
+          <t>Idempotent + logged + alerted so a double-run can't double-act.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>Guest list upload tool</t>
+          <t>Build the admin area into clean sections</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Let admins upload a guest list for an event.</t>
+          <t>Reorganize admin into Today / People / Events / Network / Money / Messages / Settings with one source of truth per question.</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>Guest list upload UI.</t>
+          <t>7-section IA; folds in nav cleanup, per-event check-in start, financial accuracy, tier tools, and guest upload.</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
@@ -2314,24 +2314,24 @@
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>Also unblocks future guest-conversion automation.</t>
+          <t>The Messages section is where the texting inbox lives.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>Fix the organization settings table</t>
+          <t>Shared admin navigation config</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>organization_settings has the wrong schema.</t>
+          <t>One shared config for admin nav so it's consistent and not duplicated.</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Correct the organization_settings schema.</t>
+          <t>Single adminNav config; remove duplicated nav definitions.</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
@@ -2341,24 +2341,24 @@
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>Schema is currently wrong; correct it.</t>
+          <t>One config; removes duplicated nav definitions.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>Route Stripe receipts to the team inbox</t>
+          <t>Guest list upload tool</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Receipt/invoice emails should also go to hello@704collective.com.</t>
+          <t>Let admins upload a guest list for an event.</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Stripe email settings -&gt; CC hello@ (or a forwarding rule).</t>
+          <t>Guest list upload UI.</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
@@ -2368,35 +2368,51 @@
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>CC hello@ on Stripe receipts, or add a forwarding rule.</t>
+          <t>Also unblocks future guest-conversion automation.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A74" s="4" t="inlineStr">
-        <is>
-          <t>MEMBER EXPERIENCE   ·   9 items</t>
-        </is>
-      </c>
-      <c r="B74" s="29" t="n"/>
-      <c r="C74" s="29" t="n"/>
-      <c r="D74" s="29" t="n"/>
-      <c r="E74" s="30" t="n"/>
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>Fix the organization settings table</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>organization_settings has the wrong schema.</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>Correct the organization_settings schema.</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>Schema is currently wrong; correct it.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A75" s="7" t="inlineStr">
         <is>
-          <t>Strip member profiles to four clean fields</t>
+          <t>Route Stripe receipts to the team inbox</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Simplify the profile to name, photo, what you do, and a one-line bio — as real columns, not JSON. Locked: archive the other 15+ fields (kept in DB, hidden) for future matchmaking.</t>
+          <t>Receipt/invoice emails should also go to hello@704collective.com.</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>4 visible fields as real columns; align onboarding + settings + directory. The 4-field data move rides with the identity foundation (same plumbing).</t>
+          <t>Stripe email settings -&gt; CC hello@ (or a forwarding rule).</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
@@ -2406,51 +2422,35 @@
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>Archive (don't delete) the rest — raw material for future matchmaking.</t>
+          <t>CC hello@ on Stripe receipts, or add a forwarding rule.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A76" s="7" t="inlineStr">
-        <is>
-          <t>Build the one merged member portal with tiered views</t>
-        </is>
-      </c>
-      <c r="B76" s="8" t="inlineStr">
-        <is>
-          <t>Locked: replace the two portals (member dashboard + business portal) with ONE codebase; business gets an elevated view, social the standard view; clear type distinction preserved.</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>One portal codebase; gate business-only modules behind member type. Replaces /dashboard vs /business-portal.</t>
-        </is>
-      </c>
-      <c r="D76" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E76" s="8" t="inlineStr">
-        <is>
-          <t>Replaces /dashboard vs /business-portal with one tier-gated codebase.</t>
-        </is>
-      </c>
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>MEMBER EXPERIENCE   ·   9 items</t>
+        </is>
+      </c>
+      <c r="B76" s="29" t="n"/>
+      <c r="C76" s="29" t="n"/>
+      <c r="D76" s="29" t="n"/>
+      <c r="E76" s="30" t="n"/>
     </row>
     <row r="77" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>Rebuild onboarding questionnaire + member brief</t>
+          <t>Strip member profiles to four clean fields</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>Store responses in their own table and generate a 'member brief' for future matchmaking/AI.</t>
+          <t>Simplify the profile to name, photo, what you do, and a one-line bio — as real columns, not JSON. Locked: archive the other 15+ fields (kept in DB, hidden) for future matchmaking.</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>Onboarding rebuild + onboarding_responses table + member_brief column.</t>
+          <t>4 visible fields as real columns; align onboarding + settings + directory. The 4-field data move rides with the identity foundation (same plumbing).</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
@@ -2460,24 +2460,24 @@
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>Responses in their own table; feeds a future member brief.</t>
+          <t>Archive (don't delete) the rest — raw material for future matchmaking.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>Member portal / dashboard redesign</t>
+          <t>Build the one merged member portal with tiered views</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>The redesign: 5-tab bottom nav, pass-first / next-event hero, onboarding checklist removed after completion, plus resources/bookings tabs. The shared activity feed is KEPT and built on (members post / share / like; event discussions surface there) — only the minor personal activity-log widget from the old dashboard is retired.</t>
+          <t>Locked: replace the two portals (member dashboard + business portal) with ONE codebase; business gets an elevated view, social the standard view; clear type distinction preserved.</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>Multi-week. SEQUENCING: the visual redesign lands AFTER the identity foundation is built and verified — not concurrent with it (one big change at a time on a no-staging system). Resources/bookings depend on vendor partnerships.</t>
+          <t>One portal codebase; gate business-only modules behind member type. Replaces /dashboard vs /business-portal.</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
@@ -2487,24 +2487,24 @@
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>Activity feed stays; only the personal activity-log widget is retired. Visual redesign sequenced after identity.</t>
+          <t>Replaces /dashboard vs /business-portal with one tier-gated codebase.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A79" s="7" t="inlineStr">
         <is>
-          <t>Member directory — people-finder for all member + partner types</t>
+          <t>Rebuild onboarding questionnaire + member brief</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>A members-only people-finder where social members, business members, and partners can all find and see each other — profiles only, WITHOUT the business-listings view. Visible to everyone logged in, regardless of type. A privacy toggle lets a member hide from it.</t>
+          <t>Store responses in their own table and generate a 'member brief' for future matchmaking/AI.</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>Logged-in directory of people (social + business + partner). Profiles only — no business view (that lives in The Network). Visible to all logged-in types; honor the privacy toggle.</t>
+          <t>Onboarding rebuild + onboarding_responses table + member_brief column.</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
@@ -2514,24 +2514,24 @@
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>Distinct from The Network (hubs + business/partner listings). Pairs with the privacy toggle below.</t>
+          <t>Responses in their own table; feeds a future member brief.</t>
         </is>
       </c>
     </row>
     <row r="80" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>Profile privacy toggle</t>
+          <t>Member portal / dashboard redesign</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>A toggle for members to control whether they appear in the directory and the internal Network member view.</t>
+          <t>The redesign: 5-tab bottom nav, pass-first / next-event hero, onboarding checklist removed after completion, plus resources/bookings tabs. The shared activity feed is KEPT and built on (members post / share / like; event discussions surface there) — only the minor personal activity-log widget from the old dashboard is retired.</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Build the opt-out toggle; default is listed, members can hide themselves.</t>
+          <t>Multi-week. SEQUENCING: the visual redesign lands AFTER the identity foundation is built and verified — not concurrent with it (one big change at a time on a no-staging system). Resources/bookings depend on vendor partnerships.</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
@@ -2541,24 +2541,24 @@
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>Confirmed feature — the directory is opt-out via this toggle.</t>
+          <t>Activity feed stays; only the personal activity-log widget is retired. Visual redesign sequenced after identity.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A81" s="7" t="inlineStr">
         <is>
-          <t>Member cancellation retention flow</t>
+          <t>Member directory — people-finder for all member + partner types</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>Improve the cancellation flow with retention UX.</t>
+          <t>A members-only people-finder where social members, business members, and partners can all find and see each other — profiles only, WITHOUT the business-listings view. Visible to everyone logged in, regardless of type. A privacy toggle lets a member hide from it.</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>Retention UX on cancellation (offers, pauses, feedback).</t>
+          <t>Logged-in directory of people (social + business + partner). Profiles only — no business view (that lives in The Network). Visible to all logged-in types; honor the privacy toggle.</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
@@ -2568,24 +2568,24 @@
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>Offers / pauses / feedback on cancellation.</t>
+          <t>Distinct from The Network (hubs + business/partner listings). Pairs with the privacy toggle below.</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A82" s="7" t="inlineStr">
         <is>
-          <t>Member spotlight on calendar/home</t>
+          <t>Profile privacy toggle</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>Feature a member spotlight on the calendar/home pages.</t>
+          <t>A toggle for members to control whether they appear in the directory and the internal Network member view.</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>Member spotlight feature.</t>
+          <t>Build the opt-out toggle; default is listed, members can hide themselves.</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
@@ -2595,100 +2595,100 @@
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>Feature a member on calendar/home.</t>
+          <t>Confirmed feature — the directory is opt-out via this toggle.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A83" s="7" t="inlineStr">
         <is>
-          <t>Unlimited guest passes for dream-team members</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="n"/>
-      <c r="C83" s="5" t="n"/>
-      <c r="D83" s="5" t="n"/>
-      <c r="E83" s="6" t="n"/>
+          <t>Member cancellation retention flow</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>Improve the cancellation flow with retention UX.</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Retention UX on cancellation (offers, pauses, feedback).</t>
+        </is>
+      </c>
+      <c r="D83" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>Offers / pauses / feedback on cancellation.</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A84" s="4" t="inlineStr">
-        <is>
-          <t>PERFORMANCE   ·   5 items</t>
-        </is>
-      </c>
-      <c r="B84" s="29" t="n"/>
-      <c r="C84" s="29" t="n"/>
-      <c r="D84" s="29" t="n"/>
-      <c r="E84" s="30" t="n"/>
+      <c r="A84" s="7" t="inlineStr">
+        <is>
+          <t>Member spotlight on calendar/home</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>Feature a member spotlight on the calendar/home pages.</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>Member spotlight feature.</t>
+        </is>
+      </c>
+      <c r="D84" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>Feature a member on calendar/home.</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A85" s="7" t="inlineStr">
         <is>
-          <t>Speed up slow list pages (Events, Tasks, Hubs)</t>
-        </is>
-      </c>
-      <c r="B85" s="8" t="inlineStr">
-        <is>
-          <t>These pages make many small repeated DB calls (N+1) that get slow as data grows.</t>
-        </is>
-      </c>
-      <c r="C85" s="8" t="inlineStr">
-        <is>
-          <t>Resolve the N+1 query patterns; batch them.</t>
-        </is>
-      </c>
-      <c r="D85" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E85" s="8" t="inlineStr">
-        <is>
-          <t>Batch the repeated calls on Events, Tasks, Hubs.</t>
-        </is>
-      </c>
+          <t>Unlimited guest passes for dream-team members</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="n"/>
+      <c r="C85" s="5" t="n"/>
+      <c r="D85" s="5" t="n"/>
+      <c r="E85" s="6" t="n"/>
     </row>
     <row r="86" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A86" s="7" t="inlineStr">
-        <is>
-          <t>Make bulk member adds all-or-nothing</t>
-        </is>
-      </c>
-      <c r="B86" s="8" t="inlineStr">
-        <is>
-          <t>Bulk add isn't transactional — a partial failure leaves half-written data.</t>
-        </is>
-      </c>
-      <c r="C86" s="8" t="inlineStr">
-        <is>
-          <t>Make add-members and hub-delete atomic.</t>
-        </is>
-      </c>
-      <c r="D86" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E86" s="8" t="inlineStr">
-        <is>
-          <t>All-or-nothing; same for hub deletes.</t>
-        </is>
-      </c>
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>PERFORMANCE   ·   5 items</t>
+        </is>
+      </c>
+      <c r="B86" s="29" t="n"/>
+      <c r="C86" s="29" t="n"/>
+      <c r="D86" s="29" t="n"/>
+      <c r="E86" s="30" t="n"/>
     </row>
     <row r="87" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A87" s="7" t="inlineStr">
         <is>
-          <t>Move heavy admin queries to the server</t>
+          <t>Speed up slow list pages (Events, Tasks, Hubs)</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>Keep the browser from doing heavy lifting on admin overview + email dashboard.</t>
+          <t>These pages make many small repeated DB calls (N+1) that get slow as data grows.</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Add server-side RPCs: admin_overview, email_dashboard.</t>
+          <t>Resolve the N+1 query patterns; batch them.</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
@@ -2698,24 +2698,24 @@
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>Move admin overview + email dashboard to server RPCs.</t>
+          <t>Batch the repeated calls on Events, Tasks, Hubs.</t>
         </is>
       </c>
     </row>
     <row r="88" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>Standardize how data is loaded (React Query)</t>
+          <t>Make bulk member adds all-or-nothing</t>
         </is>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>Make loading behavior uniform and reliable.</t>
+          <t>Bulk add isn't transactional — a partial failure leaves half-written data.</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>React Query rollout across data fetching.</t>
+          <t>Make add-members and hub-delete atomic.</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
@@ -2725,100 +2725,100 @@
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t>Uniform data-loading / caching across the app.</t>
+          <t>All-or-nothing; same for hub deletes.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A89" s="7" t="inlineStr">
         <is>
-          <t>Audit shortcut data fields for correctness</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="n"/>
-      <c r="C89" s="5" t="n"/>
-      <c r="D89" s="5" t="n"/>
-      <c r="E89" s="6" t="n"/>
+          <t>Move heavy admin queries to the server</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>Keep the browser from doing heavy lifting on admin overview + email dashboard.</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>Add server-side RPCs: admin_overview, email_dashboard.</t>
+        </is>
+      </c>
+      <c r="D89" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>Move admin overview + email dashboard to server RPCs.</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A90" s="4" t="inlineStr">
-        <is>
-          <t>AUTH   ·   7 items</t>
-        </is>
-      </c>
-      <c r="B90" s="29" t="n"/>
-      <c r="C90" s="29" t="n"/>
-      <c r="D90" s="29" t="n"/>
-      <c r="E90" s="30" t="n"/>
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>Standardize how data is loaded (React Query)</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>Make loading behavior uniform and reliable.</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>React Query rollout across data fetching.</t>
+        </is>
+      </c>
+      <c r="D90" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E90" s="8" t="inlineStr">
+        <is>
+          <t>Uniform data-loading / caching across the app.</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A91" s="7" t="inlineStr">
         <is>
-          <t>Verify magic-link login across two devices</t>
-        </is>
-      </c>
-      <c r="B91" s="8" t="inlineStr">
-        <is>
-          <t>Phone-to-desktop: request a link on a phone, type the 8-digit code on the desktop.</t>
-        </is>
-      </c>
-      <c r="C91" s="8" t="inlineStr">
-        <is>
-          <t>Cross-device OTP test; confirm same-device + resend cooldown too.</t>
-        </is>
-      </c>
-      <c r="D91" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E91" s="8" t="inlineStr">
-        <is>
-          <t>Requires a second device (owner-run).</t>
-        </is>
-      </c>
+          <t>Audit shortcut data fields for correctness</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="n"/>
+      <c r="C91" s="5" t="n"/>
+      <c r="D91" s="5" t="n"/>
+      <c r="E91" s="6" t="n"/>
     </row>
     <row r="92" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A92" s="7" t="inlineStr">
-        <is>
-          <t>Verify magic-link login works in production</t>
-        </is>
-      </c>
-      <c r="B92" s="8" t="inlineStr">
-        <is>
-          <t>End-to-end check the email magic-link round-trip works live.</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
-          <t>Test request -&gt; click -&gt; signed in, in prod.</t>
-        </is>
-      </c>
-      <c r="D92" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E92" s="8" t="inlineStr">
-        <is>
-          <t>End-to-end live round-trip check.</t>
-        </is>
-      </c>
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>AUTH   ·   7 items</t>
+        </is>
+      </c>
+      <c r="B92" s="29" t="n"/>
+      <c r="C92" s="29" t="n"/>
+      <c r="D92" s="29" t="n"/>
+      <c r="E92" s="30" t="n"/>
     </row>
     <row r="93" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A93" s="7" t="inlineStr">
         <is>
-          <t>Verify sessions refresh correctly on expiry</t>
+          <t>Verify magic-link login across two devices</t>
         </is>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>Confirm cookie-based refresh works when a token expires so members aren't kicked out.</t>
+          <t>Phone-to-desktop: request a link on a phone, type the 8-digit code on the desktop.</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>Verify @supabase/ssr middleware refreshes session on token expiry.</t>
+          <t>Cross-device OTP test; confirm same-device + resend cooldown too.</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
@@ -2828,24 +2828,24 @@
       </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t>Confirm members aren't kicked out when a token expires.</t>
+          <t>Requires a second device (owner-run).</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A94" s="7" t="inlineStr">
         <is>
-          <t>Verify Google sign-in works</t>
+          <t>Verify magic-link login works in production</t>
         </is>
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>Confirm Google login/signup paths work in production.</t>
+          <t>End-to-end check the email magic-link round-trip works live.</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t>Test Google OAuth signup + sign-in.</t>
+          <t>Test request -&gt; click -&gt; signed in, in prod.</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
@@ -2855,86 +2855,118 @@
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t>Confirm Google login/signup in production.</t>
+          <t>End-to-end live round-trip check.</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A95" s="7" t="inlineStr">
         <is>
-          <t>Apple Sign-In</t>
-        </is>
-      </c>
-      <c r="B95" s="5" t="n"/>
-      <c r="C95" s="5" t="n"/>
-      <c r="D95" s="5" t="n"/>
-      <c r="E95" s="6" t="n"/>
+          <t>Verify sessions refresh correctly on expiry</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>Confirm cookie-based refresh works when a token expires so members aren't kicked out.</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>Verify @supabase/ssr middleware refreshes session on token expiry.</t>
+        </is>
+      </c>
+      <c r="D95" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>Confirm members aren't kicked out when a token expires.</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A96" s="7" t="inlineStr">
         <is>
-          <t>Branded auth links (stop showing supabase.co URLs)</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>Build</t>
+          <t>Verify Google sign-in works</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>Confirm Google login/signup paths work in production.</t>
+        </is>
+      </c>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>Test Google OAuth signup + sign-in.</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>Confirm Google login/signup in production.</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A97" s="7" t="inlineStr">
         <is>
-          <t>Password rules hardening (min length 6 to 8, leaked-password check)</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="inlineStr">
-        <is>
-          <t>Supabase minimum password length is 6 and the leaked-password check is off. Both are weaker than they should be for a paid membership platform.</t>
-        </is>
-      </c>
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>Do the UI copy FIRST, then the dashboard toggles. Update /setup-password and every password field to state the real rule before raising the server minimum to 8, otherwise members get rejected by a rule the screen never showed them. Then enable Prevent use of leaked passwords and confirm the rejection message renders cleanly. Leave Require current password when updating OFF, it breaks the no-password comp-invite setup flow. Rehearse on develop both viewports.</t>
-        </is>
-      </c>
-      <c r="D97" s="5" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E97" s="6" t="inlineStr">
-        <is>
-          <t>Raised 2026-08-06 during the Email OTP expiration change (3600 to 86400).</t>
-        </is>
-      </c>
+          <t>Apple Sign-In</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="n"/>
+      <c r="C97" s="5" t="n"/>
+      <c r="D97" s="5" t="n"/>
+      <c r="E97" s="6" t="n"/>
     </row>
     <row r="98" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A98" s="4" t="inlineStr">
-        <is>
-          <t>BUSINESS   ·   1 item</t>
-        </is>
-      </c>
-      <c r="B98" s="29" t="n"/>
-      <c r="C98" s="29" t="n"/>
-      <c r="D98" s="29" t="n"/>
-      <c r="E98" s="30" t="n"/>
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t>Branded auth links (stop showing supabase.co URLs)</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A99" s="7" t="inlineStr">
         <is>
-          <t>Verify the business application approval works</t>
-        </is>
-      </c>
-      <c r="B99" s="5" t="n"/>
-      <c r="C99" s="5" t="n"/>
-      <c r="D99" s="5" t="n"/>
-      <c r="E99" s="6" t="n"/>
+          <t>Password rules hardening (min length 6 to 8, leaked-password check)</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Supabase minimum password length is 6 and the leaked-password check is off. Both are weaker than they should be for a paid membership platform.</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>Do the UI copy FIRST, then the dashboard toggles. Update /setup-password and every password field to state the real rule before raising the server minimum to 8, otherwise members get rejected by a rule the screen never showed them. Then enable Prevent use of leaked passwords and confirm the rejection message renders cleanly. Leave Require current password when updating OFF, it breaks the no-password comp-invite setup flow. Rehearse on develop both viewports.</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>Raised 2026-08-06 during the Email OTP expiration change (3600 to 86400).</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>FINANCIALS   ·   6 items</t>
+          <t>BUSINESS   ·   1 item</t>
         </is>
       </c>
       <c r="B100" s="29" t="n"/>
@@ -2945,208 +2977,176 @@
     <row r="101" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A101" s="7" t="inlineStr">
         <is>
-          <t>Verify the financial dashboard</t>
-        </is>
-      </c>
-      <c r="B101" s="8" t="inlineStr">
-        <is>
-          <t>Confirm it reports MRR, churn, and revenue by tier correctly (churn once showed 2055%).</t>
-        </is>
-      </c>
-      <c r="C101" s="8" t="inlineStr">
-        <is>
-          <t>Verify financial dashboard accuracy.</t>
-        </is>
-      </c>
-      <c r="D101" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E101" s="8" t="inlineStr">
-        <is>
-          <t>Built in Lovable originally — accuracy unconfirmed.</t>
-        </is>
-      </c>
+          <t>Verify the business application approval works</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="n"/>
+      <c r="C101" s="5" t="n"/>
+      <c r="D101" s="5" t="n"/>
+      <c r="E101" s="6" t="n"/>
     </row>
     <row r="102" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A102" s="7" t="inlineStr">
-        <is>
-          <t>Verify the admin financial data function</t>
-        </is>
-      </c>
-      <c r="B102" s="8" t="inlineStr">
-        <is>
-          <t>Confirm the edge function feeding admin financials returns correct numbers.</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t>Verify admin-financial-data.</t>
-        </is>
-      </c>
-      <c r="D102" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E102" s="8" t="inlineStr">
-        <is>
-          <t>Confirm the numbers it returns are correct.</t>
-        </is>
-      </c>
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>FINANCIALS   ·   6 items</t>
+        </is>
+      </c>
+      <c r="B102" s="29" t="n"/>
+      <c r="C102" s="29" t="n"/>
+      <c r="D102" s="29" t="n"/>
+      <c r="E102" s="30" t="n"/>
     </row>
     <row r="103" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A103" s="7" t="inlineStr">
         <is>
-          <t>Three-bucket revenue view</t>
+          <t>Verify the financial dashboard</t>
         </is>
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>Show revenue split three ways.</t>
+          <t>Confirm it reports MRR, churn, and revenue by tier correctly (churn once showed 2055%).</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Collected / projected / churned split.</t>
-        </is>
-      </c>
-      <c r="D103" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
+          <t>Verify financial dashboard accuracy.</t>
+        </is>
+      </c>
+      <c r="D103" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t>Collected / projected / churned.</t>
+          <t>Built in Lovable originally — accuracy unconfirmed.</t>
         </is>
       </c>
     </row>
     <row r="104" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A104" s="7" t="inlineStr">
         <is>
-          <t>Member-facing financial widget</t>
+          <t>Verify the admin financial data function</t>
         </is>
       </c>
       <c r="B104" s="8" t="inlineStr">
         <is>
-          <t>A small financial widget members can see.</t>
+          <t>Confirm the edge function feeding admin financials returns correct numbers.</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>Member-facing billing-status widget.</t>
-        </is>
-      </c>
-      <c r="D104" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
+          <t>Verify admin-financial-data.</t>
+        </is>
+      </c>
+      <c r="D104" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
         <is>
-          <t>Small billing-status widget for members.</t>
+          <t>Confirm the numbers it returns are correct.</t>
         </is>
       </c>
     </row>
     <row r="105" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A105" s="7" t="inlineStr">
         <is>
-          <t>Reduce redundant Stripe scans</t>
+          <t>Three-bucket revenue view</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>Show revenue split three ways.</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>Collected / projected / churned split.</t>
+        </is>
+      </c>
+      <c r="D105" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>Collected / projected / churned.</t>
         </is>
       </c>
     </row>
     <row r="106" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t>Past-due dismissal flow</t>
-        </is>
-      </c>
-      <c r="B106" s="5" t="n"/>
-      <c r="C106" s="5" t="n"/>
-      <c r="D106" s="5" t="n"/>
-      <c r="E106" s="6" t="n"/>
+          <t>Member-facing financial widget</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
+          <t>A small financial widget members can see.</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>Member-facing billing-status widget.</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>Small billing-status widget for members.</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A107" s="4" t="inlineStr">
-        <is>
-          <t>EMAIL &amp; DRIP   ·   13 items</t>
-        </is>
-      </c>
-      <c r="B107" s="29" t="n"/>
-      <c r="C107" s="29" t="n"/>
-      <c r="D107" s="29" t="n"/>
-      <c r="E107" s="30" t="n"/>
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>Reduce redundant Stripe scans</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t>Drip email health banner</t>
-        </is>
-      </c>
-      <c r="B108" s="8" t="inlineStr">
-        <is>
-          <t>A banner flagging when drips are silently failing or stalled.</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
-          <t>Drip health-check banner.</t>
-        </is>
-      </c>
-      <c r="D108" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E108" s="8" t="inlineStr">
-        <is>
-          <t>Flags silently failing / stalled drips.</t>
-        </is>
-      </c>
+          <t>Past-due dismissal flow</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="n"/>
+      <c r="C108" s="5" t="n"/>
+      <c r="D108" s="5" t="n"/>
+      <c r="E108" s="6" t="n"/>
     </row>
     <row r="109" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A109" s="7" t="inlineStr">
-        <is>
-          <t>Guest follow-up drip (7 + 20 day)</t>
-        </is>
-      </c>
-      <c r="B109" s="8" t="inlineStr">
-        <is>
-          <t>Automatic emails to guests at day 7 and 20 to convert them.</t>
-        </is>
-      </c>
-      <c r="C109" s="8" t="inlineStr">
-        <is>
-          <t>Guest 7-day + 20-day drip.</t>
-        </is>
-      </c>
-      <c r="D109" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E109" s="8" t="inlineStr">
-        <is>
-          <t>Converts guests at day 7 and 20.</t>
-        </is>
-      </c>
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>EMAIL &amp; DRIP   ·   13 items</t>
+        </is>
+      </c>
+      <c r="B109" s="29" t="n"/>
+      <c r="C109" s="29" t="n"/>
+      <c r="D109" s="29" t="n"/>
+      <c r="E109" s="30" t="n"/>
     </row>
     <row r="110" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t>14-day RSVP prompt for new members</t>
+          <t>Drip email health banner</t>
         </is>
       </c>
       <c r="B110" s="8" t="inlineStr">
         <is>
-          <t>Nudge new members who haven't RSVP'd within 14 days.</t>
+          <t>A banner flagging when drips are silently failing or stalled.</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t>14-day RSVP prompt drip.</t>
+          <t>Drip health-check banner.</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
@@ -3156,24 +3156,24 @@
       </c>
       <c r="E110" s="8" t="inlineStr">
         <is>
-          <t>Nudges new members who haven't RSVP'd.</t>
+          <t>Flags silently failing / stalled drips.</t>
         </is>
       </c>
     </row>
     <row r="111" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A111" s="7" t="inlineStr">
         <is>
-          <t>Confirm the email log matches actual sends</t>
+          <t>Guest follow-up drip (7 + 20 day)</t>
         </is>
       </c>
       <c r="B111" s="8" t="inlineStr">
         <is>
-          <t>Today failures are swallowed; make 'did this send' provable.</t>
+          <t>Automatic emails to guests at day 7 and 20 to convert them.</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t>email_log row matching; stop swallowing failures.</t>
+          <t>Guest 7-day + 20-day drip.</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
@@ -3183,24 +3183,24 @@
       </c>
       <c r="E111" s="8" t="inlineStr">
         <is>
-          <t>Stop swallowing failures so 'did this send' is provable.</t>
+          <t>Converts guests at day 7 and 20.</t>
         </is>
       </c>
     </row>
     <row r="112" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t>Per-email open/click analytics</t>
+          <t>14-day RSVP prompt for new members</t>
         </is>
       </c>
       <c r="B112" s="8" t="inlineStr">
         <is>
-          <t>Track opens/clicks per template so we know what works.</t>
+          <t>Nudge new members who haven't RSVP'd within 14 days.</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t>Per-template email analytics.</t>
+          <t>14-day RSVP prompt drip.</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
@@ -3210,24 +3210,24 @@
       </c>
       <c r="E112" s="8" t="inlineStr">
         <is>
-          <t>Per-template open / click tracking.</t>
+          <t>Nudges new members who haven't RSVP'd.</t>
         </is>
       </c>
     </row>
     <row r="113" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A113" s="7" t="inlineStr">
         <is>
-          <t>Per-member engagement scoring</t>
+          <t>Confirm the email log matches actual sends</t>
         </is>
       </c>
       <c r="B113" s="8" t="inlineStr">
         <is>
-          <t>Score each member's engagement from email/event activity.</t>
+          <t>Today failures are swallowed; make 'did this send' provable.</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t>Engagement scoring per member.</t>
+          <t>email_log row matching; stop swallowing failures.</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
@@ -3237,24 +3237,24 @@
       </c>
       <c r="E113" s="8" t="inlineStr">
         <is>
-          <t>Score members from email / event activity.</t>
+          <t>Stop swallowing failures so 'did this send' is provable.</t>
         </is>
       </c>
     </row>
     <row r="114" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A114" s="7" t="inlineStr">
         <is>
-          <t>Category-level unsubscribe preferences</t>
+          <t>Per-email open/click analytics</t>
         </is>
       </c>
       <c r="B114" s="8" t="inlineStr">
         <is>
-          <t>Let members opt out of specific categories, not all-or-nothing; builds on the one-flag fix.</t>
+          <t>Track opens/clicks per template so we know what works.</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t>Per-category opt-out prefs + a member settings page.</t>
+          <t>Per-template email analytics.</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
@@ -3264,24 +3264,24 @@
       </c>
       <c r="E114" s="8" t="inlineStr">
         <is>
-          <t>Builds on the one-flag opt-out fix.</t>
+          <t>Per-template open / click tracking.</t>
         </is>
       </c>
     </row>
     <row r="115" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A115" s="7" t="inlineStr">
         <is>
-          <t>Branching drips based on opens/clicks</t>
+          <t>Per-member engagement scoring</t>
         </is>
       </c>
       <c r="B115" s="8" t="inlineStr">
         <is>
-          <t>Drip sequences that branch on open/click.</t>
+          <t>Score each member's engagement from email/event activity.</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t>Open/click-branching drips.</t>
+          <t>Engagement scoring per member.</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
@@ -3291,24 +3291,24 @@
       </c>
       <c r="E115" s="8" t="inlineStr">
         <is>
-          <t>Branch sequences on open / click.</t>
+          <t>Score members from email / event activity.</t>
         </is>
       </c>
     </row>
     <row r="116" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>Send email from a contact record</t>
+          <t>Category-level unsubscribe preferences</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
         <is>
-          <t>Let an admin email directly from a member/contact record.</t>
+          <t>Let members opt out of specific categories, not all-or-nothing; builds on the one-flag fix.</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t>Send-email action on the contact record.</t>
+          <t>Per-category opt-out prefs + a member settings page.</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
@@ -3318,24 +3318,24 @@
       </c>
       <c r="E116" s="8" t="inlineStr">
         <is>
-          <t>Admin emails directly from a member record.</t>
+          <t>Builds on the one-flag opt-out fix.</t>
         </is>
       </c>
     </row>
     <row r="117" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t>Attachments and images on event email campaigns</t>
+          <t>Branching drips based on opens/clicks</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
         <is>
-          <t>Let campaign emails include attachments and images.</t>
+          <t>Drip sequences that branch on open/click.</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t>Extend the campaign editor for attachments + images.</t>
+          <t>Open/click-branching drips.</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
@@ -3345,271 +3345,271 @@
       </c>
       <c r="E117" s="8" t="inlineStr">
         <is>
-          <t>Extend the campaign editor.</t>
+          <t>Branch sequences on open / click.</t>
         </is>
       </c>
     </row>
     <row r="118" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t>Live test the guest-pass drip</t>
+          <t>Send email from a contact record</t>
         </is>
       </c>
       <c r="B118" s="8" t="inlineStr">
         <is>
-          <t>Confirm the drip fires correctly on a guest pass.</t>
+          <t>Let an admin email directly from a member/contact record.</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t>Live test the drip on guest_pass.</t>
-        </is>
-      </c>
-      <c r="D118" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
+          <t>Send-email action on the contact record.</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
         <is>
-          <t>Confirm it fires on a guest pass.</t>
+          <t>Admin emails directly from a member record.</t>
         </is>
       </c>
     </row>
     <row r="119" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A119" s="7" t="inlineStr">
         <is>
-          <t>Merge guest follow-up into the drip processor</t>
+          <t>Attachments and images on event email campaigns</t>
+        </is>
+      </c>
+      <c r="B119" s="8" t="inlineStr">
+        <is>
+          <t>Let campaign emails include attachments and images.</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>Extend the campaign editor for attachments + images.</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E119" s="8" t="inlineStr">
+        <is>
+          <t>Extend the campaign editor.</t>
         </is>
       </c>
     </row>
     <row r="120" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A120" s="7" t="inlineStr">
         <is>
+          <t>Live test the guest-pass drip</t>
+        </is>
+      </c>
+      <c r="B120" s="8" t="inlineStr">
+        <is>
+          <t>Confirm the drip fires correctly on a guest pass.</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t>Live test the drip on guest_pass.</t>
+        </is>
+      </c>
+      <c r="D120" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E120" s="8" t="inlineStr">
+        <is>
+          <t>Confirm it fires on a guest pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t>Merge guest follow-up into the drip processor</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="21.75" customFormat="1" customHeight="1" s="2">
+      <c r="A122" s="7" t="inlineStr">
+        <is>
           <t>Push current members to subscribe to the calendar + add their pass</t>
         </is>
       </c>
-      <c r="B120" s="5" t="n"/>
-      <c r="C120" s="5" t="n"/>
-      <c r="D120" s="5" t="n"/>
-      <c r="E120" s="6" t="n"/>
-    </row>
-    <row r="121" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A121" s="4" t="inlineStr">
+      <c r="B122" s="5" t="n"/>
+      <c r="C122" s="5" t="n"/>
+      <c r="D122" s="5" t="n"/>
+      <c r="E122" s="6" t="n"/>
+    </row>
+    <row r="123" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A123" s="4" t="inlineStr">
         <is>
           <t>DATA &amp; CLEANUP   ·   6 items</t>
         </is>
       </c>
-      <c r="B121" s="29" t="n"/>
-      <c r="C121" s="29" t="n"/>
-      <c r="D121" s="29" t="n"/>
-      <c r="E121" s="30" t="n"/>
-    </row>
-    <row r="122" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A122" s="17" t="inlineStr">
+      <c r="B123" s="29" t="n"/>
+      <c r="C123" s="29" t="n"/>
+      <c r="D123" s="29" t="n"/>
+      <c r="E123" s="30" t="n"/>
+    </row>
+    <row r="124" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A124" s="17" t="inlineStr">
         <is>
           <t>Add CHECK constraints incrementally (enums REJECTED — too risky)</t>
         </is>
       </c>
-      <c r="B122" s="15" t="inlineStr">
+      <c r="B124" s="15" t="inlineStr">
         <is>
           <t>Was 'convert status text -&gt; enums'. DIAGNOSED Jul 9 as too risky: ~35 tables / 60+ write paths, and profiles.subscription_status is fed by the Stripe webhook with Stripe's full status vocabulary (trialing/paused/incomplete/etc). An enum built from observed values would make the webhook UPDATE throw on the first unseen status — silent breakage in the PAYMENT path. Enums rejected.</t>
         </is>
       </c>
-      <c r="C122" s="15" t="inlineStr">
+      <c r="C124" s="15" t="inlineStr">
         <is>
           <t>If typo-prevention is wanted later: add per-table CHECK constraints (NOT enums), table-by-table, starting with attendance_credentials (values: active/used/voided). Trivially reversible. Its own scoped task — never wholesale.</t>
         </is>
       </c>
-      <c r="D122" s="18" t="inlineStr">
+      <c r="D124" s="18" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
       </c>
-      <c r="E122" s="15" t="inlineStr">
+      <c r="E124" s="15" t="inlineStr">
         <is>
           <t>Reclassified Jul 9. Do NOT rush — payment-path risk. CHECK constraints are the safe 80/20 if revisited.</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A123" s="17" t="inlineStr">
+    <row r="125" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A125" s="17" t="inlineStr">
         <is>
           <t>RSVP attribution by event ID</t>
         </is>
       </c>
-      <c r="B123" s="15" t="inlineStr">
+      <c r="B125" s="15" t="inlineStr">
         <is>
           <t>DIAGNOSED Jul 9: bigger than 'add a column'. Per-event RSVP tagging is DEAD — the code that slug-tagged events was removed; since Apr 21 a public RSVP only gets a generic 'free-event-rsvp' tag, so you can't segment 'RSVP'd to event X' for any recent event. 6 frozen slug-tags remain (105 rows) and rot on rename. contact_tags has NO event_id column.</t>
         </is>
       </c>
-      <c r="C123" s="15" t="inlineStr">
+      <c r="C125" s="15" t="inlineStr">
         <is>
           <t>HALF-DAY scoped task (not a quick close): (1) migration add nullable event_id uuid REFERENCES events(id) to contact_tags; (2) re-add per-event tagging in capture-public-rsvp (event_id already in scope) + optionally create-guest-pass; (3) backfill — 5 of 6 slug-tags map to real event_ids by title-slug match (1 unmatched: coffee-and-connect-tabbris-co-working). Deploys + tests.</t>
         </is>
       </c>
-      <c r="D123" s="19" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E123" s="15" t="inlineStr">
+      <c r="D125" s="19" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E125" s="15" t="inlineStr">
         <is>
           <t>Jul 9: revives dead per-event attribution. Own task, budget a half-day. Backfill mostly possible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A124" s="7" t="inlineStr">
-        <is>
-          <t>Drop ~35 empty leftover tables</t>
-        </is>
-      </c>
-      <c r="B124" s="8" t="inlineStr">
-        <is>
-          <t>~35 empty scaffolding tables (old CRM, social manager, feed, DMs).</t>
-        </is>
-      </c>
-      <c r="C124" s="8" t="inlineStr">
-        <is>
-          <t>Export copies as a receipt, then drop.</t>
-        </is>
-      </c>
-      <c r="D124" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E124" s="8" t="inlineStr">
-        <is>
-          <t>Don't drop without exporting copies first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A125" s="7" t="inlineStr">
-        <is>
-          <t>Drop old backup tables after soak</t>
-        </is>
-      </c>
-      <c r="B125" s="8" t="inlineStr">
-        <is>
-          <t>Backup tables from recent migrations await a 2-4 week no-regression soak.</t>
-        </is>
-      </c>
-      <c r="C125" s="8" t="inlineStr">
-        <is>
-          <t>Drop dated backup_* tables after soak; confirm stability first.</t>
-        </is>
-      </c>
-      <c r="D125" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E125" s="8" t="inlineStr">
-        <is>
-          <t>Only after a 2-4 week no-regression soak.</t>
         </is>
       </c>
     </row>
     <row r="126" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A126" s="7" t="inlineStr">
         <is>
-          <t>Delete dead admin member components</t>
+          <t>Drop ~35 empty leftover tables</t>
+        </is>
+      </c>
+      <c r="B126" s="8" t="inlineStr">
+        <is>
+          <t>~35 empty scaffolding tables (old CRM, social manager, feed, DMs).</t>
+        </is>
+      </c>
+      <c r="C126" s="8" t="inlineStr">
+        <is>
+          <t>Export copies as a receipt, then drop.</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E126" s="8" t="inlineStr">
+        <is>
+          <t>Don't drop without exporting copies first.</t>
         </is>
       </c>
     </row>
     <row r="127" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
-      <c r="A127" s="4" t="inlineStr">
-        <is>
-          <t>MARKETING &amp; FRONT-END   ·   10 items</t>
-        </is>
-      </c>
-      <c r="B127" s="29" t="n"/>
-      <c r="C127" s="29" t="n"/>
-      <c r="D127" s="29" t="n"/>
-      <c r="E127" s="30" t="n"/>
+      <c r="A127" s="7" t="inlineStr">
+        <is>
+          <t>Drop old backup tables after soak</t>
+        </is>
+      </c>
+      <c r="B127" s="8" t="inlineStr">
+        <is>
+          <t>Backup tables from recent migrations await a 2-4 week no-regression soak.</t>
+        </is>
+      </c>
+      <c r="C127" s="8" t="inlineStr">
+        <is>
+          <t>Drop dated backup_* tables after soak; confirm stability first.</t>
+        </is>
+      </c>
+      <c r="D127" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E127" s="8" t="inlineStr">
+        <is>
+          <t>Only after a 2-4 week no-regression soak.</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A128" s="7" t="inlineStr">
         <is>
-          <t>SEO + schema markup + pre-rendering (all front pages + 4 hub landers)</t>
-        </is>
-      </c>
-      <c r="B128" s="29" t="n"/>
-      <c r="C128" s="29" t="n"/>
-      <c r="D128" s="29" t="n"/>
-      <c r="E128" s="30" t="n"/>
+          <t>Delete dead admin member components</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A129" s="7" t="inlineStr">
-        <is>
-          <t>Homepage hero rebuild + image optimization</t>
-        </is>
-      </c>
-      <c r="B129" s="8" t="inlineStr">
-        <is>
-          <t>Rebuild the hero and compress oversized hero images (currently 24-30MB, should be 200-800KB).</t>
-        </is>
-      </c>
-      <c r="C129" s="8" t="inlineStr">
-        <is>
-          <t>Hero rebuild + compress images.</t>
-        </is>
-      </c>
-      <c r="D129" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E129" s="8" t="inlineStr">
-        <is>
-          <t>Includes compressing 24-30MB hero images to 200-800KB.</t>
-        </is>
-      </c>
+      <c r="A129" s="4" t="inlineStr">
+        <is>
+          <t>MARKETING &amp; FRONT-END   ·   10 items</t>
+        </is>
+      </c>
+      <c r="B129" s="29" t="n"/>
+      <c r="C129" s="29" t="n"/>
+      <c r="D129" s="29" t="n"/>
+      <c r="E129" s="30" t="n"/>
     </row>
     <row r="130" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A130" s="7" t="inlineStr">
         <is>
-          <t>Homepage copy rewrite + slogan</t>
-        </is>
-      </c>
-      <c r="B130" s="8" t="inlineStr">
-        <is>
-          <t>Rewrite homepage body/section copy and update the slogan.</t>
-        </is>
-      </c>
-      <c r="C130" s="8" t="inlineStr">
-        <is>
-          <t>Body + section copy + slogan.</t>
-        </is>
-      </c>
-      <c r="D130" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E130" s="8" t="inlineStr">
-        <is>
-          <t>Needs the copy spec.</t>
-        </is>
-      </c>
+          <t>SEO + schema markup + pre-rendering (all front pages + 4 hub landers)</t>
+        </is>
+      </c>
+      <c r="B130" s="29" t="n"/>
+      <c r="C130" s="29" t="n"/>
+      <c r="D130" s="29" t="n"/>
+      <c r="E130" s="30" t="n"/>
     </row>
     <row r="131" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A131" s="7" t="inlineStr">
         <is>
-          <t>Fix the mobile hero sliding bug</t>
+          <t>Homepage hero rebuild + image optimization</t>
         </is>
       </c>
       <c r="B131" s="8" t="inlineStr">
         <is>
-          <t>A visual bug where the hero image slides on mobile.</t>
+          <t>Rebuild the hero and compress oversized hero images (currently 24-30MB, should be 200-800KB).</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
         <is>
-          <t>Mobile hero sliding fix.</t>
+          <t>Hero rebuild + compress images.</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr">
@@ -3619,24 +3619,24 @@
       </c>
       <c r="E131" s="8" t="inlineStr">
         <is>
-          <t>Fix the hero sliding on mobile.</t>
+          <t>Includes compressing 24-30MB hero images to 200-800KB.</t>
         </is>
       </c>
     </row>
     <row r="132" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A132" s="7" t="inlineStr">
         <is>
-          <t>The Exchange page</t>
+          <t>Homepage copy rewrite + slogan</t>
         </is>
       </c>
       <c r="B132" s="8" t="inlineStr">
         <is>
-          <t>Build The Exchange page (speaker-driven business event product page).</t>
+          <t>Rewrite homepage body/section copy and update the slogan.</t>
         </is>
       </c>
       <c r="C132" s="8" t="inlineStr">
         <is>
-          <t>The Exchange page.</t>
+          <t>Body + section copy + slogan.</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr">
@@ -3646,24 +3646,24 @@
       </c>
       <c r="E132" s="8" t="inlineStr">
         <is>
-          <t>Speaker-driven business-event product page.</t>
+          <t>Needs the copy spec.</t>
         </is>
       </c>
     </row>
     <row r="133" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A133" s="7" t="inlineStr">
         <is>
-          <t>Sponsor page (likely folds into /business)</t>
+          <t>Fix the mobile hero sliding bug</t>
         </is>
       </c>
       <c r="B133" s="8" t="inlineStr">
         <is>
-          <t>Sponsor functionality — likely folds into the /business application routing.</t>
+          <t>A visual bug where the hero image slides on mobile.</t>
         </is>
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t>Probably absorbed by the /business rebuild.</t>
+          <t>Mobile hero sliding fix.</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr">
@@ -3673,24 +3673,24 @@
       </c>
       <c r="E133" s="8" t="inlineStr">
         <is>
-          <t>Likely folds into the /business rebuild — confirm first.</t>
+          <t>Fix the hero sliding on mobile.</t>
         </is>
       </c>
     </row>
     <row r="134" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A134" s="7" t="inlineStr">
         <is>
-          <t>/business page rebuild with dynamic application</t>
+          <t>The Exchange page</t>
         </is>
       </c>
       <c r="B134" s="8" t="inlineStr">
         <is>
-          <t>Rebuild /business as one page with a dynamic application routing prospects to membership, Preferred Business, or sponsorship by their answers.</t>
+          <t>Build The Exchange page (speaker-driven business event product page).</t>
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr">
         <is>
-          <t>Dynamic diagnose-before-offer application.</t>
+          <t>The Exchange page.</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
@@ -3700,24 +3700,24 @@
       </c>
       <c r="E134" s="8" t="inlineStr">
         <is>
-          <t>Routes prospects to membership, Preferred Business, or sponsorship.</t>
+          <t>Speaker-driven business-event product page.</t>
         </is>
       </c>
     </row>
     <row r="135" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
       <c r="A135" s="7" t="inlineStr">
         <is>
-          <t>Charlotte hub landing sites (4 public landers)</t>
+          <t>Sponsor page (likely folds into /business)</t>
         </is>
       </c>
       <c r="B135" s="8" t="inlineStr">
         <is>
-          <t>Four audience-specific public landers (cltarrival / cltfounded / clteatsandevents / cltreset) that funnel Charlotte audiences into the club.</t>
+          <t>Sponsor functionality — likely folds into the /business application routing.</t>
         </is>
       </c>
       <c r="C135" s="8" t="inlineStr">
         <is>
-          <t>4 public landers, shared skeleton, own design pass, fully pre-rendered + schema (see SEO item). They feed The Network.</t>
+          <t>Probably absorbed by the /business rebuild.</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
@@ -3727,24 +3727,24 @@
       </c>
       <c r="E135" s="8" t="inlineStr">
         <is>
-          <t>Public landers can ship earlier; they pair with The Network below.</t>
+          <t>Likely folds into the /business rebuild — confirm first.</t>
         </is>
       </c>
     </row>
     <row r="136" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A136" s="7" t="inlineStr">
         <is>
-          <t>The Network — four hubs + members rolled up</t>
+          <t>/business page rebuild with dynamic application</t>
         </is>
       </c>
       <c r="B136" s="8" t="inlineStr">
         <is>
-          <t>The four hubs rolled up into one view, plus all members. Two faces reading the same data: a PUBLIC face (the hub landers + business/partner listings — the sales asset) and an INTERNAL in-portal view that rolls up everyone. Social members appear ONLY on the internal in-portal view — never on the public hubs.</t>
+          <t>Rebuild /business as one page with a dynamic application routing prospects to membership, Preferred Business, or sponsorship by their answers.</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t>Roll the four hubs into one Network view + members. Public face = hubs / business + partner listings (social members excluded). Internal face = full rolled-up view including social members. Reads the same hub data as the landers.</t>
+          <t>Dynamic diagnose-before-offer application.</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
@@ -3754,70 +3754,86 @@
       </c>
       <c r="E136" s="8" t="inlineStr">
         <is>
-          <t>Depends on the portal + identity foundation. Social members are internal-only on The Network. Separate from the member directory (people-only).</t>
+          <t>Routes prospects to membership, Preferred Business, or sponsorship.</t>
         </is>
       </c>
     </row>
     <row r="137" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A137" s="7" t="inlineStr">
         <is>
-          <t>Instagram comment auto-DM (ManyChat)</t>
+          <t>Charlotte hub landing sites (4 public landers)</t>
+        </is>
+      </c>
+      <c r="B137" s="8" t="inlineStr">
+        <is>
+          <t>Four audience-specific public landers (cltarrival / cltfounded / clteatsandevents / cltreset) that funnel Charlotte audiences into the club.</t>
+        </is>
+      </c>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t>4 public landers, shared skeleton, own design pass, fully pre-rendered + schema (see SEO item). They feed The Network.</t>
+        </is>
+      </c>
+      <c r="D137" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E137" s="8" t="inlineStr">
+        <is>
+          <t>Public landers can ship earlier; they pair with The Network below.</t>
         </is>
       </c>
     </row>
     <row r="138" ht="35.05" customFormat="1" customHeight="1" s="2">
-      <c r="A138" s="4" t="inlineStr">
-        <is>
-          <t>AI / AGENTS (LATER EFFORT)   ·   2 items</t>
-        </is>
-      </c>
-      <c r="B138" s="29" t="n"/>
-      <c r="C138" s="29" t="n"/>
-      <c r="D138" s="29" t="n"/>
-      <c r="E138" s="30" t="n"/>
+      <c r="A138" s="7" t="inlineStr">
+        <is>
+          <t>The Network — four hubs + members rolled up</t>
+        </is>
+      </c>
+      <c r="B138" s="8" t="inlineStr">
+        <is>
+          <t>The four hubs rolled up into one view, plus all members. Two faces reading the same data: a PUBLIC face (the hub landers + business/partner listings — the sales asset) and an INTERNAL in-portal view that rolls up everyone. Social members appear ONLY on the internal in-portal view — never on the public hubs.</t>
+        </is>
+      </c>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t>Roll the four hubs into one Network view + members. Public face = hubs / business + partner listings (social members excluded). Internal face = full rolled-up view including social members. Reads the same hub data as the landers.</t>
+        </is>
+      </c>
+      <c r="D138" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E138" s="8" t="inlineStr">
+        <is>
+          <t>Depends on the portal + identity foundation. Social members are internal-only on The Network. Separate from the member directory (people-only).</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A139" s="7" t="inlineStr">
         <is>
+          <t>Instagram comment auto-DM (ManyChat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="21.75" customFormat="1" customHeight="1" s="2">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>AI / AGENTS (LATER EFFORT)   ·   2 items</t>
+        </is>
+      </c>
+      <c r="B140" s="29" t="n"/>
+      <c r="C140" s="29" t="n"/>
+      <c r="D140" s="29" t="n"/>
+      <c r="E140" s="30" t="n"/>
+    </row>
+    <row r="141" ht="113.4" customFormat="1" customHeight="1" s="2">
+      <c r="A141" s="7" t="inlineStr">
+        <is>
           <t>AI concierge + agent platform</t>
-        </is>
-      </c>
-      <c r="B139" s="29" t="n"/>
-      <c r="C139" s="29" t="n"/>
-      <c r="D139" s="29" t="n"/>
-      <c r="E139" s="30" t="n"/>
-    </row>
-    <row r="140" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A140" s="7" t="inlineStr">
-        <is>
-          <t>AI foundations (memory, embeddings, coordination)</t>
-        </is>
-      </c>
-      <c r="B140" s="8" t="inlineStr">
-        <is>
-          <t>Supporting infra for the agents: shared memory, member embeddings, multi-agent coordination, model routing.</t>
-        </is>
-      </c>
-      <c r="C140" s="8" t="inlineStr">
-        <is>
-          <t>pgvector + embeddings, agent_memory, multi-agent coordination, model routing.</t>
-        </is>
-      </c>
-      <c r="D140" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E140" s="8" t="inlineStr">
-        <is>
-          <t>A later effort; supports the agents (embeddings, memory, routing).</t>
-        </is>
-      </c>
-    </row>
-    <row r="141" ht="113.4" customFormat="1" customHeight="1" s="2">
-      <c r="A141" s="4" t="inlineStr">
-        <is>
-          <t>EVENT DISCUSSION &amp; NOTIFICATIONS + JUL-5/6 FINDINGS — IN-HOUSE (NOT ON THE DEVELOPER SHEET)   ·   10 items</t>
         </is>
       </c>
       <c r="B141" s="29" t="n"/>
@@ -3828,213 +3844,197 @@
     <row r="142" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A142" s="7" t="inlineStr">
         <is>
-          <t>Rotate the R2 media token (exposed key)</t>
+          <t>AI foundations (memory, embeddings, coordination)</t>
         </is>
       </c>
       <c r="B142" s="8" t="inlineStr">
         <is>
-          <t>The R2 Access Key ID + Secret for bucket 704-discussion-media were exposed in a working chat (screenshot/paste). Scope = that one media bucket only — low blast radius, but rotate.</t>
+          <t>Supporting infra for the agents: shared memory, member embeddings, multi-agent coordination, model routing.</t>
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t>After 6c ships: Cloudflare -&gt; R2 -&gt; API tokens -&gt; re-create 704-discussion-upload (Object Read &amp; Write, bucket-scoped) -&gt; supabase secrets set the two new values -&gt; confirm an upload still works.</t>
-        </is>
-      </c>
-      <c r="D142" s="20" t="inlineStr">
-        <is>
-          <t>Declined</t>
+          <t>pgvector + embeddings, agent_memory, multi-agent coordination, model routing.</t>
+        </is>
+      </c>
+      <c r="D142" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
         </is>
       </c>
       <c r="E142" s="8" t="inlineStr">
         <is>
-          <t>Adam declined rotation Jul 5 - standing watch item. Key scope = one media bucket only (no member data / money / DB). Say 'rotate' anytime: ~2 min.</t>
+          <t>A later effort; supports the agents (embeddings, memory, routing).</t>
         </is>
       </c>
     </row>
     <row r="143" ht="46.25" customFormat="1" customHeight="1" s="2">
-      <c r="A143" s="7" t="inlineStr">
-        <is>
-          <t>Verify/finish the Alerts page (full history, discussion types)</t>
-        </is>
-      </c>
-      <c r="B143" s="8" t="inlineStr">
-        <is>
-          <t>Locked: bell badge clears on open, items dismiss via X, but the ALERTS PAGE keeps every notification forever - markable read (single + all). PARTIAL Jul 5: /dashboard/notifications now honors action_url (deep-links verified end to end). Remaining: full-history + mark-read behavior verification.</t>
-        </is>
-      </c>
-      <c r="C143" s="8" t="inlineStr">
-        <is>
-          <t>Read the Alerts page code; verify full-history + mark-read behavior and that all discussion notification types display with correct deep-links; fix gaps. Desktop + mobile test.</t>
-        </is>
-      </c>
-      <c r="D143" s="20" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E143" s="8" t="inlineStr">
-        <is>
-          <t>Deep-links fixed+verified Jul 5 (commit e9f6250). Remaining: verify full-history retention + mark-read (single + all).</t>
-        </is>
-      </c>
+      <c r="A143" s="4" t="inlineStr">
+        <is>
+          <t>EVENT DISCUSSION &amp; NOTIFICATIONS + JUL-5/6 FINDINGS — IN-HOUSE (NOT ON THE DEVELOPER SHEET)   ·   10 items</t>
+        </is>
+      </c>
+      <c r="B143" s="29" t="n"/>
+      <c r="C143" s="29" t="n"/>
+      <c r="D143" s="29" t="n"/>
+      <c r="E143" s="30" t="n"/>
     </row>
     <row r="144" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A144" s="7" t="inlineStr">
         <is>
-          <t>Messaging: bells for messages in existing conversations</t>
+          <t>Rotate the R2 media token (exposed key)</t>
         </is>
       </c>
       <c r="B144" s="8" t="inlineStr">
         <is>
-          <t>Messaging was resurrected Jul 5 (DMs/groups had NEVER worked since launch: RETURNING/RLS deadlock, participants-insert policy tautology, content-vs-body + title-vs-name schema mismatches, 4 missing messages columns - all fixed and verified end to end). Remaining gap: notifyNewConversation only fires on conversation CREATION, so messages into an existing thread produce no bell.</t>
+          <t>The R2 Access Key ID + Secret for bucket 704-discussion-media were exposed in a working chat (screenshot/paste). Scope = that one media bucket only — low blast radius, but rotate.</t>
         </is>
       </c>
       <c r="C144" s="8" t="inlineStr">
         <is>
-          <t>Add a new_message bell per message into an existing conversation, throttled (e.g. skip if an unread new_message bell for that conversation already exists).</t>
+          <t>After 6c ships: Cloudflare -&gt; R2 -&gt; API tokens -&gt; re-create 704-discussion-upload (Object Read &amp; Write, bucket-scoped) -&gt; supabase secrets set the two new values -&gt; confirm an upload still works.</t>
         </is>
       </c>
       <c r="D144" s="20" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Declined</t>
         </is>
       </c>
       <c r="E144" s="8" t="inlineStr">
         <is>
-          <t>Follow-on to the Jul 5 messaging resurrection. Recipients currently only get notified on the first-ever message.</t>
+          <t>Adam declined rotation Jul 5 - standing watch item. Key scope = one media bucket only (no member data / money / DB). Say 'rotate' anytime: ~2 min.</t>
         </is>
       </c>
     </row>
     <row r="145" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A145" s="7" t="inlineStr">
         <is>
-          <t>Messaging: attachment uploads (images/files)</t>
+          <t>Verify/finish the Alerts page (full history, discussion types)</t>
         </is>
       </c>
       <c r="B145" s="8" t="inlineStr">
         <is>
-          <t>MessagingView has image/file upload code paths and messages now has image_urls/file_urls/file_names columns (added Jul 5), but the storage wiring (bucket, upload flow) has never been tested and may not exist.</t>
+          <t>Locked: bell badge clears on open, items dismiss via X, but the ALERTS PAGE keeps every notification forever - markable read (single + all). PARTIAL Jul 5: /dashboard/notifications now honors action_url (deep-links verified end to end). Remaining: full-history + mark-read behavior verification.</t>
         </is>
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t>Audit the attachment path end to end: storage bucket, upload call, render. Fix or wire what's missing. Desktop + mobile test.</t>
+          <t>Read the Alerts page code; verify full-history + mark-read behavior and that all discussion notification types display with correct deep-links; fix gaps. Desktop + mobile test.</t>
         </is>
       </c>
       <c r="D145" s="20" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Verify</t>
         </is>
       </c>
       <c r="E145" s="8" t="inlineStr">
         <is>
-          <t>Text messaging + edits verified Jul 5; attachments explicitly skipped in that test.</t>
+          <t>Deep-links fixed+verified Jul 5 (commit e9f6250). Remaining: verify full-history retention + mark-read (single + all).</t>
         </is>
       </c>
     </row>
     <row r="146" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A146" s="7" t="inlineStr">
         <is>
+          <t>Messaging: bells for messages in existing conversations</t>
+        </is>
+      </c>
+      <c r="B146" s="8" t="inlineStr">
+        <is>
+          <t>Messaging was resurrected Jul 5 (DMs/groups had NEVER worked since launch: RETURNING/RLS deadlock, participants-insert policy tautology, content-vs-body + title-vs-name schema mismatches, 4 missing messages columns - all fixed and verified end to end). Remaining gap: notifyNewConversation only fires on conversation CREATION, so messages into an existing thread produce no bell.</t>
+        </is>
+      </c>
+      <c r="C146" s="8" t="inlineStr">
+        <is>
+          <t>Add a new_message bell per message into an existing conversation, throttled (e.g. skip if an unread new_message bell for that conversation already exists).</t>
+        </is>
+      </c>
+      <c r="D146" s="20" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E146" s="8" t="inlineStr">
+        <is>
+          <t>Follow-on to the Jul 5 messaging resurrection. Recipients currently only get notified on the first-ever message.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="57.45" customFormat="1" customHeight="1" s="2">
+      <c r="A147" s="7" t="inlineStr">
+        <is>
+          <t>Messaging: attachment uploads (images/files)</t>
+        </is>
+      </c>
+      <c r="B147" s="8" t="inlineStr">
+        <is>
+          <t>MessagingView has image/file upload code paths and messages now has image_urls/file_urls/file_names columns (added Jul 5), but the storage wiring (bucket, upload flow) has never been tested and may not exist.</t>
+        </is>
+      </c>
+      <c r="C147" s="8" t="inlineStr">
+        <is>
+          <t>Audit the attachment path end to end: storage bucket, upload call, render. Fix or wire what's missing. Desktop + mobile test.</t>
+        </is>
+      </c>
+      <c r="D147" s="20" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E147" s="8" t="inlineStr">
+        <is>
+          <t>Text messaging + edits verified Jul 5; attachments explicitly skipped in that test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="57.45" customFormat="1" customHeight="1" s="2">
+      <c r="A148" s="7" t="inlineStr">
+        <is>
           <t>Verify the first real-money admin refund (Remove &amp; Refund)</t>
         </is>
       </c>
-      <c r="B146" s="8" t="inlineStr">
+      <c r="B148" s="8" t="inlineStr">
         <is>
           <t>Admin Remove &amp; Refund shipped Jul 5 (edge fn admin-refund-ticket: admin gate, Stripe refund, void credential, seat freed; + attendee-dialog button, mobile-safe). Every branch proven EXCEPT the successful real-money refund line: void-only path, 403 gate, already-voided idempotency, and the Stripe-failure 502 fail-safe (no seat freed without money returned) all tested live.</t>
         </is>
       </c>
-      <c r="C146" s="8" t="inlineStr">
+      <c r="C148" s="8" t="inlineStr">
         <is>
           <t>WAIT mode: on the next genuine member refund request, use Remove &amp; Refund in the event attendee dialog and verify: Stripe refunded, credential voided, seat freed, toast correct.</t>
         </is>
       </c>
-      <c r="D146" s="20" t="inlineStr">
+      <c r="D148" s="20" t="inlineStr">
         <is>
           <t>Verify</t>
         </is>
       </c>
-      <c r="E146" s="8" t="inlineStr">
+      <c r="E148" s="8" t="inlineStr">
         <is>
           <t>Zero-cost proof on the next real request. Sacred Walker (Jul 5) handled manually pre-feature; her case is the template.</t>
         </is>
       </c>
     </row>
-    <row r="147" ht="57.45" customFormat="1" customHeight="1" s="2">
-      <c r="A147" s="21" t="inlineStr">
+    <row r="149" ht="15" customFormat="1" customHeight="1" s="2">
+      <c r="A149" s="21" t="inlineStr">
         <is>
           <t>SESSION LOG — JUL 7–9 2026 (COMPLETED; kept as record, esp. the security fix)</t>
-        </is>
-      </c>
-    </row>
-    <row r="148" ht="57.45" customFormat="1" customHeight="1" s="2">
-      <c r="A148" s="16" t="inlineStr">
-        <is>
-          <t>[DONE] Security: dropped anon-readable active_members view + locked event_participants_view</t>
-        </is>
-      </c>
-      <c r="B148" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL FIX Jul 9: active_members and event_participants_view were SECURITY DEFINER views with ALL privileges granted to anon — an unauthenticated internet caller could read every member's email/phone/Stripe customer ID + all attendee contact info, AND active_members (auto-updatable single-table view) exposed an anon WRITE path into profiles. active_members had ZERO callers -&gt; DROPPED. event_participants_view -&gt; security_invoker=true + REVOKE anon/authenticated (sole caller send-campaign uses service-role, unaffected). member_counts left as-is (intentional).</t>
-        </is>
-      </c>
-      <c r="C148" s="23" t="inlineStr">
-        <is>
-          <t>DONE via SQL. Verified from OUTSIDE with anon key: active_members=404, event_participants_view=401 permission denied. No rows leaked. send-campaign confirmed still works.</t>
-        </is>
-      </c>
-      <c r="D148" s="24" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E148" s="23" t="inlineStr">
-        <is>
-          <t>Biggest find of the session. Was disguised as a 'review Security Definer flags' tracker row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A149" s="16" t="inlineStr">
-        <is>
-          <t>[DONE] Nine-job cron auth resurrection + 2 guards, all 10 jobs healthy</t>
-        </is>
-      </c>
-      <c r="B149" s="23" t="inlineStr">
-        <is>
-          <t>Full audit found NINE broken crons (sheet knew of 2). Fixed: Vault key was legacy JWT but runtime injects sb_secret_ (updated Vault); SQL typo value-&gt;decrypted_secret on jobs 3/4/13; event-reminder had no service-key path + a no-auth-header mass-email hole (both fixed, commit 09d637d). Then built 2 guards: business-profile-reminder 14-day cooldown via contact_activity + internal-account exclusion (503548c); guest-event-match at-capacity exclusion (d722800). Both jobs 2 &amp; 10 re-enabled. All 10 cron jobs now active + healthy.</t>
-        </is>
-      </c>
-      <c r="C149" s="23" t="inlineStr">
-        <is>
-          <t>All confirmed 200 on live ticks. Guards dry-run/logic verified. WATCH: first live ticks of job 2 (14:00 UTC every 2 days) + job 10 (13:00 UTC daily) — read-only confirm right people emailed.</t>
-        </is>
-      </c>
-      <c r="D149" s="24" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E149" s="23" t="inlineStr">
-        <is>
-          <t>Commits 09d637d, 503548c, d722800 + Vault + SQL. event-reminder security hole closed.</t>
         </is>
       </c>
     </row>
     <row r="150" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A150" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Sentry error monitoring — live + verified in prod</t>
+          <t>[DONE] Security: dropped anon-readable active_members view + locked event_participants_view</t>
         </is>
       </c>
       <c r="B150" s="23" t="inlineStr">
         <is>
-          <t>@sentry/nextjs wired (client+server+API+global-error), CSP allowance, instrumentation moved into src/ (Next ignores root-level with a src/ dir), DSN + source-map auth token in Vercel, /admin/sentry page activated. Prod capture VERIFIED (smoke-test error landed in feed).</t>
+          <t>CRITICAL FIX Jul 9: active_members and event_participants_view were SECURITY DEFINER views with ALL privileges granted to anon — an unauthenticated internet caller could read every member's email/phone/Stripe customer ID + all attendee contact info, AND active_members (auto-updatable single-table view) exposed an anon WRITE path into profiles. active_members had ZERO callers -&gt; DROPPED. event_participants_view -&gt; security_invoker=true + REVOKE anon/authenticated (sole caller send-campaign uses service-role, unaffected). member_counts left as-is (intentional).</t>
         </is>
       </c>
       <c r="C150" s="23" t="inlineStr">
         <is>
-          <t>Verified. WATCH: confirm Sentry project SLUG is exactly '704-collective' in a Vercel build log (source-map upload) — if wrong, traces stay minified (one-word fix).</t>
+          <t>DONE via SQL. Verified from OUTSIDE with anon key: active_members=404, event_participants_view=401 permission denied. No rows leaked. send-campaign confirmed still works.</t>
         </is>
       </c>
       <c r="D150" s="24" t="inlineStr">
@@ -4044,24 +4044,24 @@
       </c>
       <c r="E150" s="23" t="inlineStr">
         <is>
-          <t>Commits 417fb37/d779885/5d12aac/b437166. The safety net — Stage 1 complete.</t>
+          <t>Biggest find of the session. Was disguised as a 'review Security Definer flags' tracker row.</t>
         </is>
       </c>
     </row>
     <row r="151" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A151" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Josh Ahart full removal (exit workstream)</t>
+          <t>[DONE] Nine-job cron auth resurrection + 2 guards, all 10 jobs healthy</t>
         </is>
       </c>
       <c r="B151" s="23" t="inlineStr">
         <is>
-          <t>De-privileged (super_admin-&gt;lead), permanent ban, all 8 sessions + 64 tokens killed, profile deactivated, ambassador row disabled, removed from public /about page (0cc8c66), 2 dormant test dupe accounts hard-deleted. Stripe sub cancelled + Connect account rejected (Adam, dashboard). Platform passwords rotated (Adam).</t>
+          <t>Full audit found NINE broken crons (sheet knew of 2). Fixed: Vault key was legacy JWT but runtime injects sb_secret_ (updated Vault); SQL typo value-&gt;decrypted_secret on jobs 3/4/13; event-reminder had no service-key path + a no-auth-header mass-email hole (both fixed, commit 09d637d). Then built 2 guards: business-profile-reminder 14-day cooldown via contact_activity + internal-account exclusion (503548c); guest-event-match at-capacity exclusion (d722800). Both jobs 2 &amp; 10 re-enabled. All 10 cron jobs now active + healthy.</t>
         </is>
       </c>
       <c r="C151" s="23" t="inlineStr">
         <is>
-          <t>Verified: role=lead, 0 sessions/tokens, banned. Public site scrubbed. Dashboard-member removal confirmed by Adam.</t>
+          <t>All confirmed 200 on live ticks. Guards dry-run/logic verified. WATCH: first live ticks of job 2 (14:00 UTC every 2 days) + job 10 (13:00 UTC daily) — read-only confirm right people emailed.</t>
         </is>
       </c>
       <c r="D151" s="24" t="inlineStr">
@@ -4071,24 +4071,24 @@
       </c>
       <c r="E151" s="23" t="inlineStr">
         <is>
-          <t>NOT on the build sheet — exit workstream. Recorded here for completeness.</t>
+          <t>Commits 09d637d, 503548c, d722800 + Vault + SQL. event-reminder security hole closed.</t>
         </is>
       </c>
     </row>
     <row r="152" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A152" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Member status batch (Jul 9)</t>
+          <t>[DONE] Sentry error monitoring — live + verified in prod</t>
         </is>
       </c>
       <c r="B152" s="23" t="inlineStr">
         <is>
-          <t>Nicholas Stathopoulos + Robert Villante -&gt; non_member/inactive/override off/lead (Nick admin revoked + sessions killed). Whitney Cleland + Brenna Dunne + Kaelah Torres -&gt; ERASED (auth+profile+people+credentials deleted; all comped, no Stripe to cancel). More status changes flagged as coming.</t>
+          <t>@sentry/nextjs wired (client+server+API+global-error), CSP allowance, instrumentation moved into src/ (Next ignores root-level with a src/ dir), DSN + source-map auth token in Vercel, /admin/sentry page activated. Prod capture VERIFIED (smoke-test error landed in feed).</t>
         </is>
       </c>
       <c r="C152" s="23" t="inlineStr">
         <is>
-          <t>All verified via SQL (zeros on erase). Read-first footprint audit confirmed safe (no owned content cascaded).</t>
+          <t>Verified. WATCH: confirm Sentry project SLUG is exactly '704-collective' in a Vercel build log (source-map upload) — if wrong, traces stay minified (one-word fix).</t>
         </is>
       </c>
       <c r="D152" s="24" t="inlineStr">
@@ -4098,24 +4098,24 @@
       </c>
       <c r="E152" s="23" t="inlineStr">
         <is>
-          <t>Adam noted more member changes coming next session.</t>
+          <t>Commits 417fb37/d779885/5d12aac/b437166. The safety net — Stage 1 complete.</t>
         </is>
       </c>
     </row>
     <row r="153" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A153" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Business-event RSVP tier leak — closed + Annslee voided</t>
+          <t>[DONE] Josh Ahart full removal (exit workstream)</t>
         </is>
       </c>
       <c r="B153" s="23" t="inlineStr">
         <is>
-          <t>Social members could RSVP business-only events: create-member-rsvp never checked required_tier, and the mobile sticky RSVP bar bypassed the desktop gate. Fixed: server-side tier gate in the edge function (ff20ba9, admins exempt) + mobile CTA respects canRsvp (952fbb2). Annslee Bottoms' live breach credential on Jul-14 Business Member Meeting VOIDED. Past legacy breaches intentionally left (real attendance history).</t>
+          <t>De-privileged (super_admin-&gt;lead), permanent ban, all 8 sessions + 64 tokens killed, profile deactivated, ambassador row disabled, removed from public /about page (0cc8c66), 2 dormant test dupe accounts hard-deleted. Stripe sub cancelled + Connect account rejected (Adam, dashboard). Platform passwords rotated (Adam).</t>
         </is>
       </c>
       <c r="C153" s="23" t="inlineStr">
         <is>
-          <t>Verified: socialtest gets 403 'business members only' + red toast; direct-invoke blocked; Annslee active count on event = 0.</t>
+          <t>Verified: role=lead, 0 sessions/tokens, banned. Public site scrubbed. Dashboard-member removal confirmed by Adam.</t>
         </is>
       </c>
       <c r="D153" s="24" t="inlineStr">
@@ -4125,24 +4125,24 @@
       </c>
       <c r="E153" s="23" t="inlineStr">
         <is>
-          <t>Commits ff20ba9, 952fbb2. Guest-side email opt-out gap noted -&gt; folds into unsubscribe policy work.</t>
+          <t>NOT on the build sheet — exit workstream. Recorded here for completeness.</t>
         </is>
       </c>
     </row>
     <row r="154" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A154" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Discussion edit/delete (comments+posts+photos) + admin always-on access</t>
+          <t>[DONE] Member status batch (Jul 9)</t>
         </is>
       </c>
       <c r="B154" s="23" t="inlineStr">
         <is>
-          <t>Owners + admins can now edit/delete their own discussion comments (ecec3f8), posts (1e3adc1), and remove their own gallery photos (bcf746f); admins moderate anyone's. '(edited)' marker, soft-delete, silent removal. Also: admins now see the discussion link on any open event regardless of RSVP (583b343 — backend was already admin-exempt; was a missing-link discovery bug). Feed/comment/DM URL linkify (561403e).</t>
+          <t>Nicholas Stathopoulos + Robert Villante -&gt; non_member/inactive/override off/lead (Nick admin revoked + sessions killed). Whitney Cleland + Brenna Dunne + Kaelah Torres -&gt; ERASED (auth+profile+people+credentials deleted; all comped, no Stripe to cancel). More status changes flagged as coming.</t>
         </is>
       </c>
       <c r="C154" s="23" t="inlineStr">
         <is>
-          <t>All browser-tested desktop+mobile. Backend RLS already permitted; these were frontend gaps.</t>
+          <t>All verified via SQL (zeros on erase). Read-first footprint audit confirmed safe (no owned content cascaded).</t>
         </is>
       </c>
       <c r="D154" s="24" t="inlineStr">
@@ -4152,122 +4152,122 @@
       </c>
       <c r="E154" s="23" t="inlineStr">
         <is>
-          <t>5 commits. Discussion feature now fully moderatable.</t>
+          <t>Adam noted more member changes coming next session.</t>
         </is>
       </c>
     </row>
     <row r="155" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A155" s="16" t="inlineStr">
         <is>
+          <t>[DONE] Business-event RSVP tier leak — closed + Annslee voided</t>
+        </is>
+      </c>
+      <c r="B155" s="23" t="inlineStr">
+        <is>
+          <t>Social members could RSVP business-only events: create-member-rsvp never checked required_tier, and the mobile sticky RSVP bar bypassed the desktop gate. Fixed: server-side tier gate in the edge function (ff20ba9, admins exempt) + mobile CTA respects canRsvp (952fbb2). Annslee Bottoms' live breach credential on Jul-14 Business Member Meeting VOIDED. Past legacy breaches intentionally left (real attendance history).</t>
+        </is>
+      </c>
+      <c r="C155" s="23" t="inlineStr">
+        <is>
+          <t>Verified: socialtest gets 403 'business members only' + red toast; direct-invoke blocked; Annslee active count on event = 0.</t>
+        </is>
+      </c>
+      <c r="D155" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E155" s="23" t="inlineStr">
+        <is>
+          <t>Commits ff20ba9, 952fbb2. Guest-side email opt-out gap noted -&gt; folds into unsubscribe policy work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A156" s="16" t="inlineStr">
+        <is>
+          <t>[DONE] Discussion edit/delete (comments+posts+photos) + admin always-on access</t>
+        </is>
+      </c>
+      <c r="B156" s="23" t="inlineStr">
+        <is>
+          <t>Owners + admins can now edit/delete their own discussion comments (ecec3f8), posts (1e3adc1), and remove their own gallery photos (bcf746f); admins moderate anyone's. '(edited)' marker, soft-delete, silent removal. Also: admins now see the discussion link on any open event regardless of RSVP (583b343 — backend was already admin-exempt; was a missing-link discovery bug). Feed/comment/DM URL linkify (561403e).</t>
+        </is>
+      </c>
+      <c r="C156" s="23" t="inlineStr">
+        <is>
+          <t>All browser-tested desktop+mobile. Backend RLS already permitted; these were frontend gaps.</t>
+        </is>
+      </c>
+      <c r="D156" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E156" s="23" t="inlineStr">
+        <is>
+          <t>5 commits. Discussion feature now fully moderatable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="16" t="inlineStr">
+        <is>
           <t>[DONE] Small fixes: hubs 404, week_label, dead components, partners 400, org_settings, last_attended</t>
         </is>
       </c>
-      <c r="B155" s="23" t="inlineStr">
+      <c r="B157" s="23" t="inlineStr">
         <is>
           <t>hubs preview widget queried non-existent 'business_hubs' -&gt; fixed to 'hubs' (a00cc50, restored a silently-broken business-tier feature). ambassador-payout phantom week_label column removed (1f46e88). 3 dead admin components deleted, 1376 lines (306efa4). partners 400 fixed via column aliasing (d95a337, latent partner-disappearing bug). organization_settings tracker row was STALE (schema fine, closed). last_attended already built+firing -&gt; backfilled 17 pre-trigger rows, closed.</t>
         </is>
       </c>
-      <c r="C155" s="23" t="inlineStr">
+      <c r="C157" s="23" t="inlineStr">
         <is>
           <t>All tsc+browser verified. org_settings &amp; last_attended were already-done rows.</t>
         </is>
       </c>
-      <c r="D155" s="24" t="inlineStr">
+      <c r="D157" s="24" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="E155" s="23" t="inlineStr">
+      <c r="E157" s="23" t="inlineStr">
         <is>
           <t>Commits a00cc50, 1f46e88, 306efa4, d95a337 + 2 SQL closes.</t>
         </is>
       </c>
     </row>
-    <row r="156" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A156" s="25" t="inlineStr">
+    <row r="158">
+      <c r="A158" s="25" t="inlineStr">
         <is>
           <t>PHASE 2  ·  MAJOR BUILDS (each gets its own detailed scope before build)</t>
         </is>
       </c>
-      <c r="B156" s="29" t="n"/>
-      <c r="C156" s="29" t="n"/>
-      <c r="D156" s="29" t="n"/>
-      <c r="E156" s="30" t="n"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="4" t="inlineStr">
+      <c r="B158" s="29" t="n"/>
+      <c r="C158" s="29" t="n"/>
+      <c r="D158" s="29" t="n"/>
+      <c r="E158" s="30" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
         <is>
           <t>MAJOR BUILDS — EACH GETS ITS OWN DETAILED SCOPE BEFORE BUILD   ·   7 items</t>
         </is>
       </c>
-      <c r="B157" s="29" t="n"/>
-      <c r="C157" s="29" t="n"/>
-      <c r="D157" s="29" t="n"/>
-      <c r="E157" s="30" t="n"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="7" t="inlineStr">
-        <is>
-          <t>CRM system</t>
-        </is>
-      </c>
-      <c r="B158" s="8" t="inlineStr">
-        <is>
-          <t>Full customer-relationship system built ON the merged person record: 360-degree member view, segments/audiences, lifecycle tracking. The internal data model IS the CRM (not a re-introduced external tool).</t>
-        </is>
-      </c>
-      <c r="C158" s="8" t="inlineStr">
-        <is>
-          <t>Own detailed scope before build.</t>
-        </is>
-      </c>
-      <c r="D158" s="26" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="E158" s="8" t="inlineStr">
-        <is>
-          <t>Built on the canonical person record from Phase 1. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag (carve-out keeps /admin/crm/campaigns live for the newsletter).</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="7" t="inlineStr">
-        <is>
-          <t>Preferred Business Network</t>
-        </is>
-      </c>
-      <c r="B159" s="8" t="inlineStr">
-        <is>
-          <t>New paid product: vetted local-business listings, $300/mo to be listed. Lives in the portal first, public domains later. Includes the internal 'Seats' system. Social members browse this to find services.</t>
-        </is>
-      </c>
-      <c r="C159" s="8" t="inlineStr">
-        <is>
-          <t>Own detailed scope before build.</t>
-        </is>
-      </c>
-      <c r="D159" s="26" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="E159" s="8" t="inlineStr">
-        <is>
-          <t>Plugs into The Network surface built in Phase 1.</t>
-        </is>
-      </c>
+      <c r="B159" s="29" t="n"/>
+      <c r="C159" s="29" t="n"/>
+      <c r="D159" s="29" t="n"/>
+      <c r="E159" s="30" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
         <is>
-          <t>Partner Portal (audit, then repurpose or remove)</t>
+          <t>CRM system</t>
         </is>
       </c>
       <c r="B160" s="8" t="inlineStr">
         <is>
-          <t>An existing, mostly-built partner portal of unclear purpose. Audit it, then either repurpose it as the Preferred Business Network management surface or remove it. Frozen until then.</t>
+          <t>Full customer-relationship system built ON the merged person record: 360-degree member view, segments/audiences, lifecycle tracking. The internal data model IS the CRM (not a re-introduced external tool).</t>
         </is>
       </c>
       <c r="C160" s="8" t="inlineStr">
@@ -4282,19 +4282,19 @@
       </c>
       <c r="E160" s="8" t="inlineStr">
         <is>
-          <t>Audit first; likely becomes the Preferred Business Network management surface. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag.</t>
+          <t>Built on the canonical person record from Phase 1. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag (carve-out keeps /admin/crm/campaigns live for the newsletter).</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
         <is>
-          <t>Task center for admins (lite project tool)</t>
+          <t>Preferred Business Network</t>
         </is>
       </c>
       <c r="B161" s="8" t="inlineStr">
         <is>
-          <t>A super-light ClickUp-style task center for admins/super-admins: create, assign, track tasks.</t>
+          <t>New paid product: vetted local-business listings, $300/mo to be listed. Lives in the portal first, public domains later. Includes the internal 'Seats' system. Social members browse this to find services.</t>
         </is>
       </c>
       <c r="C161" s="8" t="inlineStr">
@@ -4309,19 +4309,19 @@
       </c>
       <c r="E161" s="8" t="inlineStr">
         <is>
-          <t>Lite task assignment + tracking for admin / super-admin.</t>
+          <t>Plugs into The Network surface built in Phase 1.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
         <is>
-          <t>Shared email inbox view for super-admins</t>
+          <t>Partner Portal (audit, then repurpose or remove)</t>
         </is>
       </c>
       <c r="B162" s="8" t="inlineStr">
         <is>
-          <t>A shared inbox view so super-admins can see the team email (hello@) in one place.</t>
+          <t>An existing, mostly-built partner portal of unclear purpose. Audit it, then either repurpose it as the Preferred Business Network management surface or remove it. Frozen until then.</t>
         </is>
       </c>
       <c r="C162" s="8" t="inlineStr">
@@ -4336,26 +4336,46 @@
       </c>
       <c r="E162" s="8" t="inlineStr">
         <is>
-          <t>Super-admin visibility into hello@.</t>
+          <t>Audit first; likely becomes the Preferred Business Network management surface. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag.</t>
         </is>
       </c>
     </row>
     <row r="163" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A163" s="7" t="inlineStr">
         <is>
-          <t>Corporate / bulk-sales floating-seats portal</t>
+          <t>Task center for admins (lite project tool)</t>
+        </is>
+      </c>
+      <c r="B163" s="8" t="inlineStr">
+        <is>
+          <t>A super-light ClickUp-style task center for admins/super-admins: create, assign, track tasks.</t>
+        </is>
+      </c>
+      <c r="C163" s="8" t="inlineStr">
+        <is>
+          <t>Own detailed scope before build.</t>
+        </is>
+      </c>
+      <c r="D163" s="26" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="E163" s="8" t="inlineStr">
+        <is>
+          <t>Lite task assignment + tracking for admin / super-admin.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
         <is>
-          <t>Full mobile app</t>
+          <t>Shared email inbox view for super-admins</t>
         </is>
       </c>
       <c r="B164" s="8" t="inlineStr">
         <is>
-          <t>A full native mobile application. The largest Phase 2 build.</t>
+          <t>A shared inbox view so super-admins can see the team email (hello@) in one place.</t>
         </is>
       </c>
       <c r="C164" s="8" t="inlineStr">
@@ -4370,89 +4390,69 @@
       </c>
       <c r="E164" s="8" t="inlineStr">
         <is>
-          <t>The final, largest Phase 2 effort.</t>
+          <t>Super-admin visibility into hello@.</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="4" t="inlineStr">
-        <is>
-          <t>OPEN WATCH ITEMS — ADDED 2026-07-19   ·   8 items</t>
-        </is>
-      </c>
-      <c r="B165" s="29" t="n"/>
-      <c r="C165" s="29" t="n"/>
-      <c r="D165" s="29" t="n"/>
-      <c r="E165" s="30" t="n"/>
+      <c r="A165" s="7" t="inlineStr">
+        <is>
+          <t>Corporate / bulk-sales floating-seats portal</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
         <is>
-          <t>Stage 5 Wave 4 - classify the ~204 guest/lead reverse-orphan profiles</t>
+          <t>Full mobile app</t>
         </is>
       </c>
       <c r="B166" s="8" t="inlineStr">
         <is>
-          <t>Waves 1-3 linked/minted the clear identity cases; the residual ~204 profiles are guests or leads that never became members and must be classified, not minted as members.</t>
+          <t>A full native mobile application. The largest Phase 2 build.</t>
         </is>
       </c>
       <c r="C166" s="8" t="inlineStr">
         <is>
-          <t>Decide the guest-vs-lead-vs-skip rule; mint people rows with the correct non-active member_status; reuse the Wave 3 additive/reversible pattern (metadata.created_by). Rehearse on develop first.</t>
-        </is>
-      </c>
-      <c r="D166" s="9" t="inlineStr">
-        <is>
-          <t>Build</t>
+          <t>Own detailed scope before build.</t>
+        </is>
+      </c>
+      <c r="D166" s="26" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="E166" s="8" t="inlineStr">
         <is>
-          <t>Waves 1-3 applied to prod. Wave 4 is the guest/lead bucket - needs a classification rule before any minting.</t>
+          <t>The final, largest Phase 2 effort.</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="7" t="inlineStr">
-        <is>
-          <t>Refill the Vercel NEXT_PUBLIC_TURNSTILE_SITE_KEY value (hardcode fallback active)</t>
-        </is>
-      </c>
-      <c r="B167" s="8" t="inlineStr">
-        <is>
-          <t>The prod env var was set to an empty string, which made the Turnstile widget render nothing and locked members out during an incident. A hardcoded public site-key fallback in TurnstileWidget.tsx currently masks the missing value.</t>
-        </is>
-      </c>
-      <c r="C167" s="8" t="inlineStr">
-        <is>
-          <t>Set the real public site key for NEXT_PUBLIC_TURNSTILE_SITE_KEY in Vercel (production), redeploy, confirm the widget renders from the env var, then optionally remove the hardcoded fallback.</t>
-        </is>
-      </c>
-      <c r="D167" s="9" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E167" s="8" t="inlineStr">
-        <is>
-          <t>Public site key (safe): 0x4AAAAAAD3gqCivsYyImeUH. Fallback keeps login working today; refill so config isn't hidden in code.</t>
-        </is>
-      </c>
+      <c r="A167" s="4" t="inlineStr">
+        <is>
+          <t>OPEN WATCH ITEMS — ADDED 2026-07-19   ·   8 items</t>
+        </is>
+      </c>
+      <c r="B167" s="29" t="n"/>
+      <c r="C167" s="29" t="n"/>
+      <c r="D167" s="29" t="n"/>
+      <c r="E167" s="30" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
         <is>
-          <t>Resolve the capacity-trigger split-brain (tickets vs attendance_credentials counting)</t>
+          <t>Stage 5 Wave 4 - classify the ~204 guest/lead reverse-orphan profiles</t>
         </is>
       </c>
       <c r="B168" s="8" t="inlineStr">
         <is>
-          <t>Event capacity is enforced by triggers on two tables (attendance_credentials and legacy tickets) that count independently, so the seated count can disagree depending on the write path.</t>
+          <t>Waves 1-3 linked/minted the clear identity cases; the residual ~204 profiles are guests or leads that never became members and must be classified, not minted as members.</t>
         </is>
       </c>
       <c r="C168" s="8" t="inlineStr">
         <is>
-          <t>Pick one source of truth (attendance_credentials); make both trigger families count consistently, or retire the legacy tickets capacity path once tickets is fully retired. Coordinates with 'Finish retiring the old ticket tables'.</t>
+          <t>Decide the guest-vs-lead-vs-skip rule; mint people rows with the correct non-active member_status; reuse the Wave 3 additive/reversible pattern (metadata.created_by). Rehearse on develop first.</t>
         </is>
       </c>
       <c r="D168" s="9" t="inlineStr">
@@ -4462,24 +4462,24 @@
       </c>
       <c r="E168" s="8" t="inlineStr">
         <is>
-          <t>The admin_override bypass now spans both trigger families; the underlying counting split remains until tickets is retired.</t>
+          <t>Waves 1-3 applied to prod. Wave 4 is the guest/lead bucket - needs a classification rule before any minting.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
         <is>
-          <t>Q6 canceled-but-paying tripwire (canceled-drift detection)</t>
+          <t>Refill the Vercel NEXT_PUBLIC_TURNSTILE_SITE_KEY value (hardcode fallback active)</t>
         </is>
       </c>
       <c r="B169" s="8" t="inlineStr">
         <is>
-          <t>Members whose app status shows canceled while Stripe still bills them (or the inverse) - a billing/status drift that should trip an alert instead of going silent.</t>
+          <t>The prod env var was set to an empty string, which made the Turnstile widget render nothing and locked members out during an incident. A hardcoded public site-key fallback in TurnstileWidget.tsx currently masks the missing value.</t>
         </is>
       </c>
       <c r="C169" s="8" t="inlineStr">
         <is>
-          <t>Add a scheduled check comparing profiles.subscription_status vs the live Stripe subscription state; alert on canceled-in-app-but-active-in-Stripe and the inverse.</t>
+          <t>Set the real public site key for NEXT_PUBLIC_TURNSTILE_SITE_KEY in Vercel (production), redeploy, confirm the widget renders from the env var, then optionally remove the hardcoded fallback.</t>
         </is>
       </c>
       <c r="D169" s="9" t="inlineStr">
@@ -4489,24 +4489,24 @@
       </c>
       <c r="E169" s="8" t="inlineStr">
         <is>
-          <t>The develop seed carries a canceled-drift (Q6) dummy for rehearsal. Folds into the DB/Stripe drift watch + admin health dashboard.</t>
+          <t>Public site key (safe): 0x4AAAAAAD3gqCivsYyImeUH. Fallback keeps login working today; refill so config isn't hidden in code.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
         <is>
-          <t>Delete the stray Stripe Connect account</t>
+          <t>Resolve the capacity-trigger split-brain (tickets vs attendance_credentials counting)</t>
         </is>
       </c>
       <c r="B170" s="8" t="inlineStr">
         <is>
-          <t>A leftover Stripe Connect (Express) account from the ambassador / exit workstream needs removing so it doesn't linger.</t>
+          <t>Event capacity is enforced by triggers on two tables (attendance_credentials and legacy tickets) that count independently, so the seated count can disagree depending on the write path.</t>
         </is>
       </c>
       <c r="C170" s="8" t="inlineStr">
         <is>
-          <t>Confirm the account has no pending balance or payouts, then delete/reject it in the Stripe dashboard. Owner task.</t>
+          <t>Pick one source of truth (attendance_credentials); make both trigger families count consistently, or retire the legacy tickets capacity path once tickets is fully retired. Coordinates with 'Finish retiring the old ticket tables'.</t>
         </is>
       </c>
       <c r="D170" s="9" t="inlineStr">
@@ -4516,24 +4516,24 @@
       </c>
       <c r="E170" s="8" t="inlineStr">
         <is>
-          <t>Cleanup item from the ambassador / Connect work; low blast radius.</t>
+          <t>The admin_override bypass now spans both trigger families; the underlying counting split remains until tickets is retired.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
         <is>
-          <t>ManyChat - disconnect the Instagram-side integration</t>
+          <t>Q6 canceled-but-paying tripwire (canceled-drift detection)</t>
         </is>
       </c>
       <c r="B171" s="8" t="inlineStr">
         <is>
-          <t>The IG-side ManyChat connection needs to be disconnected / cleaned up. This is teardown of the current Instagram link, separate from the auto-DM build.</t>
+          <t>Members whose app status shows canceled while Stripe still bills them (or the inverse) - a billing/status drift that should trip an alert instead of going silent.</t>
         </is>
       </c>
       <c r="C171" s="8" t="inlineStr">
         <is>
-          <t>Disconnect the Instagram account from ManyChat (owner task in ManyChat / Meta); confirm no active automations still reference it.</t>
+          <t>Add a scheduled check comparing profiles.subscription_status vs the live Stripe subscription state; alert on canceled-in-app-but-active-in-Stripe and the inverse.</t>
         </is>
       </c>
       <c r="D171" s="9" t="inlineStr">
@@ -4543,471 +4543,525 @@
       </c>
       <c r="E171" s="8" t="inlineStr">
         <is>
-          <t>Distinct from the 'Instagram comment auto-DM (ManyChat)' build row above - that row stays as-is.</t>
+          <t>The develop seed carries a canceled-drift (Q6) dummy for rehearsal. Folds into the DB/Stripe drift watch + admin health dashboard.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
         <is>
-          <t>DB / Stripe drift watch items</t>
+          <t>Delete the stray Stripe Connect account</t>
         </is>
       </c>
       <c r="B172" s="8" t="inlineStr">
         <is>
-          <t>Ongoing watch on the places where the database and Stripe can drift out of sync: subscription statuses, customer email on email-change, retired legacy prices, orphaned Stripe customers.</t>
+          <t>A leftover Stripe Connect (Express) account from the ambassador / exit workstream needs removing so it doesn't linger.</t>
         </is>
       </c>
       <c r="C172" s="8" t="inlineStr">
         <is>
-          <t>Track and periodically reconcile; surface on the admin health dashboard. Pairs with the Q6 tripwire and the 'email change keeps Stripe billing in sync' verify.</t>
+          <t>Confirm the account has no pending balance or payouts, then delete/reject it in the Stripe dashboard. Owner task.</t>
         </is>
       </c>
       <c r="D172" s="9" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="E172" s="8" t="inlineStr">
         <is>
-          <t>Umbrella watch item; individual drifts get their own rows as they surface.</t>
+          <t>Cleanup item from the ambassador / Connect work; low blast radius.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
         <is>
+          <t>ManyChat - disconnect the Instagram-side integration</t>
+        </is>
+      </c>
+      <c r="B173" s="8" t="inlineStr">
+        <is>
+          <t>The IG-side ManyChat connection needs to be disconnected / cleaned up. This is teardown of the current Instagram link, separate from the auto-DM build.</t>
+        </is>
+      </c>
+      <c r="C173" s="8" t="inlineStr">
+        <is>
+          <t>Disconnect the Instagram account from ManyChat (owner task in ManyChat / Meta); confirm no active automations still reference it.</t>
+        </is>
+      </c>
+      <c r="D173" s="9" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E173" s="8" t="inlineStr">
+        <is>
+          <t>Distinct from the 'Instagram comment auto-DM (ManyChat)' build row above - that row stays as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="7" t="inlineStr">
+        <is>
+          <t>DB / Stripe drift watch items</t>
+        </is>
+      </c>
+      <c r="B174" s="8" t="inlineStr">
+        <is>
+          <t>Ongoing watch on the places where the database and Stripe can drift out of sync: subscription statuses, customer email on email-change, retired legacy prices, orphaned Stripe customers.</t>
+        </is>
+      </c>
+      <c r="C174" s="8" t="inlineStr">
+        <is>
+          <t>Track and periodically reconcile; surface on the admin health dashboard. Pairs with the Q6 tripwire and the 'email change keeps Stripe billing in sync' verify.</t>
+        </is>
+      </c>
+      <c r="D174" s="9" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="E174" s="8" t="inlineStr">
+        <is>
+          <t>Umbrella watch item; individual drifts get their own rows as they surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="7" t="inlineStr">
+        <is>
           <t>Waitlist claim links - monitor first real-world use</t>
         </is>
       </c>
-      <c r="B173" s="8" t="inlineStr">
+      <c r="B175" s="8" t="inlineStr">
         <is>
           <t>Cancel frees a seat -&gt; the first waitlister is emailed a 24h claim link -&gt; they claim it. Rehearsed as a full matrix on develop and shipped to prod; needs a read-only confirm on its first genuine use.</t>
         </is>
       </c>
-      <c r="C173" s="8" t="inlineStr">
+      <c r="C175" s="8" t="inlineStr">
         <is>
           <t>On the next real cancellation that frees a seat on a full, waitlisted event, confirm: notified_at/expires_at stamped, the email sent, the claimant claimed (member_rsvp with metadata source=waitlist_claim), and the waitlist row deleted.</t>
         </is>
       </c>
-      <c r="D173" s="9" t="inlineStr">
+      <c r="D175" s="9" t="inlineStr">
         <is>
           <t>Verify</t>
         </is>
       </c>
-      <c r="E173" s="8" t="inlineStr">
+      <c r="E175" s="8" t="inlineStr">
         <is>
           <t>Shipped 2026-07-19. Zero-cost proof on first real use, like the Remove &amp; Refund WAIT-mode row.</t>
         </is>
       </c>
     </row>
-    <row r="174">
-      <c r="A174" s="27" t="inlineStr">
+    <row r="176">
+      <c r="A176" s="27" t="inlineStr">
         <is>
           <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="28" t="inlineStr">
-        <is>
-          <t>Billing views: admin billing panel + member price/renewal display</t>
-        </is>
-      </c>
-      <c r="B175" s="28" t="inlineStr">
-        <is>
-          <t>Admin contact billing panel + member-facing price/renewal display. Three new profile columns (comp_reason, external_paid_through, external_payment_note) are live on both DBs; the UI/code build is in flight.</t>
-        </is>
-      </c>
-      <c r="C175" s="28" t="inlineStr">
-        <is>
-          <t>Extend admin contact detail with live Stripe billing; surface price/renewal/discount on member settings; wire the three new profile columns into admin editors.</t>
-        </is>
-      </c>
-      <c r="D175" s="28" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
-        </is>
-      </c>
-      <c r="E175" s="28" t="inlineStr">
-        <is>
-          <t>Columns live both DBs; code build in flight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="28" t="inlineStr">
-        <is>
-          <t>Report builder: admin/super_admin any-filter member/payment reports</t>
-        </is>
-      </c>
-      <c r="B176" s="28" t="inlineStr">
-        <is>
-          <t>Admin/super_admin reporting with arbitrary filters over members and payments. Data-cleanup prerequisite is DONE; build after billing views.</t>
-        </is>
-      </c>
-      <c r="C176" s="28" t="inlineStr">
-        <is>
-          <t>Build after billing views lands. Admin/super_admin only; any-filter member + payment reports.</t>
-        </is>
-      </c>
-      <c r="D176" s="28" t="inlineStr">
-        <is>
-          <t>QUEUED-BACKLOGGED</t>
-        </is>
-      </c>
-      <c r="E176" s="28" t="inlineStr">
-        <is>
-          <t>v1 proposal complete and approved-in-principle (DB-only cut, 3 entities, column picker, CSV export, 4 presets, server-paginated, ~7 files); resume at build sign-off. Cheap adds discussed: ambassador-referred, price tier, cancel reasons.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="28" t="inlineStr">
         <is>
-          <t>Business comp invite flow: welcome template + admin invite tool</t>
+          <t>Billing views: admin billing panel + member price/renewal display</t>
         </is>
       </c>
       <c r="B177" s="28" t="inlineStr">
         <is>
-          <t>Welcome email template plus an admin tool to invite a business member (comp path).</t>
+          <t>Admin contact billing panel + member-facing price/renewal display. Three new profile columns (comp_reason, external_paid_through, external_payment_note) are live on both DBs; the UI/code build is in flight.</t>
         </is>
       </c>
       <c r="C177" s="28" t="inlineStr">
         <is>
-          <t>Blocked on Adam: invitee list + design answers. Then template + admin invite UI.</t>
+          <t>Extend admin contact detail with live Stripe billing; surface price/renewal/discount on member settings; wire the three new profile columns into admin editors.</t>
         </is>
       </c>
       <c r="D177" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: list + design answers</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="E177" s="28" t="inlineStr">
         <is>
-          <t>Needs invitee list + design answers from Adam.</t>
+          <t>Columns live both DBs; code build in flight.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="28" t="inlineStr">
         <is>
-          <t>Admin 'Invite comp member' button - form (name, company, email, phone, comp note), creates comp'd account + sends welcome email, note auto-attached to billing view (member + admin); v1 invite flow built without UI, button is the addon</t>
+          <t>Report builder: admin/super_admin any-filter member/payment reports</t>
         </is>
       </c>
       <c r="B178" s="28" t="inlineStr">
         <is>
-          <t>Admin UI button/form to invite a complimentary business member: name, company, email, phone, and comp note. Creates the comp'd account, sends the welcome email, and attaches the note to the billing view for both member and admin.</t>
+          <t>Admin/super_admin reporting with arbitrary filters over members and payments. Data-cleanup prerequisite is DONE; build after billing views.</t>
         </is>
       </c>
       <c r="C178" s="28" t="inlineStr">
         <is>
-          <t>Addon after v1 invite flow (API/ops path without UI). Build the Invite comp member button + form once the headless invite path exists.</t>
+          <t>Build after billing views lands. Admin/super_admin only; any-filter member + payment reports.</t>
         </is>
       </c>
       <c r="D178" s="28" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>QUEUED-BACKLOGGED</t>
         </is>
       </c>
       <c r="E178" s="28" t="inlineStr">
         <is>
-          <t>v1 invite flow built without UI; this button is the future addon.</t>
+          <t>v1 proposal complete and approved-in-principle (DB-only cut, 3 entities, column picker, CSV export, 4 presets, server-paginated, ~7 files); resume at build sign-off. Cheap adds discussed: ambassador-referred, price tier, cancel reasons.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="28" t="inlineStr">
         <is>
-          <t>Mike Perez: account cleanup + re-join link at $150 founding</t>
+          <t>Business comp invite flow: welcome template + admin invite tool</t>
         </is>
       </c>
       <c r="B179" s="28" t="inlineStr">
         <is>
-          <t>After Adam's conversation: clean up Mike's canceled/failed-billing account and send a founding-rate $150 re-join link.</t>
+          <t>Welcome email template plus an admin tool to invite a business member (comp path).</t>
         </is>
       </c>
       <c r="C179" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM conversation first. Then cleanup + founding $150 checkout/re-join link.</t>
+          <t>Blocked on Adam: invitee list + design answers. Then template + admin invite UI.</t>
         </is>
       </c>
       <c r="D179" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: conversation first</t>
+          <t>WAITING ON ADAM: list + design answers</t>
         </is>
       </c>
       <c r="E179" s="28" t="inlineStr">
         <is>
-          <t>Founding $150; conversation first.</t>
+          <t>Needs invitee list + design answers from Adam.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="28" t="inlineStr">
         <is>
-          <t>Zane Mackey comp_reason entry</t>
+          <t>Admin 'Invite comp member' button - form (name, company, email, phone, comp note), creates comp'd account + sends welcome email, note auto-attached to billing view (member + admin); v1 invite flow built without UI, button is the addon</t>
         </is>
       </c>
       <c r="B180" s="28" t="inlineStr">
         <is>
-          <t>Record a one-phrase comp_reason on Zane Mackey's profile now that the column exists.</t>
+          <t>Admin UI button/form to invite a complimentary business member: name, company, email, phone, and comp note. Creates the comp'd account, sends the welcome email, and attaches the note to the billing view for both member and admin.</t>
         </is>
       </c>
       <c r="C180" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: one phrase for comp_reason.</t>
+          <t>Addon after v1 invite flow (API/ops path without UI). Build the Invite comp member button + form once the headless invite path exists.</t>
         </is>
       </c>
       <c r="D180" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: one phrase</t>
+          <t>QUEUED</t>
         </is>
       </c>
       <c r="E180" s="28" t="inlineStr">
         <is>
-          <t>One phrase for comp_reason.</t>
+          <t>v1 invite flow built without UI; this button is the future addon.</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="28" t="inlineStr">
         <is>
-          <t>Zach Trusky renewal ~Nov/Dec 2026 — honored $1,034 annual</t>
+          <t>Mike Perez: account cleanup + re-join link at $150 founding</t>
         </is>
       </c>
       <c r="B181" s="28" t="inlineStr">
         <is>
-          <t>Zach's annual amount lives outside Stripe ($1,034 honored). Need reminder + collection path decision around Nov/Dec 2026.</t>
+          <t>After Adam's conversation: clean up Mike's canceled/failed-billing account and send a founding-rate $150 re-join link.</t>
         </is>
       </c>
       <c r="C181" s="28" t="inlineStr">
         <is>
-          <t>Schedule reminder; decide collection path (manual invoice vs Stripe annual vs override).</t>
+          <t>WAITING ON ADAM conversation first. Then cleanup + founding $150 checkout/re-join link.</t>
         </is>
       </c>
       <c r="D181" s="28" t="inlineStr">
         <is>
-          <t>SCHEDULED NOV 2026</t>
+          <t>WAITING ON ADAM: conversation first</t>
         </is>
       </c>
       <c r="E181" s="28" t="inlineStr">
         <is>
-          <t>Honored $1,034 annual; no Stripe customer today.</t>
+          <t>Founding $150; conversation first.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="28" t="inlineStr">
         <is>
-          <t>Security: unknown third-party script (batatatech.com) on Glue Up admin pages</t>
+          <t>Zane Mackey comp_reason entry</t>
         </is>
       </c>
       <c r="B182" s="28" t="inlineStr">
         <is>
-          <t>Unknown batatatech.com script firing on Glue Up admin pages — treat as extension/malware until proven otherwise; audit browsers + rotate passwords.</t>
+          <t>Record a one-phrase comp_reason on Zane Mackey's profile now that the column exists.</t>
         </is>
       </c>
       <c r="C182" s="28" t="inlineStr">
         <is>
-          <t>Browser extension audit on machines that use Glue Up admin; password rotation for affected accounts.</t>
+          <t>WAITING ON ADAM: one phrase for comp_reason.</t>
         </is>
       </c>
       <c r="D182" s="28" t="inlineStr">
         <is>
-          <t>OPEN - Adam chrome://extensions only</t>
+          <t>WAITING ON ADAM: one phrase</t>
         </is>
       </c>
       <c r="E182" s="28" t="inlineStr">
         <is>
-          <t>repo confirmed clean 8/4 - scope is Adam's chrome://extensions only</t>
+          <t>One phrase for comp_reason.</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>[DONE] Promo system endstate 8/5</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>Supersedes Stripe support ticket + ticket-checkout promo fast-follow (removed).</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
+      <c r="A183" s="28" t="inlineStr">
+        <is>
+          <t>Zach Trusky renewal ~Nov/Dec 2026 — honored $1,034 annual</t>
+        </is>
+      </c>
+      <c r="B183" s="28" t="inlineStr">
+        <is>
+          <t>Zach's annual amount lives outside Stripe ($1,034 honored). Need reminder + collection path decision around Nov/Dec 2026.</t>
+        </is>
+      </c>
+      <c r="C183" s="28" t="inlineStr">
+        <is>
+          <t>Schedule reminder; decide collection path (manual invoice vs Stripe annual vs override).</t>
+        </is>
+      </c>
+      <c r="D183" s="28" t="inlineStr">
+        <is>
+          <t>SCHEDULED NOV 2026</t>
+        </is>
+      </c>
+      <c r="E183" s="28" t="inlineStr">
+        <is>
+          <t>Honored $1,034 annual; no Stripe customer today.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="28" t="inlineStr">
         <is>
-          <t>Calendar update-leg verification via throwaway event</t>
+          <t>Security: unknown third-party script (batatatech.com) on Glue Up admin pages</t>
         </is>
       </c>
       <c r="B184" s="28" t="inlineStr">
         <is>
-          <t>Verify that event-edit REQUEST invites actually move real calendars (ICS sequence / update leg) using a throwaway event.</t>
+          <t>Unknown batatatech.com script firing on Glue Up admin pages — treat as extension/malware until proven otherwise; audit browsers + rotate passwords.</t>
         </is>
       </c>
       <c r="C184" s="28" t="inlineStr">
         <is>
-          <t>Create throwaway event, subscribe, edit, confirm calendars update; then delete throwaway.</t>
+          <t>Browser extension audit on machines that use Glue Up admin; password rotation for affected accounts.</t>
         </is>
       </c>
       <c r="D184" s="28" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN - Adam chrome://extensions only</t>
         </is>
       </c>
       <c r="E184" s="28" t="inlineStr">
         <is>
-          <t>Throwaway event verification of REQUEST/update path.</t>
+          <t>repo confirmed clean 8/4 - scope is Adam's chrome://extensions only</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="28" t="inlineStr">
-        <is>
-          <t>Resend click-tracking subdomain (DNS)</t>
-        </is>
-      </c>
-      <c r="B185" s="28" t="inlineStr">
-        <is>
-          <t>Configure Resend click-tracking subdomain — Adam hands / DNS.</t>
-        </is>
-      </c>
-      <c r="C185" s="28" t="inlineStr">
-        <is>
-          <t>ADAM DNS: add Resend click-tracking subdomain CNAME + add Resend to SPF include (current SPF is Google-only). Confirmed missing 8/4.</t>
-        </is>
-      </c>
-      <c r="D185" s="28" t="inlineStr">
-        <is>
-          <t>ADAM - DNS</t>
-        </is>
-      </c>
-      <c r="E185" s="28" t="inlineStr">
-        <is>
-          <t>confirmed NOT configured 8/4; also add Resend to SPF include during same DNS visit</t>
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>[DONE] Promo system endstate 8/5</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Supersedes Stripe support ticket + ticket-checkout promo fast-follow (removed).</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="28" t="inlineStr">
         <is>
-          <t>/welcome checkout-flow coverage on develop</t>
+          <t>Calendar update-leg verification via throwaway event</t>
         </is>
       </c>
       <c r="B186" s="28" t="inlineStr">
         <is>
-          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
+          <t>Verify that event-edit REQUEST invites actually move real calendars (ICS sequence / update leg) using a throwaway event.</t>
         </is>
       </c>
       <c r="C186" s="28" t="inlineStr">
         <is>
-          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
+          <t>Create throwaway event, subscribe, edit, confirm calendars update; then delete throwaway.</t>
         </is>
       </c>
       <c r="D186" s="28" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="E186" s="28" t="inlineStr">
         <is>
-          <t>Untested on develop; no Stripe checkout env.</t>
+          <t>Throwaway event verification of REQUEST/update path.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="28" t="inlineStr">
         <is>
-          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
+          <t>Resend click-tracking subdomain (DNS)</t>
         </is>
       </c>
       <c r="B187" s="28" t="inlineStr">
         <is>
-          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
+          <t>Configure Resend click-tracking subdomain — Adam hands / DNS.</t>
         </is>
       </c>
       <c r="C187" s="28" t="inlineStr">
         <is>
-          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
+          <t>ADAM DNS: add Resend click-tracking subdomain CNAME + add Resend to SPF include (current SPF is Google-only). Confirmed missing 8/4.</t>
         </is>
       </c>
       <c r="D187" s="28" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>ADAM - DNS</t>
         </is>
       </c>
       <c r="E187" s="28" t="inlineStr">
         <is>
-          <t>Revisit in identity-bridge work.</t>
+          <t>confirmed NOT configured 8/4; also add Resend to SPF include during same DNS visit</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="28" t="inlineStr">
         <is>
-          <t>Retire the Google Sheets tracker path</t>
+          <t>/welcome checkout-flow coverage on develop</t>
         </is>
       </c>
       <c r="B188" s="28" t="inlineStr">
         <is>
-          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
+          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
         </is>
       </c>
       <c r="C188" s="28" t="inlineStr">
         <is>
-          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
+          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
         </is>
       </c>
       <c r="D188" s="28" t="inlineStr">
         <is>
-          <t>QUEUED - cleanup</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="E188" s="28" t="inlineStr">
         <is>
-          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
+          <t>Untested on develop; no Stripe checkout env.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="28" t="inlineStr">
         <is>
+          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
+        </is>
+      </c>
+      <c r="B189" s="28" t="inlineStr">
+        <is>
+          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
+        </is>
+      </c>
+      <c r="C189" s="28" t="inlineStr">
+        <is>
+          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
+        </is>
+      </c>
+      <c r="D189" s="28" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="E189" s="28" t="inlineStr">
+        <is>
+          <t>Revisit in identity-bridge work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="28" t="inlineStr">
+        <is>
+          <t>Retire the Google Sheets tracker path</t>
+        </is>
+      </c>
+      <c r="B190" s="28" t="inlineStr">
+        <is>
+          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
+        </is>
+      </c>
+      <c r="C190" s="28" t="inlineStr">
+        <is>
+          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
+        </is>
+      </c>
+      <c r="D190" s="28" t="inlineStr">
+        <is>
+          <t>QUEUED - cleanup</t>
+        </is>
+      </c>
+      <c r="E190" s="28" t="inlineStr">
+        <is>
+          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="28" t="inlineStr">
+        <is>
           <t>Admin card PATCH date normalization - external dates should save as noon UTC to avoid timezone off-by-one (Zach precedent)</t>
         </is>
       </c>
-      <c r="B189" s="28" t="inlineStr">
+      <c r="B191" s="28" t="inlineStr">
         <is>
           <t>external_paid_through saved as midnight UTC displays as prior calendar day in US Eastern (Zach showed Nov 30 instead of Dec 1). Admin billing PATCH should normalize date-only inputs to noon UTC.</t>
         </is>
       </c>
-      <c r="C189" s="28" t="inlineStr">
+      <c r="C191" s="28" t="inlineStr">
         <is>
           <t>In PATCH /api/admin/members/[id]/billing (and any similar writers), coerce external_paid_through date-only values to YYYY-MM-DDT12:00:00.000Z before save. SMALL.</t>
         </is>
       </c>
-      <c r="D189" s="28" t="inlineStr">
+      <c r="D191" s="28" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="E189" s="28" t="inlineStr">
+      <c r="E191" s="28" t="inlineStr">
         <is>
           <t>SMALL/OPEN. Precedent: Zach Trusky external_paid_through 2026-12-01T00:00:00Z → Nov 30 in America/New_York.</t>
         </is>
@@ -5033,7 +5087,6 @@
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A141:E141"/>
-    <mergeCell ref="A9:E9"/>
     <mergeCell ref="A100:E100"/>
     <mergeCell ref="A156:E156"/>
     <mergeCell ref="A147:E147"/>
@@ -5041,6 +5094,7 @@
     <mergeCell ref="A121:E121"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A127:E127"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
chore: tracker - log send-email auth durable fix, dead last_attended trigger, invite token expiry decision
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E191"/>
+  <dimension ref="A1:E194"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="1" min="1" max="1"/>
@@ -1930,7 +1930,7 @@
     <row r="55" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>SECURITY &amp; MONITORING   ·   4 items</t>
+          <t>SECURITY &amp; MONITORING   ·   7 items</t>
         </is>
       </c>
       <c r="B55" s="29" t="n"/>
@@ -1941,163 +1941,179 @@
     <row r="56" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>Turn on error monitoring (Sentry)</t>
+          <t>send-email service-role auth: replace SB_SECRET_KEY duplicate with verified getClaims check</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Sentry is installed but never switched on, with no server-side capture; until it's on, no fix is provably working in production.</t>
+          <t>On 2026-08-12 the sb_secret_ prefix grant and the unverified-JWT-payload grant were removed from send-email and ambassador-payout (both were forgeable). That broke every restricted-template send on prod for about 10 minutes, because the app's legacy eyJ service-role JWT does NOT equal the SUPABASE_SERVICE_ROLE_KEY the function runtime sees - it had been passing via the unverified decode all along. Mitigated by setting SB_SECRET_KEY on prod to the same legacy JWT the app sends, restoring an exact match. That works but stores one credential under two names.</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Initialize across client + server + API routes + a root ErrorBoundary. Company-owned.</t>
+          <t>Replace the SB_SECRET_KEY exact-match branch with supabase.auth.getClaims(token) plus a claims.role === 'service_role' check. getClaims verifies the signature, so it is not forgeable, unlike the removed base64 decode. Confirm a user-scoped token can never surface role service_role in verified claims before relying on it. Then delete the SB_SECRET_KEY secret from prod. CRITICAL: test with the REAL prod service-role key against PROD before deploying - develop cannot catch this class of bug because develop's key is the new sb_secret_ format which the gateway rejects outright. Restricted templates affected if this breaks again: password-setup, welcome-new, welcome-back, welcome-setup, guest-pass, admin-invite, public-rsvp-confirmation and 22 others.</t>
         </is>
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="E56" s="15" t="inlineStr">
         <is>
-          <t>DONE Jul 9: @sentry/nextjs wired (client+server+API+global-error), CSP allowance added, DSN in Vercel, source-map upload configured, admin /admin/sentry page activated. Prod capture VERIFIED (smoke-test error landed). Commits 417fb37/d779885/5d12aac/b437166/a00cc50-adjacent. Until it's on, no fix is provable in production — it's the verification backbone.</t>
+          <t>Raised 2026-08-12 after causing and resolving a live 10-minute prod outage on restricted-template email. Prod currently healthy via SB_SECRET_KEY. Verified: Vercel prod and .env.local hold the same 219-char legacy JWT.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>Add a deploy pipeline so changes go live safely</t>
+          <t>Dead trigger: last_attended_at never updates from public check-ins</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>DB/function changes are pushed by hand today — the root cause of code/live drift. Locked: hand-patching stops once this lands (with a written emergency lane).</t>
+          <t>The trigger trg_update_last_attended_from_public_rsvp fires on event_public_rsvps check-in and is meant to stamp profiles.last_attended_at. It looks up contacts.converted_to_member_id first, and NO code anywhere writes that column (0 of 207 rows on prod have it set), so the trigger always exits early. Members who check in through the public RSVP path never get their last-attended date updated.</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>GitHub Actions: merge to main -&gt; db push + functions deploy. Needs 3 repo secrets.</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>Once in, hand-patching stops; needed before two people touch production in parallel.</t>
+          <t>Two options. Either populate contacts.converted_to_member_id when a contact becomes a member (a real CRM flow that does not currently exist), or rewrite the trigger to resolve the profile by email or through the people bridge instead of the dead column. The second is far smaller. Note the conversion-rate report widget that depended on the same column was removed on 2026-08-12 because it always rendered 0 percent.</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E57" s="15" t="inlineStr">
+        <is>
+          <t>Raised 2026-08-12 during a contacts table audit. Fails safe - does nothing rather than something wrong.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>Make the code able to rebuild the live database</t>
+          <t>Exchange invite tokens never expire</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Several live DB objects were made by hand and aren't in migration history, so the repo can't recreate prod.</t>
+          <t>The 12 personalized Form C links sent to members on 2026-08-12 (format https://704collective.com/exchange/i/EX-XXXXXXXXXXXX) have no expiry. Anyone holding a forwarded link can submit answers on that member's behalf indefinitely. They cannot see stored data, change an RSVP, or register anyone.</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Snapshot prod schema, diff vs migrations, commit a baseline migration.</t>
-        </is>
-      </c>
-      <c r="D58" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Absorbs recent hand-made objects (RSVP backfill, a few functions, the unsubscribe function).</t>
+          <t>DELIBERATE DECISION 2026-08-12: leave them alone through Aug 27. Adding expiry now risks a member opening their email late and finding a dead link, which costs the exact data the form exists to collect. Revisit only if the intake pattern is reused for a future event, at which point add an expires_at column to exchange_intake and check it in the invited path of exchange-intake-submit.</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="E58" s="15" t="inlineStr">
+        <is>
+          <t>Logged so nobody reopens this as a bug. Low risk, intentional.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>Add three safety tests on the things that can't break</t>
+          <t>Turn on error monitoring (Sentry)</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>Effectively no automated testing exists.</t>
+          <t>Sentry is installed but never switched on, with no server-side capture; until it's on, no fix is provably working in production.</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Three critical-path tests — (1) checkout -&gt; webhook -&gt; activated, (2) RSVP -&gt; attendance, (3) unsubscribe honored — and remove passWithNoTests so CI gates.</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="inlineStr">
-        <is>
-          <t>The three failures that hurt most; flips CI from passing with zero tests.</t>
+          <t>Initialize across client + server + API routes + a root ErrorBoundary. Company-owned.</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E59" s="15" t="inlineStr">
+        <is>
+          <t>DONE Jul 9: @sentry/nextjs wired (client+server+API+global-error), CSP allowance added, DSN in Vercel, source-map upload configured, admin /admin/sentry page activated. Prod capture VERIFIED (smoke-test error landed). Commits 417fb37/d779885/5d12aac/b437166/a00cc50-adjacent. Until it's on, no fix is provable in production — it's the verification backbone.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>EMAIL &amp; COMPLIANCE   ·   3 items</t>
-        </is>
-      </c>
-      <c r="B60" s="29" t="n"/>
-      <c r="C60" s="29" t="n"/>
-      <c r="D60" s="29" t="n"/>
-      <c r="E60" s="30" t="n"/>
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>Add a deploy pipeline so changes go live safely</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>DB/function changes are pushed by hand today — the root cause of code/live drift. Locked: hand-patching stops once this lands (with a written emergency lane).</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>GitHub Actions: merge to main -&gt; db push + functions deploy. Needs 3 repo secrets.</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Once in, hand-patching stops; needed before two people touch production in parallel.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>Make every email sender respect unsubscribes</t>
+          <t>Make the code able to rebuild the live database</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>The unsubscribe page/link policy is fixed, but two senders (drip processor, renewal reminders) still don't check the opt-out flag, and one reminder may skip members on a null value.</t>
+          <t>Several live DB objects were made by hand and aren't in migration history, so the repo can't recreate prod.</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Add opt-out filtering to process-drips + renewal-reminders; fix event-reminder null handling. One opt-out flag is the source of truth.</t>
+          <t>Snapshot prod schema, diff vs migrations, commit a baseline migration.</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>send-email unsubscribe-block work is in flight; process-drips + renewal-reminders filtering to confirm/finish.</t>
+          <t>Absorbs recent hand-made objects (RSVP backfill, a few functions, the unsubscribe function).</t>
         </is>
       </c>
     </row>
     <row r="62" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>Make unsubscribe links forgery-proof</t>
+          <t>Add three safety tests on the things that can't break</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>The unsubscribe token is currently guessable/forgeable (low stakes).</t>
+          <t>Effectively no automated testing exists.</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>HMAC-sign the token; align format across send-campaign, send-email, and unsubscribe.</t>
+          <t>Three critical-path tests — (1) checkout -&gt; webhook -&gt; activated, (2) RSVP -&gt; attendance, (3) unsubscribe honored — and remove passWithNoTests so CI gates.</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
@@ -2107,42 +2123,62 @@
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>Align the token format across the three places that generate/read it.</t>
+          <t>The three failures that hurt most; flips CI from passing with zero tests.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A63" s="16" t="inlineStr">
-        <is>
-          <t>Remove unsubscribe links from ALL emails; members cannot unsubscribe (manual-only)</t>
-        </is>
-      </c>
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>EMAIL &amp; COMPLIANCE   ·   3 items</t>
+        </is>
+      </c>
+      <c r="B63" s="29" t="n"/>
+      <c r="C63" s="29" t="n"/>
+      <c r="D63" s="29" t="n"/>
+      <c r="E63" s="30" t="n"/>
     </row>
     <row r="64" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>ADMIN &amp; OPERATIONS   ·   12 items</t>
-        </is>
-      </c>
-      <c r="B64" s="29" t="n"/>
-      <c r="C64" s="29" t="n"/>
-      <c r="D64" s="29" t="n"/>
-      <c r="E64" s="30" t="n"/>
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>Make every email sender respect unsubscribes</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>The unsubscribe page/link policy is fixed, but two senders (drip processor, renewal reminders) still don't check the opt-out flag, and one reminder may skip members on a null value.</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>Add opt-out filtering to process-drips + renewal-reminders; fix event-reminder null handling. One opt-out flag is the source of truth.</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>send-email unsubscribe-block work is in flight; process-drips + renewal-reminders filtering to confirm/finish.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>PRIORITY 1: Exchange intake viewer (admin)</t>
+          <t>Make unsubscribe links forgery-proof</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>The Exchange intake forms are live and collecting registrations into the exchange_intake table, but there is NO way to see any of it in the admin UI. Right now the only way to read who registered, what they answered, or how full each pool is, is to run raw SQL. This is needed before Aug 27 and is the foundation the speed-networking matching engine will read from.</t>
+          <t>The unsubscribe token is currently guessable/forgeable (low stakes).</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>Build an admin page (suggested /admin/exchange or a tab on the event detail admin view) that lists exchange_intake rows for a given event. Must show: name, email, phone, form_variant (public / commonwealth / invited), pool (house / commonwealth), participation (business_and_social / social_only), member_status_at_submit, status (invited / submitted), submitted_at, and all four free-text answers (q_role_title, q_company, q_years_charlotte, q_seeking). Needs: live pool counters (house X of 60, commonwealth Y of 60), filter by pool and participation, CSV export, and a view of which invited members have not yet submitted. RLS already allows admin/super_admin SELECT on exchange_intake. Read before write - the table already exists on both prod and develop.</t>
+          <t>HMAC-sign the token; align format across send-campaign, send-email, and unsubscribe.</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
@@ -2152,78 +2188,42 @@
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>TOP PRIORITY. Raised 2026-08-12 immediately after the intake forms shipped. Event is Aug 27 2026. Table: exchange_intake, event id 02afde72-33c4-4c99-8dba-0ea5a8c0a723.</t>
+          <t>Align the token format across the three places that generate/read it.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A66" s="7" t="inlineStr">
-        <is>
-          <t>PRIORITY 2: send-campaign all_contacts audience includes paying members</t>
-        </is>
-      </c>
-      <c r="B66" s="8" t="inlineStr">
-        <is>
-          <t>The 'All Contacts' audience in the campaign tool pulls every row from the contacts table and filters ONLY on unsubscribed. It does not exclude members. On prod, 89 of 207 contacts are also active members (over 40 percent overlap), so any All Contacts campaign sends prospect-facing copy to people who already pay. A 'join 704 Collective' style blast would pitch membership to existing members.</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>In supabase/functions/send-campaign/index.ts, the all_contacts branch (approx lines 478-489) selects contacts where unsubscribed is null or false, with no membership filter. Add an exclusion so contacts whose email matches a non-deleted profile with subscription_status active or trialing or membership_override true are removed from that audience. Consider whether the segment audience (tag-based, approx lines 490-506) needs the same treatment. Related dead code found the same night: converted_to_member_id is never written by any code, so the conversion-rate report on /admin/crm/reports measures nothing, and the campaigns audience preview counts contact_type = 'guest' which zero rows have, so it always shows 0. Rehearse on develop both viewports before shipping.</t>
-        </is>
-      </c>
-      <c r="D66" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>Raised 2026-08-12 during a contacts table audit. Not known whether any past campaign used this audience. Timi should be told to avoid All Contacts until fixed.</t>
+      <c r="A66" s="16" t="inlineStr">
+        <is>
+          <t>Remove unsubscribe links from ALL emails; members cannot unsubscribe (manual-only)</t>
         </is>
       </c>
     </row>
     <row r="67" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A67" s="7" t="inlineStr">
-        <is>
-          <t>Add a private notes section on each member</t>
-        </is>
-      </c>
-      <c r="B67" s="8" t="inlineStr">
-        <is>
-          <t>Internal request: a notes area per member for context (e.g. 'comped through August').</t>
-        </is>
-      </c>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>Read: admin + super-admin. Write/edit: super-admin only. Not member-visible.</t>
-        </is>
-      </c>
-      <c r="D67" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>Internal-only; super-admin writes, admins read, members never see it.</t>
-        </is>
-      </c>
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>ADMIN &amp; OPERATIONS   ·   12 items</t>
+        </is>
+      </c>
+      <c r="B67" s="29" t="n"/>
+      <c r="C67" s="29" t="n"/>
+      <c r="D67" s="29" t="n"/>
+      <c r="E67" s="30" t="n"/>
     </row>
     <row r="68" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>Build the admin health dashboard</t>
+          <t>PRIORITY 1: Exchange intake viewer (admin)</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>One screen showing system health at a glance; catches silent failures before members do.</t>
+          <t>The Exchange intake forms are live and collecting registrations into the exchange_intake table, but there is NO way to see any of it in the admin UI. Right now the only way to read who registered, what they answered, or how full each pool is, is to run raw SQL. This is needed before Aug 27 and is the foundation the speed-networking matching engine will read from.</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>5 widgets — cron, webhooks, drip health, email tracking, payment sync. Sits on /api/health.</t>
+          <t>Build an admin page (suggested /admin/exchange or a tab on the event detail admin view) that lists exchange_intake rows for a given event. Must show: name, email, phone, form_variant (public / commonwealth / invited), pool (house / commonwealth), participation (business_and_social / social_only), member_status_at_submit, status (invited / submitted), submitted_at, and all four free-text answers (q_role_title, q_company, q_years_charlotte, q_seeking). Needs: live pool counters (house X of 60, commonwealth Y of 60), filter by pool and participation, CSV export, and a view of which invited members have not yet submitted. RLS already allows admin/super_admin SELECT on exchange_intake. Read before write - the table already exists on both prod and develop.</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
@@ -2233,24 +2233,24 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>Reads /api/health + checks; surfaces silent failures.</t>
+          <t>TOP PRIORITY. Raised 2026-08-12 immediately after the intake forms shipped. Event is Aug 27 2026. Table: exchange_intake, event id 02afde72-33c4-4c99-8dba-0ea5a8c0a723.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>Let admins change a member's tier and have billing follow</t>
+          <t>PRIORITY 2: send-campaign all_contacts audience includes paying members</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>App-side tier change/comp exists; the Stripe billing side doesn't follow.</t>
+          <t>The 'All Contacts' audience in the campaign tool pulls every row from the contacts table and filters ONLY on unsubscribed. It does not exclude members. On prod, 89 of 207 contacts are also active members (over 40 percent overlap), so any All Contacts campaign sends prospect-facing copy to people who already pay. A 'join 704 Collective' style blast would pitch membership to existing members.</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>Wire admin tier-change to Stripe subscription cancel/modify/start.</t>
+          <t>In supabase/functions/send-campaign/index.ts, the all_contacts branch (approx lines 478-489) selects contacts where unsubscribed is null or false, with no membership filter. Add an exclusion so contacts whose email matches a non-deleted profile with subscription_status active or trialing or membership_override true are removed from that audience. Consider whether the segment audience (tag-based, approx lines 490-506) needs the same treatment. Related dead code found the same night: converted_to_member_id is never written by any code, so the conversion-rate report on /admin/crm/reports measures nothing, and the campaigns audience preview counts contact_type = 'guest' which zero rows have, so it always shows 0. Rehearse on develop both viewports before shipping.</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
@@ -2260,24 +2260,24 @@
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>App-side override already exists; this is the Stripe billing reconciliation.</t>
+          <t>Raised 2026-08-12 during a contacts table audit. Not known whether any past campaign used this audience. Timi should be told to avoid All Contacts until fixed.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>Harden the admin cancel-subscription flow</t>
+          <t>Add a private notes section on each member</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>Make admin cancel safe (running twice shouldn't double-act).</t>
+          <t>Internal request: a notes area per member for context (e.g. 'comped through August').</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>Add idempotency + structured logging + alert to admin-cancel-subscription.</t>
+          <t>Read: admin + super-admin. Write/edit: super-admin only. Not member-visible.</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
@@ -2287,24 +2287,24 @@
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>Idempotent + logged + alerted so a double-run can't double-act.</t>
+          <t>Internal-only; super-admin writes, admins read, members never see it.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>Build the admin area into clean sections</t>
+          <t>Build the admin health dashboard</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Reorganize admin into Today / People / Events / Network / Money / Messages / Settings with one source of truth per question.</t>
+          <t>One screen showing system health at a glance; catches silent failures before members do.</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>7-section IA; folds in nav cleanup, per-event check-in start, financial accuracy, tier tools, and guest upload.</t>
+          <t>5 widgets — cron, webhooks, drip health, email tracking, payment sync. Sits on /api/health.</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
@@ -2314,24 +2314,24 @@
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>The Messages section is where the texting inbox lives.</t>
+          <t>Reads /api/health + checks; surfaces silent failures.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>Shared admin navigation config</t>
+          <t>Let admins change a member's tier and have billing follow</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>One shared config for admin nav so it's consistent and not duplicated.</t>
+          <t>App-side tier change/comp exists; the Stripe billing side doesn't follow.</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>Single adminNav config; remove duplicated nav definitions.</t>
+          <t>Wire admin tier-change to Stripe subscription cancel/modify/start.</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
@@ -2341,24 +2341,24 @@
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
-          <t>One config; removes duplicated nav definitions.</t>
+          <t>App-side override already exists; this is the Stripe billing reconciliation.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>Guest list upload tool</t>
+          <t>Harden the admin cancel-subscription flow</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Let admins upload a guest list for an event.</t>
+          <t>Make admin cancel safe (running twice shouldn't double-act).</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Guest list upload UI.</t>
+          <t>Add idempotency + structured logging + alert to admin-cancel-subscription.</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
@@ -2368,24 +2368,24 @@
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>Also unblocks future guest-conversion automation.</t>
+          <t>Idempotent + logged + alerted so a double-run can't double-act.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>Fix the organization settings table</t>
+          <t>Build the admin area into clean sections</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>organization_settings has the wrong schema.</t>
+          <t>Reorganize admin into Today / People / Events / Network / Money / Messages / Settings with one source of truth per question.</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>Correct the organization_settings schema.</t>
+          <t>7-section IA; folds in nav cleanup, per-event check-in start, financial accuracy, tier tools, and guest upload.</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
@@ -2395,24 +2395,24 @@
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
-          <t>Schema is currently wrong; correct it.</t>
+          <t>The Messages section is where the texting inbox lives.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A75" s="7" t="inlineStr">
         <is>
-          <t>Route Stripe receipts to the team inbox</t>
+          <t>Shared admin navigation config</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Receipt/invoice emails should also go to hello@704collective.com.</t>
+          <t>One shared config for admin nav so it's consistent and not duplicated.</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>Stripe email settings -&gt; CC hello@ (or a forwarding rule).</t>
+          <t>Single adminNav config; remove duplicated nav definitions.</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
@@ -2422,62 +2422,62 @@
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>CC hello@ on Stripe receipts, or add a forwarding rule.</t>
+          <t>One config; removes duplicated nav definitions.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>MEMBER EXPERIENCE   ·   9 items</t>
-        </is>
-      </c>
-      <c r="B76" s="29" t="n"/>
-      <c r="C76" s="29" t="n"/>
-      <c r="D76" s="29" t="n"/>
-      <c r="E76" s="30" t="n"/>
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>Guest list upload tool</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>Let admins upload a guest list for an event.</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>Guest list upload UI.</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>Also unblocks future guest-conversion automation.</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>Strip member profiles to four clean fields</t>
-        </is>
-      </c>
-      <c r="B77" s="8" t="inlineStr">
-        <is>
-          <t>Simplify the profile to name, photo, what you do, and a one-line bio — as real columns, not JSON. Locked: archive the other 15+ fields (kept in DB, hidden) for future matchmaking.</t>
-        </is>
-      </c>
-      <c r="C77" s="8" t="inlineStr">
-        <is>
-          <t>4 visible fields as real columns; align onboarding + settings + directory. The 4-field data move rides with the identity foundation (same plumbing).</t>
-        </is>
-      </c>
-      <c r="D77" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E77" s="8" t="inlineStr">
-        <is>
-          <t>Archive (don't delete) the rest — raw material for future matchmaking.</t>
-        </is>
-      </c>
+          <t>Fix the organization settings table</t>
+        </is>
+      </c>
+      <c r="B77" s="29" t="n"/>
+      <c r="C77" s="29" t="n"/>
+      <c r="D77" s="29" t="n"/>
+      <c r="E77" s="30" t="n"/>
     </row>
     <row r="78" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>Build the one merged member portal with tiered views</t>
+          <t>Route Stripe receipts to the team inbox</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>Locked: replace the two portals (member dashboard + business portal) with ONE codebase; business gets an elevated view, social the standard view; clear type distinction preserved.</t>
+          <t>Receipt/invoice emails should also go to hello@704collective.com.</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>One portal codebase; gate business-only modules behind member type. Replaces /dashboard vs /business-portal.</t>
+          <t>Stripe email settings -&gt; CC hello@ (or a forwarding rule).</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
@@ -2487,51 +2487,35 @@
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>Replaces /dashboard vs /business-portal with one tier-gated codebase.</t>
+          <t>CC hello@ on Stripe receipts, or add a forwarding rule.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="57.45" customFormat="1" customHeight="1" s="2">
-      <c r="A79" s="7" t="inlineStr">
-        <is>
-          <t>Rebuild onboarding questionnaire + member brief</t>
-        </is>
-      </c>
-      <c r="B79" s="8" t="inlineStr">
-        <is>
-          <t>Store responses in their own table and generate a 'member brief' for future matchmaking/AI.</t>
-        </is>
-      </c>
-      <c r="C79" s="8" t="inlineStr">
-        <is>
-          <t>Onboarding rebuild + onboarding_responses table + member_brief column.</t>
-        </is>
-      </c>
-      <c r="D79" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E79" s="8" t="inlineStr">
-        <is>
-          <t>Responses in their own table; feeds a future member brief.</t>
-        </is>
-      </c>
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>MEMBER EXPERIENCE   ·   9 items</t>
+        </is>
+      </c>
+      <c r="B79" s="29" t="n"/>
+      <c r="C79" s="29" t="n"/>
+      <c r="D79" s="29" t="n"/>
+      <c r="E79" s="30" t="n"/>
     </row>
     <row r="80" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>Member portal / dashboard redesign</t>
+          <t>Strip member profiles to four clean fields</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>The redesign: 5-tab bottom nav, pass-first / next-event hero, onboarding checklist removed after completion, plus resources/bookings tabs. The shared activity feed is KEPT and built on (members post / share / like; event discussions surface there) — only the minor personal activity-log widget from the old dashboard is retired.</t>
+          <t>Simplify the profile to name, photo, what you do, and a one-line bio — as real columns, not JSON. Locked: archive the other 15+ fields (kept in DB, hidden) for future matchmaking.</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>Multi-week. SEQUENCING: the visual redesign lands AFTER the identity foundation is built and verified — not concurrent with it (one big change at a time on a no-staging system). Resources/bookings depend on vendor partnerships.</t>
+          <t>4 visible fields as real columns; align onboarding + settings + directory. The 4-field data move rides with the identity foundation (same plumbing).</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
@@ -2541,24 +2525,24 @@
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>Activity feed stays; only the personal activity-log widget is retired. Visual redesign sequenced after identity.</t>
+          <t>Archive (don't delete) the rest — raw material for future matchmaking.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A81" s="7" t="inlineStr">
         <is>
-          <t>Member directory — people-finder for all member + partner types</t>
+          <t>Build the one merged member portal with tiered views</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>A members-only people-finder where social members, business members, and partners can all find and see each other — profiles only, WITHOUT the business-listings view. Visible to everyone logged in, regardless of type. A privacy toggle lets a member hide from it.</t>
+          <t>Locked: replace the two portals (member dashboard + business portal) with ONE codebase; business gets an elevated view, social the standard view; clear type distinction preserved.</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>Logged-in directory of people (social + business + partner). Profiles only — no business view (that lives in The Network). Visible to all logged-in types; honor the privacy toggle.</t>
+          <t>One portal codebase; gate business-only modules behind member type. Replaces /dashboard vs /business-portal.</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
@@ -2568,24 +2552,24 @@
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>Distinct from The Network (hubs + business/partner listings). Pairs with the privacy toggle below.</t>
+          <t>Replaces /dashboard vs /business-portal with one tier-gated codebase.</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A82" s="7" t="inlineStr">
         <is>
-          <t>Profile privacy toggle</t>
+          <t>Rebuild onboarding questionnaire + member brief</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>A toggle for members to control whether they appear in the directory and the internal Network member view.</t>
+          <t>Store responses in their own table and generate a 'member brief' for future matchmaking/AI.</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>Build the opt-out toggle; default is listed, members can hide themselves.</t>
+          <t>Onboarding rebuild + onboarding_responses table + member_brief column.</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
@@ -2595,24 +2579,24 @@
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>Confirmed feature — the directory is opt-out via this toggle.</t>
+          <t>Responses in their own table; feeds a future member brief.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A83" s="7" t="inlineStr">
         <is>
-          <t>Member cancellation retention flow</t>
+          <t>Member portal / dashboard redesign</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Improve the cancellation flow with retention UX.</t>
+          <t>The redesign: 5-tab bottom nav, pass-first / next-event hero, onboarding checklist removed after completion, plus resources/bookings tabs. The shared activity feed is KEPT and built on (members post / share / like; event discussions surface there) — only the minor personal activity-log widget from the old dashboard is retired.</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>Retention UX on cancellation (offers, pauses, feedback).</t>
+          <t>Multi-week. SEQUENCING: the visual redesign lands AFTER the identity foundation is built and verified — not concurrent with it (one big change at a time on a no-staging system). Resources/bookings depend on vendor partnerships.</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
@@ -2622,24 +2606,24 @@
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>Offers / pauses / feedback on cancellation.</t>
+          <t>Activity feed stays; only the personal activity-log widget is retired. Visual redesign sequenced after identity.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A84" s="7" t="inlineStr">
         <is>
-          <t>Member spotlight on calendar/home</t>
+          <t>Member directory — people-finder for all member + partner types</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>Feature a member spotlight on the calendar/home pages.</t>
+          <t>A members-only people-finder where social members, business members, and partners can all find and see each other — profiles only, WITHOUT the business-listings view. Visible to everyone logged in, regardless of type. A privacy toggle lets a member hide from it.</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>Member spotlight feature.</t>
+          <t>Logged-in directory of people (social + business + partner). Profiles only — no business view (that lives in The Network). Visible to all logged-in types; honor the privacy toggle.</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
@@ -2649,127 +2633,111 @@
       </c>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t>Feature a member on calendar/home.</t>
+          <t>Distinct from The Network (hubs + business/partner listings). Pairs with the privacy toggle below.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A85" s="7" t="inlineStr">
         <is>
-          <t>Unlimited guest passes for dream-team members</t>
-        </is>
-      </c>
-      <c r="B85" s="5" t="n"/>
-      <c r="C85" s="5" t="n"/>
-      <c r="D85" s="5" t="n"/>
-      <c r="E85" s="6" t="n"/>
+          <t>Profile privacy toggle</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>A toggle for members to control whether they appear in the directory and the internal Network member view.</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Build the opt-out toggle; default is listed, members can hide themselves.</t>
+        </is>
+      </c>
+      <c r="D85" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>Confirmed feature — the directory is opt-out via this toggle.</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A86" s="4" t="inlineStr">
-        <is>
-          <t>PERFORMANCE   ·   5 items</t>
-        </is>
-      </c>
-      <c r="B86" s="29" t="n"/>
-      <c r="C86" s="29" t="n"/>
-      <c r="D86" s="29" t="n"/>
-      <c r="E86" s="30" t="n"/>
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>Member cancellation retention flow</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>Improve the cancellation flow with retention UX.</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>Retention UX on cancellation (offers, pauses, feedback).</t>
+        </is>
+      </c>
+      <c r="D86" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="inlineStr">
+        <is>
+          <t>Offers / pauses / feedback on cancellation.</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A87" s="7" t="inlineStr">
         <is>
-          <t>Speed up slow list pages (Events, Tasks, Hubs)</t>
-        </is>
-      </c>
-      <c r="B87" s="8" t="inlineStr">
-        <is>
-          <t>These pages make many small repeated DB calls (N+1) that get slow as data grows.</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
-          <t>Resolve the N+1 query patterns; batch them.</t>
-        </is>
-      </c>
-      <c r="D87" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E87" s="8" t="inlineStr">
-        <is>
-          <t>Batch the repeated calls on Events, Tasks, Hubs.</t>
-        </is>
-      </c>
+          <t>Member spotlight on calendar/home</t>
+        </is>
+      </c>
+      <c r="B87" s="29" t="n"/>
+      <c r="C87" s="29" t="n"/>
+      <c r="D87" s="29" t="n"/>
+      <c r="E87" s="30" t="n"/>
     </row>
     <row r="88" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>Make bulk member adds all-or-nothing</t>
-        </is>
-      </c>
-      <c r="B88" s="8" t="inlineStr">
-        <is>
-          <t>Bulk add isn't transactional — a partial failure leaves half-written data.</t>
-        </is>
-      </c>
-      <c r="C88" s="8" t="inlineStr">
-        <is>
-          <t>Make add-members and hub-delete atomic.</t>
-        </is>
-      </c>
-      <c r="D88" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E88" s="8" t="inlineStr">
-        <is>
-          <t>All-or-nothing; same for hub deletes.</t>
-        </is>
-      </c>
+          <t>Unlimited guest passes for dream-team members</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="n"/>
+      <c r="C88" s="5" t="n"/>
+      <c r="D88" s="5" t="n"/>
+      <c r="E88" s="6" t="n"/>
     </row>
     <row r="89" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A89" s="7" t="inlineStr">
-        <is>
-          <t>Move heavy admin queries to the server</t>
-        </is>
-      </c>
-      <c r="B89" s="8" t="inlineStr">
-        <is>
-          <t>Keep the browser from doing heavy lifting on admin overview + email dashboard.</t>
-        </is>
-      </c>
-      <c r="C89" s="8" t="inlineStr">
-        <is>
-          <t>Add server-side RPCs: admin_overview, email_dashboard.</t>
-        </is>
-      </c>
-      <c r="D89" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E89" s="8" t="inlineStr">
-        <is>
-          <t>Move admin overview + email dashboard to server RPCs.</t>
-        </is>
-      </c>
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>PERFORMANCE   ·   5 items</t>
+        </is>
+      </c>
+      <c r="B89" s="29" t="n"/>
+      <c r="C89" s="29" t="n"/>
+      <c r="D89" s="29" t="n"/>
+      <c r="E89" s="30" t="n"/>
     </row>
     <row r="90" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t>Standardize how data is loaded (React Query)</t>
+          <t>Speed up slow list pages (Events, Tasks, Hubs)</t>
         </is>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>Make loading behavior uniform and reliable.</t>
+          <t>These pages make many small repeated DB calls (N+1) that get slow as data grows.</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>React Query rollout across data fetching.</t>
+          <t>Resolve the N+1 query patterns; batch them.</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
@@ -2779,127 +2747,111 @@
       </c>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t>Uniform data-loading / caching across the app.</t>
+          <t>Batch the repeated calls on Events, Tasks, Hubs.</t>
         </is>
       </c>
     </row>
     <row r="91" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A91" s="7" t="inlineStr">
         <is>
-          <t>Audit shortcut data fields for correctness</t>
-        </is>
-      </c>
-      <c r="B91" s="5" t="n"/>
-      <c r="C91" s="5" t="n"/>
-      <c r="D91" s="5" t="n"/>
-      <c r="E91" s="6" t="n"/>
+          <t>Make bulk member adds all-or-nothing</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>Bulk add isn't transactional — a partial failure leaves half-written data.</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>Make add-members and hub-delete atomic.</t>
+        </is>
+      </c>
+      <c r="D91" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>All-or-nothing; same for hub deletes.</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A92" s="4" t="inlineStr">
-        <is>
-          <t>AUTH   ·   7 items</t>
-        </is>
-      </c>
-      <c r="B92" s="29" t="n"/>
-      <c r="C92" s="29" t="n"/>
-      <c r="D92" s="29" t="n"/>
-      <c r="E92" s="30" t="n"/>
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>Move heavy admin queries to the server</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t>Keep the browser from doing heavy lifting on admin overview + email dashboard.</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>Add server-side RPCs: admin_overview, email_dashboard.</t>
+        </is>
+      </c>
+      <c r="D92" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>Move admin overview + email dashboard to server RPCs.</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A93" s="7" t="inlineStr">
         <is>
-          <t>Verify magic-link login across two devices</t>
-        </is>
-      </c>
-      <c r="B93" s="8" t="inlineStr">
-        <is>
-          <t>Phone-to-desktop: request a link on a phone, type the 8-digit code on the desktop.</t>
-        </is>
-      </c>
-      <c r="C93" s="8" t="inlineStr">
-        <is>
-          <t>Cross-device OTP test; confirm same-device + resend cooldown too.</t>
-        </is>
-      </c>
-      <c r="D93" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E93" s="8" t="inlineStr">
-        <is>
-          <t>Requires a second device (owner-run).</t>
-        </is>
-      </c>
+          <t>Standardize how data is loaded (React Query)</t>
+        </is>
+      </c>
+      <c r="B93" s="29" t="n"/>
+      <c r="C93" s="29" t="n"/>
+      <c r="D93" s="29" t="n"/>
+      <c r="E93" s="30" t="n"/>
     </row>
     <row r="94" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A94" s="7" t="inlineStr">
         <is>
-          <t>Verify magic-link login works in production</t>
-        </is>
-      </c>
-      <c r="B94" s="8" t="inlineStr">
-        <is>
-          <t>End-to-end check the email magic-link round-trip works live.</t>
-        </is>
-      </c>
-      <c r="C94" s="8" t="inlineStr">
-        <is>
-          <t>Test request -&gt; click -&gt; signed in, in prod.</t>
-        </is>
-      </c>
-      <c r="D94" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E94" s="8" t="inlineStr">
-        <is>
-          <t>End-to-end live round-trip check.</t>
-        </is>
-      </c>
+          <t>Audit shortcut data fields for correctness</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="n"/>
+      <c r="C94" s="5" t="n"/>
+      <c r="D94" s="5" t="n"/>
+      <c r="E94" s="6" t="n"/>
     </row>
     <row r="95" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A95" s="7" t="inlineStr">
-        <is>
-          <t>Verify sessions refresh correctly on expiry</t>
-        </is>
-      </c>
-      <c r="B95" s="8" t="inlineStr">
-        <is>
-          <t>Confirm cookie-based refresh works when a token expires so members aren't kicked out.</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
-          <t>Verify @supabase/ssr middleware refreshes session on token expiry.</t>
-        </is>
-      </c>
-      <c r="D95" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E95" s="8" t="inlineStr">
-        <is>
-          <t>Confirm members aren't kicked out when a token expires.</t>
-        </is>
-      </c>
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>AUTH   ·   7 items</t>
+        </is>
+      </c>
+      <c r="B95" s="29" t="n"/>
+      <c r="C95" s="29" t="n"/>
+      <c r="D95" s="29" t="n"/>
+      <c r="E95" s="30" t="n"/>
     </row>
     <row r="96" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A96" s="7" t="inlineStr">
         <is>
-          <t>Verify Google sign-in works</t>
+          <t>Verify magic-link login across two devices</t>
         </is>
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>Confirm Google login/signup paths work in production.</t>
+          <t>Phone-to-desktop: request a link on a phone, type the 8-digit code on the desktop.</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>Test Google OAuth signup + sign-in.</t>
+          <t>Cross-device OTP test; confirm same-device + resend cooldown too.</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
@@ -2909,325 +2861,328 @@
       </c>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t>Confirm Google login/signup in production.</t>
+          <t>Requires a second device (owner-run).</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A97" s="7" t="inlineStr">
         <is>
-          <t>Apple Sign-In</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="n"/>
-      <c r="C97" s="5" t="n"/>
-      <c r="D97" s="5" t="n"/>
-      <c r="E97" s="6" t="n"/>
+          <t>Verify magic-link login works in production</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>End-to-end check the email magic-link round-trip works live.</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>Test request -&gt; click -&gt; signed in, in prod.</t>
+        </is>
+      </c>
+      <c r="D97" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>End-to-end live round-trip check.</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A98" s="7" t="inlineStr">
         <is>
-          <t>Branded auth links (stop showing supabase.co URLs)</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>Build</t>
+          <t>Verify sessions refresh correctly on expiry</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>Confirm cookie-based refresh works when a token expires so members aren't kicked out.</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>Verify @supabase/ssr middleware refreshes session on token expiry.</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>Confirm members aren't kicked out when a token expires.</t>
         </is>
       </c>
     </row>
     <row r="99" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A99" s="7" t="inlineStr">
         <is>
-          <t>Password rules hardening (min length 6 to 8, leaked-password check)</t>
-        </is>
-      </c>
-      <c r="B99" s="5" t="inlineStr">
-        <is>
-          <t>Supabase minimum password length is 6 and the leaked-password check is off. Both are weaker than they should be for a paid membership platform.</t>
-        </is>
-      </c>
-      <c r="C99" s="5" t="inlineStr">
-        <is>
-          <t>Do the UI copy FIRST, then the dashboard toggles. Update /setup-password and every password field to state the real rule before raising the server minimum to 8, otherwise members get rejected by a rule the screen never showed them. Then enable Prevent use of leaked passwords and confirm the rejection message renders cleanly. Leave Require current password when updating OFF, it breaks the no-password comp-invite setup flow. Rehearse on develop both viewports.</t>
-        </is>
-      </c>
-      <c r="D99" s="5" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E99" s="6" t="inlineStr">
-        <is>
-          <t>Raised 2026-08-06 during the Email OTP expiration change (3600 to 86400).</t>
+          <t>Verify Google sign-in works</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Confirm Google login/signup paths work in production.</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Test Google OAuth signup + sign-in.</t>
+        </is>
+      </c>
+      <c r="D99" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>Confirm Google login/signup in production.</t>
         </is>
       </c>
     </row>
     <row r="100" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A100" s="4" t="inlineStr">
-        <is>
-          <t>BUSINESS   ·   1 item</t>
-        </is>
-      </c>
-      <c r="B100" s="29" t="n"/>
-      <c r="C100" s="29" t="n"/>
-      <c r="D100" s="29" t="n"/>
-      <c r="E100" s="30" t="n"/>
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t>Apple Sign-In</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="n"/>
+      <c r="C100" s="5" t="n"/>
+      <c r="D100" s="5" t="n"/>
+      <c r="E100" s="6" t="n"/>
     </row>
     <row r="101" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A101" s="7" t="inlineStr">
         <is>
-          <t>Verify the business application approval works</t>
-        </is>
-      </c>
-      <c r="B101" s="5" t="n"/>
-      <c r="C101" s="5" t="n"/>
-      <c r="D101" s="5" t="n"/>
-      <c r="E101" s="6" t="n"/>
+          <t>Branded auth links (stop showing supabase.co URLs)</t>
+        </is>
+      </c>
+      <c r="B101" s="29" t="n"/>
+      <c r="C101" s="29" t="n"/>
+      <c r="D101" s="29" t="n"/>
+      <c r="E101" s="30" t="n"/>
     </row>
     <row r="102" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A102" s="4" t="inlineStr">
-        <is>
-          <t>FINANCIALS   ·   6 items</t>
-        </is>
-      </c>
-      <c r="B102" s="29" t="n"/>
-      <c r="C102" s="29" t="n"/>
-      <c r="D102" s="29" t="n"/>
-      <c r="E102" s="30" t="n"/>
+      <c r="A102" s="7" t="inlineStr">
+        <is>
+          <t>Password rules hardening (min length 6 to 8, leaked-password check)</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Supabase minimum password length is 6 and the leaked-password check is off. Both are weaker than they should be for a paid membership platform.</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Do the UI copy FIRST, then the dashboard toggles. Update /setup-password and every password field to state the real rule before raising the server minimum to 8, otherwise members get rejected by a rule the screen never showed them. Then enable Prevent use of leaked passwords and confirm the rejection message renders cleanly. Leave Require current password when updating OFF, it breaks the no-password comp-invite setup flow. Rehearse on develop both viewports.</t>
+        </is>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E102" s="6" t="inlineStr">
+        <is>
+          <t>Raised 2026-08-06 during the Email OTP expiration change (3600 to 86400).</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A103" s="7" t="inlineStr">
-        <is>
-          <t>Verify the financial dashboard</t>
-        </is>
-      </c>
-      <c r="B103" s="8" t="inlineStr">
-        <is>
-          <t>Confirm it reports MRR, churn, and revenue by tier correctly (churn once showed 2055%).</t>
-        </is>
-      </c>
-      <c r="C103" s="8" t="inlineStr">
-        <is>
-          <t>Verify financial dashboard accuracy.</t>
-        </is>
-      </c>
-      <c r="D103" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E103" s="8" t="inlineStr">
-        <is>
-          <t>Built in Lovable originally — accuracy unconfirmed.</t>
-        </is>
-      </c>
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>BUSINESS   ·   1 item</t>
+        </is>
+      </c>
+      <c r="B103" s="29" t="n"/>
+      <c r="C103" s="29" t="n"/>
+      <c r="D103" s="29" t="n"/>
+      <c r="E103" s="30" t="n"/>
     </row>
     <row r="104" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A104" s="7" t="inlineStr">
         <is>
-          <t>Verify the admin financial data function</t>
-        </is>
-      </c>
-      <c r="B104" s="8" t="inlineStr">
-        <is>
-          <t>Confirm the edge function feeding admin financials returns correct numbers.</t>
-        </is>
-      </c>
-      <c r="C104" s="8" t="inlineStr">
-        <is>
-          <t>Verify admin-financial-data.</t>
-        </is>
-      </c>
-      <c r="D104" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E104" s="8" t="inlineStr">
-        <is>
-          <t>Confirm the numbers it returns are correct.</t>
-        </is>
-      </c>
+          <t>Verify the business application approval works</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="n"/>
+      <c r="C104" s="5" t="n"/>
+      <c r="D104" s="5" t="n"/>
+      <c r="E104" s="6" t="n"/>
     </row>
     <row r="105" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A105" s="7" t="inlineStr">
-        <is>
-          <t>Three-bucket revenue view</t>
-        </is>
-      </c>
-      <c r="B105" s="8" t="inlineStr">
-        <is>
-          <t>Show revenue split three ways.</t>
-        </is>
-      </c>
-      <c r="C105" s="8" t="inlineStr">
-        <is>
-          <t>Collected / projected / churned split.</t>
-        </is>
-      </c>
-      <c r="D105" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E105" s="8" t="inlineStr">
-        <is>
-          <t>Collected / projected / churned.</t>
-        </is>
-      </c>
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>FINANCIALS   ·   6 items</t>
+        </is>
+      </c>
+      <c r="B105" s="29" t="n"/>
+      <c r="C105" s="29" t="n"/>
+      <c r="D105" s="29" t="n"/>
+      <c r="E105" s="30" t="n"/>
     </row>
     <row r="106" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t>Member-facing financial widget</t>
+          <t>Verify the financial dashboard</t>
         </is>
       </c>
       <c r="B106" s="8" t="inlineStr">
         <is>
-          <t>A small financial widget members can see.</t>
+          <t>Confirm it reports MRR, churn, and revenue by tier correctly (churn once showed 2055%).</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t>Member-facing billing-status widget.</t>
-        </is>
-      </c>
-      <c r="D106" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
+          <t>Verify financial dashboard accuracy.</t>
+        </is>
+      </c>
+      <c r="D106" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
         <is>
-          <t>Small billing-status widget for members.</t>
+          <t>Built in Lovable originally — accuracy unconfirmed.</t>
         </is>
       </c>
     </row>
     <row r="107" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A107" s="7" t="inlineStr">
         <is>
-          <t>Reduce redundant Stripe scans</t>
+          <t>Verify the admin financial data function</t>
+        </is>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
+          <t>Confirm the edge function feeding admin financials returns correct numbers.</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>Verify admin-financial-data.</t>
+        </is>
+      </c>
+      <c r="D107" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E107" s="8" t="inlineStr">
+        <is>
+          <t>Confirm the numbers it returns are correct.</t>
         </is>
       </c>
     </row>
     <row r="108" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t>Past-due dismissal flow</t>
-        </is>
-      </c>
-      <c r="B108" s="5" t="n"/>
-      <c r="C108" s="5" t="n"/>
-      <c r="D108" s="5" t="n"/>
-      <c r="E108" s="6" t="n"/>
+          <t>Three-bucket revenue view</t>
+        </is>
+      </c>
+      <c r="B108" s="8" t="inlineStr">
+        <is>
+          <t>Show revenue split three ways.</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>Collected / projected / churned split.</t>
+        </is>
+      </c>
+      <c r="D108" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E108" s="8" t="inlineStr">
+        <is>
+          <t>Collected / projected / churned.</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A109" s="4" t="inlineStr">
-        <is>
-          <t>EMAIL &amp; DRIP   ·   13 items</t>
-        </is>
-      </c>
-      <c r="B109" s="29" t="n"/>
-      <c r="C109" s="29" t="n"/>
-      <c r="D109" s="29" t="n"/>
-      <c r="E109" s="30" t="n"/>
+      <c r="A109" s="7" t="inlineStr">
+        <is>
+          <t>Member-facing financial widget</t>
+        </is>
+      </c>
+      <c r="B109" s="8" t="inlineStr">
+        <is>
+          <t>A small financial widget members can see.</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>Member-facing billing-status widget.</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E109" s="8" t="inlineStr">
+        <is>
+          <t>Small billing-status widget for members.</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t>Drip email health banner</t>
-        </is>
-      </c>
-      <c r="B110" s="8" t="inlineStr">
-        <is>
-          <t>A banner flagging when drips are silently failing or stalled.</t>
-        </is>
-      </c>
-      <c r="C110" s="8" t="inlineStr">
-        <is>
-          <t>Drip health-check banner.</t>
-        </is>
-      </c>
-      <c r="D110" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E110" s="8" t="inlineStr">
-        <is>
-          <t>Flags silently failing / stalled drips.</t>
-        </is>
-      </c>
+          <t>Reduce redundant Stripe scans</t>
+        </is>
+      </c>
+      <c r="B110" s="29" t="n"/>
+      <c r="C110" s="29" t="n"/>
+      <c r="D110" s="29" t="n"/>
+      <c r="E110" s="30" t="n"/>
     </row>
     <row r="111" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A111" s="7" t="inlineStr">
         <is>
-          <t>Guest follow-up drip (7 + 20 day)</t>
-        </is>
-      </c>
-      <c r="B111" s="8" t="inlineStr">
-        <is>
-          <t>Automatic emails to guests at day 7 and 20 to convert them.</t>
-        </is>
-      </c>
-      <c r="C111" s="8" t="inlineStr">
-        <is>
-          <t>Guest 7-day + 20-day drip.</t>
-        </is>
-      </c>
-      <c r="D111" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E111" s="8" t="inlineStr">
-        <is>
-          <t>Converts guests at day 7 and 20.</t>
-        </is>
-      </c>
+          <t>Past-due dismissal flow</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="n"/>
+      <c r="C111" s="5" t="n"/>
+      <c r="D111" s="5" t="n"/>
+      <c r="E111" s="6" t="n"/>
     </row>
     <row r="112" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A112" s="7" t="inlineStr">
-        <is>
-          <t>14-day RSVP prompt for new members</t>
-        </is>
-      </c>
-      <c r="B112" s="8" t="inlineStr">
-        <is>
-          <t>Nudge new members who haven't RSVP'd within 14 days.</t>
-        </is>
-      </c>
-      <c r="C112" s="8" t="inlineStr">
-        <is>
-          <t>14-day RSVP prompt drip.</t>
-        </is>
-      </c>
-      <c r="D112" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E112" s="8" t="inlineStr">
-        <is>
-          <t>Nudges new members who haven't RSVP'd.</t>
-        </is>
-      </c>
+      <c r="A112" s="4" t="inlineStr">
+        <is>
+          <t>EMAIL &amp; DRIP   ·   13 items</t>
+        </is>
+      </c>
+      <c r="B112" s="29" t="n"/>
+      <c r="C112" s="29" t="n"/>
+      <c r="D112" s="29" t="n"/>
+      <c r="E112" s="30" t="n"/>
     </row>
     <row r="113" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A113" s="7" t="inlineStr">
         <is>
-          <t>Confirm the email log matches actual sends</t>
+          <t>Drip email health banner</t>
         </is>
       </c>
       <c r="B113" s="8" t="inlineStr">
         <is>
-          <t>Today failures are swallowed; make 'did this send' provable.</t>
+          <t>A banner flagging when drips are silently failing or stalled.</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t>email_log row matching; stop swallowing failures.</t>
+          <t>Drip health-check banner.</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
@@ -3237,24 +3192,24 @@
       </c>
       <c r="E113" s="8" t="inlineStr">
         <is>
-          <t>Stop swallowing failures so 'did this send' is provable.</t>
+          <t>Flags silently failing / stalled drips.</t>
         </is>
       </c>
     </row>
     <row r="114" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A114" s="7" t="inlineStr">
         <is>
-          <t>Per-email open/click analytics</t>
+          <t>Guest follow-up drip (7 + 20 day)</t>
         </is>
       </c>
       <c r="B114" s="8" t="inlineStr">
         <is>
-          <t>Track opens/clicks per template so we know what works.</t>
+          <t>Automatic emails to guests at day 7 and 20 to convert them.</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t>Per-template email analytics.</t>
+          <t>Guest 7-day + 20-day drip.</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
@@ -3264,24 +3219,24 @@
       </c>
       <c r="E114" s="8" t="inlineStr">
         <is>
-          <t>Per-template open / click tracking.</t>
+          <t>Converts guests at day 7 and 20.</t>
         </is>
       </c>
     </row>
     <row r="115" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A115" s="7" t="inlineStr">
         <is>
-          <t>Per-member engagement scoring</t>
+          <t>14-day RSVP prompt for new members</t>
         </is>
       </c>
       <c r="B115" s="8" t="inlineStr">
         <is>
-          <t>Score each member's engagement from email/event activity.</t>
+          <t>Nudge new members who haven't RSVP'd within 14 days.</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t>Engagement scoring per member.</t>
+          <t>14-day RSVP prompt drip.</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr">
@@ -3291,24 +3246,24 @@
       </c>
       <c r="E115" s="8" t="inlineStr">
         <is>
-          <t>Score members from email / event activity.</t>
+          <t>Nudges new members who haven't RSVP'd.</t>
         </is>
       </c>
     </row>
     <row r="116" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>Category-level unsubscribe preferences</t>
+          <t>Confirm the email log matches actual sends</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
         <is>
-          <t>Let members opt out of specific categories, not all-or-nothing; builds on the one-flag fix.</t>
+          <t>Today failures are swallowed; make 'did this send' provable.</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t>Per-category opt-out prefs + a member settings page.</t>
+          <t>email_log row matching; stop swallowing failures.</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr">
@@ -3318,24 +3273,24 @@
       </c>
       <c r="E116" s="8" t="inlineStr">
         <is>
-          <t>Builds on the one-flag opt-out fix.</t>
+          <t>Stop swallowing failures so 'did this send' is provable.</t>
         </is>
       </c>
     </row>
     <row r="117" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t>Branching drips based on opens/clicks</t>
+          <t>Per-email open/click analytics</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
         <is>
-          <t>Drip sequences that branch on open/click.</t>
+          <t>Track opens/clicks per template so we know what works.</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t>Open/click-branching drips.</t>
+          <t>Per-template email analytics.</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr">
@@ -3345,24 +3300,24 @@
       </c>
       <c r="E117" s="8" t="inlineStr">
         <is>
-          <t>Branch sequences on open / click.</t>
+          <t>Per-template open / click tracking.</t>
         </is>
       </c>
     </row>
     <row r="118" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t>Send email from a contact record</t>
+          <t>Per-member engagement scoring</t>
         </is>
       </c>
       <c r="B118" s="8" t="inlineStr">
         <is>
-          <t>Let an admin email directly from a member/contact record.</t>
+          <t>Score each member's engagement from email/event activity.</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t>Send-email action on the contact record.</t>
+          <t>Engagement scoring per member.</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr">
@@ -3372,24 +3327,24 @@
       </c>
       <c r="E118" s="8" t="inlineStr">
         <is>
-          <t>Admin emails directly from a member record.</t>
+          <t>Score members from email / event activity.</t>
         </is>
       </c>
     </row>
     <row r="119" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A119" s="7" t="inlineStr">
         <is>
-          <t>Attachments and images on event email campaigns</t>
+          <t>Category-level unsubscribe preferences</t>
         </is>
       </c>
       <c r="B119" s="8" t="inlineStr">
         <is>
-          <t>Let campaign emails include attachments and images.</t>
+          <t>Let members opt out of specific categories, not all-or-nothing; builds on the one-flag fix.</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t>Extend the campaign editor for attachments + images.</t>
+          <t>Per-category opt-out prefs + a member settings page.</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr">
@@ -3399,196 +3354,236 @@
       </c>
       <c r="E119" s="8" t="inlineStr">
         <is>
-          <t>Extend the campaign editor.</t>
+          <t>Builds on the one-flag opt-out fix.</t>
         </is>
       </c>
     </row>
     <row r="120" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A120" s="7" t="inlineStr">
         <is>
-          <t>Live test the guest-pass drip</t>
+          <t>Branching drips based on opens/clicks</t>
         </is>
       </c>
       <c r="B120" s="8" t="inlineStr">
         <is>
-          <t>Confirm the drip fires correctly on a guest pass.</t>
+          <t>Drip sequences that branch on open/click.</t>
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t>Live test the drip on guest_pass.</t>
-        </is>
-      </c>
-      <c r="D120" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
+          <t>Open/click-branching drips.</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
         </is>
       </c>
       <c r="E120" s="8" t="inlineStr">
         <is>
-          <t>Confirm it fires on a guest pass.</t>
+          <t>Branch sequences on open / click.</t>
         </is>
       </c>
     </row>
     <row r="121" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A121" s="7" t="inlineStr">
         <is>
-          <t>Merge guest follow-up into the drip processor</t>
+          <t>Send email from a contact record</t>
+        </is>
+      </c>
+      <c r="B121" s="8" t="inlineStr">
+        <is>
+          <t>Let an admin email directly from a member/contact record.</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>Send-email action on the contact record.</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E121" s="8" t="inlineStr">
+        <is>
+          <t>Admin emails directly from a member record.</t>
         </is>
       </c>
     </row>
     <row r="122" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A122" s="7" t="inlineStr">
         <is>
+          <t>Attachments and images on event email campaigns</t>
+        </is>
+      </c>
+      <c r="B122" s="8" t="inlineStr">
+        <is>
+          <t>Let campaign emails include attachments and images.</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>Extend the campaign editor for attachments + images.</t>
+        </is>
+      </c>
+      <c r="D122" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E122" s="8" t="inlineStr">
+        <is>
+          <t>Extend the campaign editor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A123" s="7" t="inlineStr">
+        <is>
+          <t>Live test the guest-pass drip</t>
+        </is>
+      </c>
+      <c r="B123" s="8" t="inlineStr">
+        <is>
+          <t>Confirm the drip fires correctly on a guest pass.</t>
+        </is>
+      </c>
+      <c r="C123" s="8" t="inlineStr">
+        <is>
+          <t>Live test the drip on guest_pass.</t>
+        </is>
+      </c>
+      <c r="D123" s="11" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E123" s="8" t="inlineStr">
+        <is>
+          <t>Confirm it fires on a guest pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A124" s="7" t="inlineStr">
+        <is>
+          <t>Merge guest follow-up into the drip processor</t>
+        </is>
+      </c>
+      <c r="B124" s="29" t="n"/>
+      <c r="C124" s="29" t="n"/>
+      <c r="D124" s="29" t="n"/>
+      <c r="E124" s="30" t="n"/>
+    </row>
+    <row r="125" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A125" s="7" t="inlineStr">
+        <is>
           <t>Push current members to subscribe to the calendar + add their pass</t>
         </is>
       </c>
-      <c r="B122" s="5" t="n"/>
-      <c r="C122" s="5" t="n"/>
-      <c r="D122" s="5" t="n"/>
-      <c r="E122" s="6" t="n"/>
-    </row>
-    <row r="123" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A123" s="4" t="inlineStr">
+      <c r="B125" s="5" t="n"/>
+      <c r="C125" s="5" t="n"/>
+      <c r="D125" s="5" t="n"/>
+      <c r="E125" s="6" t="n"/>
+    </row>
+    <row r="126" ht="15" customFormat="1" customHeight="1" s="2">
+      <c r="A126" s="4" t="inlineStr">
         <is>
           <t>DATA &amp; CLEANUP   ·   6 items</t>
         </is>
       </c>
-      <c r="B123" s="29" t="n"/>
-      <c r="C123" s="29" t="n"/>
-      <c r="D123" s="29" t="n"/>
-      <c r="E123" s="30" t="n"/>
-    </row>
-    <row r="124" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A124" s="17" t="inlineStr">
+      <c r="B126" s="29" t="n"/>
+      <c r="C126" s="29" t="n"/>
+      <c r="D126" s="29" t="n"/>
+      <c r="E126" s="30" t="n"/>
+    </row>
+    <row r="127" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
+      <c r="A127" s="17" t="inlineStr">
         <is>
           <t>Add CHECK constraints incrementally (enums REJECTED — too risky)</t>
         </is>
       </c>
-      <c r="B124" s="15" t="inlineStr">
+      <c r="B127" s="15" t="inlineStr">
         <is>
           <t>Was 'convert status text -&gt; enums'. DIAGNOSED Jul 9 as too risky: ~35 tables / 60+ write paths, and profiles.subscription_status is fed by the Stripe webhook with Stripe's full status vocabulary (trialing/paused/incomplete/etc). An enum built from observed values would make the webhook UPDATE throw on the first unseen status — silent breakage in the PAYMENT path. Enums rejected.</t>
         </is>
       </c>
-      <c r="C124" s="15" t="inlineStr">
+      <c r="C127" s="15" t="inlineStr">
         <is>
           <t>If typo-prevention is wanted later: add per-table CHECK constraints (NOT enums), table-by-table, starting with attendance_credentials (values: active/used/voided). Trivially reversible. Its own scoped task — never wholesale.</t>
         </is>
       </c>
-      <c r="D124" s="18" t="inlineStr">
+      <c r="D127" s="18" t="inlineStr">
         <is>
           <t>Deferred</t>
         </is>
       </c>
-      <c r="E124" s="15" t="inlineStr">
+      <c r="E127" s="15" t="inlineStr">
         <is>
           <t>Reclassified Jul 9. Do NOT rush — payment-path risk. CHECK constraints are the safe 80/20 if revisited.</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A125" s="17" t="inlineStr">
+    <row r="128" ht="23.85" customFormat="1" customHeight="1" s="2">
+      <c r="A128" s="17" t="inlineStr">
         <is>
           <t>RSVP attribution by event ID</t>
         </is>
       </c>
-      <c r="B125" s="15" t="inlineStr">
+      <c r="B128" s="15" t="inlineStr">
         <is>
           <t>DIAGNOSED Jul 9: bigger than 'add a column'. Per-event RSVP tagging is DEAD — the code that slug-tagged events was removed; since Apr 21 a public RSVP only gets a generic 'free-event-rsvp' tag, so you can't segment 'RSVP'd to event X' for any recent event. 6 frozen slug-tags remain (105 rows) and rot on rename. contact_tags has NO event_id column.</t>
         </is>
       </c>
-      <c r="C125" s="15" t="inlineStr">
+      <c r="C128" s="15" t="inlineStr">
         <is>
           <t>HALF-DAY scoped task (not a quick close): (1) migration add nullable event_id uuid REFERENCES events(id) to contact_tags; (2) re-add per-event tagging in capture-public-rsvp (event_id already in scope) + optionally create-guest-pass; (3) backfill — 5 of 6 slug-tags map to real event_ids by title-slug match (1 unmatched: coffee-and-connect-tabbris-co-working). Deploys + tests.</t>
         </is>
       </c>
-      <c r="D125" s="19" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E125" s="15" t="inlineStr">
+      <c r="D128" s="19" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E128" s="15" t="inlineStr">
         <is>
           <t>Jul 9: revives dead per-event attribution. Own task, budget a half-day. Backfill mostly possible.</t>
         </is>
       </c>
     </row>
-    <row r="126" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A126" s="7" t="inlineStr">
+    <row r="129" ht="21.75" customFormat="1" customHeight="1" s="2">
+      <c r="A129" s="7" t="inlineStr">
         <is>
           <t>Drop ~35 empty leftover tables</t>
         </is>
       </c>
-      <c r="B126" s="8" t="inlineStr">
+      <c r="B129" s="8" t="inlineStr">
         <is>
           <t>~35 empty scaffolding tables (old CRM, social manager, feed, DMs).</t>
         </is>
       </c>
-      <c r="C126" s="8" t="inlineStr">
+      <c r="C129" s="8" t="inlineStr">
         <is>
           <t>Export copies as a receipt, then drop.</t>
         </is>
       </c>
-      <c r="D126" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E126" s="8" t="inlineStr">
+      <c r="D129" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E129" s="8" t="inlineStr">
         <is>
           <t>Don't drop without exporting copies first.</t>
         </is>
       </c>
-    </row>
-    <row r="127" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
-      <c r="A127" s="7" t="inlineStr">
-        <is>
-          <t>Drop old backup tables after soak</t>
-        </is>
-      </c>
-      <c r="B127" s="8" t="inlineStr">
-        <is>
-          <t>Backup tables from recent migrations await a 2-4 week no-regression soak.</t>
-        </is>
-      </c>
-      <c r="C127" s="8" t="inlineStr">
-        <is>
-          <t>Drop dated backup_* tables after soak; confirm stability first.</t>
-        </is>
-      </c>
-      <c r="D127" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E127" s="8" t="inlineStr">
-        <is>
-          <t>Only after a 2-4 week no-regression soak.</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A128" s="7" t="inlineStr">
-        <is>
-          <t>Delete dead admin member components</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A129" s="4" t="inlineStr">
-        <is>
-          <t>MARKETING &amp; FRONT-END   ·   10 items</t>
-        </is>
-      </c>
-      <c r="B129" s="29" t="n"/>
-      <c r="C129" s="29" t="n"/>
-      <c r="D129" s="29" t="n"/>
-      <c r="E129" s="30" t="n"/>
     </row>
     <row r="130" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A130" s="7" t="inlineStr">
         <is>
-          <t>SEO + schema markup + pre-rendering (all front pages + 4 hub landers)</t>
+          <t>Drop old backup tables after soak</t>
         </is>
       </c>
       <c r="B130" s="29" t="n"/>
@@ -3599,98 +3594,46 @@
     <row r="131" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A131" s="7" t="inlineStr">
         <is>
-          <t>Homepage hero rebuild + image optimization</t>
-        </is>
-      </c>
-      <c r="B131" s="8" t="inlineStr">
-        <is>
-          <t>Rebuild the hero and compress oversized hero images (currently 24-30MB, should be 200-800KB).</t>
-        </is>
-      </c>
-      <c r="C131" s="8" t="inlineStr">
-        <is>
-          <t>Hero rebuild + compress images.</t>
-        </is>
-      </c>
-      <c r="D131" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E131" s="8" t="inlineStr">
-        <is>
-          <t>Includes compressing 24-30MB hero images to 200-800KB.</t>
+          <t>Delete dead admin member components</t>
         </is>
       </c>
     </row>
     <row r="132" ht="23.85" customFormat="1" customHeight="1" s="2">
-      <c r="A132" s="7" t="inlineStr">
-        <is>
-          <t>Homepage copy rewrite + slogan</t>
-        </is>
-      </c>
-      <c r="B132" s="8" t="inlineStr">
-        <is>
-          <t>Rewrite homepage body/section copy and update the slogan.</t>
-        </is>
-      </c>
-      <c r="C132" s="8" t="inlineStr">
-        <is>
-          <t>Body + section copy + slogan.</t>
-        </is>
-      </c>
-      <c r="D132" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E132" s="8" t="inlineStr">
-        <is>
-          <t>Needs the copy spec.</t>
-        </is>
-      </c>
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>MARKETING &amp; FRONT-END   ·   10 items</t>
+        </is>
+      </c>
+      <c r="B132" s="29" t="n"/>
+      <c r="C132" s="29" t="n"/>
+      <c r="D132" s="29" t="n"/>
+      <c r="E132" s="30" t="n"/>
     </row>
     <row r="133" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A133" s="7" t="inlineStr">
         <is>
-          <t>Fix the mobile hero sliding bug</t>
-        </is>
-      </c>
-      <c r="B133" s="8" t="inlineStr">
-        <is>
-          <t>A visual bug where the hero image slides on mobile.</t>
-        </is>
-      </c>
-      <c r="C133" s="8" t="inlineStr">
-        <is>
-          <t>Mobile hero sliding fix.</t>
-        </is>
-      </c>
-      <c r="D133" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E133" s="8" t="inlineStr">
-        <is>
-          <t>Fix the hero sliding on mobile.</t>
-        </is>
-      </c>
+          <t>SEO + schema markup + pre-rendering (all front pages + 4 hub landers)</t>
+        </is>
+      </c>
+      <c r="B133" s="29" t="n"/>
+      <c r="C133" s="29" t="n"/>
+      <c r="D133" s="29" t="n"/>
+      <c r="E133" s="30" t="n"/>
     </row>
     <row r="134" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A134" s="7" t="inlineStr">
         <is>
-          <t>The Exchange page</t>
+          <t>Homepage hero rebuild + image optimization</t>
         </is>
       </c>
       <c r="B134" s="8" t="inlineStr">
         <is>
-          <t>Build The Exchange page (speaker-driven business event product page).</t>
+          <t>Rebuild the hero and compress oversized hero images (currently 24-30MB, should be 200-800KB).</t>
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr">
         <is>
-          <t>The Exchange page.</t>
+          <t>Hero rebuild + compress images.</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr">
@@ -3700,24 +3643,24 @@
       </c>
       <c r="E134" s="8" t="inlineStr">
         <is>
-          <t>Speaker-driven business-event product page.</t>
+          <t>Includes compressing 24-30MB hero images to 200-800KB.</t>
         </is>
       </c>
     </row>
     <row r="135" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
       <c r="A135" s="7" t="inlineStr">
         <is>
-          <t>Sponsor page (likely folds into /business)</t>
+          <t>Homepage copy rewrite + slogan</t>
         </is>
       </c>
       <c r="B135" s="8" t="inlineStr">
         <is>
-          <t>Sponsor functionality — likely folds into the /business application routing.</t>
+          <t>Rewrite homepage body/section copy and update the slogan.</t>
         </is>
       </c>
       <c r="C135" s="8" t="inlineStr">
         <is>
-          <t>Probably absorbed by the /business rebuild.</t>
+          <t>Body + section copy + slogan.</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr">
@@ -3727,24 +3670,24 @@
       </c>
       <c r="E135" s="8" t="inlineStr">
         <is>
-          <t>Likely folds into the /business rebuild — confirm first.</t>
+          <t>Needs the copy spec.</t>
         </is>
       </c>
     </row>
     <row r="136" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A136" s="7" t="inlineStr">
         <is>
-          <t>/business page rebuild with dynamic application</t>
+          <t>Fix the mobile hero sliding bug</t>
         </is>
       </c>
       <c r="B136" s="8" t="inlineStr">
         <is>
-          <t>Rebuild /business as one page with a dynamic application routing prospects to membership, Preferred Business, or sponsorship by their answers.</t>
+          <t>A visual bug where the hero image slides on mobile.</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t>Dynamic diagnose-before-offer application.</t>
+          <t>Mobile hero sliding fix.</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr">
@@ -3754,24 +3697,24 @@
       </c>
       <c r="E136" s="8" t="inlineStr">
         <is>
-          <t>Routes prospects to membership, Preferred Business, or sponsorship.</t>
+          <t>Fix the hero sliding on mobile.</t>
         </is>
       </c>
     </row>
     <row r="137" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A137" s="7" t="inlineStr">
         <is>
-          <t>Charlotte hub landing sites (4 public landers)</t>
+          <t>The Exchange page</t>
         </is>
       </c>
       <c r="B137" s="8" t="inlineStr">
         <is>
-          <t>Four audience-specific public landers (cltarrival / cltfounded / clteatsandevents / cltreset) that funnel Charlotte audiences into the club.</t>
+          <t>Build The Exchange page (speaker-driven business event product page).</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t>4 public landers, shared skeleton, own design pass, fully pre-rendered + schema (see SEO item). They feed The Network.</t>
+          <t>The Exchange page.</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
@@ -3781,24 +3724,24 @@
       </c>
       <c r="E137" s="8" t="inlineStr">
         <is>
-          <t>Public landers can ship earlier; they pair with The Network below.</t>
+          <t>Speaker-driven business-event product page.</t>
         </is>
       </c>
     </row>
     <row r="138" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A138" s="7" t="inlineStr">
         <is>
-          <t>The Network — four hubs + members rolled up</t>
+          <t>Sponsor page (likely folds into /business)</t>
         </is>
       </c>
       <c r="B138" s="8" t="inlineStr">
         <is>
-          <t>The four hubs rolled up into one view, plus all members. Two faces reading the same data: a PUBLIC face (the hub landers + business/partner listings — the sales asset) and an INTERNAL in-portal view that rolls up everyone. Social members appear ONLY on the internal in-portal view — never on the public hubs.</t>
+          <t>Sponsor functionality — likely folds into the /business application routing.</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t>Roll the four hubs into one Network view + members. Public face = hubs / business + partner listings (social members excluded). Internal face = full rolled-up view including social members. Reads the same hub data as the landers.</t>
+          <t>Probably absorbed by the /business rebuild.</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr">
@@ -3808,32 +3751,68 @@
       </c>
       <c r="E138" s="8" t="inlineStr">
         <is>
-          <t>Depends on the portal + identity foundation. Social members are internal-only on The Network. Separate from the member directory (people-only).</t>
+          <t>Likely folds into the /business rebuild — confirm first.</t>
         </is>
       </c>
     </row>
     <row r="139" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A139" s="7" t="inlineStr">
         <is>
-          <t>Instagram comment auto-DM (ManyChat)</t>
+          <t>/business page rebuild with dynamic application</t>
+        </is>
+      </c>
+      <c r="B139" s="8" t="inlineStr">
+        <is>
+          <t>Rebuild /business as one page with a dynamic application routing prospects to membership, Preferred Business, or sponsorship by their answers.</t>
+        </is>
+      </c>
+      <c r="C139" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic diagnose-before-offer application.</t>
+        </is>
+      </c>
+      <c r="D139" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E139" s="8" t="inlineStr">
+        <is>
+          <t>Routes prospects to membership, Preferred Business, or sponsorship.</t>
         </is>
       </c>
     </row>
     <row r="140" ht="21.75" customFormat="1" customHeight="1" s="2">
-      <c r="A140" s="4" t="inlineStr">
-        <is>
-          <t>AI / AGENTS (LATER EFFORT)   ·   2 items</t>
-        </is>
-      </c>
-      <c r="B140" s="29" t="n"/>
-      <c r="C140" s="29" t="n"/>
-      <c r="D140" s="29" t="n"/>
-      <c r="E140" s="30" t="n"/>
+      <c r="A140" s="7" t="inlineStr">
+        <is>
+          <t>Charlotte hub landing sites (4 public landers)</t>
+        </is>
+      </c>
+      <c r="B140" s="8" t="inlineStr">
+        <is>
+          <t>Four audience-specific public landers (cltarrival / cltfounded / clteatsandevents / cltreset) that funnel Charlotte audiences into the club.</t>
+        </is>
+      </c>
+      <c r="C140" s="8" t="inlineStr">
+        <is>
+          <t>4 public landers, shared skeleton, own design pass, fully pre-rendered + schema (see SEO item). They feed The Network.</t>
+        </is>
+      </c>
+      <c r="D140" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E140" s="8" t="inlineStr">
+        <is>
+          <t>Public landers can ship earlier; they pair with The Network below.</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="113.4" customFormat="1" customHeight="1" s="2">
       <c r="A141" s="7" t="inlineStr">
         <is>
-          <t>AI concierge + agent platform</t>
+          <t>The Network — four hubs + members rolled up</t>
         </is>
       </c>
       <c r="B141" s="29" t="n"/>
@@ -3844,34 +3823,14 @@
     <row r="142" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A142" s="7" t="inlineStr">
         <is>
-          <t>AI foundations (memory, embeddings, coordination)</t>
-        </is>
-      </c>
-      <c r="B142" s="8" t="inlineStr">
-        <is>
-          <t>Supporting infra for the agents: shared memory, member embeddings, multi-agent coordination, model routing.</t>
-        </is>
-      </c>
-      <c r="C142" s="8" t="inlineStr">
-        <is>
-          <t>pgvector + embeddings, agent_memory, multi-agent coordination, model routing.</t>
-        </is>
-      </c>
-      <c r="D142" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E142" s="8" t="inlineStr">
-        <is>
-          <t>A later effort; supports the agents (embeddings, memory, routing).</t>
+          <t>Instagram comment auto-DM (ManyChat)</t>
         </is>
       </c>
     </row>
     <row r="143" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>EVENT DISCUSSION &amp; NOTIFICATIONS + JUL-5/6 FINDINGS — IN-HOUSE (NOT ON THE DEVELOPER SHEET)   ·   10 items</t>
+          <t>AI / AGENTS (LATER EFFORT)   ·   2 items</t>
         </is>
       </c>
       <c r="B143" s="29" t="n"/>
@@ -3882,240 +3841,192 @@
     <row r="144" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A144" s="7" t="inlineStr">
         <is>
-          <t>Rotate the R2 media token (exposed key)</t>
-        </is>
-      </c>
-      <c r="B144" s="8" t="inlineStr">
-        <is>
-          <t>The R2 Access Key ID + Secret for bucket 704-discussion-media were exposed in a working chat (screenshot/paste). Scope = that one media bucket only — low blast radius, but rotate.</t>
-        </is>
-      </c>
-      <c r="C144" s="8" t="inlineStr">
-        <is>
-          <t>After 6c ships: Cloudflare -&gt; R2 -&gt; API tokens -&gt; re-create 704-discussion-upload (Object Read &amp; Write, bucket-scoped) -&gt; supabase secrets set the two new values -&gt; confirm an upload still works.</t>
-        </is>
-      </c>
-      <c r="D144" s="20" t="inlineStr">
-        <is>
-          <t>Declined</t>
-        </is>
-      </c>
-      <c r="E144" s="8" t="inlineStr">
-        <is>
-          <t>Adam declined rotation Jul 5 - standing watch item. Key scope = one media bucket only (no member data / money / DB). Say 'rotate' anytime: ~2 min.</t>
-        </is>
-      </c>
+          <t>AI concierge + agent platform</t>
+        </is>
+      </c>
+      <c r="B144" s="29" t="n"/>
+      <c r="C144" s="29" t="n"/>
+      <c r="D144" s="29" t="n"/>
+      <c r="E144" s="30" t="n"/>
     </row>
     <row r="145" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A145" s="7" t="inlineStr">
         <is>
-          <t>Verify/finish the Alerts page (full history, discussion types)</t>
+          <t>AI foundations (memory, embeddings, coordination)</t>
         </is>
       </c>
       <c r="B145" s="8" t="inlineStr">
         <is>
-          <t>Locked: bell badge clears on open, items dismiss via X, but the ALERTS PAGE keeps every notification forever - markable read (single + all). PARTIAL Jul 5: /dashboard/notifications now honors action_url (deep-links verified end to end). Remaining: full-history + mark-read behavior verification.</t>
+          <t>Supporting infra for the agents: shared memory, member embeddings, multi-agent coordination, model routing.</t>
         </is>
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t>Read the Alerts page code; verify full-history + mark-read behavior and that all discussion notification types display with correct deep-links; fix gaps. Desktop + mobile test.</t>
-        </is>
-      </c>
-      <c r="D145" s="20" t="inlineStr">
-        <is>
-          <t>Verify</t>
+          <t>pgvector + embeddings, agent_memory, multi-agent coordination, model routing.</t>
+        </is>
+      </c>
+      <c r="D145" s="10" t="inlineStr">
+        <is>
+          <t>Build</t>
         </is>
       </c>
       <c r="E145" s="8" t="inlineStr">
         <is>
-          <t>Deep-links fixed+verified Jul 5 (commit e9f6250). Remaining: verify full-history retention + mark-read (single + all).</t>
+          <t>A later effort; supports the agents (embeddings, memory, routing).</t>
         </is>
       </c>
     </row>
     <row r="146" ht="57.45" customFormat="1" customHeight="1" s="2">
-      <c r="A146" s="7" t="inlineStr">
-        <is>
-          <t>Messaging: bells for messages in existing conversations</t>
-        </is>
-      </c>
-      <c r="B146" s="8" t="inlineStr">
-        <is>
-          <t>Messaging was resurrected Jul 5 (DMs/groups had NEVER worked since launch: RETURNING/RLS deadlock, participants-insert policy tautology, content-vs-body + title-vs-name schema mismatches, 4 missing messages columns - all fixed and verified end to end). Remaining gap: notifyNewConversation only fires on conversation CREATION, so messages into an existing thread produce no bell.</t>
-        </is>
-      </c>
-      <c r="C146" s="8" t="inlineStr">
-        <is>
-          <t>Add a new_message bell per message into an existing conversation, throttled (e.g. skip if an unread new_message bell for that conversation already exists).</t>
-        </is>
-      </c>
-      <c r="D146" s="20" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E146" s="8" t="inlineStr">
-        <is>
-          <t>Follow-on to the Jul 5 messaging resurrection. Recipients currently only get notified on the first-ever message.</t>
-        </is>
-      </c>
+      <c r="A146" s="4" t="inlineStr">
+        <is>
+          <t>EVENT DISCUSSION &amp; NOTIFICATIONS + JUL-5/6 FINDINGS — IN-HOUSE (NOT ON THE DEVELOPER SHEET)   ·   10 items</t>
+        </is>
+      </c>
+      <c r="B146" s="29" t="n"/>
+      <c r="C146" s="29" t="n"/>
+      <c r="D146" s="29" t="n"/>
+      <c r="E146" s="30" t="n"/>
     </row>
     <row r="147" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A147" s="7" t="inlineStr">
         <is>
-          <t>Messaging: attachment uploads (images/files)</t>
+          <t>Rotate the R2 media token (exposed key)</t>
         </is>
       </c>
       <c r="B147" s="8" t="inlineStr">
         <is>
-          <t>MessagingView has image/file upload code paths and messages now has image_urls/file_urls/file_names columns (added Jul 5), but the storage wiring (bucket, upload flow) has never been tested and may not exist.</t>
+          <t>The R2 Access Key ID + Secret for bucket 704-discussion-media were exposed in a working chat (screenshot/paste). Scope = that one media bucket only — low blast radius, but rotate.</t>
         </is>
       </c>
       <c r="C147" s="8" t="inlineStr">
         <is>
-          <t>Audit the attachment path end to end: storage bucket, upload call, render. Fix or wire what's missing. Desktop + mobile test.</t>
+          <t>After 6c ships: Cloudflare -&gt; R2 -&gt; API tokens -&gt; re-create 704-discussion-upload (Object Read &amp; Write, bucket-scoped) -&gt; supabase secrets set the two new values -&gt; confirm an upload still works.</t>
         </is>
       </c>
       <c r="D147" s="20" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Declined</t>
         </is>
       </c>
       <c r="E147" s="8" t="inlineStr">
         <is>
-          <t>Text messaging + edits verified Jul 5; attachments explicitly skipped in that test.</t>
+          <t>Adam declined rotation Jul 5 - standing watch item. Key scope = one media bucket only (no member data / money / DB). Say 'rotate' anytime: ~2 min.</t>
         </is>
       </c>
     </row>
     <row r="148" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A148" s="7" t="inlineStr">
         <is>
+          <t>Verify/finish the Alerts page (full history, discussion types)</t>
+        </is>
+      </c>
+      <c r="B148" s="8" t="inlineStr">
+        <is>
+          <t>Locked: bell badge clears on open, items dismiss via X, but the ALERTS PAGE keeps every notification forever - markable read (single + all). PARTIAL Jul 5: /dashboard/notifications now honors action_url (deep-links verified end to end). Remaining: full-history + mark-read behavior verification.</t>
+        </is>
+      </c>
+      <c r="C148" s="8" t="inlineStr">
+        <is>
+          <t>Read the Alerts page code; verify full-history + mark-read behavior and that all discussion notification types display with correct deep-links; fix gaps. Desktop + mobile test.</t>
+        </is>
+      </c>
+      <c r="D148" s="20" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E148" s="8" t="inlineStr">
+        <is>
+          <t>Deep-links fixed+verified Jul 5 (commit e9f6250). Remaining: verify full-history retention + mark-read (single + all).</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="15" customFormat="1" customHeight="1" s="2">
+      <c r="A149" s="7" t="inlineStr">
+        <is>
+          <t>Messaging: bells for messages in existing conversations</t>
+        </is>
+      </c>
+      <c r="B149" s="8" t="inlineStr">
+        <is>
+          <t>Messaging was resurrected Jul 5 (DMs/groups had NEVER worked since launch: RETURNING/RLS deadlock, participants-insert policy tautology, content-vs-body + title-vs-name schema mismatches, 4 missing messages columns - all fixed and verified end to end). Remaining gap: notifyNewConversation only fires on conversation CREATION, so messages into an existing thread produce no bell.</t>
+        </is>
+      </c>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t>Add a new_message bell per message into an existing conversation, throttled (e.g. skip if an unread new_message bell for that conversation already exists).</t>
+        </is>
+      </c>
+      <c r="D149" s="20" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E149" s="8" t="inlineStr">
+        <is>
+          <t>Follow-on to the Jul 5 messaging resurrection. Recipients currently only get notified on the first-ever message.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="57.45" customFormat="1" customHeight="1" s="2">
+      <c r="A150" s="7" t="inlineStr">
+        <is>
+          <t>Messaging: attachment uploads (images/files)</t>
+        </is>
+      </c>
+      <c r="B150" s="29" t="n"/>
+      <c r="C150" s="29" t="n"/>
+      <c r="D150" s="29" t="n"/>
+      <c r="E150" s="30" t="n"/>
+    </row>
+    <row r="151" ht="46.25" customFormat="1" customHeight="1" s="2">
+      <c r="A151" s="7" t="inlineStr">
+        <is>
           <t>Verify the first real-money admin refund (Remove &amp; Refund)</t>
         </is>
       </c>
-      <c r="B148" s="8" t="inlineStr">
+      <c r="B151" s="8" t="inlineStr">
         <is>
           <t>Admin Remove &amp; Refund shipped Jul 5 (edge fn admin-refund-ticket: admin gate, Stripe refund, void credential, seat freed; + attendee-dialog button, mobile-safe). Every branch proven EXCEPT the successful real-money refund line: void-only path, 403 gate, already-voided idempotency, and the Stripe-failure 502 fail-safe (no seat freed without money returned) all tested live.</t>
         </is>
       </c>
-      <c r="C148" s="8" t="inlineStr">
+      <c r="C151" s="8" t="inlineStr">
         <is>
           <t>WAIT mode: on the next genuine member refund request, use Remove &amp; Refund in the event attendee dialog and verify: Stripe refunded, credential voided, seat freed, toast correct.</t>
         </is>
       </c>
-      <c r="D148" s="20" t="inlineStr">
+      <c r="D151" s="20" t="inlineStr">
         <is>
           <t>Verify</t>
         </is>
       </c>
-      <c r="E148" s="8" t="inlineStr">
+      <c r="E151" s="8" t="inlineStr">
         <is>
           <t>Zero-cost proof on the next real request. Sacred Walker (Jul 5) handled manually pre-feature; her case is the template.</t>
         </is>
       </c>
     </row>
-    <row r="149" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A149" s="21" t="inlineStr">
+    <row r="152" ht="57.45" customFormat="1" customHeight="1" s="2">
+      <c r="A152" s="21" t="inlineStr">
         <is>
           <t>SESSION LOG — JUL 7–9 2026 (COMPLETED; kept as record, esp. the security fix)</t>
-        </is>
-      </c>
-    </row>
-    <row r="150" ht="57.45" customFormat="1" customHeight="1" s="2">
-      <c r="A150" s="16" t="inlineStr">
-        <is>
-          <t>[DONE] Security: dropped anon-readable active_members view + locked event_participants_view</t>
-        </is>
-      </c>
-      <c r="B150" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL FIX Jul 9: active_members and event_participants_view were SECURITY DEFINER views with ALL privileges granted to anon — an unauthenticated internet caller could read every member's email/phone/Stripe customer ID + all attendee contact info, AND active_members (auto-updatable single-table view) exposed an anon WRITE path into profiles. active_members had ZERO callers -&gt; DROPPED. event_participants_view -&gt; security_invoker=true + REVOKE anon/authenticated (sole caller send-campaign uses service-role, unaffected). member_counts left as-is (intentional).</t>
-        </is>
-      </c>
-      <c r="C150" s="23" t="inlineStr">
-        <is>
-          <t>DONE via SQL. Verified from OUTSIDE with anon key: active_members=404, event_participants_view=401 permission denied. No rows leaked. send-campaign confirmed still works.</t>
-        </is>
-      </c>
-      <c r="D150" s="24" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E150" s="23" t="inlineStr">
-        <is>
-          <t>Biggest find of the session. Was disguised as a 'review Security Definer flags' tracker row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="46.25" customFormat="1" customHeight="1" s="2">
-      <c r="A151" s="16" t="inlineStr">
-        <is>
-          <t>[DONE] Nine-job cron auth resurrection + 2 guards, all 10 jobs healthy</t>
-        </is>
-      </c>
-      <c r="B151" s="23" t="inlineStr">
-        <is>
-          <t>Full audit found NINE broken crons (sheet knew of 2). Fixed: Vault key was legacy JWT but runtime injects sb_secret_ (updated Vault); SQL typo value-&gt;decrypted_secret on jobs 3/4/13; event-reminder had no service-key path + a no-auth-header mass-email hole (both fixed, commit 09d637d). Then built 2 guards: business-profile-reminder 14-day cooldown via contact_activity + internal-account exclusion (503548c); guest-event-match at-capacity exclusion (d722800). Both jobs 2 &amp; 10 re-enabled. All 10 cron jobs now active + healthy.</t>
-        </is>
-      </c>
-      <c r="C151" s="23" t="inlineStr">
-        <is>
-          <t>All confirmed 200 on live ticks. Guards dry-run/logic verified. WATCH: first live ticks of job 2 (14:00 UTC every 2 days) + job 10 (13:00 UTC daily) — read-only confirm right people emailed.</t>
-        </is>
-      </c>
-      <c r="D151" s="24" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E151" s="23" t="inlineStr">
-        <is>
-          <t>Commits 09d637d, 503548c, d722800 + Vault + SQL. event-reminder security hole closed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="57.45" customFormat="1" customHeight="1" s="2">
-      <c r="A152" s="16" t="inlineStr">
-        <is>
-          <t>[DONE] Sentry error monitoring — live + verified in prod</t>
-        </is>
-      </c>
-      <c r="B152" s="23" t="inlineStr">
-        <is>
-          <t>@sentry/nextjs wired (client+server+API+global-error), CSP allowance, instrumentation moved into src/ (Next ignores root-level with a src/ dir), DSN + source-map auth token in Vercel, /admin/sentry page activated. Prod capture VERIFIED (smoke-test error landed in feed).</t>
-        </is>
-      </c>
-      <c r="C152" s="23" t="inlineStr">
-        <is>
-          <t>Verified. WATCH: confirm Sentry project SLUG is exactly '704-collective' in a Vercel build log (source-map upload) — if wrong, traces stay minified (one-word fix).</t>
-        </is>
-      </c>
-      <c r="D152" s="24" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E152" s="23" t="inlineStr">
-        <is>
-          <t>Commits 417fb37/d779885/5d12aac/b437166. The safety net — Stage 1 complete.</t>
         </is>
       </c>
     </row>
     <row r="153" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A153" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Josh Ahart full removal (exit workstream)</t>
+          <t>[DONE] Security: dropped anon-readable active_members view + locked event_participants_view</t>
         </is>
       </c>
       <c r="B153" s="23" t="inlineStr">
         <is>
-          <t>De-privileged (super_admin-&gt;lead), permanent ban, all 8 sessions + 64 tokens killed, profile deactivated, ambassador row disabled, removed from public /about page (0cc8c66), 2 dormant test dupe accounts hard-deleted. Stripe sub cancelled + Connect account rejected (Adam, dashboard). Platform passwords rotated (Adam).</t>
+          <t>CRITICAL FIX Jul 9: active_members and event_participants_view were SECURITY DEFINER views with ALL privileges granted to anon — an unauthenticated internet caller could read every member's email/phone/Stripe customer ID + all attendee contact info, AND active_members (auto-updatable single-table view) exposed an anon WRITE path into profiles. active_members had ZERO callers -&gt; DROPPED. event_participants_view -&gt; security_invoker=true + REVOKE anon/authenticated (sole caller send-campaign uses service-role, unaffected). member_counts left as-is (intentional).</t>
         </is>
       </c>
       <c r="C153" s="23" t="inlineStr">
         <is>
-          <t>Verified: role=lead, 0 sessions/tokens, banned. Public site scrubbed. Dashboard-member removal confirmed by Adam.</t>
+          <t>DONE via SQL. Verified from OUTSIDE with anon key: active_members=404, event_participants_view=401 permission denied. No rows leaked. send-campaign confirmed still works.</t>
         </is>
       </c>
       <c r="D153" s="24" t="inlineStr">
@@ -4125,24 +4036,24 @@
       </c>
       <c r="E153" s="23" t="inlineStr">
         <is>
-          <t>NOT on the build sheet — exit workstream. Recorded here for completeness.</t>
+          <t>Biggest find of the session. Was disguised as a 'review Security Definer flags' tracker row.</t>
         </is>
       </c>
     </row>
     <row r="154" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A154" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Member status batch (Jul 9)</t>
+          <t>[DONE] Nine-job cron auth resurrection + 2 guards, all 10 jobs healthy</t>
         </is>
       </c>
       <c r="B154" s="23" t="inlineStr">
         <is>
-          <t>Nicholas Stathopoulos + Robert Villante -&gt; non_member/inactive/override off/lead (Nick admin revoked + sessions killed). Whitney Cleland + Brenna Dunne + Kaelah Torres -&gt; ERASED (auth+profile+people+credentials deleted; all comped, no Stripe to cancel). More status changes flagged as coming.</t>
+          <t>Full audit found NINE broken crons (sheet knew of 2). Fixed: Vault key was legacy JWT but runtime injects sb_secret_ (updated Vault); SQL typo value-&gt;decrypted_secret on jobs 3/4/13; event-reminder had no service-key path + a no-auth-header mass-email hole (both fixed, commit 09d637d). Then built 2 guards: business-profile-reminder 14-day cooldown via contact_activity + internal-account exclusion (503548c); guest-event-match at-capacity exclusion (d722800). Both jobs 2 &amp; 10 re-enabled. All 10 cron jobs now active + healthy.</t>
         </is>
       </c>
       <c r="C154" s="23" t="inlineStr">
         <is>
-          <t>All verified via SQL (zeros on erase). Read-first footprint audit confirmed safe (no owned content cascaded).</t>
+          <t>All confirmed 200 on live ticks. Guards dry-run/logic verified. WATCH: first live ticks of job 2 (14:00 UTC every 2 days) + job 10 (13:00 UTC daily) — read-only confirm right people emailed.</t>
         </is>
       </c>
       <c r="D154" s="24" t="inlineStr">
@@ -4152,24 +4063,24 @@
       </c>
       <c r="E154" s="23" t="inlineStr">
         <is>
-          <t>Adam noted more member changes coming next session.</t>
+          <t>Commits 09d637d, 503548c, d722800 + Vault + SQL. event-reminder security hole closed.</t>
         </is>
       </c>
     </row>
     <row r="155" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A155" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Business-event RSVP tier leak — closed + Annslee voided</t>
+          <t>[DONE] Sentry error monitoring — live + verified in prod</t>
         </is>
       </c>
       <c r="B155" s="23" t="inlineStr">
         <is>
-          <t>Social members could RSVP business-only events: create-member-rsvp never checked required_tier, and the mobile sticky RSVP bar bypassed the desktop gate. Fixed: server-side tier gate in the edge function (ff20ba9, admins exempt) + mobile CTA respects canRsvp (952fbb2). Annslee Bottoms' live breach credential on Jul-14 Business Member Meeting VOIDED. Past legacy breaches intentionally left (real attendance history).</t>
+          <t>@sentry/nextjs wired (client+server+API+global-error), CSP allowance, instrumentation moved into src/ (Next ignores root-level with a src/ dir), DSN + source-map auth token in Vercel, /admin/sentry page activated. Prod capture VERIFIED (smoke-test error landed in feed).</t>
         </is>
       </c>
       <c r="C155" s="23" t="inlineStr">
         <is>
-          <t>Verified: socialtest gets 403 'business members only' + red toast; direct-invoke blocked; Annslee active count on event = 0.</t>
+          <t>Verified. WATCH: confirm Sentry project SLUG is exactly '704-collective' in a Vercel build log (source-map upload) — if wrong, traces stay minified (one-word fix).</t>
         </is>
       </c>
       <c r="D155" s="24" t="inlineStr">
@@ -4179,24 +4090,24 @@
       </c>
       <c r="E155" s="23" t="inlineStr">
         <is>
-          <t>Commits ff20ba9, 952fbb2. Guest-side email opt-out gap noted -&gt; folds into unsubscribe policy work.</t>
+          <t>Commits 417fb37/d779885/5d12aac/b437166. The safety net — Stage 1 complete.</t>
         </is>
       </c>
     </row>
     <row r="156" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A156" s="16" t="inlineStr">
         <is>
-          <t>[DONE] Discussion edit/delete (comments+posts+photos) + admin always-on access</t>
+          <t>[DONE] Josh Ahart full removal (exit workstream)</t>
         </is>
       </c>
       <c r="B156" s="23" t="inlineStr">
         <is>
-          <t>Owners + admins can now edit/delete their own discussion comments (ecec3f8), posts (1e3adc1), and remove their own gallery photos (bcf746f); admins moderate anyone's. '(edited)' marker, soft-delete, silent removal. Also: admins now see the discussion link on any open event regardless of RSVP (583b343 — backend was already admin-exempt; was a missing-link discovery bug). Feed/comment/DM URL linkify (561403e).</t>
+          <t>De-privileged (super_admin-&gt;lead), permanent ban, all 8 sessions + 64 tokens killed, profile deactivated, ambassador row disabled, removed from public /about page (0cc8c66), 2 dormant test dupe accounts hard-deleted. Stripe sub cancelled + Connect account rejected (Adam, dashboard). Platform passwords rotated (Adam).</t>
         </is>
       </c>
       <c r="C156" s="23" t="inlineStr">
         <is>
-          <t>All browser-tested desktop+mobile. Backend RLS already permitted; these were frontend gaps.</t>
+          <t>Verified: role=lead, 0 sessions/tokens, banned. Public site scrubbed. Dashboard-member removal confirmed by Adam.</t>
         </is>
       </c>
       <c r="D156" s="24" t="inlineStr">
@@ -4206,149 +4117,109 @@
       </c>
       <c r="E156" s="23" t="inlineStr">
         <is>
-          <t>5 commits. Discussion feature now fully moderatable.</t>
+          <t>NOT on the build sheet — exit workstream. Recorded here for completeness.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="16" t="inlineStr">
         <is>
+          <t>[DONE] Member status batch (Jul 9)</t>
+        </is>
+      </c>
+      <c r="B157" s="23" t="inlineStr">
+        <is>
+          <t>Nicholas Stathopoulos + Robert Villante -&gt; non_member/inactive/override off/lead (Nick admin revoked + sessions killed). Whitney Cleland + Brenna Dunne + Kaelah Torres -&gt; ERASED (auth+profile+people+credentials deleted; all comped, no Stripe to cancel). More status changes flagged as coming.</t>
+        </is>
+      </c>
+      <c r="C157" s="23" t="inlineStr">
+        <is>
+          <t>All verified via SQL (zeros on erase). Read-first footprint audit confirmed safe (no owned content cascaded).</t>
+        </is>
+      </c>
+      <c r="D157" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E157" s="23" t="inlineStr">
+        <is>
+          <t>Adam noted more member changes coming next session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="16" t="inlineStr">
+        <is>
+          <t>[DONE] Business-event RSVP tier leak — closed + Annslee voided</t>
+        </is>
+      </c>
+      <c r="B158" s="23" t="inlineStr">
+        <is>
+          <t>Social members could RSVP business-only events: create-member-rsvp never checked required_tier, and the mobile sticky RSVP bar bypassed the desktop gate. Fixed: server-side tier gate in the edge function (ff20ba9, admins exempt) + mobile CTA respects canRsvp (952fbb2). Annslee Bottoms' live breach credential on Jul-14 Business Member Meeting VOIDED. Past legacy breaches intentionally left (real attendance history).</t>
+        </is>
+      </c>
+      <c r="C158" s="23" t="inlineStr">
+        <is>
+          <t>Verified: socialtest gets 403 'business members only' + red toast; direct-invoke blocked; Annslee active count on event = 0.</t>
+        </is>
+      </c>
+      <c r="D158" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E158" s="23" t="inlineStr">
+        <is>
+          <t>Commits ff20ba9, 952fbb2. Guest-side email opt-out gap noted -&gt; folds into unsubscribe policy work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="16" t="inlineStr">
+        <is>
+          <t>[DONE] Discussion edit/delete (comments+posts+photos) + admin always-on access</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="16" t="inlineStr">
+        <is>
           <t>[DONE] Small fixes: hubs 404, week_label, dead components, partners 400, org_settings, last_attended</t>
         </is>
       </c>
-      <c r="B157" s="23" t="inlineStr">
-        <is>
-          <t>hubs preview widget queried non-existent 'business_hubs' -&gt; fixed to 'hubs' (a00cc50, restored a silently-broken business-tier feature). ambassador-payout phantom week_label column removed (1f46e88). 3 dead admin components deleted, 1376 lines (306efa4). partners 400 fixed via column aliasing (d95a337, latent partner-disappearing bug). organization_settings tracker row was STALE (schema fine, closed). last_attended already built+firing -&gt; backfilled 17 pre-trigger rows, closed.</t>
-        </is>
-      </c>
-      <c r="C157" s="23" t="inlineStr">
-        <is>
-          <t>All tsc+browser verified. org_settings &amp; last_attended were already-done rows.</t>
-        </is>
-      </c>
-      <c r="D157" s="24" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E157" s="23" t="inlineStr">
-        <is>
-          <t>Commits a00cc50, 1f46e88, 306efa4, d95a337 + 2 SQL closes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="25" t="inlineStr">
+    </row>
+    <row r="161">
+      <c r="A161" s="25" t="inlineStr">
         <is>
           <t>PHASE 2  ·  MAJOR BUILDS (each gets its own detailed scope before build)</t>
         </is>
       </c>
-      <c r="B158" s="29" t="n"/>
-      <c r="C158" s="29" t="n"/>
-      <c r="D158" s="29" t="n"/>
-      <c r="E158" s="30" t="n"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="4" t="inlineStr">
+      <c r="B161" s="29" t="n"/>
+      <c r="C161" s="29" t="n"/>
+      <c r="D161" s="29" t="n"/>
+      <c r="E161" s="30" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="4" t="inlineStr">
         <is>
           <t>MAJOR BUILDS — EACH GETS ITS OWN DETAILED SCOPE BEFORE BUILD   ·   7 items</t>
         </is>
       </c>
-      <c r="B159" s="29" t="n"/>
-      <c r="C159" s="29" t="n"/>
-      <c r="D159" s="29" t="n"/>
-      <c r="E159" s="30" t="n"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="7" t="inlineStr">
-        <is>
-          <t>CRM system</t>
-        </is>
-      </c>
-      <c r="B160" s="8" t="inlineStr">
-        <is>
-          <t>Full customer-relationship system built ON the merged person record: 360-degree member view, segments/audiences, lifecycle tracking. The internal data model IS the CRM (not a re-introduced external tool).</t>
-        </is>
-      </c>
-      <c r="C160" s="8" t="inlineStr">
-        <is>
-          <t>Own detailed scope before build.</t>
-        </is>
-      </c>
-      <c r="D160" s="26" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="E160" s="8" t="inlineStr">
-        <is>
-          <t>Built on the canonical person record from Phase 1. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag (carve-out keeps /admin/crm/campaigns live for the newsletter).</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="7" t="inlineStr">
-        <is>
-          <t>Preferred Business Network</t>
-        </is>
-      </c>
-      <c r="B161" s="8" t="inlineStr">
-        <is>
-          <t>New paid product: vetted local-business listings, $300/mo to be listed. Lives in the portal first, public domains later. Includes the internal 'Seats' system. Social members browse this to find services.</t>
-        </is>
-      </c>
-      <c r="C161" s="8" t="inlineStr">
-        <is>
-          <t>Own detailed scope before build.</t>
-        </is>
-      </c>
-      <c r="D161" s="26" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="E161" s="8" t="inlineStr">
-        <is>
-          <t>Plugs into The Network surface built in Phase 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="7" t="inlineStr">
-        <is>
-          <t>Partner Portal (audit, then repurpose or remove)</t>
-        </is>
-      </c>
-      <c r="B162" s="8" t="inlineStr">
-        <is>
-          <t>An existing, mostly-built partner portal of unclear purpose. Audit it, then either repurpose it as the Preferred Business Network management surface or remove it. Frozen until then.</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
-        <is>
-          <t>Own detailed scope before build.</t>
-        </is>
-      </c>
-      <c r="D162" s="26" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="E162" s="8" t="inlineStr">
-        <is>
-          <t>Audit first; likely becomes the Preferred Business Network management surface. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag.</t>
-        </is>
-      </c>
+      <c r="B162" s="29" t="n"/>
+      <c r="C162" s="29" t="n"/>
+      <c r="D162" s="29" t="n"/>
+      <c r="E162" s="30" t="n"/>
     </row>
     <row r="163" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A163" s="7" t="inlineStr">
         <is>
-          <t>Task center for admins (lite project tool)</t>
+          <t>CRM system</t>
         </is>
       </c>
       <c r="B163" s="8" t="inlineStr">
         <is>
-          <t>A super-light ClickUp-style task center for admins/super-admins: create, assign, track tasks.</t>
+          <t>Full customer-relationship system built ON the merged person record: 360-degree member view, segments/audiences, lifecycle tracking. The internal data model IS the CRM (not a re-introduced external tool).</t>
         </is>
       </c>
       <c r="C163" s="8" t="inlineStr">
@@ -4363,19 +4234,19 @@
       </c>
       <c r="E163" s="8" t="inlineStr">
         <is>
-          <t>Lite task assignment + tracking for admin / super-admin.</t>
+          <t>Built on the canonical person record from Phase 1. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag (carve-out keeps /admin/crm/campaigns live for the newsletter).</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
         <is>
-          <t>Shared email inbox view for super-admins</t>
+          <t>Preferred Business Network</t>
         </is>
       </c>
       <c r="B164" s="8" t="inlineStr">
         <is>
-          <t>A shared inbox view so super-admins can see the team email (hello@) in one place.</t>
+          <t>New paid product: vetted local-business listings, $300/mo to be listed. Lives in the portal first, public domains later. Includes the internal 'Seats' system. Social members browse this to find services.</t>
         </is>
       </c>
       <c r="C164" s="8" t="inlineStr">
@@ -4390,26 +4261,46 @@
       </c>
       <c r="E164" s="8" t="inlineStr">
         <is>
-          <t>Super-admin visibility into hello@.</t>
+          <t>Plugs into The Network surface built in Phase 1.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
         <is>
-          <t>Corporate / bulk-sales floating-seats portal</t>
+          <t>Partner Portal (audit, then repurpose or remove)</t>
+        </is>
+      </c>
+      <c r="B165" s="8" t="inlineStr">
+        <is>
+          <t>An existing, mostly-built partner portal of unclear purpose. Audit it, then either repurpose it as the Preferred Business Network management surface or remove it. Frozen until then.</t>
+        </is>
+      </c>
+      <c r="C165" s="8" t="inlineStr">
+        <is>
+          <t>Own detailed scope before build.</t>
+        </is>
+      </c>
+      <c r="D165" s="26" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="E165" s="8" t="inlineStr">
+        <is>
+          <t>Audit first; likely becomes the Preferred Business Network management surface. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag.</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
         <is>
-          <t>Full mobile app</t>
+          <t>Task center for admins (lite project tool)</t>
         </is>
       </c>
       <c r="B166" s="8" t="inlineStr">
         <is>
-          <t>A full native mobile application. The largest Phase 2 build.</t>
+          <t>A super-light ClickUp-style task center for admins/super-admins: create, assign, track tasks.</t>
         </is>
       </c>
       <c r="C166" s="8" t="inlineStr">
@@ -4424,116 +4315,100 @@
       </c>
       <c r="E166" s="8" t="inlineStr">
         <is>
-          <t>The final, largest Phase 2 effort.</t>
+          <t>Lite task assignment + tracking for admin / super-admin.</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="4" t="inlineStr">
-        <is>
-          <t>OPEN WATCH ITEMS — ADDED 2026-07-19   ·   8 items</t>
-        </is>
-      </c>
-      <c r="B167" s="29" t="n"/>
-      <c r="C167" s="29" t="n"/>
-      <c r="D167" s="29" t="n"/>
-      <c r="E167" s="30" t="n"/>
+      <c r="A167" s="7" t="inlineStr">
+        <is>
+          <t>Shared email inbox view for super-admins</t>
+        </is>
+      </c>
+      <c r="B167" s="8" t="inlineStr">
+        <is>
+          <t>A shared inbox view so super-admins can see the team email (hello@) in one place.</t>
+        </is>
+      </c>
+      <c r="C167" s="8" t="inlineStr">
+        <is>
+          <t>Own detailed scope before build.</t>
+        </is>
+      </c>
+      <c r="D167" s="26" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="E167" s="8" t="inlineStr">
+        <is>
+          <t>Super-admin visibility into hello@.</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
         <is>
-          <t>Stage 5 Wave 4 - classify the ~204 guest/lead reverse-orphan profiles</t>
-        </is>
-      </c>
-      <c r="B168" s="8" t="inlineStr">
-        <is>
-          <t>Waves 1-3 linked/minted the clear identity cases; the residual ~204 profiles are guests or leads that never became members and must be classified, not minted as members.</t>
-        </is>
-      </c>
-      <c r="C168" s="8" t="inlineStr">
-        <is>
-          <t>Decide the guest-vs-lead-vs-skip rule; mint people rows with the correct non-active member_status; reuse the Wave 3 additive/reversible pattern (metadata.created_by). Rehearse on develop first.</t>
-        </is>
-      </c>
-      <c r="D168" s="9" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E168" s="8" t="inlineStr">
-        <is>
-          <t>Waves 1-3 applied to prod. Wave 4 is the guest/lead bucket - needs a classification rule before any minting.</t>
-        </is>
-      </c>
+          <t>Corporate / bulk-sales floating-seats portal</t>
+        </is>
+      </c>
+      <c r="B168" s="29" t="n"/>
+      <c r="C168" s="29" t="n"/>
+      <c r="D168" s="29" t="n"/>
+      <c r="E168" s="30" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
         <is>
-          <t>Refill the Vercel NEXT_PUBLIC_TURNSTILE_SITE_KEY value (hardcode fallback active)</t>
+          <t>Full mobile app</t>
         </is>
       </c>
       <c r="B169" s="8" t="inlineStr">
         <is>
-          <t>The prod env var was set to an empty string, which made the Turnstile widget render nothing and locked members out during an incident. A hardcoded public site-key fallback in TurnstileWidget.tsx currently masks the missing value.</t>
+          <t>A full native mobile application. The largest Phase 2 build.</t>
         </is>
       </c>
       <c r="C169" s="8" t="inlineStr">
         <is>
-          <t>Set the real public site key for NEXT_PUBLIC_TURNSTILE_SITE_KEY in Vercel (production), redeploy, confirm the widget renders from the env var, then optionally remove the hardcoded fallback.</t>
-        </is>
-      </c>
-      <c r="D169" s="9" t="inlineStr">
-        <is>
-          <t>Build</t>
+          <t>Own detailed scope before build.</t>
+        </is>
+      </c>
+      <c r="D169" s="26" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="E169" s="8" t="inlineStr">
         <is>
-          <t>Public site key (safe): 0x4AAAAAAD3gqCivsYyImeUH. Fallback keeps login working today; refill so config isn't hidden in code.</t>
+          <t>The final, largest Phase 2 effort.</t>
         </is>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="7" t="inlineStr">
-        <is>
-          <t>Resolve the capacity-trigger split-brain (tickets vs attendance_credentials counting)</t>
-        </is>
-      </c>
-      <c r="B170" s="8" t="inlineStr">
-        <is>
-          <t>Event capacity is enforced by triggers on two tables (attendance_credentials and legacy tickets) that count independently, so the seated count can disagree depending on the write path.</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
-          <t>Pick one source of truth (attendance_credentials); make both trigger families count consistently, or retire the legacy tickets capacity path once tickets is fully retired. Coordinates with 'Finish retiring the old ticket tables'.</t>
-        </is>
-      </c>
-      <c r="D170" s="9" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E170" s="8" t="inlineStr">
-        <is>
-          <t>The admin_override bypass now spans both trigger families; the underlying counting split remains until tickets is retired.</t>
-        </is>
-      </c>
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>OPEN WATCH ITEMS — ADDED 2026-07-19   ·   8 items</t>
+        </is>
+      </c>
+      <c r="B170" s="29" t="n"/>
+      <c r="C170" s="29" t="n"/>
+      <c r="D170" s="29" t="n"/>
+      <c r="E170" s="30" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
         <is>
-          <t>Q6 canceled-but-paying tripwire (canceled-drift detection)</t>
+          <t>Stage 5 Wave 4 - classify the ~204 guest/lead reverse-orphan profiles</t>
         </is>
       </c>
       <c r="B171" s="8" t="inlineStr">
         <is>
-          <t>Members whose app status shows canceled while Stripe still bills them (or the inverse) - a billing/status drift that should trip an alert instead of going silent.</t>
+          <t>Waves 1-3 linked/minted the clear identity cases; the residual ~204 profiles are guests or leads that never became members and must be classified, not minted as members.</t>
         </is>
       </c>
       <c r="C171" s="8" t="inlineStr">
         <is>
-          <t>Add a scheduled check comparing profiles.subscription_status vs the live Stripe subscription state; alert on canceled-in-app-but-active-in-Stripe and the inverse.</t>
+          <t>Decide the guest-vs-lead-vs-skip rule; mint people rows with the correct non-active member_status; reuse the Wave 3 additive/reversible pattern (metadata.created_by). Rehearse on develop first.</t>
         </is>
       </c>
       <c r="D171" s="9" t="inlineStr">
@@ -4543,24 +4418,24 @@
       </c>
       <c r="E171" s="8" t="inlineStr">
         <is>
-          <t>The develop seed carries a canceled-drift (Q6) dummy for rehearsal. Folds into the DB/Stripe drift watch + admin health dashboard.</t>
+          <t>Waves 1-3 applied to prod. Wave 4 is the guest/lead bucket - needs a classification rule before any minting.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
         <is>
-          <t>Delete the stray Stripe Connect account</t>
+          <t>Refill the Vercel NEXT_PUBLIC_TURNSTILE_SITE_KEY value (hardcode fallback active)</t>
         </is>
       </c>
       <c r="B172" s="8" t="inlineStr">
         <is>
-          <t>A leftover Stripe Connect (Express) account from the ambassador / exit workstream needs removing so it doesn't linger.</t>
+          <t>The prod env var was set to an empty string, which made the Turnstile widget render nothing and locked members out during an incident. A hardcoded public site-key fallback in TurnstileWidget.tsx currently masks the missing value.</t>
         </is>
       </c>
       <c r="C172" s="8" t="inlineStr">
         <is>
-          <t>Confirm the account has no pending balance or payouts, then delete/reject it in the Stripe dashboard. Owner task.</t>
+          <t>Set the real public site key for NEXT_PUBLIC_TURNSTILE_SITE_KEY in Vercel (production), redeploy, confirm the widget renders from the env var, then optionally remove the hardcoded fallback.</t>
         </is>
       </c>
       <c r="D172" s="9" t="inlineStr">
@@ -4570,24 +4445,24 @@
       </c>
       <c r="E172" s="8" t="inlineStr">
         <is>
-          <t>Cleanup item from the ambassador / Connect work; low blast radius.</t>
+          <t>Public site key (safe): 0x4AAAAAAD3gqCivsYyImeUH. Fallback keeps login working today; refill so config isn't hidden in code.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
         <is>
-          <t>ManyChat - disconnect the Instagram-side integration</t>
+          <t>Resolve the capacity-trigger split-brain (tickets vs attendance_credentials counting)</t>
         </is>
       </c>
       <c r="B173" s="8" t="inlineStr">
         <is>
-          <t>The IG-side ManyChat connection needs to be disconnected / cleaned up. This is teardown of the current Instagram link, separate from the auto-DM build.</t>
+          <t>Event capacity is enforced by triggers on two tables (attendance_credentials and legacy tickets) that count independently, so the seated count can disagree depending on the write path.</t>
         </is>
       </c>
       <c r="C173" s="8" t="inlineStr">
         <is>
-          <t>Disconnect the Instagram account from ManyChat (owner task in ManyChat / Meta); confirm no active automations still reference it.</t>
+          <t>Pick one source of truth (attendance_credentials); make both trigger families count consistently, or retire the legacy tickets capacity path once tickets is fully retired. Coordinates with 'Finish retiring the old ticket tables'.</t>
         </is>
       </c>
       <c r="D173" s="9" t="inlineStr">
@@ -4597,471 +4472,536 @@
       </c>
       <c r="E173" s="8" t="inlineStr">
         <is>
-          <t>Distinct from the 'Instagram comment auto-DM (ManyChat)' build row above - that row stays as-is.</t>
+          <t>The admin_override bypass now spans both trigger families; the underlying counting split remains until tickets is retired.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
         <is>
-          <t>DB / Stripe drift watch items</t>
+          <t>Q6 canceled-but-paying tripwire (canceled-drift detection)</t>
         </is>
       </c>
       <c r="B174" s="8" t="inlineStr">
         <is>
-          <t>Ongoing watch on the places where the database and Stripe can drift out of sync: subscription statuses, customer email on email-change, retired legacy prices, orphaned Stripe customers.</t>
+          <t>Members whose app status shows canceled while Stripe still bills them (or the inverse) - a billing/status drift that should trip an alert instead of going silent.</t>
         </is>
       </c>
       <c r="C174" s="8" t="inlineStr">
         <is>
-          <t>Track and periodically reconcile; surface on the admin health dashboard. Pairs with the Q6 tripwire and the 'email change keeps Stripe billing in sync' verify.</t>
+          <t>Add a scheduled check comparing profiles.subscription_status vs the live Stripe subscription state; alert on canceled-in-app-but-active-in-Stripe and the inverse.</t>
         </is>
       </c>
       <c r="D174" s="9" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="E174" s="8" t="inlineStr">
         <is>
-          <t>Umbrella watch item; individual drifts get their own rows as they surface.</t>
+          <t>The develop seed carries a canceled-drift (Q6) dummy for rehearsal. Folds into the DB/Stripe drift watch + admin health dashboard.</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
         <is>
+          <t>Delete the stray Stripe Connect account</t>
+        </is>
+      </c>
+      <c r="B175" s="8" t="inlineStr">
+        <is>
+          <t>A leftover Stripe Connect (Express) account from the ambassador / exit workstream needs removing so it doesn't linger.</t>
+        </is>
+      </c>
+      <c r="C175" s="8" t="inlineStr">
+        <is>
+          <t>Confirm the account has no pending balance or payouts, then delete/reject it in the Stripe dashboard. Owner task.</t>
+        </is>
+      </c>
+      <c r="D175" s="9" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E175" s="8" t="inlineStr">
+        <is>
+          <t>Cleanup item from the ambassador / Connect work; low blast radius.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="7" t="inlineStr">
+        <is>
+          <t>ManyChat - disconnect the Instagram-side integration</t>
+        </is>
+      </c>
+      <c r="B176" s="8" t="inlineStr">
+        <is>
+          <t>The IG-side ManyChat connection needs to be disconnected / cleaned up. This is teardown of the current Instagram link, separate from the auto-DM build.</t>
+        </is>
+      </c>
+      <c r="C176" s="8" t="inlineStr">
+        <is>
+          <t>Disconnect the Instagram account from ManyChat (owner task in ManyChat / Meta); confirm no active automations still reference it.</t>
+        </is>
+      </c>
+      <c r="D176" s="9" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E176" s="8" t="inlineStr">
+        <is>
+          <t>Distinct from the 'Instagram comment auto-DM (ManyChat)' build row above - that row stays as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="7" t="inlineStr">
+        <is>
+          <t>DB / Stripe drift watch items</t>
+        </is>
+      </c>
+      <c r="B177" s="29" t="n"/>
+      <c r="C177" s="29" t="n"/>
+      <c r="D177" s="29" t="n"/>
+      <c r="E177" s="30" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="7" t="inlineStr">
+        <is>
           <t>Waitlist claim links - monitor first real-world use</t>
         </is>
       </c>
-      <c r="B175" s="8" t="inlineStr">
+      <c r="B178" s="8" t="inlineStr">
         <is>
           <t>Cancel frees a seat -&gt; the first waitlister is emailed a 24h claim link -&gt; they claim it. Rehearsed as a full matrix on develop and shipped to prod; needs a read-only confirm on its first genuine use.</t>
         </is>
       </c>
-      <c r="C175" s="8" t="inlineStr">
+      <c r="C178" s="8" t="inlineStr">
         <is>
           <t>On the next real cancellation that frees a seat on a full, waitlisted event, confirm: notified_at/expires_at stamped, the email sent, the claimant claimed (member_rsvp with metadata source=waitlist_claim), and the waitlist row deleted.</t>
         </is>
       </c>
-      <c r="D175" s="9" t="inlineStr">
+      <c r="D178" s="9" t="inlineStr">
         <is>
           <t>Verify</t>
         </is>
       </c>
-      <c r="E175" s="8" t="inlineStr">
+      <c r="E178" s="8" t="inlineStr">
         <is>
           <t>Shipped 2026-07-19. Zero-cost proof on first real use, like the Remove &amp; Refund WAIT-mode row.</t>
         </is>
       </c>
     </row>
-    <row r="176">
-      <c r="A176" s="27" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="27" t="inlineStr">
         <is>
           <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="28" t="inlineStr">
-        <is>
-          <t>Billing views: admin billing panel + member price/renewal display</t>
-        </is>
-      </c>
-      <c r="B177" s="28" t="inlineStr">
-        <is>
-          <t>Admin contact billing panel + member-facing price/renewal display. Three new profile columns (comp_reason, external_paid_through, external_payment_note) are live on both DBs; the UI/code build is in flight.</t>
-        </is>
-      </c>
-      <c r="C177" s="28" t="inlineStr">
-        <is>
-          <t>Extend admin contact detail with live Stripe billing; surface price/renewal/discount on member settings; wire the three new profile columns into admin editors.</t>
-        </is>
-      </c>
-      <c r="D177" s="28" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
-        </is>
-      </c>
-      <c r="E177" s="28" t="inlineStr">
-        <is>
-          <t>Columns live both DBs; code build in flight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="28" t="inlineStr">
-        <is>
-          <t>Report builder: admin/super_admin any-filter member/payment reports</t>
-        </is>
-      </c>
-      <c r="B178" s="28" t="inlineStr">
-        <is>
-          <t>Admin/super_admin reporting with arbitrary filters over members and payments. Data-cleanup prerequisite is DONE; build after billing views.</t>
-        </is>
-      </c>
-      <c r="C178" s="28" t="inlineStr">
-        <is>
-          <t>Build after billing views lands. Admin/super_admin only; any-filter member + payment reports.</t>
-        </is>
-      </c>
-      <c r="D178" s="28" t="inlineStr">
-        <is>
-          <t>QUEUED-BACKLOGGED</t>
-        </is>
-      </c>
-      <c r="E178" s="28" t="inlineStr">
-        <is>
-          <t>v1 proposal complete and approved-in-principle (DB-only cut, 3 entities, column picker, CSV export, 4 presets, server-paginated, ~7 files); resume at build sign-off. Cheap adds discussed: ambassador-referred, price tier, cancel reasons.</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="28" t="inlineStr">
-        <is>
-          <t>Business comp invite flow: welcome template + admin invite tool</t>
-        </is>
-      </c>
-      <c r="B179" s="28" t="inlineStr">
-        <is>
-          <t>Welcome email template plus an admin tool to invite a business member (comp path).</t>
-        </is>
-      </c>
-      <c r="C179" s="28" t="inlineStr">
-        <is>
-          <t>Blocked on Adam: invitee list + design answers. Then template + admin invite UI.</t>
-        </is>
-      </c>
-      <c r="D179" s="28" t="inlineStr">
-        <is>
-          <t>WAITING ON ADAM: list + design answers</t>
-        </is>
-      </c>
-      <c r="E179" s="28" t="inlineStr">
-        <is>
-          <t>Needs invitee list + design answers from Adam.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="28" t="inlineStr">
         <is>
-          <t>Admin 'Invite comp member' button - form (name, company, email, phone, comp note), creates comp'd account + sends welcome email, note auto-attached to billing view (member + admin); v1 invite flow built without UI, button is the addon</t>
+          <t>Billing views: admin billing panel + member price/renewal display</t>
         </is>
       </c>
       <c r="B180" s="28" t="inlineStr">
         <is>
-          <t>Admin UI button/form to invite a complimentary business member: name, company, email, phone, and comp note. Creates the comp'd account, sends the welcome email, and attaches the note to the billing view for both member and admin.</t>
+          <t>Admin contact billing panel + member-facing price/renewal display. Three new profile columns (comp_reason, external_paid_through, external_payment_note) are live on both DBs; the UI/code build is in flight.</t>
         </is>
       </c>
       <c r="C180" s="28" t="inlineStr">
         <is>
-          <t>Addon after v1 invite flow (API/ops path without UI). Build the Invite comp member button + form once the headless invite path exists.</t>
+          <t>Extend admin contact detail with live Stripe billing; surface price/renewal/discount on member settings; wire the three new profile columns into admin editors.</t>
         </is>
       </c>
       <c r="D180" s="28" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="E180" s="28" t="inlineStr">
         <is>
-          <t>v1 invite flow built without UI; this button is the future addon.</t>
+          <t>Columns live both DBs; code build in flight.</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="28" t="inlineStr">
         <is>
-          <t>Mike Perez: account cleanup + re-join link at $150 founding</t>
+          <t>Report builder: admin/super_admin any-filter member/payment reports</t>
         </is>
       </c>
       <c r="B181" s="28" t="inlineStr">
         <is>
-          <t>After Adam's conversation: clean up Mike's canceled/failed-billing account and send a founding-rate $150 re-join link.</t>
+          <t>Admin/super_admin reporting with arbitrary filters over members and payments. Data-cleanup prerequisite is DONE; build after billing views.</t>
         </is>
       </c>
       <c r="C181" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM conversation first. Then cleanup + founding $150 checkout/re-join link.</t>
+          <t>Build after billing views lands. Admin/super_admin only; any-filter member + payment reports.</t>
         </is>
       </c>
       <c r="D181" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: conversation first</t>
+          <t>QUEUED-BACKLOGGED</t>
         </is>
       </c>
       <c r="E181" s="28" t="inlineStr">
         <is>
-          <t>Founding $150; conversation first.</t>
+          <t>v1 proposal complete and approved-in-principle (DB-only cut, 3 entities, column picker, CSV export, 4 presets, server-paginated, ~7 files); resume at build sign-off. Cheap adds discussed: ambassador-referred, price tier, cancel reasons.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="28" t="inlineStr">
         <is>
-          <t>Zane Mackey comp_reason entry</t>
+          <t>Business comp invite flow: welcome template + admin invite tool</t>
         </is>
       </c>
       <c r="B182" s="28" t="inlineStr">
         <is>
-          <t>Record a one-phrase comp_reason on Zane Mackey's profile now that the column exists.</t>
+          <t>Welcome email template plus an admin tool to invite a business member (comp path).</t>
         </is>
       </c>
       <c r="C182" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: one phrase for comp_reason.</t>
+          <t>Blocked on Adam: invitee list + design answers. Then template + admin invite UI.</t>
         </is>
       </c>
       <c r="D182" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM: one phrase</t>
+          <t>WAITING ON ADAM: list + design answers</t>
         </is>
       </c>
       <c r="E182" s="28" t="inlineStr">
         <is>
-          <t>One phrase for comp_reason.</t>
+          <t>Needs invitee list + design answers from Adam.</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="28" t="inlineStr">
         <is>
-          <t>Zach Trusky renewal ~Nov/Dec 2026 — honored $1,034 annual</t>
+          <t>Admin 'Invite comp member' button - form (name, company, email, phone, comp note), creates comp'd account + sends welcome email, note auto-attached to billing view (member + admin); v1 invite flow built without UI, button is the addon</t>
         </is>
       </c>
       <c r="B183" s="28" t="inlineStr">
         <is>
-          <t>Zach's annual amount lives outside Stripe ($1,034 honored). Need reminder + collection path decision around Nov/Dec 2026.</t>
+          <t>Admin UI button/form to invite a complimentary business member: name, company, email, phone, and comp note. Creates the comp'd account, sends the welcome email, and attaches the note to the billing view for both member and admin.</t>
         </is>
       </c>
       <c r="C183" s="28" t="inlineStr">
         <is>
-          <t>Schedule reminder; decide collection path (manual invoice vs Stripe annual vs override).</t>
+          <t>Addon after v1 invite flow (API/ops path without UI). Build the Invite comp member button + form once the headless invite path exists.</t>
         </is>
       </c>
       <c r="D183" s="28" t="inlineStr">
         <is>
-          <t>SCHEDULED NOV 2026</t>
+          <t>QUEUED</t>
         </is>
       </c>
       <c r="E183" s="28" t="inlineStr">
         <is>
-          <t>Honored $1,034 annual; no Stripe customer today.</t>
+          <t>v1 invite flow built without UI; this button is the future addon.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="28" t="inlineStr">
         <is>
-          <t>Security: unknown third-party script (batatatech.com) on Glue Up admin pages</t>
+          <t>Mike Perez: account cleanup + re-join link at $150 founding</t>
         </is>
       </c>
       <c r="B184" s="28" t="inlineStr">
         <is>
-          <t>Unknown batatatech.com script firing on Glue Up admin pages — treat as extension/malware until proven otherwise; audit browsers + rotate passwords.</t>
+          <t>After Adam's conversation: clean up Mike's canceled/failed-billing account and send a founding-rate $150 re-join link.</t>
         </is>
       </c>
       <c r="C184" s="28" t="inlineStr">
         <is>
-          <t>Browser extension audit on machines that use Glue Up admin; password rotation for affected accounts.</t>
+          <t>WAITING ON ADAM conversation first. Then cleanup + founding $150 checkout/re-join link.</t>
         </is>
       </c>
       <c r="D184" s="28" t="inlineStr">
         <is>
-          <t>OPEN - Adam chrome://extensions only</t>
+          <t>WAITING ON ADAM: conversation first</t>
         </is>
       </c>
       <c r="E184" s="28" t="inlineStr">
         <is>
-          <t>repo confirmed clean 8/4 - scope is Adam's chrome://extensions only</t>
+          <t>Founding $150; conversation first.</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>[DONE] Promo system endstate 8/5</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
-        </is>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>Supersedes Stripe support ticket + ticket-checkout promo fast-follow (removed).</t>
-        </is>
-      </c>
-      <c r="D185" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="E185" t="inlineStr">
-        <is>
-          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
+      <c r="A185" s="28" t="inlineStr">
+        <is>
+          <t>Zane Mackey comp_reason entry</t>
+        </is>
+      </c>
+      <c r="B185" s="28" t="inlineStr">
+        <is>
+          <t>Record a one-phrase comp_reason on Zane Mackey's profile now that the column exists.</t>
+        </is>
+      </c>
+      <c r="C185" s="28" t="inlineStr">
+        <is>
+          <t>WAITING ON ADAM: one phrase for comp_reason.</t>
+        </is>
+      </c>
+      <c r="D185" s="28" t="inlineStr">
+        <is>
+          <t>WAITING ON ADAM: one phrase</t>
+        </is>
+      </c>
+      <c r="E185" s="28" t="inlineStr">
+        <is>
+          <t>One phrase for comp_reason.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="28" t="inlineStr">
         <is>
-          <t>Calendar update-leg verification via throwaway event</t>
+          <t>Zach Trusky renewal ~Nov/Dec 2026 — honored $1,034 annual</t>
         </is>
       </c>
       <c r="B186" s="28" t="inlineStr">
         <is>
-          <t>Verify that event-edit REQUEST invites actually move real calendars (ICS sequence / update leg) using a throwaway event.</t>
+          <t>Zach's annual amount lives outside Stripe ($1,034 honored). Need reminder + collection path decision around Nov/Dec 2026.</t>
         </is>
       </c>
       <c r="C186" s="28" t="inlineStr">
         <is>
-          <t>Create throwaway event, subscribe, edit, confirm calendars update; then delete throwaway.</t>
+          <t>Schedule reminder; decide collection path (manual invoice vs Stripe annual vs override).</t>
         </is>
       </c>
       <c r="D186" s="28" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>SCHEDULED NOV 2026</t>
         </is>
       </c>
       <c r="E186" s="28" t="inlineStr">
         <is>
-          <t>Throwaway event verification of REQUEST/update path.</t>
+          <t>Honored $1,034 annual; no Stripe customer today.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="28" t="inlineStr">
         <is>
-          <t>Resend click-tracking subdomain (DNS)</t>
+          <t>Security: unknown third-party script (batatatech.com) on Glue Up admin pages</t>
         </is>
       </c>
       <c r="B187" s="28" t="inlineStr">
         <is>
-          <t>Configure Resend click-tracking subdomain — Adam hands / DNS.</t>
+          <t>Unknown batatatech.com script firing on Glue Up admin pages — treat as extension/malware until proven otherwise; audit browsers + rotate passwords.</t>
         </is>
       </c>
       <c r="C187" s="28" t="inlineStr">
         <is>
-          <t>ADAM DNS: add Resend click-tracking subdomain CNAME + add Resend to SPF include (current SPF is Google-only). Confirmed missing 8/4.</t>
+          <t>Browser extension audit on machines that use Glue Up admin; password rotation for affected accounts.</t>
         </is>
       </c>
       <c r="D187" s="28" t="inlineStr">
         <is>
-          <t>ADAM - DNS</t>
+          <t>OPEN - Adam chrome://extensions only</t>
         </is>
       </c>
       <c r="E187" s="28" t="inlineStr">
         <is>
-          <t>confirmed NOT configured 8/4; also add Resend to SPF include during same DNS visit</t>
+          <t>repo confirmed clean 8/4 - scope is Adam's chrome://extensions only</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="28" t="inlineStr">
-        <is>
-          <t>/welcome checkout-flow coverage on develop</t>
-        </is>
-      </c>
-      <c r="B188" s="28" t="inlineStr">
-        <is>
-          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
-        </is>
-      </c>
-      <c r="C188" s="28" t="inlineStr">
-        <is>
-          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
-        </is>
-      </c>
-      <c r="D188" s="28" t="inlineStr">
-        <is>
-          <t>WATCH</t>
-        </is>
-      </c>
-      <c r="E188" s="28" t="inlineStr">
-        <is>
-          <t>Untested on develop; no Stripe checkout env.</t>
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>[DONE] Promo system endstate 8/5</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Supersedes Stripe support ticket + ticket-checkout promo fast-follow (removed).</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Promo endstate 8/5: server-side attach only, native box removed everywhere (create-checkout v64, create-ticket-checkout v65), Josh coupon shadow eliminated (2 free subs + 5 customers deleted, 3 abuse codes deactivated), 3 live promos + ambassador system verified.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="28" t="inlineStr">
         <is>
-          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
+          <t>Calendar update-leg verification via throwaway event</t>
         </is>
       </c>
       <c r="B189" s="28" t="inlineStr">
         <is>
-          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
+          <t>Verify that event-edit REQUEST invites actually move real calendars (ICS sequence / update leg) using a throwaway event.</t>
         </is>
       </c>
       <c r="C189" s="28" t="inlineStr">
         <is>
-          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
+          <t>Create throwaway event, subscribe, edit, confirm calendars update; then delete throwaway.</t>
         </is>
       </c>
       <c r="D189" s="28" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="E189" s="28" t="inlineStr">
         <is>
-          <t>Revisit in identity-bridge work.</t>
+          <t>Throwaway event verification of REQUEST/update path.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="28" t="inlineStr">
         <is>
-          <t>Retire the Google Sheets tracker path</t>
+          <t>Resend click-tracking subdomain (DNS)</t>
         </is>
       </c>
       <c r="B190" s="28" t="inlineStr">
         <is>
-          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
+          <t>Configure Resend click-tracking subdomain — Adam hands / DNS.</t>
         </is>
       </c>
       <c r="C190" s="28" t="inlineStr">
         <is>
-          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
+          <t>ADAM DNS: add Resend click-tracking subdomain CNAME + add Resend to SPF include (current SPF is Google-only). Confirmed missing 8/4.</t>
         </is>
       </c>
       <c r="D190" s="28" t="inlineStr">
         <is>
-          <t>QUEUED - cleanup</t>
+          <t>ADAM - DNS</t>
         </is>
       </c>
       <c r="E190" s="28" t="inlineStr">
         <is>
-          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
+          <t>confirmed NOT configured 8/4; also add Resend to SPF include during same DNS visit</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="28" t="inlineStr">
         <is>
+          <t>/welcome checkout-flow coverage on develop</t>
+        </is>
+      </c>
+      <c r="B191" s="28" t="inlineStr">
+        <is>
+          <t>/welcome checkout flow is still untested on develop (no Stripe checkout env there).</t>
+        </is>
+      </c>
+      <c r="C191" s="28" t="inlineStr">
+        <is>
+          <t>WATCH until develop has a Stripe checkout path; then cover /welcome end to end.</t>
+        </is>
+      </c>
+      <c r="D191" s="28" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="E191" s="28" t="inlineStr">
+        <is>
+          <t>Untested on develop; no Stripe checkout env.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="28" t="inlineStr">
+        <is>
+          <t>Stripe/DB drift duo: admin-delete-user + cleanup-business-members</t>
+        </is>
+      </c>
+      <c r="B192" s="28" t="inlineStr">
+        <is>
+          <t>admin-delete-user leaves unlinked Stripe subs; cleanup-business-members does not cancel in Stripe. Drift risk until identity-bridge work.</t>
+        </is>
+      </c>
+      <c r="C192" s="28" t="inlineStr">
+        <is>
+          <t>WATCH — revisit in identity-bridge work. Ensure deletes/cancels hit Stripe or leave an explicit orphan alert.</t>
+        </is>
+      </c>
+      <c r="D192" s="28" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="E192" s="28" t="inlineStr">
+        <is>
+          <t>Revisit in identity-bridge work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="28" t="inlineStr">
+        <is>
+          <t>Retire the Google Sheets tracker path</t>
+        </is>
+      </c>
+      <c r="B193" s="28" t="inlineStr">
+        <is>
+          <t>Repo xlsx under docs/ is the source of truth. Remove/deprecate update-backlog-sheet edge function, its secrets (BACKLOG_*, GOOGLE_SHEETS_SERVICE_ACCOUNT_JSON if unused elsewhere), and the delete/agent-auth additions.</t>
+        </is>
+      </c>
+      <c r="C193" s="28" t="inlineStr">
+        <is>
+          <t>QUEUED cleanup: delete the edge function (or stub 410), remove BACKLOG_AUTH_SECRET / BACKLOG_AGENT_SECRET / BACKLOG_SHEET_ID (and SA JSON if unused), scrub temp scripts.</t>
+        </is>
+      </c>
+      <c r="D193" s="28" t="inlineStr">
+        <is>
+          <t>QUEUED - cleanup</t>
+        </is>
+      </c>
+      <c r="E193" s="28" t="inlineStr">
+        <is>
+          <t>debug_env already stripped 2026-08-03; full retirement queued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="28" t="inlineStr">
+        <is>
           <t>Admin card PATCH date normalization - external dates should save as noon UTC to avoid timezone off-by-one (Zach precedent)</t>
         </is>
       </c>
-      <c r="B191" s="28" t="inlineStr">
+      <c r="B194" s="28" t="inlineStr">
         <is>
           <t>external_paid_through saved as midnight UTC displays as prior calendar day in US Eastern (Zach showed Nov 30 instead of Dec 1). Admin billing PATCH should normalize date-only inputs to noon UTC.</t>
         </is>
       </c>
-      <c r="C191" s="28" t="inlineStr">
+      <c r="C194" s="28" t="inlineStr">
         <is>
           <t>In PATCH /api/admin/members/[id]/billing (and any similar writers), coerce external_paid_through date-only values to YYYY-MM-DDT12:00:00.000Z before save. SMALL.</t>
         </is>
       </c>
-      <c r="D191" s="28" t="inlineStr">
+      <c r="D194" s="28" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="E191" s="28" t="inlineStr">
+      <c r="E194" s="28" t="inlineStr">
         <is>
           <t>SMALL/OPEN. Precedent: Zach Trusky external_paid_through 2026-12-01T00:00:00Z → Nov 30 in America/New_York.</t>
         </is>

</xml_diff>

<commit_message>
fix: tracker - realign merged header ranges drifted by row inserts
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -2052,26 +2052,6 @@
           <t>Add a deploy pipeline so changes go live safely</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>DB/function changes are pushed by hand today — the root cause of code/live drift. Locked: hand-patching stops once this lands (with a written emergency lane).</t>
-        </is>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>GitHub Actions: merge to main -&gt; db push + functions deploy. Needs 3 repo secrets.</t>
-        </is>
-      </c>
-      <c r="D60" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Once in, hand-patching stops; needed before two people touch production in parallel.</t>
-        </is>
-      </c>
     </row>
     <row r="61" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A61" s="7" t="inlineStr">
@@ -2144,26 +2124,6 @@
           <t>Make every email sender respect unsubscribes</t>
         </is>
       </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>The unsubscribe page/link policy is fixed, but two senders (drip processor, renewal reminders) still don't check the opt-out flag, and one reminder may skip members on a null value.</t>
-        </is>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>Add opt-out filtering to process-drips + renewal-reminders; fix event-reminder null handling. One opt-out flag is the source of truth.</t>
-        </is>
-      </c>
-      <c r="D64" s="10" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>send-email unsubscribe-block work is in flight; process-drips + renewal-reminders filtering to confirm/finish.</t>
-        </is>
-      </c>
     </row>
     <row r="65" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A65" s="7" t="inlineStr">
@@ -2378,26 +2338,6 @@
           <t>Build the admin area into clean sections</t>
         </is>
       </c>
-      <c r="B74" s="8" t="inlineStr">
-        <is>
-          <t>Reorganize admin into Today / People / Events / Network / Money / Messages / Settings with one source of truth per question.</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>7-section IA; folds in nav cleanup, per-event check-in start, financial accuracy, tier tools, and guest upload.</t>
-        </is>
-      </c>
-      <c r="D74" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="inlineStr">
-        <is>
-          <t>The Messages section is where the texting inbox lives.</t>
-        </is>
-      </c>
     </row>
     <row r="75" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A75" s="7" t="inlineStr">
@@ -2616,26 +2556,6 @@
           <t>Member directory — people-finder for all member + partner types</t>
         </is>
       </c>
-      <c r="B84" s="8" t="inlineStr">
-        <is>
-          <t>A members-only people-finder where social members, business members, and partners can all find and see each other — profiles only, WITHOUT the business-listings view. Visible to everyone logged in, regardless of type. A privacy toggle lets a member hide from it.</t>
-        </is>
-      </c>
-      <c r="C84" s="8" t="inlineStr">
-        <is>
-          <t>Logged-in directory of people (social + business + partner). Profiles only — no business view (that lives in The Network). Visible to all logged-in types; honor the privacy toggle.</t>
-        </is>
-      </c>
-      <c r="D84" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E84" s="8" t="inlineStr">
-        <is>
-          <t>Distinct from The Network (hubs + business/partner listings). Pairs with the privacy toggle below.</t>
-        </is>
-      </c>
     </row>
     <row r="85" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A85" s="7" t="inlineStr">
@@ -2730,26 +2650,6 @@
           <t>Speed up slow list pages (Events, Tasks, Hubs)</t>
         </is>
       </c>
-      <c r="B90" s="8" t="inlineStr">
-        <is>
-          <t>These pages make many small repeated DB calls (N+1) that get slow as data grows.</t>
-        </is>
-      </c>
-      <c r="C90" s="8" t="inlineStr">
-        <is>
-          <t>Resolve the N+1 query patterns; batch them.</t>
-        </is>
-      </c>
-      <c r="D90" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E90" s="8" t="inlineStr">
-        <is>
-          <t>Batch the repeated calls on Events, Tasks, Hubs.</t>
-        </is>
-      </c>
     </row>
     <row r="91" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A91" s="7" t="inlineStr">
@@ -2898,26 +2798,6 @@
           <t>Verify sessions refresh correctly on expiry</t>
         </is>
       </c>
-      <c r="B98" s="8" t="inlineStr">
-        <is>
-          <t>Confirm cookie-based refresh works when a token expires so members aren't kicked out.</t>
-        </is>
-      </c>
-      <c r="C98" s="8" t="inlineStr">
-        <is>
-          <t>Verify @supabase/ssr middleware refreshes session on token expiry.</t>
-        </is>
-      </c>
-      <c r="D98" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E98" s="8" t="inlineStr">
-        <is>
-          <t>Confirm members aren't kicked out when a token expires.</t>
-        </is>
-      </c>
     </row>
     <row r="99" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A99" s="7" t="inlineStr">
@@ -2952,10 +2832,6 @@
           <t>Apple Sign-In</t>
         </is>
       </c>
-      <c r="B100" s="5" t="n"/>
-      <c r="C100" s="5" t="n"/>
-      <c r="D100" s="5" t="n"/>
-      <c r="E100" s="6" t="n"/>
     </row>
     <row r="101" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A101" s="7" t="inlineStr">
@@ -3061,26 +2937,6 @@
           <t>Verify the admin financial data function</t>
         </is>
       </c>
-      <c r="B107" s="8" t="inlineStr">
-        <is>
-          <t>Confirm the edge function feeding admin financials returns correct numbers.</t>
-        </is>
-      </c>
-      <c r="C107" s="8" t="inlineStr">
-        <is>
-          <t>Verify admin-financial-data.</t>
-        </is>
-      </c>
-      <c r="D107" s="11" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="E107" s="8" t="inlineStr">
-        <is>
-          <t>Confirm the numbers it returns are correct.</t>
-        </is>
-      </c>
     </row>
     <row r="108" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A108" s="7" t="inlineStr">
@@ -3391,26 +3247,6 @@
           <t>Send email from a contact record</t>
         </is>
       </c>
-      <c r="B121" s="8" t="inlineStr">
-        <is>
-          <t>Let an admin email directly from a member/contact record.</t>
-        </is>
-      </c>
-      <c r="C121" s="8" t="inlineStr">
-        <is>
-          <t>Send-email action on the contact record.</t>
-        </is>
-      </c>
-      <c r="D121" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E121" s="8" t="inlineStr">
-        <is>
-          <t>Admin emails directly from a member record.</t>
-        </is>
-      </c>
     </row>
     <row r="122" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A122" s="7" t="inlineStr">
@@ -3505,26 +3341,6 @@
           <t>Add CHECK constraints incrementally (enums REJECTED — too risky)</t>
         </is>
       </c>
-      <c r="B127" s="15" t="inlineStr">
-        <is>
-          <t>Was 'convert status text -&gt; enums'. DIAGNOSED Jul 9 as too risky: ~35 tables / 60+ write paths, and profiles.subscription_status is fed by the Stripe webhook with Stripe's full status vocabulary (trialing/paused/incomplete/etc). An enum built from observed values would make the webhook UPDATE throw on the first unseen status — silent breakage in the PAYMENT path. Enums rejected.</t>
-        </is>
-      </c>
-      <c r="C127" s="15" t="inlineStr">
-        <is>
-          <t>If typo-prevention is wanted later: add per-table CHECK constraints (NOT enums), table-by-table, starting with attendance_credentials (values: active/used/voided). Trivially reversible. Its own scoped task — never wholesale.</t>
-        </is>
-      </c>
-      <c r="D127" s="18" t="inlineStr">
-        <is>
-          <t>Deferred</t>
-        </is>
-      </c>
-      <c r="E127" s="15" t="inlineStr">
-        <is>
-          <t>Reclassified Jul 9. Do NOT rush — payment-path risk. CHECK constraints are the safe 80/20 if revisited.</t>
-        </is>
-      </c>
     </row>
     <row r="128" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A128" s="17" t="inlineStr">
@@ -3734,26 +3550,6 @@
           <t>Sponsor page (likely folds into /business)</t>
         </is>
       </c>
-      <c r="B138" s="8" t="inlineStr">
-        <is>
-          <t>Sponsor functionality — likely folds into the /business application routing.</t>
-        </is>
-      </c>
-      <c r="C138" s="8" t="inlineStr">
-        <is>
-          <t>Probably absorbed by the /business rebuild.</t>
-        </is>
-      </c>
-      <c r="D138" s="10" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E138" s="8" t="inlineStr">
-        <is>
-          <t>Likely folds into the /business rebuild — confirm first.</t>
-        </is>
-      </c>
     </row>
     <row r="139" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A139" s="7" t="inlineStr">
@@ -3815,10 +3611,6 @@
           <t>The Network — four hubs + members rolled up</t>
         </is>
       </c>
-      <c r="B141" s="29" t="n"/>
-      <c r="C141" s="29" t="n"/>
-      <c r="D141" s="29" t="n"/>
-      <c r="E141" s="30" t="n"/>
     </row>
     <row r="142" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A142" s="7" t="inlineStr">
@@ -3893,26 +3685,6 @@
           <t>Rotate the R2 media token (exposed key)</t>
         </is>
       </c>
-      <c r="B147" s="8" t="inlineStr">
-        <is>
-          <t>The R2 Access Key ID + Secret for bucket 704-discussion-media were exposed in a working chat (screenshot/paste). Scope = that one media bucket only — low blast radius, but rotate.</t>
-        </is>
-      </c>
-      <c r="C147" s="8" t="inlineStr">
-        <is>
-          <t>After 6c ships: Cloudflare -&gt; R2 -&gt; API tokens -&gt; re-create 704-discussion-upload (Object Read &amp; Write, bucket-scoped) -&gt; supabase secrets set the two new values -&gt; confirm an upload still works.</t>
-        </is>
-      </c>
-      <c r="D147" s="20" t="inlineStr">
-        <is>
-          <t>Declined</t>
-        </is>
-      </c>
-      <c r="E147" s="8" t="inlineStr">
-        <is>
-          <t>Adam declined rotation Jul 5 - standing watch item. Key scope = one media bucket only (no member data / money / DB). Say 'rotate' anytime: ~2 min.</t>
-        </is>
-      </c>
     </row>
     <row r="148" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A148" s="7" t="inlineStr">
@@ -4100,51 +3872,11 @@
           <t>[DONE] Josh Ahart full removal (exit workstream)</t>
         </is>
       </c>
-      <c r="B156" s="23" t="inlineStr">
-        <is>
-          <t>De-privileged (super_admin-&gt;lead), permanent ban, all 8 sessions + 64 tokens killed, profile deactivated, ambassador row disabled, removed from public /about page (0cc8c66), 2 dormant test dupe accounts hard-deleted. Stripe sub cancelled + Connect account rejected (Adam, dashboard). Platform passwords rotated (Adam).</t>
-        </is>
-      </c>
-      <c r="C156" s="23" t="inlineStr">
-        <is>
-          <t>Verified: role=lead, 0 sessions/tokens, banned. Public site scrubbed. Dashboard-member removal confirmed by Adam.</t>
-        </is>
-      </c>
-      <c r="D156" s="24" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E156" s="23" t="inlineStr">
-        <is>
-          <t>NOT on the build sheet — exit workstream. Recorded here for completeness.</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" s="16" t="inlineStr">
         <is>
           <t>[DONE] Member status batch (Jul 9)</t>
-        </is>
-      </c>
-      <c r="B157" s="23" t="inlineStr">
-        <is>
-          <t>Nicholas Stathopoulos + Robert Villante -&gt; non_member/inactive/override off/lead (Nick admin revoked + sessions killed). Whitney Cleland + Brenna Dunne + Kaelah Torres -&gt; ERASED (auth+profile+people+credentials deleted; all comped, no Stripe to cancel). More status changes flagged as coming.</t>
-        </is>
-      </c>
-      <c r="C157" s="23" t="inlineStr">
-        <is>
-          <t>All verified via SQL (zeros on erase). Read-first footprint audit confirmed safe (no owned content cascaded).</t>
-        </is>
-      </c>
-      <c r="D157" s="24" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E157" s="23" t="inlineStr">
-        <is>
-          <t>Adam noted more member changes coming next session.</t>
         </is>
       </c>
     </row>
@@ -4271,26 +4003,6 @@
           <t>Partner Portal (audit, then repurpose or remove)</t>
         </is>
       </c>
-      <c r="B165" s="8" t="inlineStr">
-        <is>
-          <t>An existing, mostly-built partner portal of unclear purpose. Audit it, then either repurpose it as the Preferred Business Network management surface or remove it. Frozen until then.</t>
-        </is>
-      </c>
-      <c r="C165" s="8" t="inlineStr">
-        <is>
-          <t>Own detailed scope before build.</t>
-        </is>
-      </c>
-      <c r="D165" s="26" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="E165" s="8" t="inlineStr">
-        <is>
-          <t>Audit first; likely becomes the Preferred Business Network management surface. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag.</t>
-        </is>
-      </c>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -4482,26 +4194,6 @@
           <t>Q6 canceled-but-paying tripwire (canceled-drift detection)</t>
         </is>
       </c>
-      <c r="B174" s="8" t="inlineStr">
-        <is>
-          <t>Members whose app status shows canceled while Stripe still bills them (or the inverse) - a billing/status drift that should trip an alert instead of going silent.</t>
-        </is>
-      </c>
-      <c r="C174" s="8" t="inlineStr">
-        <is>
-          <t>Add a scheduled check comparing profiles.subscription_status vs the live Stripe subscription state; alert on canceled-in-app-but-active-in-Stripe and the inverse.</t>
-        </is>
-      </c>
-      <c r="D174" s="9" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-      <c r="E174" s="8" t="inlineStr">
-        <is>
-          <t>The develop seed carries a canceled-drift (Q6) dummy for rehearsal. Folds into the DB/Stripe drift watch + admin health dashboard.</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -5011,30 +4703,30 @@
   <mergeCells count="26">
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A157:E157"/>
-    <mergeCell ref="A64:E64"/>
-    <mergeCell ref="A98:E98"/>
-    <mergeCell ref="A60:E60"/>
     <mergeCell ref="A51:E51"/>
-    <mergeCell ref="A107:E107"/>
-    <mergeCell ref="A138:E138"/>
-    <mergeCell ref="A90:E90"/>
-    <mergeCell ref="A174:E174"/>
-    <mergeCell ref="A84:E84"/>
-    <mergeCell ref="A74:E74"/>
+    <mergeCell ref="A103:E103"/>
+    <mergeCell ref="A132:E132"/>
+    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A146:E146"/>
+    <mergeCell ref="A162:E162"/>
+    <mergeCell ref="A89:E89"/>
+    <mergeCell ref="A105:E105"/>
     <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A143:E143"/>
+    <mergeCell ref="A95:E95"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A179:E179"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A141:E141"/>
-    <mergeCell ref="A100:E100"/>
-    <mergeCell ref="A156:E156"/>
-    <mergeCell ref="A147:E147"/>
-    <mergeCell ref="A165:E165"/>
-    <mergeCell ref="A121:E121"/>
+    <mergeCell ref="A126:E126"/>
+    <mergeCell ref="A161:E161"/>
+    <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A152:E152"/>
+    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A170:E170"/>
     <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A127:E127"/>
     <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A67:E67"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
fix: tracker - recover cells written after baseline and lost to merge drift
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -248,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
@@ -330,6 +330,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -630,10 +634,10 @@
           <t>ONBOARDING &amp; SIGNUP   ·   2 items</t>
         </is>
       </c>
-      <c r="B2" s="29" t="n"/>
-      <c r="C2" s="29" t="n"/>
-      <c r="D2" s="29" t="n"/>
-      <c r="E2" s="30" t="n"/>
+      <c r="B2" s="31" t="n"/>
+      <c r="C2" s="31" t="n"/>
+      <c r="D2" s="31" t="n"/>
+      <c r="E2" s="31" t="n"/>
     </row>
     <row r="3" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A3" s="7" t="inlineStr">
@@ -695,10 +699,10 @@
           <t>MEMBERS &amp; MONEY   ·   3 items</t>
         </is>
       </c>
-      <c r="B5" s="29" t="n"/>
-      <c r="C5" s="29" t="n"/>
-      <c r="D5" s="29" t="n"/>
-      <c r="E5" s="30" t="n"/>
+      <c r="B5" s="31" t="n"/>
+      <c r="C5" s="31" t="n"/>
+      <c r="D5" s="31" t="n"/>
+      <c r="E5" s="31" t="n"/>
     </row>
     <row r="6" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A6" s="7" t="inlineStr">
@@ -787,10 +791,10 @@
           <t>IDENTITY FOUNDATION   ·   3 items</t>
         </is>
       </c>
-      <c r="B9" s="29" t="n"/>
-      <c r="C9" s="29" t="n"/>
-      <c r="D9" s="29" t="n"/>
-      <c r="E9" s="30" t="n"/>
+      <c r="B9" s="31" t="n"/>
+      <c r="C9" s="31" t="n"/>
+      <c r="D9" s="31" t="n"/>
+      <c r="E9" s="31" t="n"/>
     </row>
     <row r="10" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
       <c r="A10" s="7" t="inlineStr">
@@ -879,10 +883,10 @@
           <t>EVENTS &amp; CALENDAR   ·   19 items</t>
         </is>
       </c>
-      <c r="B13" s="29" t="n"/>
-      <c r="C13" s="29" t="n"/>
-      <c r="D13" s="29" t="n"/>
-      <c r="E13" s="30" t="n"/>
+      <c r="B13" s="31" t="n"/>
+      <c r="C13" s="31" t="n"/>
+      <c r="D13" s="31" t="n"/>
+      <c r="E13" s="31" t="n"/>
     </row>
     <row r="14" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A14" s="7" t="inlineStr">
@@ -1403,10 +1407,10 @@
           <t>WALLET PASS   ·   5 items</t>
         </is>
       </c>
-      <c r="B33" s="29" t="n"/>
-      <c r="C33" s="29" t="n"/>
-      <c r="D33" s="29" t="n"/>
-      <c r="E33" s="30" t="n"/>
+      <c r="B33" s="31" t="n"/>
+      <c r="C33" s="31" t="n"/>
+      <c r="D33" s="31" t="n"/>
+      <c r="E33" s="31" t="n"/>
     </row>
     <row r="34" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A34" s="7" t="inlineStr">
@@ -1549,10 +1553,10 @@
           <t>AMBASSADORS   ·   8 items</t>
         </is>
       </c>
-      <c r="B39" s="29" t="n"/>
-      <c r="C39" s="29" t="n"/>
-      <c r="D39" s="29" t="n"/>
-      <c r="E39" s="30" t="n"/>
+      <c r="B39" s="31" t="n"/>
+      <c r="C39" s="31" t="n"/>
+      <c r="D39" s="31" t="n"/>
+      <c r="E39" s="31" t="n"/>
     </row>
     <row r="40" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A40" s="7" t="inlineStr">
@@ -1776,10 +1780,10 @@
           <t>MEMBER TEXTING   ·   2 items</t>
         </is>
       </c>
-      <c r="B48" s="29" t="n"/>
-      <c r="C48" s="29" t="n"/>
-      <c r="D48" s="29" t="n"/>
-      <c r="E48" s="30" t="n"/>
+      <c r="B48" s="31" t="n"/>
+      <c r="C48" s="31" t="n"/>
+      <c r="D48" s="31" t="n"/>
+      <c r="E48" s="31" t="n"/>
     </row>
     <row r="49" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A49" s="7" t="inlineStr">
@@ -1841,10 +1845,10 @@
           <t>SECURITY   ·   3 items</t>
         </is>
       </c>
-      <c r="B51" s="29" t="n"/>
-      <c r="C51" s="29" t="n"/>
-      <c r="D51" s="29" t="n"/>
-      <c r="E51" s="30" t="n"/>
+      <c r="B51" s="31" t="n"/>
+      <c r="C51" s="31" t="n"/>
+      <c r="D51" s="31" t="n"/>
+      <c r="E51" s="31" t="n"/>
     </row>
     <row r="52" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A52" s="7" t="inlineStr">
@@ -1933,10 +1937,10 @@
           <t>SECURITY &amp; MONITORING   ·   7 items</t>
         </is>
       </c>
-      <c r="B55" s="29" t="n"/>
-      <c r="C55" s="29" t="n"/>
-      <c r="D55" s="29" t="n"/>
-      <c r="E55" s="30" t="n"/>
+      <c r="B55" s="31" t="n"/>
+      <c r="C55" s="31" t="n"/>
+      <c r="D55" s="31" t="n"/>
+      <c r="E55" s="31" t="n"/>
     </row>
     <row r="56" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A56" s="7" t="inlineStr">
@@ -2052,6 +2056,26 @@
           <t>Add a deploy pipeline so changes go live safely</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>DB/function changes are pushed by hand today — the root cause of code/live drift. Locked: hand-patching stops once this lands (with a written emergency lane).</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>GitHub Actions: merge to main -&gt; db push + functions deploy. Needs 3 repo secrets.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Once in, hand-patching stops; needed before two people touch production in parallel.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A61" s="7" t="inlineStr">
@@ -2113,10 +2137,10 @@
           <t>EMAIL &amp; COMPLIANCE   ·   3 items</t>
         </is>
       </c>
-      <c r="B63" s="29" t="n"/>
-      <c r="C63" s="29" t="n"/>
-      <c r="D63" s="29" t="n"/>
-      <c r="E63" s="30" t="n"/>
+      <c r="B63" s="31" t="n"/>
+      <c r="C63" s="31" t="n"/>
+      <c r="D63" s="31" t="n"/>
+      <c r="E63" s="31" t="n"/>
     </row>
     <row r="64" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A64" s="7" t="inlineStr">
@@ -2124,6 +2148,26 @@
           <t>Make every email sender respect unsubscribes</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>The unsubscribe page/link policy is fixed, but two senders (drip processor, renewal reminders) still don't check the opt-out flag, and one reminder may skip members on a null value.</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Add opt-out filtering to process-drips + renewal-reminders; fix event-reminder null handling. One opt-out flag is the source of truth.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>send-email unsubscribe-block work is in flight; process-drips + renewal-reminders filtering to confirm/finish.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A65" s="7" t="inlineStr">
@@ -2165,10 +2209,10 @@
           <t>ADMIN &amp; OPERATIONS   ·   12 items</t>
         </is>
       </c>
-      <c r="B67" s="29" t="n"/>
-      <c r="C67" s="29" t="n"/>
-      <c r="D67" s="29" t="n"/>
-      <c r="E67" s="30" t="n"/>
+      <c r="B67" s="31" t="n"/>
+      <c r="C67" s="31" t="n"/>
+      <c r="D67" s="31" t="n"/>
+      <c r="E67" s="31" t="n"/>
     </row>
     <row r="68" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A68" s="7" t="inlineStr">
@@ -2338,6 +2382,26 @@
           <t>Build the admin area into clean sections</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Reorganize admin into Today / People / Events / Network / Money / Messages / Settings with one source of truth per question.</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>7-section IA; folds in nav cleanup, per-event check-in start, financial accuracy, tier tools, and guest upload.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>The Messages section is where the texting inbox lives.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A75" s="7" t="inlineStr">
@@ -2399,10 +2463,26 @@
           <t>Fix the organization settings table</t>
         </is>
       </c>
-      <c r="B77" s="29" t="n"/>
-      <c r="C77" s="29" t="n"/>
-      <c r="D77" s="29" t="n"/>
-      <c r="E77" s="30" t="n"/>
+      <c r="B77" s="29" t="inlineStr">
+        <is>
+          <t>organization_settings has the wrong schema.</t>
+        </is>
+      </c>
+      <c r="C77" s="29" t="inlineStr">
+        <is>
+          <t>Correct the organization_settings schema.</t>
+        </is>
+      </c>
+      <c r="D77" s="29" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E77" s="30" t="inlineStr">
+        <is>
+          <t>Schema is currently wrong; correct it.</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
       <c r="A78" s="7" t="inlineStr">
@@ -2437,10 +2517,10 @@
           <t>MEMBER EXPERIENCE   ·   9 items</t>
         </is>
       </c>
-      <c r="B79" s="29" t="n"/>
-      <c r="C79" s="29" t="n"/>
-      <c r="D79" s="29" t="n"/>
-      <c r="E79" s="30" t="n"/>
+      <c r="B79" s="31" t="n"/>
+      <c r="C79" s="31" t="n"/>
+      <c r="D79" s="31" t="n"/>
+      <c r="E79" s="31" t="n"/>
     </row>
     <row r="80" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A80" s="7" t="inlineStr">
@@ -2556,6 +2636,26 @@
           <t>Member directory — people-finder for all member + partner types</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>A members-only people-finder where social members, business members, and partners can all find and see each other — profiles only, WITHOUT the business-listings view. Visible to everyone logged in, regardless of type. A privacy toggle lets a member hide from it.</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Logged-in directory of people (social + business + partner). Profiles only — no business view (that lives in The Network). Visible to all logged-in types; honor the privacy toggle.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Distinct from The Network (hubs + business/partner listings). Pairs with the privacy toggle below.</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A85" s="7" t="inlineStr">
@@ -2617,10 +2717,26 @@
           <t>Member spotlight on calendar/home</t>
         </is>
       </c>
-      <c r="B87" s="29" t="n"/>
-      <c r="C87" s="29" t="n"/>
-      <c r="D87" s="29" t="n"/>
-      <c r="E87" s="30" t="n"/>
+      <c r="B87" s="29" t="inlineStr">
+        <is>
+          <t>Feature a member spotlight on the calendar/home pages.</t>
+        </is>
+      </c>
+      <c r="C87" s="29" t="inlineStr">
+        <is>
+          <t>Member spotlight feature.</t>
+        </is>
+      </c>
+      <c r="D87" s="29" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E87" s="30" t="inlineStr">
+        <is>
+          <t>Feature a member on calendar/home.</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A88" s="7" t="inlineStr">
@@ -2639,10 +2755,10 @@
           <t>PERFORMANCE   ·   5 items</t>
         </is>
       </c>
-      <c r="B89" s="29" t="n"/>
-      <c r="C89" s="29" t="n"/>
-      <c r="D89" s="29" t="n"/>
-      <c r="E89" s="30" t="n"/>
+      <c r="B89" s="31" t="n"/>
+      <c r="C89" s="31" t="n"/>
+      <c r="D89" s="31" t="n"/>
+      <c r="E89" s="31" t="n"/>
     </row>
     <row r="90" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A90" s="7" t="inlineStr">
@@ -2650,6 +2766,26 @@
           <t>Speed up slow list pages (Events, Tasks, Hubs)</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>These pages make many small repeated DB calls (N+1) that get slow as data grows.</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Resolve the N+1 query patterns; batch them.</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Batch the repeated calls on Events, Tasks, Hubs.</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A91" s="7" t="inlineStr">
@@ -2711,10 +2847,26 @@
           <t>Standardize how data is loaded (React Query)</t>
         </is>
       </c>
-      <c r="B93" s="29" t="n"/>
-      <c r="C93" s="29" t="n"/>
-      <c r="D93" s="29" t="n"/>
-      <c r="E93" s="30" t="n"/>
+      <c r="B93" s="29" t="inlineStr">
+        <is>
+          <t>Make loading behavior uniform and reliable.</t>
+        </is>
+      </c>
+      <c r="C93" s="29" t="inlineStr">
+        <is>
+          <t>React Query rollout across data fetching.</t>
+        </is>
+      </c>
+      <c r="D93" s="29" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E93" s="30" t="inlineStr">
+        <is>
+          <t>Uniform data-loading / caching across the app.</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A94" s="7" t="inlineStr">
@@ -2733,10 +2885,10 @@
           <t>AUTH   ·   7 items</t>
         </is>
       </c>
-      <c r="B95" s="29" t="n"/>
-      <c r="C95" s="29" t="n"/>
-      <c r="D95" s="29" t="n"/>
-      <c r="E95" s="30" t="n"/>
+      <c r="B95" s="31" t="n"/>
+      <c r="C95" s="31" t="n"/>
+      <c r="D95" s="31" t="n"/>
+      <c r="E95" s="31" t="n"/>
     </row>
     <row r="96" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A96" s="7" t="inlineStr">
@@ -2798,6 +2950,26 @@
           <t>Verify sessions refresh correctly on expiry</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Confirm cookie-based refresh works when a token expires so members aren't kicked out.</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Verify @supabase/ssr middleware refreshes session on token expiry.</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Confirm members aren't kicked out when a token expires.</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A99" s="7" t="inlineStr">
@@ -2841,7 +3013,11 @@
       </c>
       <c r="B101" s="29" t="n"/>
       <c r="C101" s="29" t="n"/>
-      <c r="D101" s="29" t="n"/>
+      <c r="D101" s="29" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
       <c r="E101" s="30" t="n"/>
     </row>
     <row r="102" ht="15" customFormat="1" customHeight="1" s="2">
@@ -2877,10 +3053,10 @@
           <t>BUSINESS   ·   1 item</t>
         </is>
       </c>
-      <c r="B103" s="29" t="n"/>
-      <c r="C103" s="29" t="n"/>
-      <c r="D103" s="29" t="n"/>
-      <c r="E103" s="30" t="n"/>
+      <c r="B103" s="31" t="n"/>
+      <c r="C103" s="31" t="n"/>
+      <c r="D103" s="31" t="n"/>
+      <c r="E103" s="31" t="n"/>
     </row>
     <row r="104" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A104" s="7" t="inlineStr">
@@ -2899,10 +3075,10 @@
           <t>FINANCIALS   ·   6 items</t>
         </is>
       </c>
-      <c r="B105" s="29" t="n"/>
-      <c r="C105" s="29" t="n"/>
-      <c r="D105" s="29" t="n"/>
-      <c r="E105" s="30" t="n"/>
+      <c r="B105" s="31" t="n"/>
+      <c r="C105" s="31" t="n"/>
+      <c r="D105" s="31" t="n"/>
+      <c r="E105" s="31" t="n"/>
     </row>
     <row r="106" ht="15" customFormat="1" customHeight="1" s="2">
       <c r="A106" s="7" t="inlineStr">
@@ -2937,6 +3113,26 @@
           <t>Verify the admin financial data function</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Confirm the edge function feeding admin financials returns correct numbers.</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Verify admin-financial-data.</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Confirm the numbers it returns are correct.</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A108" s="7" t="inlineStr">
@@ -2998,10 +3194,26 @@
           <t>Reduce redundant Stripe scans</t>
         </is>
       </c>
-      <c r="B110" s="29" t="n"/>
-      <c r="C110" s="29" t="n"/>
-      <c r="D110" s="29" t="n"/>
-      <c r="E110" s="30" t="n"/>
+      <c r="B110" s="29" t="inlineStr">
+        <is>
+          <t>Cut how often the system scans Stripe, for performance/cost.</t>
+        </is>
+      </c>
+      <c r="C110" s="29" t="inlineStr">
+        <is>
+          <t>Reduce Stripe API scan frequency.</t>
+        </is>
+      </c>
+      <c r="D110" s="29" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E110" s="30" t="inlineStr">
+        <is>
+          <t>Cut scan frequency for cost / performance.</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A111" s="7" t="inlineStr">
@@ -3020,10 +3232,10 @@
           <t>EMAIL &amp; DRIP   ·   13 items</t>
         </is>
       </c>
-      <c r="B112" s="29" t="n"/>
-      <c r="C112" s="29" t="n"/>
-      <c r="D112" s="29" t="n"/>
-      <c r="E112" s="30" t="n"/>
+      <c r="B112" s="31" t="n"/>
+      <c r="C112" s="31" t="n"/>
+      <c r="D112" s="31" t="n"/>
+      <c r="E112" s="31" t="n"/>
     </row>
     <row r="113" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A113" s="7" t="inlineStr">
@@ -3247,6 +3459,26 @@
           <t>Send email from a contact record</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Let an admin email directly from a member/contact record.</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Send-email action on the contact record.</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Admin emails directly from a member record.</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A122" s="7" t="inlineStr">
@@ -3308,10 +3540,26 @@
           <t>Merge guest follow-up into the drip processor</t>
         </is>
       </c>
-      <c r="B124" s="29" t="n"/>
-      <c r="C124" s="29" t="n"/>
-      <c r="D124" s="29" t="n"/>
-      <c r="E124" s="30" t="n"/>
+      <c r="B124" s="29" t="inlineStr">
+        <is>
+          <t>Retire the separate guest-followup function and fold it into the main processor.</t>
+        </is>
+      </c>
+      <c r="C124" s="29" t="inlineStr">
+        <is>
+          <t>Consolidate guest-followup into process-drips.</t>
+        </is>
+      </c>
+      <c r="D124" s="29" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E124" s="30" t="inlineStr">
+        <is>
+          <t>Fold guest-followup into process-drips.</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A125" s="7" t="inlineStr">
@@ -3330,10 +3578,10 @@
           <t>DATA &amp; CLEANUP   ·   6 items</t>
         </is>
       </c>
-      <c r="B126" s="29" t="n"/>
-      <c r="C126" s="29" t="n"/>
-      <c r="D126" s="29" t="n"/>
-      <c r="E126" s="30" t="n"/>
+      <c r="B126" s="31" t="n"/>
+      <c r="C126" s="31" t="n"/>
+      <c r="D126" s="31" t="n"/>
+      <c r="E126" s="31" t="n"/>
     </row>
     <row r="127" ht="68.65000000000001" customFormat="1" customHeight="1" s="2">
       <c r="A127" s="17" t="inlineStr">
@@ -3341,6 +3589,26 @@
           <t>Add CHECK constraints incrementally (enums REJECTED — too risky)</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Was 'convert status text -&gt; enums'. DIAGNOSED Jul 9 as too risky: ~35 tables / 60+ write paths, and profiles.subscription_status is fed by the Stripe webhook with Stripe's full status vocabulary (trialing/paused/incomplete/etc). An enum built from observed values would make the webhook UPDATE throw on the first unseen status — silent breakage in the PAYMENT path. Enums rejected.</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>If typo-prevention is wanted later: add per-table CHECK constraints (NOT enums), table-by-table, starting with attendance_credentials (values: active/used/voided). Trivially reversible. Its own scoped task — never wholesale.</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Reclassified Jul 9. Do NOT rush — payment-path risk. CHECK constraints are the safe 80/20 if revisited.</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A128" s="17" t="inlineStr">
@@ -3402,10 +3670,26 @@
           <t>Drop old backup tables after soak</t>
         </is>
       </c>
-      <c r="B130" s="29" t="n"/>
-      <c r="C130" s="29" t="n"/>
-      <c r="D130" s="29" t="n"/>
-      <c r="E130" s="30" t="n"/>
+      <c r="B130" s="29" t="inlineStr">
+        <is>
+          <t>Backup tables from recent migrations await a 2-4 week no-regression soak.</t>
+        </is>
+      </c>
+      <c r="C130" s="29" t="inlineStr">
+        <is>
+          <t>Drop dated backup_* tables after soak; confirm stability first.</t>
+        </is>
+      </c>
+      <c r="D130" s="29" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E130" s="30" t="inlineStr">
+        <is>
+          <t>Only after a 2-4 week no-regression soak.</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A131" s="7" t="inlineStr">
@@ -3420,10 +3704,10 @@
           <t>MARKETING &amp; FRONT-END   ·   10 items</t>
         </is>
       </c>
-      <c r="B132" s="29" t="n"/>
-      <c r="C132" s="29" t="n"/>
-      <c r="D132" s="29" t="n"/>
-      <c r="E132" s="30" t="n"/>
+      <c r="B132" s="31" t="n"/>
+      <c r="C132" s="31" t="n"/>
+      <c r="D132" s="31" t="n"/>
+      <c r="E132" s="31" t="n"/>
     </row>
     <row r="133" ht="35.05" customFormat="1" customHeight="1" s="2">
       <c r="A133" s="7" t="inlineStr">
@@ -3550,6 +3834,26 @@
           <t>Sponsor page (likely folds into /business)</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Sponsor functionality — likely folds into the /business application routing.</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Probably absorbed by the /business rebuild.</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Likely folds into the /business rebuild — confirm first.</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A139" s="7" t="inlineStr">
@@ -3611,6 +3915,26 @@
           <t>The Network — four hubs + members rolled up</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>The four hubs rolled up into one view, plus all members. Two faces reading the same data: a PUBLIC face (the hub landers + business/partner listings — the sales asset) and an INTERNAL in-portal view that rolls up everyone. Social members appear ONLY on the internal in-portal view — never on the public hubs.</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Roll the four hubs into one Network view + members. Public face = hubs / business + partner listings (social members excluded). Internal face = full rolled-up view including social members. Reads the same hub data as the landers.</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Depends on the portal + identity foundation. Social members are internal-only on The Network. Separate from the member directory (people-only).</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A142" s="7" t="inlineStr">
@@ -3625,10 +3949,10 @@
           <t>AI / AGENTS (LATER EFFORT)   ·   2 items</t>
         </is>
       </c>
-      <c r="B143" s="29" t="n"/>
-      <c r="C143" s="29" t="n"/>
-      <c r="D143" s="29" t="n"/>
-      <c r="E143" s="30" t="n"/>
+      <c r="B143" s="31" t="n"/>
+      <c r="C143" s="31" t="n"/>
+      <c r="D143" s="31" t="n"/>
+      <c r="E143" s="31" t="n"/>
     </row>
     <row r="144" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A144" s="7" t="inlineStr">
@@ -3674,10 +3998,10 @@
           <t>EVENT DISCUSSION &amp; NOTIFICATIONS + JUL-5/6 FINDINGS — IN-HOUSE (NOT ON THE DEVELOPER SHEET)   ·   10 items</t>
         </is>
       </c>
-      <c r="B146" s="29" t="n"/>
-      <c r="C146" s="29" t="n"/>
-      <c r="D146" s="29" t="n"/>
-      <c r="E146" s="30" t="n"/>
+      <c r="B146" s="31" t="n"/>
+      <c r="C146" s="31" t="n"/>
+      <c r="D146" s="31" t="n"/>
+      <c r="E146" s="31" t="n"/>
     </row>
     <row r="147" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A147" s="7" t="inlineStr">
@@ -3685,6 +4009,26 @@
           <t>Rotate the R2 media token (exposed key)</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>The R2 Access Key ID + Secret for bucket 704-discussion-media were exposed in a working chat (screenshot/paste). Scope = that one media bucket only — low blast radius, but rotate.</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>After 6c ships: Cloudflare -&gt; R2 -&gt; API tokens -&gt; re-create 704-discussion-upload (Object Read &amp; Write, bucket-scoped) -&gt; supabase secrets set the two new values -&gt; confirm an upload still works.</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Declined</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Adam declined rotation Jul 5 - standing watch item. Key scope = one media bucket only (no member data / money / DB). Say 'rotate' anytime: ~2 min.</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="57.45" customFormat="1" customHeight="1" s="2">
       <c r="A148" s="7" t="inlineStr">
@@ -3746,10 +4090,26 @@
           <t>Messaging: attachment uploads (images/files)</t>
         </is>
       </c>
-      <c r="B150" s="29" t="n"/>
-      <c r="C150" s="29" t="n"/>
-      <c r="D150" s="29" t="n"/>
-      <c r="E150" s="30" t="n"/>
+      <c r="B150" s="29" t="inlineStr">
+        <is>
+          <t>MessagingView has image/file upload code paths and messages now has image_urls/file_urls/file_names columns (added Jul 5), but the storage wiring (bucket, upload flow) has never been tested and may not exist.</t>
+        </is>
+      </c>
+      <c r="C150" s="29" t="inlineStr">
+        <is>
+          <t>Audit the attachment path end to end: storage bucket, upload call, render. Fix or wire what's missing. Desktop + mobile test.</t>
+        </is>
+      </c>
+      <c r="D150" s="29" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E150" s="30" t="inlineStr">
+        <is>
+          <t>Text messaging + edits verified Jul 5; attachments explicitly skipped in that test.</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="46.25" customFormat="1" customHeight="1" s="2">
       <c r="A151" s="7" t="inlineStr">
@@ -3784,6 +4144,10 @@
           <t>SESSION LOG — JUL 7–9 2026 (COMPLETED; kept as record, esp. the security fix)</t>
         </is>
       </c>
+      <c r="B152" s="32" t="n"/>
+      <c r="C152" s="32" t="n"/>
+      <c r="D152" s="32" t="n"/>
+      <c r="E152" s="32" t="n"/>
     </row>
     <row r="153" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A153" s="16" t="inlineStr">
@@ -3872,6 +4236,26 @@
           <t>[DONE] Josh Ahart full removal (exit workstream)</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>De-privileged (super_admin-&gt;lead), permanent ban, all 8 sessions + 64 tokens killed, profile deactivated, ambassador row disabled, removed from public /about page (0cc8c66), 2 dormant test dupe accounts hard-deleted. Stripe sub cancelled + Connect account rejected (Adam, dashboard). Platform passwords rotated (Adam).</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Verified: role=lead, 0 sessions/tokens, banned. Public site scrubbed. Dashboard-member removal confirmed by Adam.</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>NOT on the build sheet — exit workstream. Recorded here for completeness.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="16" t="inlineStr">
@@ -3879,6 +4263,26 @@
           <t>[DONE] Member status batch (Jul 9)</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Nicholas Stathopoulos + Robert Villante -&gt; non_member/inactive/override off/lead (Nick admin revoked + sessions killed). Whitney Cleland + Brenna Dunne + Kaelah Torres -&gt; ERASED (auth+profile+people+credentials deleted; all comped, no Stripe to cancel). More status changes flagged as coming.</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>All verified via SQL (zeros on erase). Read-first footprint audit confirmed safe (no owned content cascaded).</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Adam noted more member changes coming next session.</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="16" t="inlineStr">
@@ -3913,6 +4317,26 @@
           <t>[DONE] Discussion edit/delete (comments+posts+photos) + admin always-on access</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Owners + admins can now edit/delete their own discussion comments (ecec3f8), posts (1e3adc1), and remove their own gallery photos (bcf746f); admins moderate anyone's. '(edited)' marker, soft-delete, silent removal. Also: admins now see the discussion link on any open event regardless of RSVP (583b343 — backend was already admin-exempt; was a missing-link discovery bug). Feed/comment/DM URL linkify (561403e).</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>All browser-tested desktop+mobile. Backend RLS already permitted; these were frontend gaps.</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>5 commits. Discussion feature now fully moderatable.</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="16" t="inlineStr">
@@ -3920,6 +4344,26 @@
           <t>[DONE] Small fixes: hubs 404, week_label, dead components, partners 400, org_settings, last_attended</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>hubs preview widget queried non-existent 'business_hubs' -&gt; fixed to 'hubs' (a00cc50, restored a silently-broken business-tier feature). ambassador-payout phantom week_label column removed (1f46e88). 3 dead admin components deleted, 1376 lines (306efa4). partners 400 fixed via column aliasing (d95a337, latent partner-disappearing bug). organization_settings tracker row was STALE (schema fine, closed). last_attended already built+firing -&gt; backfilled 17 pre-trigger rows, closed.</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>All tsc+browser verified. org_settings &amp; last_attended were already-done rows.</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Commits a00cc50, 1f46e88, 306efa4, d95a337 + 2 SQL closes.</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="25" t="inlineStr">
@@ -3927,10 +4371,10 @@
           <t>PHASE 2  ·  MAJOR BUILDS (each gets its own detailed scope before build)</t>
         </is>
       </c>
-      <c r="B161" s="29" t="n"/>
-      <c r="C161" s="29" t="n"/>
-      <c r="D161" s="29" t="n"/>
-      <c r="E161" s="30" t="n"/>
+      <c r="B161" s="33" t="n"/>
+      <c r="C161" s="33" t="n"/>
+      <c r="D161" s="33" t="n"/>
+      <c r="E161" s="33" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -3938,10 +4382,10 @@
           <t>MAJOR BUILDS — EACH GETS ITS OWN DETAILED SCOPE BEFORE BUILD   ·   7 items</t>
         </is>
       </c>
-      <c r="B162" s="29" t="n"/>
-      <c r="C162" s="29" t="n"/>
-      <c r="D162" s="29" t="n"/>
-      <c r="E162" s="30" t="n"/>
+      <c r="B162" s="31" t="n"/>
+      <c r="C162" s="31" t="n"/>
+      <c r="D162" s="31" t="n"/>
+      <c r="E162" s="31" t="n"/>
     </row>
     <row r="163" ht="21.75" customFormat="1" customHeight="1" s="2">
       <c r="A163" s="7" t="inlineStr">
@@ -4003,6 +4447,26 @@
           <t>Partner Portal (audit, then repurpose or remove)</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>An existing, mostly-built partner portal of unclear purpose. Audit it, then either repurpose it as the Preferred Business Network management surface or remove it. Frozen until then.</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Own detailed scope before build.</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Audit first; likely becomes the Preferred Business Network management surface. Currently hidden behind the reversible HIDE_CRM_AND_PARTNERS middleware flag.</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -4064,10 +4528,26 @@
           <t>Corporate / bulk-sales floating-seats portal</t>
         </is>
       </c>
-      <c r="B168" s="29" t="n"/>
-      <c r="C168" s="29" t="n"/>
-      <c r="D168" s="29" t="n"/>
-      <c r="E168" s="30" t="n"/>
+      <c r="B168" s="29" t="inlineStr">
+        <is>
+          <t>A portal for selling memberships in bulk to companies, with reassignable 'floating' seats.</t>
+        </is>
+      </c>
+      <c r="C168" s="29" t="inlineStr">
+        <is>
+          <t>Own detailed scope before build.</t>
+        </is>
+      </c>
+      <c r="D168" s="29" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="E168" s="30" t="inlineStr">
+        <is>
+          <t>Reassignable floating seats for companies.</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -4102,10 +4582,10 @@
           <t>OPEN WATCH ITEMS — ADDED 2026-07-19   ·   8 items</t>
         </is>
       </c>
-      <c r="B170" s="29" t="n"/>
-      <c r="C170" s="29" t="n"/>
-      <c r="D170" s="29" t="n"/>
-      <c r="E170" s="30" t="n"/>
+      <c r="B170" s="31" t="n"/>
+      <c r="C170" s="31" t="n"/>
+      <c r="D170" s="31" t="n"/>
+      <c r="E170" s="31" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -4194,6 +4674,26 @@
           <t>Q6 canceled-but-paying tripwire (canceled-drift detection)</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Members whose app status shows canceled while Stripe still bills them (or the inverse) - a billing/status drift that should trip an alert instead of going silent.</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Add a scheduled check comparing profiles.subscription_status vs the live Stripe subscription state; alert on canceled-in-app-but-active-in-Stripe and the inverse.</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>The develop seed carries a canceled-drift (Q6) dummy for rehearsal. Folds into the DB/Stripe drift watch + admin health dashboard.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -4255,10 +4755,26 @@
           <t>DB / Stripe drift watch items</t>
         </is>
       </c>
-      <c r="B177" s="29" t="n"/>
-      <c r="C177" s="29" t="n"/>
-      <c r="D177" s="29" t="n"/>
-      <c r="E177" s="30" t="n"/>
+      <c r="B177" s="29" t="inlineStr">
+        <is>
+          <t>Ongoing watch on the places where the database and Stripe can drift out of sync: subscription statuses, customer email on email-change, retired legacy prices, orphaned Stripe customers.</t>
+        </is>
+      </c>
+      <c r="C177" s="29" t="inlineStr">
+        <is>
+          <t>Track and periodically reconcile; surface on the admin health dashboard. Pairs with the Q6 tripwire and the 'email change keeps Stripe billing in sync' verify.</t>
+        </is>
+      </c>
+      <c r="D177" s="29" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="E177" s="30" t="inlineStr">
+        <is>
+          <t>Umbrella watch item; individual drifts get their own rows as they surface.</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -4293,6 +4809,10 @@
           <t>BILLING-VIEWS ERA — ADDED 2026-08-03   ·   15 items</t>
         </is>
       </c>
+      <c r="B179" s="34" t="n"/>
+      <c r="C179" s="34" t="n"/>
+      <c r="D179" s="34" t="n"/>
+      <c r="E179" s="34" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="28" t="inlineStr">
@@ -4700,34 +5220,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="A103:E103"/>
-    <mergeCell ref="A132:E132"/>
-    <mergeCell ref="A79:E79"/>
-    <mergeCell ref="A146:E146"/>
-    <mergeCell ref="A162:E162"/>
-    <mergeCell ref="A89:E89"/>
-    <mergeCell ref="A105:E105"/>
-    <mergeCell ref="A55:E55"/>
-    <mergeCell ref="A143:E143"/>
-    <mergeCell ref="A95:E95"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A179:E179"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A126:E126"/>
-    <mergeCell ref="A161:E161"/>
-    <mergeCell ref="A112:E112"/>
-    <mergeCell ref="A152:E152"/>
-    <mergeCell ref="A63:E63"/>
-    <mergeCell ref="A170:E170"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A67:E67"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: tracker - mark send-campaign audience fixes shipped, correct the member overlap figure
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -2244,27 +2244,27 @@
     <row r="69" ht="23.85" customFormat="1" customHeight="1" s="2">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>PRIORITY 2: send-campaign all_contacts audience includes paying members</t>
+          <t>send-campaign audience fixes - SHIPPED 2026-08-12</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>The 'All Contacts' audience in the campaign tool pulls every row from the contacts table and filters ONLY on unsubscribed. It does not exclude members. On prod, 89 of 207 contacts are also active members (over 40 percent overlap), so any All Contacts campaign sends prospect-facing copy to people who already pay. A 'join 704 Collective' style blast would pitch membership to existing members.</t>
+          <t>Three defects in the campaign audience resolver, all shipped to production on 2026-08-12. (1) all_contacts and segment both selected contacts.first_name and contacts.last_name, columns that have never existed on that table. PostgREST returned 400, the code discarded the error, and both audiences silently resolved to ZERO recipients while reporting success. all_contacts reached 0 of 214 people; segment reached 0 of 212. (2) all_contacts had no membership filter, so once the column bug was fixed it would have reached 47 active or comped members with prospect-facing copy. (3) The member exclusion lookup had no explicit limit and would have silently truncated past PostgREST's 1000-row default.</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>In supabase/functions/send-campaign/index.ts, the all_contacts branch (approx lines 478-489) selects contacts where unsubscribed is null or false, with no membership filter. Add an exclusion so contacts whose email matches a non-deleted profile with subscription_status active or trialing or membership_override true are removed from that audience. Consider whether the segment audience (tag-based, approx lines 490-506) needs the same treatment. Related dead code found the same night: converted_to_member_id is never written by any code, so the conversion-rate report on /admin/crm/reports measures nothing, and the campaigns audience preview counts contact_type = 'guest' which zero rows have, so it always shows 0. Rehearse on develop both viewports before shipping.</t>
+          <t>DONE. Commits b43d59c (full_name plus error propagation on both branches), a2fe05a (exclude active and comped members from all_contacts), f453dd4 (explicit limit on the exclusion lookup). Verified on develop against independently computed ground truth, then deployed to prod and confirmed by reading the deployed source. The segment branch deliberately does NOT exclude members - tag-driven audiences are explicitly targeted and filtering them would break legitimate use.</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>Raised 2026-08-12 during a contacts table audit. Not known whether any past campaign used this audience. Timi should be told to avoid All Contacts until fixed.</t>
+          <t>Prod all_contacts now resolves to 167 prospects (214 minus 47 members) with real names from full_name. The campaigns page preview will jump from 0 to 167 - that is the fix, not a bug. NOTE the earlier '89 members' figure in this row was wrong: it counted any profile match including cancelled and non-member accounts. The correct active/comped figure is 47. Neither audience had worked for an unknown period, so any past all_contacts campaign that appeared to send reached nobody.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(tracker): financial truth project + tonight's repairs
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E202"/>
+  <dimension ref="A1:E212"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="1" min="1" max="1"/>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>NOT on the build sheet — exit workstream. Recorded here for completeness.</t>
+          <t>NOT on the build sheet — exit workstream. Recorded here for completeness. Aug 25: Josh hub purge done — the hubs he created were removed deliberately rather than left to a profile delete, which would have cascaded (see the hubs.created_by row). Closes the owned-content residue of the exit.</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Adam noted more member changes coming next session.</t>
+          <t>Adam noted more member changes coming next session. Aug 25: Audrey converted to non-member — done, and recorded here as the next entry in this running member-status record.</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="E200" s="28" t="inlineStr">
         <is>
-          <t>Time-boxed: this row closes after the Aug 27 Exchange, either resolved or converted into an ordinary billing follow-up.</t>
+          <t>Time-boxed: this row closes after the Aug 27 Exchange, either resolved or converted into an ordinary billing follow-up. Aug 25: the 3+1 member_tier repairs done tonight included the tier-null row the payment-failure webhook re-created on this account Aug 24 — see the member_tier invariant row. The past_due watch itself still stands through Aug 27.</t>
         </is>
       </c>
     </row>
@@ -5416,6 +5416,260 @@
       <c r="E202" s="28" t="inlineStr">
         <is>
           <t>Written down so nobody later reads a UTM column and believes it is full-funnel attribution. Related: the RSVP-attribution-by-event-ID row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="27" t="inlineStr">
+        <is>
+          <t>[P0] FINANCIAL TRUTH PROJECT + AUG 25 FINDINGS — ADDED 2026-08-25   ·   9 items</t>
+        </is>
+      </c>
+      <c r="B203" s="34" t="n"/>
+      <c r="C203" s="34" t="n"/>
+      <c r="D203" s="34" t="n"/>
+      <c r="E203" s="34" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="28" t="inlineStr">
+        <is>
+          <t>[P0] Financial truth phase 1 — backfill the payment ledger from Stripe (all-time)</t>
+        </is>
+      </c>
+      <c r="B204" s="28" t="inlineStr">
+        <is>
+          <t>The database has never held a complete record of money received. 62 payment rows are confirmed missing, and the gap is not a single window: it spans the pre-app era (money collected before this application existed and therefore never written anywhere), the 5 subscribers who were never migrated into the app, and ordinary in-app payments the webhook dropped. Trinity French is the worked case study — $225 paid to Stripe, $0 of it in the ledger — and she is one of 62, not an exception. Every downstream number (MRR, churn, revenue by tier, the financial dashboard, any report built on payments) is computed from this incomplete table, so all of them are wrong by an unknown amount until the ledger is whole.</t>
+        </is>
+      </c>
+      <c r="C204" s="28" t="inlineStr">
+        <is>
+          <t>Backfill from Stripe as the source of truth, all-time, before touching anything downstream. Pull every charge / invoice / payment_intent from account creation forward, match to the person record through the unified resolver, and write the missing rows idempotently keyed on the Stripe object id so a re-run cannot double-post. Cover the three populations explicitly: pre-app-era payments, the 5 unmigrated subscribers, and the 62 confirmed misses. Reconcile the $809 of open invoices in the same pass — $645 is stranded on canceled subscriptions and should be voided, $170 is pre-app era, and only $114 is genuinely collectible. Rehearse the whole backfill on develop and diff the resulting totals against Stripe before running it against prod.</t>
+        </is>
+      </c>
+      <c r="D204" s="28" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E204" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1 of 4. Blocks phases 2-4 and every financial number in the product. Evidence: 62 confirmed missing payment rows; Trinity French $225 paid / $0 recorded; $809 open invoices ($645 to void on canceled subs, $170 pre-app era, $114 real). Backfill must be idempotent — it will be run more than once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="28" t="inlineStr">
+        <is>
+          <t>[P0] Financial truth phase 2 — fix the webhook silent-skip defect + add stripe_payment_intent_id</t>
+        </is>
+      </c>
+      <c r="B205" s="28" t="inlineStr">
+        <is>
+          <t>The Stripe webhook silently skips payments rather than failing loudly, which is why the ledger drifted without anyone noticing: a dropped payment produces no error, no alert and no row, so the only evidence is an absence nobody is looking for. The payments table also has no stripe_payment_intent_id column, so there is no durable key tying a stored row back to the Stripe object it came from — which makes both deduplication and reconciliation guesswork.</t>
+        </is>
+      </c>
+      <c r="C205" s="28" t="inlineStr">
+        <is>
+          <t>Two changes, both prerequisites for the reconciliation in phase 3. (1) Replace every silent skip in the webhook handler with a loud failure: log the Stripe event id, the reason, and alert — never return 200 on an unwritten payment. (2) Add stripe_payment_intent_id to the payments table with a unique index, populate it in the phase 1 backfill, and write it on every new payment. Prove the fix with a Stripe-CLI replay of the exact event shapes that were being skipped, on develop first.</t>
+        </is>
+      </c>
+      <c r="D205" s="28" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E205" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2 of 4. This is the defect that created the hole — fixing it stops the ledger re-diverging the moment phase 1 finishes. The new column is what phase 3 joins on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="28" t="inlineStr">
+        <is>
+          <t>[P0] Financial truth phase 3 — nightly two-way reconciliation with loud mismatch alerts</t>
+        </is>
+      </c>
+      <c r="B206" s="28" t="inlineStr">
+        <is>
+          <t>Once the ledger is whole (phase 1) and the webhook stops dropping rows (phase 2), the remaining risk is silent drift: any future gap between Stripe and the database is invisible until someone audits by hand, which is exactly how 62 rows accumulated. Nothing today compares the two systems on a schedule.</t>
+        </is>
+      </c>
+      <c r="C206" s="28" t="inlineStr">
+        <is>
+          <t>Scheduled nightly job that reconciles in BOTH directions — every Stripe payment must exist in the ledger, and every ledger row must exist in Stripe — joined on stripe_payment_intent_id. Any mismatch alerts loudly (not a log line nobody reads) with the offending ids attached, and surfaces on the admin health dashboard alongside the cron / webhook widgets. Pairs with the Q6 canceled-drift tripwire and the DB/Stripe drift watch rows; consider folding them into one money-drift check rather than three.</t>
+        </is>
+      </c>
+      <c r="D206" s="28" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E206" s="28" t="inlineStr">
+        <is>
+          <t>Phase 3 of 4. Turns 'the numbers are right tonight' into 'the numbers stay right'. Depends on the stripe_payment_intent_id column from phase 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="28" t="inlineStr">
+        <is>
+          <t>[P0] Financial truth phase 4 — rebuild the financial dashboard on the clean ledger</t>
+        </is>
+      </c>
+      <c r="B207" s="28" t="inlineStr">
+        <is>
+          <t>The financial dashboard was built in Lovable on the incomplete payments table and has never been trusted (churn once displayed 2055%). Rebuilding it before the ledger is whole would only re-derive wrong numbers from a wrong source, so it is deliberately sequenced last.</t>
+        </is>
+      </c>
+      <c r="C207" s="28" t="inlineStr">
+        <is>
+          <t>After phases 1-3 land, rebuild MRR, churn and revenue-by-tier directly on the reconciled ledger, then verify each figure against Stripe by hand once before trusting it. Absorbs the existing 'verify the financial dashboard' and 'verify the admin financial data function' rows, and is where the three-bucket collected / projected / churned view should land.</t>
+        </is>
+      </c>
+      <c r="D207" s="28" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E207" s="28" t="inlineStr">
+        <is>
+          <t>Phase 4 of 4. Do NOT start before phase 1 completes — a dashboard on a partial ledger is the current problem, rebuilt. Supersedes the older FINANCIALS verify rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="28" t="inlineStr">
+        <is>
+          <t>Rich Lavner subscription is send_invoice mode — never dunned, $65 open, needs a human decision</t>
+        </is>
+      </c>
+      <c r="B208" s="28" t="inlineStr">
+        <is>
+          <t>Rich Lavner's subscription is set to collection_method = send_invoice rather than charge_automatically. Stripe therefore emails an invoice and waits: no card is charged, no dunning sequence runs, no payment-failure webhook fires, and no past_due state ever appears in the app. He currently sits at $65 open with nothing chasing it, and nothing in the product would have surfaced that — the money is simply not being collected.</t>
+        </is>
+      </c>
+      <c r="C208" s="28" t="inlineStr">
+        <is>
+          <t>Two steps, in order. First a human decision from Adam on the $65 already outstanding (collect, write off, or comp). Then flip the subscription to charge_automatically so it enters normal billing and dunning like every other member. Afterwards, sweep Stripe for any other send_invoice subscriptions — this mode is invisible to every app-side billing state, so a second one would be equally silent.</t>
+        </is>
+      </c>
+      <c r="D208" s="28" t="inlineStr">
+        <is>
+          <t>WAITING ON ADAM</t>
+        </is>
+      </c>
+      <c r="E208" s="28" t="inlineStr">
+        <is>
+          <t>Found during the Aug 25 financial audit. Part of the $809 open-invoice bucket. The real lesson is the class, not the case: send_invoice subscriptions bypass dunning entirely and are invisible to the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="28" t="inlineStr">
+        <is>
+          <t>member_tier invariant hole: an active member can hold a null tier, and the webhook re-creates them</t>
+        </is>
+      </c>
+      <c r="B209" s="28" t="inlineStr">
+        <is>
+          <t>Nothing in the schema forbids the broken state. There is no CHECK constraint and no default preventing an active member from having a null member_tier, the partner member type has no tier mapping at all (so partners are structurally tier-null), and the payment-failure webhook re-creates tier-null rows even after they have been repaired by hand — Andrea's Aug 24 case is the proof that manual repair alone does not hold. Anything that gates on tier (event access, portal views, pricing) behaves unpredictably against a null.</t>
+        </is>
+      </c>
+      <c r="C209" s="28" t="inlineStr">
+        <is>
+          <t>Close the hole at the database level rather than by repeated repair. Decide the correct tier for the partner type first (it needs a real mapping, not a null), then add a CHECK constraint or default that makes 'active with null tier' unrepresentable, and fix the payment-failure webhook path so it preserves the existing tier instead of writing a row without one. Repair the outstanding rows in the same pass and re-check after the next real payment failure. Follow the incremental CHECK-constraint approach already agreed on the enums row — one table, carefully, not a schema-wide sweep.</t>
+        </is>
+      </c>
+      <c r="D209" s="28" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E209" s="28" t="inlineStr">
+        <is>
+          <t>Aug 25: the 3+1 tier repairs were done tonight, but they are repairs, not a fix — the webhook will re-create tier-null rows until the write path and the constraint both change. Partner-type mapping is the open decision inside this row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="28" t="inlineStr">
+        <is>
+          <t>hubs.created_by is NOT NULL ON DELETE CASCADE — deleting a creator profile destroys their hubs</t>
+        </is>
+      </c>
+      <c r="B210" s="28" t="inlineStr">
+        <is>
+          <t>The hubs.created_by foreign key is NOT NULL with ON DELETE CASCADE, so hard-deleting a profile deletes every hub that person created and everything those hubs contain. This is a live footgun on any exit or cleanup workstream: an ordinary-looking profile delete silently takes member-facing content with it, and there is nothing in the admin UI that warns about it.</t>
+        </is>
+      </c>
+      <c r="C210" s="28" t="inlineStr">
+        <is>
+          <t>Change the cascade to something survivable: make created_by nullable with ON DELETE SET NULL, or repoint deleted creators to an organisation-owned system account, so hubs outlive the person who made them. Until that lands, treat any profile hard-delete as a two-step operation — audit owned content first (the read-first footprint audit already used on member removals), reassign or purge deliberately, then delete.</t>
+        </is>
+      </c>
+      <c r="D210" s="28" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E210" s="28" t="inlineStr">
+        <is>
+          <t>Aug 25: surfaced while purging Josh's hubs — the purge was done deliberately for that reason rather than by deleting the profile. Same class as the bulk-delete atomicity row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="28" t="inlineStr">
+        <is>
+          <t>Retention watch: 7 members exiting by Sep 13 — $287/mo MRR at risk</t>
+        </is>
+      </c>
+      <c r="B211" s="28" t="inlineStr">
+        <is>
+          <t>Seven members are on track to exit by Sep 13, representing $287 per month of recurring revenue. Recorded as a dated watch so the number is tracked deliberately rather than discovered in a month-end total.</t>
+        </is>
+      </c>
+      <c r="C211" s="28" t="inlineStr">
+        <is>
+          <t>Track through Sep 13. Decide per member whether anything is worth doing (conversation, offer, pause instead of cancel) before the exits land, and confirm the actual outcome against this figure afterwards. Feeds the member-cancellation retention flow row — that build should be scoped by what these seven actually say.</t>
+        </is>
+      </c>
+      <c r="D211" s="28" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+      <c r="E211" s="28" t="inlineStr">
+        <is>
+          <t>Time-boxed: this row closes after Sep 13, either as a recorded loss or as retained members. $287/mo across 7 members. Note the financial figures here come from Stripe, not from the ledger the financial-truth project is fixing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="28" t="inlineStr">
+        <is>
+          <t>Members-by-type admin view — spec discussion in progress, build pending Adam's five answers</t>
+        </is>
+      </c>
+      <c r="B212" s="28" t="inlineStr">
+        <is>
+          <t>An admin view of members broken out by type. The spec conversation with Adam is underway but not finished: five questions remain open, and the build is deliberately not started until they are answered, so that the view is built once against a settled definition rather than reworked.</t>
+        </is>
+      </c>
+      <c r="C212" s="28" t="inlineStr">
+        <is>
+          <t>Finish the spec discussion with Adam and capture the five answers here, then build. Reuse the canonical person record and the existing member-type vocabulary rather than inventing a parallel definition — the same classification that the member_counts view and the directory work already use.</t>
+        </is>
+      </c>
+      <c r="D212" s="28" t="inlineStr">
+        <is>
+          <t>WAITING ON ADAM: five answers</t>
+        </is>
+      </c>
+      <c r="E212" s="28" t="inlineStr">
+        <is>
+          <t>Spec in progress as of Aug 25. Build is intentionally blocked, not forgotten. Related to the unified admin users view and the member directory rows.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(tracker): financial truth project + tonight's repairs (note corrections)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -4172,7 +4172,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>NOT on the build sheet — exit workstream. Recorded here for completeness. Aug 25: Josh hub purge done — the hubs he created were removed deliberately rather than left to a profile delete, which would have cascaded (see the hubs.created_by row). Closes the owned-content residue of the exit.</t>
+          <t>NOT on the build sheet — exit workstream. Recorded here for completeness. Aug 25: Josh hub purge DONE - his 4 remaining hub_members rows (one per hub, all joined 2026-05-21 03:11:32, all added by Adam) were deleted; verified afterwards at 0 hub memberships, 0 posts, 0 comments, 0 likes, 0 resources. CORRECTION to an earlier wording of this note: Josh created NO hubs. All four hubs are created_by Adam, so nothing was owned by him and the purge was membership rows only - the cascade risk on hubs.created_by is a separate finding about Adam's profile (see that row). Also noted while verifying: the hub display queries in dashboard/hubs/[id] and admin/hubs join profiles without a deleted_at filter, which is why his soft-deleted profile kept rendering and inflated each hub's member count by one. Closes the hub residue of the exit.</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Adam noted more member changes coming next session. Aug 25: Audrey converted to non-member — done, and recorded here as the next entry in this running member-status record.</t>
+          <t>Adam noted more member changes coming next session. Aug 25: Audrey Handleton converted to non-member - DONE, and recorded here as the next entry in this running member-status record. Verified end state: profiles reads non_member / inactive / membership_override false; the people row reads roles ['prospect'] with member_tier and member_status both null (never-was, not canceled). She was a comp who had drifted - profile said social while her people row still said business - and she never paid a cent, so there was no Stripe side to cancel.</t>
         </is>
       </c>
     </row>
@@ -5334,7 +5334,7 @@
       </c>
       <c r="E199" s="28" t="inlineStr">
         <is>
-          <t>Labeled during the Aug 19 status pass and deliberately left unmerged. Six rows, two humans. Folds naturally into the contacts fold (6B-6E).</t>
+          <t>Labeled during the Aug 19 status pass and deliberately left unmerged. Six rows, two humans. Folds naturally into the contacts fold (6B-6E). 2026-08-25: Josh's 4 hub_members rows were purged on the primary identity (a5f1b294) only; both duplicate rows held zero hub memberships, so that cleanup did not depend on this adjudication and does not constrain it.</t>
         </is>
       </c>
     </row>
@@ -5588,7 +5588,7 @@
       </c>
       <c r="E209" s="28" t="inlineStr">
         <is>
-          <t>Aug 25: the 3+1 tier repairs were done tonight, but they are repairs, not a fix — the webhook will re-create tier-null rows until the write path and the constraint both change. Partner-type mapping is the open decision inside this row.</t>
+          <t>Aug 25: the 3+1 tier repairs were done tonight, but they are repairs, not a fix — the webhook will re-create tier-null rows until the write path and the constraint both change. Partner-type mapping is the open decision inside this row. Verified end state 2026-08-25: Jacob Cohen, JD Davis and Vaishali Willis all read member_tier 'social'; Andrea Baquero's row reads social too (updated 20:19:51 UTC) but she is still past_due, so the Stripe retry did not clear the money. 13 people rows holding a member role still carry a null tier, and exactly ONE of those is active - partnertest@704collective.com - which is the partner-type mapping hole above rather than a missed repair.</t>
         </is>
       </c>
     </row>
@@ -5615,7 +5615,7 @@
       </c>
       <c r="E210" s="28" t="inlineStr">
         <is>
-          <t>Aug 25: surfaced while purging Josh's hubs — the purge was done deliberately for that reason rather than by deleting the profile. Same class as the bulk-delete atomicity row.</t>
+          <t>Aug 25: surfaced during the Josh hub-membership cleanup forensics, not because Josh owned anything - he created zero hubs. All four hubs (The Arrival, Business Founders, Eats &amp; Experiences, The Wellness) are created_by Adam, so the whole Network content structure hangs off one profile row and that is where the exposure sits. Soft deletes are safe; the hard-delete path (admin-delete-user, manual profile delete) is the footgun. Same class as the bulk-delete atomicity row.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: tracker true-up 3 + social_only_scope v2 capture
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
+++ b/docs/704_Collective___Internal_Tracker__Phase_1___Phase_2___UPDATED_2026-08-03.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E212"/>
+  <dimension ref="A1:E216"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="1" min="1" max="1"/>
@@ -846,7 +846,7 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Now identity Wave 9 (tickets), queued behind the contacts fold (6B-6E) and the auth cutover (8); resumes Aug 28. Still do not drop before the soak confirms nothing else reads them. Closes together with the capacity-trigger split-brain row.</t>
+          <t>Now identity Wave 9 (tickets), queued behind the contacts fold (6B-6E) and the auth cutover (8); resumes Aug 28. Still do not drop before the soak confirms nothing else reads them. Closes together with the capacity-trigger split-brain row. Wave 9 recon Aug 25: create-guest-pass writes legacy tickets PRIMARY; dashboard guest-pass list + get_community_stats (frozen 416 since Jul 19 vs live 969) read legacy; capacity trigger pair mapped; retirement order + mandatory backfill (8 of 26 mirrored).</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4556,7 @@
       </c>
       <c r="E169" s="8" t="inlineStr">
         <is>
-          <t>The admin_override bypass now spans both trigger families; the underlying counting split remains until tickets is retired. Closes with identity Wave 9 (tickets); resumes Aug 28.</t>
+          <t>The admin_override bypass now spans both trigger families; the underlying counting split remains until tickets is retired. Closes with identity Wave 9 (tickets); resumes Aug 28. Wave 9 recon Aug 25: create-guest-pass writes legacy tickets PRIMARY; dashboard guest-pass list + get_community_stats (frozen 416 since Jul 19 vs live 969) read legacy; capacity trigger pair mapped; retirement order + mandatory backfill (8 of 26 mirrored).</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="E200" s="28" t="inlineStr">
         <is>
-          <t>Time-boxed: this row closes after the Aug 27 Exchange, either resolved or converted into an ordinary billing follow-up. Aug 25: the 3+1 member_tier repairs done tonight included the tier-null row the payment-failure webhook re-created on this account Aug 24 — see the member_tier invariant row. The past_due watch itself still stands through Aug 27.</t>
+          <t>Time-boxed: this row closes after the Aug 27 Exchange, either resolved or converted into an ordinary billing follow-up. Aug 25: the 3+1 member_tier repairs done tonight included the tier-null row the payment-failure webhook re-created on this account Aug 24 — see the member_tier invariant row. The past_due watch itself still stands through Aug 27. Aug 26: RESOLVED to watch-only — billing email sent Aug 26; card in Stripe auto-retry; attends Aug 27 event; Adam reports ~2 attended events never captured at check-in.</t>
         </is>
       </c>
     </row>
@@ -5422,13 +5422,17 @@
     <row r="203">
       <c r="A203" s="27" t="inlineStr">
         <is>
-          <t>[P0] FINANCIAL TRUTH PROJECT + AUG 25 FINDINGS — ADDED 2026-08-25   ·   9 items</t>
+          <t>[P0] FINANCIAL TRUTH PROJECT + AUG 25 FINDINGS — ADDED 2026-08-25   ·   8 items</t>
         </is>
       </c>
       <c r="B203" s="34" t="n"/>
       <c r="C203" s="34" t="n"/>
       <c r="D203" s="34" t="n"/>
-      <c r="E203" s="34" t="n"/>
+      <c r="E203" s="34" t="inlineStr">
+        <is>
+          <t>Requirement: journal invoice.voided (Stripe currently sole truth on voids, Rich case Aug 26).</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="28" t="inlineStr">
@@ -5541,44 +5545,44 @@
     <row r="208">
       <c r="A208" s="28" t="inlineStr">
         <is>
-          <t>Rich Lavner subscription is send_invoice mode — never dunned, $65 open, needs a human decision</t>
+          <t>member_tier invariant hole: an active member can hold a null tier, and the webhook re-creates them</t>
         </is>
       </c>
       <c r="B208" s="28" t="inlineStr">
         <is>
-          <t>Rich Lavner's subscription is set to collection_method = send_invoice rather than charge_automatically. Stripe therefore emails an invoice and waits: no card is charged, no dunning sequence runs, no payment-failure webhook fires, and no past_due state ever appears in the app. He currently sits at $65 open with nothing chasing it, and nothing in the product would have surfaced that — the money is simply not being collected.</t>
+          <t>Nothing in the schema forbids the broken state. There is no CHECK constraint and no default preventing an active member from having a null member_tier, the partner member type has no tier mapping at all (so partners are structurally tier-null), and the payment-failure webhook re-creates tier-null rows even after they have been repaired by hand — Andrea's Aug 24 case is the proof that manual repair alone does not hold. Anything that gates on tier (event access, portal views, pricing) behaves unpredictably against a null.</t>
         </is>
       </c>
       <c r="C208" s="28" t="inlineStr">
         <is>
-          <t>Two steps, in order. First a human decision from Adam on the $65 already outstanding (collect, write off, or comp). Then flip the subscription to charge_automatically so it enters normal billing and dunning like every other member. Afterwards, sweep Stripe for any other send_invoice subscriptions — this mode is invisible to every app-side billing state, so a second one would be equally silent.</t>
+          <t>Close the hole at the database level rather than by repeated repair. Decide the correct tier for the partner type first (it needs a real mapping, not a null), then add a CHECK constraint or default that makes 'active with null tier' unrepresentable, and fix the payment-failure webhook path so it preserves the existing tier instead of writing a row without one. Repair the outstanding rows in the same pass and re-check after the next real payment failure. Follow the incremental CHECK-constraint approach already agreed on the enums row — one table, carefully, not a schema-wide sweep.</t>
         </is>
       </c>
       <c r="D208" s="28" t="inlineStr">
         <is>
-          <t>WAITING ON ADAM</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="E208" s="28" t="inlineStr">
         <is>
-          <t>Found during the Aug 25 financial audit. Part of the $809 open-invoice bucket. The real lesson is the class, not the case: send_invoice subscriptions bypass dunning entirely and are invisible to the app.</t>
+          <t>Aug 25: the 3+1 tier repairs were done tonight, but they are repairs, not a fix — the webhook will re-create tier-null rows until the write path and the constraint both change. Partner-type mapping is the open decision inside this row. Verified end state 2026-08-25: Jacob Cohen, JD Davis and Vaishali Willis all read member_tier 'social'; Andrea Baquero's row reads social too (updated 20:19:51 UTC) but she is still past_due, so the Stripe retry did not clear the money. 13 people rows holding a member role still carry a null tier, and exactly ONE of those is active - partnertest@704collective.com - which is the partner-type mapping hole above rather than a missed repair. ~20 people rows carry member role with null status; partnertest maps to no tier; normalize during invariant fix.</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="28" t="inlineStr">
         <is>
-          <t>member_tier invariant hole: an active member can hold a null tier, and the webhook re-creates them</t>
+          <t>hubs.created_by is NOT NULL ON DELETE CASCADE — deleting a creator profile destroys their hubs</t>
         </is>
       </c>
       <c r="B209" s="28" t="inlineStr">
         <is>
-          <t>Nothing in the schema forbids the broken state. There is no CHECK constraint and no default preventing an active member from having a null member_tier, the partner member type has no tier mapping at all (so partners are structurally tier-null), and the payment-failure webhook re-creates tier-null rows even after they have been repaired by hand — Andrea's Aug 24 case is the proof that manual repair alone does not hold. Anything that gates on tier (event access, portal views, pricing) behaves unpredictably against a null.</t>
+          <t>The hubs.created_by foreign key is NOT NULL with ON DELETE CASCADE, so hard-deleting a profile deletes every hub that person created and everything those hubs contain. This is a live footgun on any exit or cleanup workstream: an ordinary-looking profile delete silently takes member-facing content with it, and there is nothing in the admin UI that warns about it.</t>
         </is>
       </c>
       <c r="C209" s="28" t="inlineStr">
         <is>
-          <t>Close the hole at the database level rather than by repeated repair. Decide the correct tier for the partner type first (it needs a real mapping, not a null), then add a CHECK constraint or default that makes 'active with null tier' unrepresentable, and fix the payment-failure webhook path so it preserves the existing tier instead of writing a row without one. Repair the outstanding rows in the same pass and re-check after the next real payment failure. Follow the incremental CHECK-constraint approach already agreed on the enums row — one table, carefully, not a schema-wide sweep.</t>
+          <t>Change the cascade to something survivable: make created_by nullable with ON DELETE SET NULL, or repoint deleted creators to an organisation-owned system account, so hubs outlive the person who made them. Until that lands, treat any profile hard-delete as a two-step operation — audit owned content first (the read-first footprint audit already used on member removals), reassign or purge deliberately, then delete.</t>
         </is>
       </c>
       <c r="D209" s="28" t="inlineStr">
@@ -5588,88 +5592,180 @@
       </c>
       <c r="E209" s="28" t="inlineStr">
         <is>
-          <t>Aug 25: the 3+1 tier repairs were done tonight, but they are repairs, not a fix — the webhook will re-create tier-null rows until the write path and the constraint both change. Partner-type mapping is the open decision inside this row. Verified end state 2026-08-25: Jacob Cohen, JD Davis and Vaishali Willis all read member_tier 'social'; Andrea Baquero's row reads social too (updated 20:19:51 UTC) but she is still past_due, so the Stripe retry did not clear the money. 13 people rows holding a member role still carry a null tier, and exactly ONE of those is active - partnertest@704collective.com - which is the partner-type mapping hole above rather than a missed repair.</t>
+          <t>Aug 25: surfaced during the Josh hub-membership cleanup forensics, not because Josh owned anything - he created zero hubs. All four hubs (The Arrival, Business Founders, Eats &amp; Experiences, The Wellness) are created_by Adam, so the whole Network content structure hangs off one profile row and that is where the exposure sits. Soft deletes are safe; the hard-delete path (admin-delete-user, manual profile delete) is the footgun. Same class as the bulk-delete atomicity row.</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="28" t="inlineStr">
         <is>
-          <t>hubs.created_by is NOT NULL ON DELETE CASCADE — deleting a creator profile destroys their hubs</t>
+          <t>Retention watch: 7 members exiting by Sep 13 — $287/mo MRR at risk</t>
         </is>
       </c>
       <c r="B210" s="28" t="inlineStr">
         <is>
-          <t>The hubs.created_by foreign key is NOT NULL with ON DELETE CASCADE, so hard-deleting a profile deletes every hub that person created and everything those hubs contain. This is a live footgun on any exit or cleanup workstream: an ordinary-looking profile delete silently takes member-facing content with it, and there is nothing in the admin UI that warns about it.</t>
+          <t>Seven members are on track to exit by Sep 13, representing $287 per month of recurring revenue. Recorded as a dated watch so the number is tracked deliberately rather than discovered in a month-end total.</t>
         </is>
       </c>
       <c r="C210" s="28" t="inlineStr">
         <is>
-          <t>Change the cascade to something survivable: make created_by nullable with ON DELETE SET NULL, or repoint deleted creators to an organisation-owned system account, so hubs outlive the person who made them. Until that lands, treat any profile hard-delete as a two-step operation — audit owned content first (the read-first footprint audit already used on member removals), reassign or purge deliberately, then delete.</t>
+          <t>Track through Sep 13. Decide per member whether anything is worth doing (conversation, offer, pause instead of cancel) before the exits land, and confirm the actual outcome against this figure afterwards. Feeds the member-cancellation retention flow row — that build should be scoped by what these seven actually say.</t>
         </is>
       </c>
       <c r="D210" s="28" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="E210" s="28" t="inlineStr">
         <is>
-          <t>Aug 25: surfaced during the Josh hub-membership cleanup forensics, not because Josh owned anything - he created zero hubs. All four hubs (The Arrival, Business Founders, Eats &amp; Experiences, The Wellness) are created_by Adam, so the whole Network content structure hangs off one profile row and that is where the exposure sits. Soft deletes are safe; the hard-delete path (admin-delete-user, manual profile delete) is the footgun. Same class as the bulk-delete atomicity row.</t>
+          <t>Time-boxed: this row closes after Sep 13, either as a recorded loss or as retained members. $287/mo across 7 members. Note the financial figures here come from Stripe, not from the ledger the financial-truth project is fixing.</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="28" t="inlineStr">
         <is>
-          <t>Retention watch: 7 members exiting by Sep 13 — $287/mo MRR at risk</t>
+          <t>Members-by-type admin view — spec discussion in progress, build pending Adam's five answers</t>
         </is>
       </c>
       <c r="B211" s="28" t="inlineStr">
         <is>
-          <t>Seven members are on track to exit by Sep 13, representing $287 per month of recurring revenue. Recorded as a dated watch so the number is tracked deliberately rather than discovered in a month-end total.</t>
+          <t>An admin view of members broken out by type. The spec conversation with Adam is underway but not finished: five questions remain open, and the build is deliberately not started until they are answered, so that the view is built once against a settled definition rather than reworked.</t>
         </is>
       </c>
       <c r="C211" s="28" t="inlineStr">
         <is>
-          <t>Track through Sep 13. Decide per member whether anything is worth doing (conversation, offer, pause instead of cancel) before the exits land, and confirm the actual outcome against this figure afterwards. Feeds the member-cancellation retention flow row — that build should be scoped by what these seven actually say.</t>
+          <t>Finish the spec discussion with Adam and capture the five answers here, then build. Reuse the canonical person record and the existing member-type vocabulary rather than inventing a parallel definition — the same classification that the member_counts view and the directory work already use.</t>
         </is>
       </c>
       <c r="D211" s="28" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>WAITING ON ADAM: five answers</t>
         </is>
       </c>
       <c r="E211" s="28" t="inlineStr">
         <is>
-          <t>Time-boxed: this row closes after Sep 13, either as a recorded loss or as retained members. $287/mo across 7 members. Note the financial figures here come from Stripe, not from the ledger the financial-truth project is fixing.</t>
+          <t>Spec in progress as of Aug 25. Build is intentionally blocked, not forgotten. Related to the unified admin users view and the member directory rows.</t>
         </is>
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="28" t="inlineStr">
-        <is>
-          <t>Members-by-type admin view — spec discussion in progress, build pending Adam's five answers</t>
-        </is>
-      </c>
-      <c r="B212" s="28" t="inlineStr">
-        <is>
-          <t>An admin view of members broken out by type. The spec conversation with Adam is underway but not finished: five questions remain open, and the build is deliberately not started until they are answered, so that the view is built once against a settled definition rather than reworked.</t>
-        </is>
-      </c>
-      <c r="C212" s="28" t="inlineStr">
-        <is>
-          <t>Finish the spec discussion with Adam and capture the five answers here, then build. Reuse the canonical person record and the existing member-type vocabulary rather than inventing a parallel definition — the same classification that the member_counts view and the directory work already use.</t>
-        </is>
-      </c>
-      <c r="D212" s="28" t="inlineStr">
-        <is>
-          <t>WAITING ON ADAM: five answers</t>
-        </is>
-      </c>
-      <c r="E212" s="28" t="inlineStr">
-        <is>
-          <t>Spec in progress as of Aug 25. Build is intentionally blocked, not forgotten. Related to the unified admin users view and the member directory rows.</t>
+      <c r="A212" s="27" t="inlineStr">
+        <is>
+          <t>AUG 26 FINDINGS — ADDED 2026-08-26   ·   4 items</t>
+        </is>
+      </c>
+      <c r="B212" s="34" t="n"/>
+      <c r="C212" s="34" t="n"/>
+      <c r="D212" s="34" t="n"/>
+      <c r="E212" s="34" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="28" t="inlineStr">
+        <is>
+          <t>Attendance undercount is systemic — door discipline, not a data bug</t>
+        </is>
+      </c>
+      <c r="B213" s="28" t="inlineStr">
+        <is>
+          <t>Attendance is only ever as true as the door. Adam reports roughly two events Andrea Baquero attended that were never captured at check-in, and the same gap exists for anyone scanned inconsistently. This is not a reporting defect: the records are never written at all, so every downstream number that rests on attendance is quietly low and nothing signals it. It is event-critical for the Exchange specifically, because the mixer roster is built from check-ins — an uncaptured arrival is a person the engine will never seat.</t>
+        </is>
+      </c>
+      <c r="C213" s="28" t="inlineStr">
+        <is>
+          <t>Treat as an operations fix first, not a code fix. Add an explicit check-in line to the run-of-show for the Aug 27 Exchange so every arrival is scanned or recorded by hand, then measure that night's capture against the known headcount. Only if capture is still short does this become an instrumentation problem in the door path. Backfilling historical attendance is a separate decision, and not worth making until live capture is trustworthy.</t>
+        </is>
+      </c>
+      <c r="D213" s="28" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E213" s="28" t="inlineStr">
+        <is>
+          <t>Raised Aug 26 from the Andrea Baquero case (~2 attended events never captured). Immediate lever is the Aug 27 run-of-show line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="28" t="inlineStr">
+        <is>
+          <t>Hub add-member search still surfaces banned business members</t>
+        </is>
+      </c>
+      <c r="B214" s="28" t="inlineStr">
+        <is>
+          <t>The add-member search on /admin/hubs was narrowed Aug 26 to active business members with is_internal false, but banned was deliberately left out of the filter set. A banned business member with an active subscription therefore still appears in the search and can still be added to a hub. The member-facing hub tab hides them correctly, so the effect is an invisible member occupying a row rather than a data leak.</t>
+        </is>
+      </c>
+      <c r="C214" s="28" t="inlineStr">
+        <is>
+          <t>One line in the add-member search query: .eq('banned', false), alongside the existing deleted_at, member_type and is_internal filters. Same rehearsal shape as the Aug 26 hub work — seed a banned business member, confirm it is absent from the search, and confirm the member-facing tab is unchanged.</t>
+        </is>
+      </c>
+      <c r="D214" s="28" t="inlineStr">
+        <is>
+          <t>WAITING ON ADAM</t>
+        </is>
+      </c>
+      <c r="E214" s="28" t="inlineStr">
+        <is>
+          <t>Left open on purpose Aug 26: the shipped scope named member_type and is_internal only, so the gap was reported rather than silently widened. One-line change whenever Adam approves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="28" t="inlineStr">
+        <is>
+          <t>Email logo still partially inverts in Gmail dark mode</t>
+        </is>
+      </c>
+      <c r="B215" s="28" t="inlineStr">
+        <is>
+          <t>The member blast logo was changed Aug 26 from the white-on-dark mark to the circular badge on an opaque white circle. That fixed the logo disappearing entirely and was render-verified for contrast in both light and dark-emulated views. In real Gmail, dark-mode inversion still partially affects the surrounding shell, so the badge is legible but the treatment is an improvement rather than a complete answer.</t>
+        </is>
+      </c>
+      <c r="C215" s="28" t="inlineStr">
+        <is>
+          <t>Next lever is a dark-mode-aware CSS asset: prefers-color-scheme rules plus explicit background locks on the shell, and where Gmail ignores those, a pre-composited image asset that cannot be inverted. Verify against a real Gmail dark-mode client, not only an emulated render — the emulated view is what passed while the real client still differed.</t>
+        </is>
+      </c>
+      <c r="D215" s="28" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E215" s="28" t="inlineStr">
+        <is>
+          <t>Badge shipped Aug 26 and is legible; this row covers the remaining shell inversion. Cosmetic and low urgency, but it touches every member-facing send.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="28" t="inlineStr">
+        <is>
+          <t>Sentry: "load" error thrown on /dashboard (~Aug 24), undiagnosed</t>
+        </is>
+      </c>
+      <c r="B216" s="28" t="inlineStr">
+        <is>
+          <t>Sentry reports an error on the member dashboard in which a Supabase error object appears to be thrown rather than handled, surfacing with the message "load". It first appears around Aug 24. Nothing else is known — frequency, affected users, and whether the page actually degrades are all unread, because the issue detail has not been opened.</t>
+        </is>
+      </c>
+      <c r="C216" s="28" t="inlineStr">
+        <is>
+          <t>Blocked on evidence, not on effort. Adam sends the Sentry issue-detail screenshot (stack, breadcrumbs, event count, affected users) and diagnosis follows from there. Likely shape is an unchecked Supabase call whose error object is thrown as-is, which is why the message reads as the object rather than a cause — but that is a guess until the throw site is visible.</t>
+        </is>
+      </c>
+      <c r="D216" s="28" t="inlineStr">
+        <is>
+          <t>WAITING ON ADAM: issue-detail screenshot</t>
+        </is>
+      </c>
+      <c r="E216" s="28" t="inlineStr">
+        <is>
+          <t>Raised Aug 26. Cannot be triaged from the title alone; the throw site is what identifies it. First seen ~Aug 24.</t>
         </is>
       </c>
     </row>

</xml_diff>